<commit_message>
Aba Vídeos: ranking do YouTube, busca nas transcrições e vídeos de referência no FAQ e guias
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/times.xlsx
+++ b/times.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="312">
   <si>
     <t>GUIA DE ROTAÇÃO &amp; METAGAME - POKEALLIANCE(PKA)</t>
   </si>
@@ -22,58 +22,22 @@
     <t>RECOMENDAÇÃO DE TIME PARA HUNTS!</t>
   </si>
   <si>
+    <t>GUIA VISUAL DE HUNT: CARDS - ELEMENTOS</t>
+  </si>
+  <si>
+    <t>GUIA RÁPIDO</t>
+  </si>
+  <si>
     <t>Requisitos de Entrada e Progressão 2x2x2.</t>
   </si>
   <si>
     <t>https://www.twitch.tv/safnaww</t>
   </si>
   <si>
-    <t>📌 REQUISITOS INICIAIS (START DE ROTAÇÃO)</t>
-  </si>
-  <si>
-    <t>GUIA RÁPIDO</t>
-  </si>
-  <si>
-    <t>GUIA VISUAL DE HUNT: CARDS - ELEMENTOS</t>
-  </si>
-  <si>
-    <t>⚡ UPGRADE: ROTAÇÃO 2x2x2</t>
-  </si>
-  <si>
-    <t>Nível &amp; Held:</t>
-  </si>
-  <si>
-    <t>Todos os Pokémon +15 com Atk 4</t>
-  </si>
-  <si>
-    <t>Todos os Pokémon +25 com Atk 5</t>
-  </si>
-  <si>
-    <t>Atalho / Dica:</t>
-  </si>
-  <si>
-    <t>Runas de Atk no Pokelog ajudam a adiantar a meta</t>
-  </si>
-  <si>
-    <t>Estrelas Mínimas:</t>
-  </si>
-  <si>
     <t>Com algumas exceções, todos os restantes são SHINYS.</t>
   </si>
   <si>
-    <t>Tier 1: 2★ (estrelas)  |  SR: 1★ (estrela)</t>
-  </si>
-  <si>
-    <t>Meta no Dummy:</t>
-  </si>
-  <si>
-    <t>★ METAGROSS</t>
-  </si>
-  <si>
-    <t>Bater 560k de dano com 3 Pokémon</t>
-  </si>
-  <si>
-    <t>Bater 560k de dano com apenas 2 Pokémon</t>
+    <t>Segue lá!</t>
   </si>
   <si>
     <r>
@@ -97,604 +61,679 @@
     </r>
   </si>
   <si>
+    <t>★ METAGROSS</t>
+  </si>
+  <si>
+    <t>ELEMENTO / HUNT</t>
+  </si>
+  <si>
+    <t>ALVO (HUNT)</t>
+  </si>
+  <si>
+    <t>🛡️ LURAR (T1)</t>
+  </si>
+  <si>
+    <t>⚔️ DPS (SR)</t>
+  </si>
+  <si>
+    <t>🎨 TIPO SMEARGLE</t>
+  </si>
+  <si>
+    <t>Bug</t>
+  </si>
+  <si>
+    <t>📌 REQUISITOS INICIAIS (START DE ROTAÇÃO)</t>
+  </si>
+  <si>
+    <t>★ LUCARIO</t>
+  </si>
+  <si>
+    <t>★ GENGAR</t>
+  </si>
+  <si>
+    <t>⚡ UPGRADE: ROTAÇÃO 2x2x2</t>
+  </si>
+  <si>
+    <t>Nessa planilha não indicaremos pokémons T2 ou T3 para a rotação.</t>
+  </si>
+  <si>
+    <t>Nível &amp; Held:</t>
+  </si>
+  <si>
+    <t>Em breve</t>
+  </si>
+  <si>
+    <t>★ BUG</t>
+  </si>
+  <si>
+    <t>Hunt: Steel / Psychic</t>
+  </si>
+  <si>
+    <t>Todos os Pokémon +15 com Atk 4</t>
+  </si>
+  <si>
+    <t>★ FAIRY</t>
+  </si>
+  <si>
+    <t>Rapidash, Typhlosion, Magcargo</t>
+  </si>
+  <si>
+    <t>★ FIRE</t>
+  </si>
+  <si>
+    <t>Hunt: Fighting / Steel</t>
+  </si>
+  <si>
+    <t>Hunt: Ghost / Poison</t>
+  </si>
+  <si>
+    <t>Todos os Pokémon +25 com Atk 5</t>
+  </si>
+  <si>
+    <t>Atalho / Dica:</t>
+  </si>
+  <si>
+    <t>Arcanine, Infernape, Armaldo</t>
+  </si>
+  <si>
+    <t>Runas de Atk no Pokelog ajudam a adiantar a meta</t>
+  </si>
+  <si>
+    <t>🛡️ LURAR / TANQUE (T1)</t>
+  </si>
+  <si>
+    <t>Hunt: Em breve</t>
+  </si>
+  <si>
+    <t>Fire, Rock</t>
+  </si>
+  <si>
+    <t>Fairy</t>
+  </si>
+  <si>
+    <t>Hunt: Shiny Sylveon (Lendário)</t>
+  </si>
+  <si>
+    <t>Hunt: Magmar (Lendário) / Torkoal (UR)</t>
+  </si>
+  <si>
+    <t>Estrelas Mínimas:</t>
+  </si>
+  <si>
+    <t>Tier 1: 2★ (estrelas)  |  SR: 1★ (estrela)</t>
+  </si>
+  <si>
+    <t>Meta no Dummy:</t>
+  </si>
+  <si>
+    <t>Bater 560k de dano com 3 Pokémon</t>
+  </si>
+  <si>
+    <t>⚔️ DPS / DANO (SR)</t>
+  </si>
+  <si>
+    <t>Shiny Sylveon (Lendário)</t>
+  </si>
+  <si>
+    <t>Bater 560k de dano com apenas 2 Pokémon</t>
+  </si>
+  <si>
     <t>Regra de Prey:</t>
   </si>
   <si>
+    <t>⭐ S.Rapidash, S.Typhlosion, S.Steelix</t>
+  </si>
+  <si>
     <t>Obrigatório Prey de Atk na hunt (já calculada no dummy)</t>
   </si>
   <si>
     <t>Manter sempre Prey de Atk ativa na hunt</t>
   </si>
   <si>
-    <t>★ LUCARIO</t>
-  </si>
-  <si>
     <t>💡 POR QUE COMPOSIÇÕES COM 2 A 3 ELEMENTOS SÃO SUPERIORES? (ANTI-MONO)</t>
   </si>
   <si>
-    <t>★ GENGAR</t>
-  </si>
-  <si>
-    <t>Hunt: Steel / Psychic</t>
-  </si>
-  <si>
-    <t>ELEMENTO / HUNT</t>
+    <t>Muk, Tentacruel, Mawile</t>
+  </si>
+  <si>
+    <t>Aggron, Skarmory, Toxicroak</t>
   </si>
   <si>
     <t>⏱️ Cooldown Reduzido por Tier</t>
   </si>
   <si>
-    <t>Hunt: Fighting / Steel</t>
-  </si>
-  <si>
-    <t>ALVO (HUNT)</t>
-  </si>
-  <si>
-    <t>Hunt: Ghost / Poison</t>
-  </si>
-  <si>
-    <t>🛡️ LURAR / TANQUE (T1)</t>
-  </si>
-  <si>
-    <t>Nessa planilha não indicaremos pokémons T2 ou T3 para a rotação.</t>
-  </si>
-  <si>
-    <t>⚔️ DPS / DANO (SR)</t>
+    <t>Poison, Metal</t>
+  </si>
+  <si>
+    <t>⭐ Arcanine, Houndoom, Pupitar</t>
+  </si>
+  <si>
+    <t>⭐S.Rapidash, S.Typhlosion, S.Magcargo</t>
+  </si>
+  <si>
+    <t>⭐ Arcanine, Infernape, Armaldo</t>
+  </si>
+  <si>
+    <t>⭐ Muk, Tentacruel, Mawile</t>
+  </si>
+  <si>
+    <t>Fire</t>
+  </si>
+  <si>
+    <t>Magmar (Lendário) / Torkoal (UR)</t>
+  </si>
+  <si>
+    <t>Blastoise, Feraligatr, Omastar</t>
+  </si>
+  <si>
+    <t>Pupitar, Torterra, Kingdra</t>
+  </si>
+  <si>
+    <t>Rock, Water, Ground</t>
+  </si>
+  <si>
+    <t>Fighting</t>
   </si>
   <si>
     <t>No PKA, tiers mais altos não dão só dano: reduzem o cooldown das skills, deixando a rotação muito mais rápida.</t>
   </si>
   <si>
-    <t>★ BUG</t>
-  </si>
-  <si>
-    <t>⭐ S.Rapidash, S.Typhlosion, S.Steelix</t>
-  </si>
-  <si>
-    <t>🛡️ LURAR (T1)</t>
-  </si>
-  <si>
-    <t>⚔️ DPS (SR)</t>
-  </si>
-  <si>
-    <t>🎨 TIPO SMEARGLE</t>
-  </si>
-  <si>
-    <t>Bug</t>
+    <t>Mega Clefable, Pidgeot, Espeon</t>
+  </si>
+  <si>
+    <t>Wobbuffet, Mimikyu, Gliscor</t>
+  </si>
+  <si>
+    <t>⭐ Hitmontop, Typhlosion, Rapidash</t>
+  </si>
+  <si>
+    <t>Psychic, Flying, Fairy</t>
+  </si>
+  <si>
+    <t>Dark</t>
+  </si>
+  <si>
+    <t>Absol (Lendário) / Mightyena (UR)</t>
+  </si>
+  <si>
+    <t>Hitmontop, Hitmonchan, Poliwrath</t>
+  </si>
+  <si>
+    <t>Machamp, Scyther, Mimikyu</t>
+  </si>
+  <si>
+    <t>Fighting, Fairy, Bug</t>
+  </si>
+  <si>
+    <t>Water</t>
+  </si>
+  <si>
+    <t>Milotic (UR)</t>
+  </si>
+  <si>
+    <t>Tangrowth, Ampharos, Venusaur</t>
+  </si>
+  <si>
+    <t>Tangrowth, Gogoat, Luxray</t>
+  </si>
+  <si>
+    <t>Grass, Electric</t>
   </si>
   <si>
     <t>📈 Mais Mobs e Brokes / Hora</t>
   </si>
   <si>
-    <t>★ FAIRY</t>
-  </si>
-  <si>
-    <t>⭐ Arcanine, Houndoom, Pupitar</t>
+    <t>Grass</t>
+  </si>
+  <si>
+    <t>Leafeon (Lendário) / Sceptile (UR)</t>
+  </si>
+  <si>
+    <t>Typhlosion, Rapidash, Pidgeot</t>
+  </si>
+  <si>
+    <t>Arcanine, Infernape, Scyther</t>
+  </si>
+  <si>
+    <t>Poison, Bug, Fire, Fly, Ice</t>
+  </si>
+  <si>
+    <t>Electric</t>
   </si>
   <si>
     <t>Rotação mais fluida = mais mobs derrotados/hora, aumentando drasticamente a chance de Shiny/hr e lucro.</t>
   </si>
   <si>
-    <t>Em breve</t>
-  </si>
-  <si>
-    <t>⭐ Hitmontop, Typhlosion, Rapidash</t>
-  </si>
-  <si>
-    <t>Rapidash, Typhlosion, Magcargo</t>
-  </si>
-  <si>
-    <t>★ FIRE</t>
-  </si>
-  <si>
-    <t>Arcanine, Infernape, Armaldo</t>
+    <t>⭐ Aggron, Skarmory, Toxicroak</t>
+  </si>
+  <si>
+    <t>Electabuzz (Lendário) / Manectric (UR)</t>
+  </si>
+  <si>
+    <t>⭐ Blastoise, Feraligatr, Omastar</t>
+  </si>
+  <si>
+    <t>Steelix, Nidoqueen, Torterra</t>
+  </si>
+  <si>
+    <t>⭐ Pupitar, Torterra, Kingdra</t>
   </si>
   <si>
     <t>⭐ Arcanine, Machamp, Pupitar</t>
   </si>
   <si>
+    <t>Torterra, Pupitar, Smeargle</t>
+  </si>
+  <si>
+    <t>⚔️ Hazards Mais Altos</t>
+  </si>
+  <si>
+    <t>Outras Opções T1:</t>
+  </si>
+  <si>
+    <t>Ground</t>
+  </si>
+  <si>
+    <t>Ghost</t>
+  </si>
+  <si>
     <t>⭐ Umbreon, Crawdaunt, Sableye</t>
   </si>
   <si>
+    <t>Mesmo encurtando o número total de hunts, permite solar níveis de Hazard superiores com segurança e eficiência.</t>
+  </si>
+  <si>
     <t>⭐ Houndoom, Hydreigon, Pupitar</t>
   </si>
   <si>
-    <t>Outras Opções T1:</t>
-  </si>
-  <si>
-    <t>⚔️ Hazards Mais Altos</t>
-  </si>
-  <si>
-    <t>Fire, Rock</t>
+    <t>Umbreon, Crawdaunt, Dusknoir</t>
+  </si>
+  <si>
+    <t>Dusknoir, Houndoom, Hydreigon</t>
+  </si>
+  <si>
+    <t>Dark, Ghost</t>
+  </si>
+  <si>
+    <t>Ice</t>
+  </si>
+  <si>
+    <t>Glaceon (Lendário) / Glalie (UR)</t>
+  </si>
+  <si>
+    <t>🏆 Futuro &amp; Escalabilidade (Endgame)</t>
   </si>
   <si>
     <t>Outras Opções SR:</t>
   </si>
   <si>
-    <t>Mesmo encurtando o número total de hunts, permite solar níveis de Hazard superiores com segurança e eficiência.</t>
+    <t>S.Charizard, Kabutops, Golem</t>
+  </si>
+  <si>
+    <t>Typhlosion, Rapidash, Hitmontop</t>
+  </si>
+  <si>
+    <t>Trabalhar com 2 ou 3 elementos abre um catálogo amplo de opções viáveis para evoluir: T1, SR, UR e Lendários.</t>
   </si>
   <si>
     <t>Umbreon</t>
   </si>
   <si>
-    <t>🏆 Futuro &amp; Escalabilidade (Endgame)</t>
-  </si>
-  <si>
-    <t>Fairy</t>
-  </si>
-  <si>
-    <t>Hunt: Em breve</t>
-  </si>
-  <si>
-    <t>Trabalhar com 2 ou 3 elementos abre um catálogo amplo de opções viáveis para evoluir: T1, SR, UR e Lendários.</t>
+    <t>—</t>
+  </si>
+  <si>
+    <t>Infernape, Machamp, Skarmory</t>
+  </si>
+  <si>
+    <t>Fighting, Fire, Metal</t>
+  </si>
+  <si>
+    <t>Poison</t>
+  </si>
+  <si>
+    <t>Garbodor (Lendário) / Swalot (UR)</t>
+  </si>
+  <si>
+    <t>Steelix, Espeon, Nidoqueen</t>
+  </si>
+  <si>
+    <t>Metang, Magneton Estrelado</t>
+  </si>
+  <si>
+    <t>Wobbuffet, Mr. Mime, Pupitar</t>
+  </si>
+  <si>
+    <t>Ground, Psychic</t>
+  </si>
+  <si>
+    <t>SevIper</t>
+  </si>
+  <si>
+    <t>Normal</t>
+  </si>
+  <si>
+    <t>Snorlax (Lendário) / Exploud (UR)</t>
+  </si>
+  <si>
+    <t>Poliwrath, Hitmontop, Medicham</t>
+  </si>
+  <si>
+    <t>Machamp, Kangaskhan, Smeargle</t>
+  </si>
+  <si>
+    <t>Vaporeon, Rhyperior, Magcargo</t>
   </si>
   <si>
     <t>Torterra, Misdreavus</t>
   </si>
   <si>
+    <t>Sharpedo</t>
+  </si>
+  <si>
     <t>Poliwrath, Medicham, Hariyama</t>
   </si>
   <si>
+    <t>Rock</t>
+  </si>
+  <si>
+    <t>Rampardos (UR)</t>
+  </si>
+  <si>
     <t>Infernape, Kangaskhan, Torterra</t>
   </si>
   <si>
+    <t>Tangrowth, Steelix, Blastoise</t>
+  </si>
+  <si>
+    <t>🎨 Smeargle: Fire, Rock</t>
+  </si>
+  <si>
+    <t>Tangrowth, Machamp, Gogoat</t>
+  </si>
+  <si>
     <t>Cacturne, Banette, Dusclops</t>
   </si>
   <si>
+    <t>Fighting, Ground, Water, Grass</t>
+  </si>
+  <si>
+    <t>Steel</t>
+  </si>
+  <si>
     <t>Misdreavus, Dusknoir, Torterra</t>
   </si>
   <si>
-    <t>Hunt: Shiny Sylveon (Lendário)</t>
+    <t>Hitmontop, Rapidash, Typhlosion</t>
+  </si>
+  <si>
+    <t>Arcanine, Machamp, Infernape</t>
+  </si>
+  <si>
+    <t>Ground, Fighting, Fire</t>
+  </si>
+  <si>
+    <t>Blastoise, Tangrowth, Gogoat</t>
+  </si>
+  <si>
+    <t>🎨 Smeargle: Poison, Metal</t>
+  </si>
+  <si>
+    <t>Tangrowth, Kingdra, Sharpedo</t>
   </si>
   <si>
     <t>🎨 Smeargle: Fire, Ground, Ghost, Dark</t>
   </si>
   <si>
-    <t>Shiny Sylveon (Lendário)</t>
-  </si>
-  <si>
-    <t>Hunt: Magmar (Lendário) / Torkoal (UR)</t>
-  </si>
-  <si>
-    <t>Muk, Tentacruel, Mawile</t>
-  </si>
-  <si>
-    <t>Aggron, Skarmory, Toxicroak</t>
-  </si>
-  <si>
-    <t>Poison, Metal</t>
+    <t>Water, Ice, Grass</t>
+  </si>
+  <si>
+    <t>Dragon</t>
+  </si>
+  <si>
+    <t>Salamence (UR) / Flygon (Lendário)</t>
+  </si>
+  <si>
+    <t>Lapras, Mega Clefable, Jynx</t>
+  </si>
+  <si>
+    <t>Mimikyu, Florges, Walrein</t>
+  </si>
+  <si>
+    <t>Dragon, Ice, Fairy</t>
+  </si>
+  <si>
+    <t>🎨 Smeargle: Rock, Water, Ground</t>
+  </si>
+  <si>
+    <t>Psychic</t>
+  </si>
+  <si>
+    <t>Alakazam (Lendário)</t>
   </si>
   <si>
     <t>🎨 Smeargle: Fighting, Fire, Ground</t>
   </si>
   <si>
-    <t>Fire</t>
-  </si>
-  <si>
-    <t>Magmar (Lendário) / Torkoal (UR)</t>
-  </si>
-  <si>
-    <t>Blastoise, Feraligatr, Omastar</t>
-  </si>
-  <si>
-    <t>Pupitar, Torterra, Kingdra</t>
-  </si>
-  <si>
-    <t>Rock, Water, Ground</t>
-  </si>
-  <si>
-    <t>Fighting</t>
-  </si>
-  <si>
-    <t>Mega Clefable, Pidgeot, Espeon</t>
-  </si>
-  <si>
-    <t>Wobbuffet, Mimikyu, Gliscor</t>
-  </si>
-  <si>
-    <t>Psychic, Flying, Fairy</t>
-  </si>
-  <si>
-    <t>Dark</t>
-  </si>
-  <si>
-    <t>Absol (Lendário) / Mightyena (UR)</t>
-  </si>
-  <si>
-    <t>Hitmontop, Hitmonchan, Poliwrath</t>
-  </si>
-  <si>
-    <t>Machamp, Scyther, Mimikyu</t>
-  </si>
-  <si>
-    <t>Fighting, Fairy, Bug</t>
-  </si>
-  <si>
-    <t>Water</t>
-  </si>
-  <si>
-    <t>Milotic (UR)</t>
-  </si>
-  <si>
-    <t>⭐S.Rapidash, S.Typhlosion, S.Magcargo</t>
-  </si>
-  <si>
-    <t>Tangrowth, Ampharos, Venusaur</t>
-  </si>
-  <si>
-    <t>Tangrowth, Gogoat, Luxray</t>
-  </si>
-  <si>
-    <t>⭐ Arcanine, Infernape, Armaldo</t>
-  </si>
-  <si>
-    <t>Grass, Electric</t>
-  </si>
-  <si>
-    <t>Grass</t>
-  </si>
-  <si>
-    <t>Leafeon (Lendário) / Sceptile (UR)</t>
-  </si>
-  <si>
-    <t>Typhlosion, Rapidash, Pidgeot</t>
-  </si>
-  <si>
-    <t>Arcanine, Infernape, Scyther</t>
-  </si>
-  <si>
-    <t>Poison, Bug, Fire, Fly, Ice</t>
-  </si>
-  <si>
-    <t>⭐ Muk, Tentacruel, Mawile</t>
-  </si>
-  <si>
-    <t>Electric</t>
-  </si>
-  <si>
-    <t>Electabuzz (Lendário) / Manectric (UR)</t>
-  </si>
-  <si>
-    <t>Steelix, Nidoqueen, Torterra</t>
-  </si>
-  <si>
-    <t>Torterra, Pupitar, Smeargle</t>
-  </si>
-  <si>
-    <t>⭐ Aggron, Skarmory, Toxicroak</t>
-  </si>
-  <si>
-    <t>Ground</t>
-  </si>
-  <si>
-    <t>⭐ Blastoise, Feraligatr, Omastar</t>
-  </si>
-  <si>
-    <t>⭐ Pupitar, Torterra, Kingdra</t>
+    <t>Umbreon, Crawdaunt, Sableye</t>
+  </si>
+  <si>
+    <t>Houndoom, Scyther, Dusknoir</t>
+  </si>
+  <si>
+    <t>Ghost, Dark, Bug</t>
+  </si>
+  <si>
+    <t>Flying</t>
+  </si>
+  <si>
+    <t>Ampharos, Magcargo, Lapras</t>
+  </si>
+  <si>
+    <t>Walrein, Luxray, Pachirisu</t>
+  </si>
+  <si>
+    <t>Electric, Ice, Rock</t>
   </si>
   <si>
     <t>🎨 Smeargle: Dark, Ghost, Ground</t>
   </si>
   <si>
+    <t>Metagross</t>
+  </si>
+  <si>
+    <t>Steel / Psychic</t>
+  </si>
+  <si>
+    <t>Rapidash, Typhlosion, Steelix</t>
+  </si>
+  <si>
+    <t>★ FIGHTING</t>
+  </si>
+  <si>
+    <t>Arcanine, Houndoom, Pupitar</t>
+  </si>
+  <si>
+    <t>Fire, Ground, Ghost, Dark</t>
+  </si>
+  <si>
+    <t>Lucario</t>
+  </si>
+  <si>
+    <t>Fighting / Steel</t>
+  </si>
+  <si>
+    <t>Hitmontop, Typhlosion, Rapidash</t>
+  </si>
+  <si>
+    <t>Arcanine, Machamp, Pupitar</t>
+  </si>
+  <si>
     <t>★ GARDEVOIR</t>
   </si>
   <si>
-    <t>S.Charizard, Kabutops, Golem</t>
-  </si>
-  <si>
-    <t>Ghost</t>
+    <t>Fighting, Fire, Ground</t>
+  </si>
+  <si>
+    <t>Gengar</t>
+  </si>
+  <si>
+    <t>Ghost / Poison</t>
+  </si>
+  <si>
+    <t>★ DARK</t>
+  </si>
+  <si>
+    <t>Houndoom, Hydreigon, Pupitar</t>
   </si>
   <si>
     <t>★ GYARADOS</t>
   </si>
   <si>
-    <t>Umbreon, Crawdaunt, Dusknoir</t>
-  </si>
-  <si>
-    <t>Dusknoir, Houndoom, Hydreigon</t>
-  </si>
-  <si>
-    <t>Dark, Ghost</t>
-  </si>
-  <si>
-    <t>—</t>
-  </si>
-  <si>
-    <t>Ice</t>
-  </si>
-  <si>
-    <t>Glaceon (Lendário) / Glalie (UR)</t>
-  </si>
-  <si>
-    <t>Typhlosion, Rapidash, Hitmontop</t>
-  </si>
-  <si>
-    <t>Metang, Magneton Estrelado</t>
-  </si>
-  <si>
-    <t>Infernape, Machamp, Skarmory</t>
-  </si>
-  <si>
-    <t>Fighting, Fire, Metal</t>
+    <t>Dark, Ghost, Ground</t>
+  </si>
+  <si>
+    <t>Gardevoir</t>
+  </si>
+  <si>
+    <t>Psychic / Fairy</t>
+  </si>
+  <si>
+    <t>Mawile, Muk, Tentacruel</t>
+  </si>
+  <si>
+    <t>Toxicroak, Seviper, Misdreavus</t>
+  </si>
+  <si>
+    <t>Poison, Ghost, Metal</t>
+  </si>
+  <si>
+    <t>Gyarados</t>
+  </si>
+  <si>
+    <t>Water / Flying</t>
   </si>
   <si>
     <t>★ SWAMPERT</t>
   </si>
   <si>
-    <t>Poison</t>
-  </si>
-  <si>
-    <t>SevIper</t>
-  </si>
-  <si>
-    <t>Garbodor (Lendário) / Swalot (UR)</t>
-  </si>
-  <si>
-    <t>Steelix, Espeon, Nidoqueen</t>
-  </si>
-  <si>
-    <t>Wobbuffet, Mr. Mime, Pupitar</t>
-  </si>
-  <si>
-    <t>Ground, Psychic</t>
-  </si>
-  <si>
-    <t>Vaporeon, Rhyperior, Magcargo</t>
-  </si>
-  <si>
-    <t>Normal</t>
-  </si>
-  <si>
-    <t>Snorlax (Lendário) / Exploud (UR)</t>
-  </si>
-  <si>
-    <t>Sharpedo</t>
-  </si>
-  <si>
-    <t>Poliwrath, Hitmontop, Medicham</t>
-  </si>
-  <si>
-    <t>Machamp, Kangaskhan, Smeargle</t>
-  </si>
-  <si>
-    <t>Rock</t>
+    <t>★ WATER</t>
+  </si>
+  <si>
+    <t>Ampharos, Luxray, Jolteon</t>
+  </si>
+  <si>
+    <t>Luxray, Pachirisu, Smeargle Eletric</t>
   </si>
   <si>
     <t>Hunt: Psychic / Fairy</t>
   </si>
   <si>
-    <t>Rampardos (UR)</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Fire, Rock</t>
-  </si>
-  <si>
-    <t>Tangrowth, Steelix, Blastoise</t>
-  </si>
-  <si>
-    <t>Tangrowth, Machamp, Gogoat</t>
-  </si>
-  <si>
-    <t>Fighting, Ground, Water, Grass</t>
-  </si>
-  <si>
-    <t>Steel</t>
-  </si>
-  <si>
     <t>Hunt: Water / Flying</t>
   </si>
   <si>
-    <t>Hitmontop, Rapidash, Typhlosion</t>
-  </si>
-  <si>
-    <t>Arcanine, Machamp, Infernape</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Poison, Metal</t>
-  </si>
-  <si>
-    <t>Ground, Fighting, Fire</t>
-  </si>
-  <si>
-    <t>Blastoise, Tangrowth, Gogoat</t>
-  </si>
-  <si>
-    <t>Tangrowth, Kingdra, Sharpedo</t>
-  </si>
-  <si>
-    <t>Water, Ice, Grass</t>
-  </si>
-  <si>
     <t>Hunt: Water / Ground</t>
   </si>
   <si>
-    <t>Dragon</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Rock, Water, Ground</t>
-  </si>
-  <si>
-    <t>Salamence (UR) / Flygon (Lendário)</t>
-  </si>
-  <si>
-    <t>Lapras, Mega Clefable, Jynx</t>
-  </si>
-  <si>
-    <t>Mimikyu, Florges, Walrein</t>
-  </si>
-  <si>
-    <t>Dragon, Ice, Fairy</t>
-  </si>
-  <si>
-    <t>Psychic</t>
-  </si>
-  <si>
-    <t>Alakazam (Lendário)</t>
-  </si>
-  <si>
-    <t>Umbreon, Crawdaunt, Sableye</t>
-  </si>
-  <si>
-    <t>Houndoom, Scyther, Dusknoir</t>
-  </si>
-  <si>
-    <t>Ghost, Dark, Bug</t>
-  </si>
-  <si>
-    <t>Flying</t>
-  </si>
-  <si>
-    <t>★ FIGHTING</t>
-  </si>
-  <si>
-    <t>Ampharos, Magcargo, Lapras</t>
-  </si>
-  <si>
-    <t>Walrein, Luxray, Pachirisu</t>
-  </si>
-  <si>
-    <t>Electric, Ice, Rock</t>
+    <t>Hunt: Absol (Lendário) / Mightyena (UR)</t>
+  </si>
+  <si>
+    <t>Hunt: Milotic (UR)</t>
   </si>
   <si>
     <t>⭐ Mawile, Muk, Tentacruel</t>
   </si>
   <si>
-    <t>Metagross</t>
-  </si>
-  <si>
     <t>⭐ Toxicroak, Seviper, Misdreavus</t>
   </si>
   <si>
-    <t>Steel / Psychic</t>
+    <t>⭐ Mega Clefable, Pidgeot, Espeon</t>
   </si>
   <si>
     <t>⭐ Ampharos, Luxray, Jolteon</t>
   </si>
   <si>
-    <t>Rapidash, Typhlosion, Steelix</t>
-  </si>
-  <si>
-    <t>Arcanine, Houndoom, Pupitar</t>
-  </si>
-  <si>
-    <t>Fire, Ground, Ghost, Dark</t>
-  </si>
-  <si>
-    <t>★ DARK</t>
-  </si>
-  <si>
-    <t>Lucario</t>
+    <t>⭐ Wobbuffet, Mimikyu, Gliscor</t>
+  </si>
+  <si>
+    <t>⭐ Hitmontop, Hitmonchan, Poliwrath</t>
+  </si>
+  <si>
+    <t>⭐ Machamp, Scyther, Mimikyu</t>
+  </si>
+  <si>
+    <t>⭐ Tangrowth, Ampharos, Venusaur</t>
   </si>
   <si>
     <t>⭐ S.Luxray, S.Pachirisu, Smeargle Eletric</t>
   </si>
   <si>
-    <t>Fighting / Steel</t>
-  </si>
-  <si>
-    <t>Hitmontop, Typhlosion, Rapidash</t>
-  </si>
-  <si>
-    <t>Arcanine, Machamp, Pupitar</t>
-  </si>
-  <si>
-    <t>Fighting, Fire, Ground</t>
-  </si>
-  <si>
-    <t>Gengar</t>
+    <t>⭐ Tangrowth, Gogoat, Luxray</t>
   </si>
   <si>
     <t>⭐Venusaur, Gogoat, Tangrowth</t>
   </si>
   <si>
-    <t>Ghost / Poison</t>
-  </si>
-  <si>
     <t>⭐ S.Tangrowth,S. Gogoat, Smeargle Grass</t>
   </si>
   <si>
-    <t>★ WATER</t>
-  </si>
-  <si>
-    <t>Houndoom, Hydreigon, Pupitar</t>
-  </si>
-  <si>
-    <t>Dark, Ghost, Ground</t>
-  </si>
-  <si>
-    <t>Gardevoir</t>
-  </si>
-  <si>
-    <t>Psychic / Fairy</t>
-  </si>
-  <si>
-    <t>Mawile, Muk, Tentacruel</t>
+    <t>Farfetch'd, Gliscor</t>
+  </si>
+  <si>
+    <t>Mr. Mime, Florges, Swellow</t>
+  </si>
+  <si>
+    <t>Mega Clefable, Hitmonlee</t>
+  </si>
+  <si>
+    <t>Florges, Kangaskhan, Pinsir</t>
+  </si>
+  <si>
+    <t>Luxray, Gogoat</t>
+  </si>
+  <si>
+    <t>Pachirisu</t>
+  </si>
+  <si>
+    <t>🎨 Smeargle: Psychic, Flying, Fairy</t>
   </si>
   <si>
     <t>Metang, Banette, Dusclops, Nidoking</t>
   </si>
   <si>
-    <t>Toxicroak, Seviper, Misdreavus</t>
-  </si>
-  <si>
     <t>Aggron, Skarmory</t>
   </si>
   <si>
-    <t>Poison, Ghost, Metal</t>
-  </si>
-  <si>
-    <t>Gyarados</t>
-  </si>
-  <si>
-    <t>Water / Flying</t>
-  </si>
-  <si>
-    <t>Ampharos, Luxray, Jolteon</t>
-  </si>
-  <si>
-    <t>Luxray, Pachirisu, Smeargle Eletric</t>
-  </si>
-  <si>
     <t>Raichu</t>
   </si>
   <si>
+    <t>🎨 Smeargle: Fighting, Fairy, Bug</t>
+  </si>
+  <si>
     <t>🎨 Smeargle: Poison, Ghost, Metal</t>
   </si>
   <si>
-    <t>Hunt: Absol (Lendário) / Mightyena (UR)</t>
-  </si>
-  <si>
     <t>🎨 Smeargle: Electric</t>
   </si>
   <si>
-    <t>Hunt: Milotic (UR)</t>
+    <t>🎨 Smeargle: Grass, Electric</t>
   </si>
   <si>
     <t>🎨 Smeargle: Grass</t>
   </si>
   <si>
+    <t>★ GRASS</t>
+  </si>
+  <si>
     <t>★ SCIZOR</t>
   </si>
   <si>
-    <t>⭐ Mega Clefable, Pidgeot, Espeon</t>
-  </si>
-  <si>
-    <t>⭐ Wobbuffet, Mimikyu, Gliscor</t>
+    <t>★ ELECTRIC</t>
   </si>
   <si>
     <t>Hunt: Bug</t>
   </si>
   <si>
-    <t>⭐ Hitmontop, Hitmonchan, Poliwrath</t>
-  </si>
-  <si>
-    <t>⭐ Machamp, Scyther, Mimikyu</t>
-  </si>
-  <si>
-    <t>⭐ Tangrowth, Ampharos, Venusaur</t>
-  </si>
-  <si>
-    <t>⭐ Tangrowth, Gogoat, Luxray</t>
+    <t>★ GHOST</t>
   </si>
   <si>
     <t>⭐ S.Rapidash, S.Typhlosion, S.Zard</t>
@@ -703,46 +742,10 @@
     <t>⭐S.Arcanine, S.Infernape, Smeargle Fire</t>
   </si>
   <si>
-    <t>Farfetch'd, Gliscor</t>
-  </si>
-  <si>
-    <t>Mr. Mime, Florges, Swellow</t>
-  </si>
-  <si>
-    <t>Mega Clefable, Hitmonlee</t>
-  </si>
-  <si>
-    <t>Florges, Kangaskhan, Pinsir</t>
-  </si>
-  <si>
-    <t>Luxray, Gogoat</t>
-  </si>
-  <si>
-    <t>Pachirisu</t>
+    <t>Hunt: Leafeon (Lendário) / Sceptile (UR)</t>
   </si>
   <si>
     <t>🎨 Smeargle: Fire</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Psychic, Flying, Fairy</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Fighting, Fairy, Bug</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Grass, Electric</t>
-  </si>
-  <si>
-    <t>★ GRASS</t>
-  </si>
-  <si>
-    <t>★ ELECTRIC</t>
-  </si>
-  <si>
-    <t>★ GHOST</t>
-  </si>
-  <si>
-    <t>Hunt: Leafeon (Lendário) / Sceptile (UR)</t>
   </si>
   <si>
     <t>Hunt: Electabuzz (Lendário) / Manectric (UR)</t>
@@ -986,34 +989,21 @@
     </font>
     <font/>
     <font>
+      <b/>
+      <sz val="13.0"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
       <i/>
       <sz val="9.0"/>
       <color rgb="FF94A3B8"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
-      <b/>
-      <sz val="10.0"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13.0"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9.0"/>
-      <color rgb="FF334155"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9.0"/>
-      <color rgb="FF0F172A"/>
-      <name val="Quattrocento Sans"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <i/>
@@ -1029,14 +1019,8 @@
       <name val="Quattrocento Sans"/>
     </font>
     <font>
-      <sz val="9.0"/>
-      <color rgb="FF0F172A"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
+      <u/>
+      <color rgb="FF0000FF"/>
     </font>
     <font>
       <b/>
@@ -1045,19 +1029,9 @@
       <name val="Quattrocento Sans"/>
     </font>
     <font>
-      <u/>
-      <color rgb="FF0000FF"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="9.0"/>
-      <color rgb="FFF3F4F6"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
       <b/>
-      <sz val="9.0"/>
-      <color rgb="FF1E3A8A"/>
+      <sz val="10.0"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1069,30 +1043,31 @@
     </font>
     <font>
       <b/>
-      <sz val="9.0"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <sz val="9.0"/>
-      <color rgb="FF1F2937"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10.0"/>
-      <color rgb="FF1A1A1A"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
       <sz val="10.0"/>
       <color rgb="FF1E293B"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
+      <b/>
+      <sz val="9.0"/>
+      <color rgb="FF334155"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
       <sz val="9.0"/>
       <color rgb="FF475569"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9.0"/>
+      <color rgb="FFF3F4F6"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9.0"/>
+      <color rgb="FF0F172A"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1109,14 +1084,42 @@
     </font>
     <font>
       <b/>
-      <sz val="8.0"/>
-      <color rgb="FF4B5563"/>
+      <sz val="9.0"/>
+      <color rgb="FF1E40AF"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <sz val="9.0"/>
+      <color rgb="FF0F172A"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
       <b/>
       <sz val="9.0"/>
-      <color rgb="FF1E40AF"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10.0"/>
+      <color rgb="FF1A1A1A"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9.0"/>
+      <color rgb="FF1E3A8A"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <sz val="9.0"/>
+      <color rgb="FF1F2937"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8.0"/>
+      <color rgb="FF4B5563"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1127,13 +1130,13 @@
     <font>
       <b/>
       <sz val="8.0"/>
-      <color rgb="FF1E3A8A"/>
+      <color rgb="FF4A4A4A"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
       <b/>
       <sz val="8.0"/>
-      <color rgb="FF4A4A4A"/>
+      <color rgb="FF1E3A8A"/>
       <name val="Quattrocento Sans"/>
     </font>
   </fonts>
@@ -1158,6 +1161,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+        <bgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF334155"/>
         <bgColor rgb="FF334155"/>
       </patternFill>
@@ -1170,8 +1185,50 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <fgColor rgb="FF8DAA34"/>
+        <bgColor rgb="FF8DAA34"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE68D9C"/>
+        <bgColor rgb="FFE68D9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF374151"/>
+        <bgColor rgb="FF374151"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF0FDF4"/>
+        <bgColor rgb="FFF0FDF4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEA6C2D"/>
+        <bgColor rgb="FFEA6C2D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF2F2"/>
+        <bgColor rgb="FFFEF2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E7D32"/>
+        <bgColor rgb="FF2E7D32"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8FAFC"/>
+        <bgColor rgb="FFF8FAFC"/>
       </patternFill>
     </fill>
     <fill>
@@ -1182,8 +1239,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E78"/>
-        <bgColor rgb="FF1F4E78"/>
+        <fgColor rgb="FFC62828"/>
+        <bgColor rgb="FFC62828"/>
       </patternFill>
     </fill>
     <fill>
@@ -1200,36 +1257,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF374151"/>
-        <bgColor rgb="FF374151"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEFF6FF"/>
-        <bgColor rgb="FFEFF6FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF2E7D32"/>
-        <bgColor rgb="FF2E7D32"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC62828"/>
-        <bgColor rgb="FFC62828"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF8DAA34"/>
-        <bgColor rgb="FF8DAA34"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFE8F5E9"/>
         <bgColor rgb="FFE8F5E9"/>
       </patternFill>
@@ -1242,20 +1269,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE68D9C"/>
-        <bgColor rgb="FFE68D9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF0FDF4"/>
-        <bgColor rgb="FFF0FDF4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFEF2F2"/>
-        <bgColor rgb="FFFEF2F2"/>
+        <fgColor rgb="FFEFF6FF"/>
+        <bgColor rgb="FFEFF6FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -1266,20 +1281,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEA6C2D"/>
-        <bgColor rgb="FFEA6C2D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFF9FAFB"/>
         <bgColor rgb="FFF9FAFB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF8FAFC"/>
-        <bgColor rgb="FFF8FAFC"/>
       </patternFill>
     </fill>
     <fill>
@@ -1397,22 +1400,22 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFCBD5E1"/>
+        <color rgb="FFD1D5DB"/>
       </left>
-      <right style="thin">
-        <color rgb="FFCBD5E1"/>
-      </right>
       <top style="thin">
-        <color rgb="FFCBD5E1"/>
+        <color rgb="FFD1D5DB"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFCBD5E1"/>
+        <color rgb="FFD1D5DB"/>
       </bottom>
     </border>
     <border>
       <left style="thin">
         <color rgb="FFD1D5DB"/>
       </left>
+      <right style="thin">
+        <color rgb="FFD1D5DB"/>
+      </right>
       <top style="thin">
         <color rgb="FFD1D5DB"/>
       </top>
@@ -1433,16 +1436,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFD1D5DB"/>
+        <color rgb="FFCBD5E1"/>
       </left>
       <right style="thin">
-        <color rgb="FFD1D5DB"/>
+        <color rgb="FFCBD5E1"/>
       </right>
       <top style="thin">
-        <color rgb="FFD1D5DB"/>
+        <color rgb="FFCBD5E1"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFD1D5DB"/>
+        <color rgb="FFCBD5E1"/>
       </bottom>
     </border>
     <border>
@@ -1479,7 +1482,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="70">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1490,189 +1493,192 @@
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="5" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="6" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
     <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="6" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="6" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="5" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="6" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="6" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="6" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="3" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="6" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="4" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="7" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="8" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="4" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="9" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="10" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="4" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf borderId="5" fillId="11" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="7" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="12" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="13" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="4" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="4" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="5" fillId="8" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="9" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="6" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="10" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="11" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="7" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="8" fillId="12" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="14" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="7" fillId="13" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="9" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="7" fillId="14" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="8" fillId="6" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="7" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="5" fillId="15" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="10" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="7" fillId="16" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="7" fillId="16" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="5" fillId="17" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="18" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="5" fillId="15" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="19" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="20" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="7" fillId="6" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="15" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="17" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="21" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="7" fillId="6" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="8" fillId="22" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="9" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="8" fillId="4" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="10" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="5" fillId="20" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="5" fillId="23" fontId="25" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="5" fillId="24" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="5" fillId="24" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="5" fillId="24" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="25" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="18" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="26" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="19" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="7" fillId="16" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="7" fillId="20" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="7" fillId="21" fontId="24" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="5" fillId="22" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="27" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="6" fontId="25" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="5" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="28" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="23" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="4" fillId="10" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="24" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="21" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="25" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="29" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="24" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="30" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="25" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="31" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="24" fontId="25" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="32" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="23" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="7" fillId="23" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="5" fillId="8" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="11" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="26" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="33" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="17" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="5" fillId="27" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="34" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="28" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="35" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="25" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="29" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="36" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="30" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="37" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="31" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="38" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="32" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="39" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="33" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="34" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="35" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="36" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="37" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="38" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="39" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="40" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="40" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1920,135 +1926,149 @@
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
-      <c r="F2" s="4"/>
+      <c r="F2" s="5"/>
     </row>
     <row r="3" ht="19.5" customHeight="1">
-      <c r="B3" s="5" t="s">
-        <v>2</v>
+      <c r="B3" s="7" t="s">
+        <v>4</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
-      <c r="F3" s="4"/>
+      <c r="F3" s="5"/>
+    </row>
+    <row r="4">
+      <c r="B4" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="5" ht="24.0" customHeight="1">
-      <c r="B5" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="4"/>
-      <c r="E5" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F5" s="4"/>
+      <c r="B5" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="5"/>
+      <c r="E5" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="5"/>
     </row>
     <row r="6" ht="24.75" customHeight="1">
-      <c r="B6" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>10</v>
+      <c r="B6" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="25" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="7" ht="24.75" customHeight="1">
-      <c r="B7" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="13" t="s">
-        <v>15</v>
+      <c r="B7" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="F7" s="30" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="8" ht="24.75" customHeight="1">
-      <c r="B8" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="F8" s="17" t="s">
-        <v>19</v>
+      <c r="B8" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" s="33" t="s">
+        <v>44</v>
+      </c>
+      <c r="E8" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="F8" s="35" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="9" ht="24.75" customHeight="1">
-      <c r="B9" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="F9" s="13" t="s">
-        <v>23</v>
+      <c r="B9" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="C9" s="30" t="s">
+        <v>50</v>
+      </c>
+      <c r="E9" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="F9" s="30" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="11" ht="24.0" customHeight="1">
-      <c r="B11" s="20" t="s">
-        <v>25</v>
+      <c r="B11" s="37" t="s">
+        <v>52</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
-      <c r="F11" s="4"/>
+      <c r="F11" s="5"/>
     </row>
     <row r="12" ht="24.0" customHeight="1">
-      <c r="B12" s="23" t="s">
-        <v>29</v>
-      </c>
-      <c r="C12" s="26"/>
-      <c r="D12" s="28" t="s">
-        <v>36</v>
-      </c>
-      <c r="E12" s="31"/>
-      <c r="F12" s="26"/>
+      <c r="B12" s="41" t="s">
+        <v>55</v>
+      </c>
+      <c r="C12" s="42"/>
+      <c r="D12" s="43" t="s">
+        <v>67</v>
+      </c>
+      <c r="E12" s="44"/>
+      <c r="F12" s="42"/>
     </row>
     <row r="13" ht="24.0" customHeight="1">
-      <c r="B13" s="23" t="s">
-        <v>43</v>
-      </c>
-      <c r="C13" s="26"/>
-      <c r="D13" s="28" t="s">
-        <v>46</v>
-      </c>
-      <c r="E13" s="31"/>
-      <c r="F13" s="26"/>
+      <c r="B13" s="41" t="s">
+        <v>82</v>
+      </c>
+      <c r="C13" s="42"/>
+      <c r="D13" s="43" t="s">
+        <v>89</v>
+      </c>
+      <c r="E13" s="44"/>
+      <c r="F13" s="42"/>
     </row>
     <row r="14" ht="24.0" customHeight="1">
-      <c r="B14" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="C14" s="26"/>
-      <c r="D14" s="28" t="s">
-        <v>59</v>
-      </c>
-      <c r="E14" s="31"/>
-      <c r="F14" s="26"/>
+      <c r="B14" s="41" t="s">
+        <v>97</v>
+      </c>
+      <c r="C14" s="42"/>
+      <c r="D14" s="43" t="s">
+        <v>102</v>
+      </c>
+      <c r="E14" s="44"/>
+      <c r="F14" s="42"/>
     </row>
     <row r="15" ht="24.0" customHeight="1">
-      <c r="B15" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C15" s="26"/>
-      <c r="D15" s="28" t="s">
-        <v>64</v>
-      </c>
-      <c r="E15" s="31"/>
-      <c r="F15" s="26"/>
+      <c r="B15" s="41" t="s">
+        <v>109</v>
+      </c>
+      <c r="C15" s="42"/>
+      <c r="D15" s="43" t="s">
+        <v>113</v>
+      </c>
+      <c r="E15" s="44"/>
+      <c r="F15" s="42"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -3046,10 +3066,14 @@
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="D12:F12"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="C4"/>
+    <hyperlink r:id="rId2" ref="E4"/>
+  </hyperlinks>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -3070,8 +3094,8 @@
   </cols>
   <sheetData>
     <row r="1" ht="31.5" customHeight="1">
-      <c r="A1" s="10" t="s">
-        <v>6</v>
+      <c r="A1" s="4" t="s">
+        <v>2</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -3079,14 +3103,14 @@
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="14" t="s">
-        <v>14</v>
+      <c r="H1" s="5"/>
+      <c r="I1" s="8" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="2" ht="19.5" customHeight="1">
-      <c r="A2" s="24" t="s">
-        <v>20</v>
+      <c r="A2" s="17" t="s">
+        <v>8</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -3094,754 +3118,754 @@
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="14" t="s">
-        <v>34</v>
+      <c r="H2" s="5"/>
+      <c r="I2" s="8" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="4" ht="21.75" customHeight="1">
-      <c r="A4" s="30" t="s">
-        <v>37</v>
-      </c>
-      <c r="B4" s="18"/>
-      <c r="D4" s="36" t="s">
-        <v>44</v>
-      </c>
-      <c r="E4" s="18"/>
-      <c r="G4" s="41" t="s">
-        <v>50</v>
-      </c>
-      <c r="H4" s="18"/>
+      <c r="A4" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="16"/>
+      <c r="D4" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="16"/>
+      <c r="G4" s="27" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" s="16"/>
     </row>
     <row r="5" ht="18.0" customHeight="1">
-      <c r="A5" s="21" t="s">
-        <v>63</v>
-      </c>
-      <c r="B5" s="18"/>
-      <c r="D5" s="21" t="s">
-        <v>70</v>
-      </c>
-      <c r="E5" s="18"/>
-      <c r="G5" s="21" t="s">
-        <v>73</v>
-      </c>
-      <c r="H5" s="18"/>
+      <c r="A5" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="16"/>
+      <c r="D5" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" s="16"/>
+      <c r="G5" s="24" t="s">
+        <v>40</v>
+      </c>
+      <c r="H5" s="16"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="B6" s="27" t="s">
+      <c r="A6" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="D6" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="E6" s="27" t="s">
+      <c r="B6" s="34" t="s">
+        <v>45</v>
+      </c>
+      <c r="D6" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="G6" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="H6" s="27" t="s">
+      <c r="E6" s="34" t="s">
+        <v>45</v>
+      </c>
+      <c r="G6" s="31" t="s">
         <v>35</v>
       </c>
+      <c r="H6" s="34" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="7" ht="42.0" customHeight="1">
-      <c r="A7" s="32" t="s">
+      <c r="A7" s="38" t="s">
+        <v>58</v>
+      </c>
+      <c r="B7" s="40" t="s">
+        <v>59</v>
+      </c>
+      <c r="D7" s="45" t="s">
+        <v>60</v>
+      </c>
+      <c r="E7" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="G7" s="45" t="s">
+        <v>92</v>
+      </c>
+      <c r="H7" s="40" t="s">
         <v>94</v>
       </c>
-      <c r="B7" s="34" t="s">
-        <v>97</v>
-      </c>
-      <c r="D7" s="38" t="s">
-        <v>104</v>
-      </c>
-      <c r="E7" s="34" t="s">
-        <v>109</v>
-      </c>
-      <c r="G7" s="38" t="s">
+    </row>
+    <row r="8" ht="15.0" customHeight="1">
+      <c r="A8" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="B8" s="46" t="s">
+        <v>110</v>
+      </c>
+      <c r="D8" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="E8" s="46" t="s">
+        <v>110</v>
+      </c>
+      <c r="G8" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="H8" s="46" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="9" ht="27.75" customHeight="1">
+      <c r="A9" s="47" t="s">
         <v>111</v>
       </c>
-      <c r="H7" s="34" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="B8" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="D8" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="E8" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="G8" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="H8" s="40" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" ht="27.75" customHeight="1">
-      <c r="A9" s="48" t="s">
+      <c r="B9" s="48" t="s">
         <v>115</v>
       </c>
-      <c r="B9" s="43" t="s">
+      <c r="D9" s="48" t="s">
         <v>121</v>
       </c>
-      <c r="D9" s="43" t="s">
-        <v>125</v>
-      </c>
       <c r="E9" s="49" t="s">
-        <v>130</v>
-      </c>
-      <c r="G9" s="43" t="s">
-        <v>135</v>
-      </c>
-      <c r="H9" s="43" t="s">
-        <v>138</v>
+        <v>124</v>
+      </c>
+      <c r="G9" s="48" t="s">
+        <v>129</v>
+      </c>
+      <c r="H9" s="48" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="10" ht="18.0" customHeight="1">
-      <c r="A10" s="46" t="s">
-        <v>144</v>
-      </c>
-      <c r="B10" s="18"/>
-      <c r="D10" s="46" t="s">
-        <v>152</v>
-      </c>
-      <c r="E10" s="18"/>
-      <c r="G10" s="46" t="s">
-        <v>159</v>
-      </c>
-      <c r="H10" s="18"/>
+      <c r="A10" s="50" t="s">
+        <v>137</v>
+      </c>
+      <c r="B10" s="16"/>
+      <c r="D10" s="50" t="s">
+        <v>147</v>
+      </c>
+      <c r="E10" s="16"/>
+      <c r="G10" s="50" t="s">
+        <v>156</v>
+      </c>
+      <c r="H10" s="16"/>
     </row>
     <row r="14" ht="21.75" customHeight="1">
-      <c r="A14" s="52" t="s">
-        <v>170</v>
-      </c>
-      <c r="B14" s="18"/>
-      <c r="D14" s="54" t="s">
+      <c r="A14" s="51" t="s">
+        <v>171</v>
+      </c>
+      <c r="B14" s="16"/>
+      <c r="D14" s="52" t="s">
         <v>182</v>
       </c>
-      <c r="E14" s="18"/>
-      <c r="G14" s="55" t="s">
-        <v>193</v>
-      </c>
-      <c r="H14" s="18"/>
+      <c r="E14" s="16"/>
+      <c r="G14" s="54" t="s">
+        <v>194</v>
+      </c>
+      <c r="H14" s="16"/>
     </row>
     <row r="15" ht="18.0" customHeight="1">
-      <c r="A15" s="21" t="s">
-        <v>63</v>
-      </c>
-      <c r="B15" s="18"/>
-      <c r="D15" s="21" t="s">
+      <c r="A15" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" s="16"/>
+      <c r="D15" s="24" t="s">
+        <v>200</v>
+      </c>
+      <c r="E15" s="16"/>
+      <c r="G15" s="24" t="s">
+        <v>201</v>
+      </c>
+      <c r="H15" s="16"/>
+    </row>
+    <row r="16" ht="19.5" customHeight="1">
+      <c r="A16" s="31" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="34" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" s="31" t="s">
+        <v>35</v>
+      </c>
+      <c r="E16" s="34" t="s">
+        <v>45</v>
+      </c>
+      <c r="G16" s="31" t="s">
+        <v>35</v>
+      </c>
+      <c r="H16" s="34" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="17" ht="42.0" customHeight="1">
+      <c r="A17" s="45" t="s">
+        <v>204</v>
+      </c>
+      <c r="B17" s="40" t="s">
+        <v>206</v>
+      </c>
+      <c r="D17" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="E17" s="40" t="s">
+        <v>208</v>
+      </c>
+      <c r="G17" s="45" t="s">
         <v>209</v>
       </c>
-      <c r="E15" s="18"/>
-      <c r="G15" s="21" t="s">
+      <c r="H17" s="40" t="s">
         <v>211</v>
       </c>
-      <c r="H15" s="18"/>
-    </row>
-    <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="B16" s="27" t="s">
-        <v>35</v>
-      </c>
-      <c r="D16" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="E16" s="27" t="s">
-        <v>35</v>
-      </c>
-      <c r="G16" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="H16" s="27" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="17" ht="42.0" customHeight="1">
-      <c r="A17" s="38" t="s">
+    </row>
+    <row r="18" ht="15.0" customHeight="1">
+      <c r="A18" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="B18" s="46" t="s">
+        <v>110</v>
+      </c>
+      <c r="D18" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="E18" s="46" t="s">
+        <v>110</v>
+      </c>
+      <c r="G18" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="H18" s="46" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="19" ht="27.75" customHeight="1">
+      <c r="A19" s="48" t="s">
         <v>214</v>
       </c>
-      <c r="B17" s="34" t="s">
+      <c r="B19" s="48" t="s">
         <v>215</v>
       </c>
-      <c r="D17" s="38" t="s">
+      <c r="D19" s="48" t="s">
+        <v>216</v>
+      </c>
+      <c r="E19" s="48" t="s">
         <v>217</v>
       </c>
-      <c r="E17" s="34" t="s">
+      <c r="G19" s="48" t="s">
         <v>218</v>
       </c>
-      <c r="G17" s="38" t="s">
+      <c r="H19" s="48" t="s">
         <v>219</v>
       </c>
-      <c r="H17" s="34" t="s">
+    </row>
+    <row r="20" ht="18.0" customHeight="1">
+      <c r="A20" s="50" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="18" ht="15.0" customHeight="1">
-      <c r="A18" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="B18" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="D18" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="E18" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="G18" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="H18" s="40" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="19" ht="27.75" customHeight="1">
-      <c r="A19" s="43" t="s">
-        <v>223</v>
-      </c>
-      <c r="B19" s="43" t="s">
+      <c r="B20" s="16"/>
+      <c r="D20" s="50" t="s">
         <v>224</v>
       </c>
-      <c r="D19" s="43" t="s">
-        <v>225</v>
-      </c>
-      <c r="E19" s="43" t="s">
-        <v>226</v>
-      </c>
-      <c r="G19" s="43" t="s">
+      <c r="E20" s="16"/>
+      <c r="G20" s="50" t="s">
         <v>227</v>
       </c>
-      <c r="H19" s="43" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="20" ht="18.0" customHeight="1">
-      <c r="A20" s="46" t="s">
-        <v>230</v>
-      </c>
-      <c r="B20" s="18"/>
-      <c r="D20" s="46" t="s">
-        <v>231</v>
-      </c>
-      <c r="E20" s="18"/>
-      <c r="G20" s="46" t="s">
-        <v>232</v>
-      </c>
-      <c r="H20" s="18"/>
+      <c r="H20" s="16"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
     <row r="23" ht="15.75" customHeight="1"/>
     <row r="24" ht="21.75" customHeight="1">
-      <c r="A24" s="57" t="s">
+      <c r="A24" s="58" t="s">
+        <v>229</v>
+      </c>
+      <c r="B24" s="16"/>
+      <c r="D24" s="59" t="s">
+        <v>231</v>
+      </c>
+      <c r="E24" s="16"/>
+      <c r="G24" s="60" t="s">
         <v>233</v>
       </c>
-      <c r="B24" s="18"/>
-      <c r="D24" s="58" t="s">
-        <v>234</v>
-      </c>
-      <c r="E24" s="18"/>
-      <c r="G24" s="59" t="s">
-        <v>235</v>
-      </c>
-      <c r="H24" s="18"/>
+      <c r="H24" s="16"/>
     </row>
     <row r="25" ht="18.0" customHeight="1">
-      <c r="A25" s="21" t="s">
+      <c r="A25" s="24" t="s">
         <v>236</v>
       </c>
-      <c r="B25" s="18"/>
-      <c r="D25" s="21" t="s">
-        <v>237</v>
-      </c>
-      <c r="E25" s="18"/>
-      <c r="G25" s="21" t="s">
-        <v>63</v>
-      </c>
-      <c r="H25" s="18"/>
+      <c r="B25" s="16"/>
+      <c r="D25" s="24" t="s">
+        <v>238</v>
+      </c>
+      <c r="E25" s="16"/>
+      <c r="G25" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="H25" s="16"/>
     </row>
     <row r="26" ht="19.5" customHeight="1">
-      <c r="A26" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="B26" s="27" t="s">
+      <c r="A26" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="D26" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="E26" s="27" t="s">
+      <c r="B26" s="34" t="s">
+        <v>45</v>
+      </c>
+      <c r="D26" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="G26" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="H26" s="27" t="s">
+      <c r="E26" s="34" t="s">
+        <v>45</v>
+      </c>
+      <c r="G26" s="31" t="s">
         <v>35</v>
       </c>
+      <c r="H26" s="34" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="27" ht="42.0" customHeight="1">
-      <c r="A27" s="38" t="s">
-        <v>238</v>
-      </c>
-      <c r="B27" s="34" t="s">
+      <c r="A27" s="45" t="s">
         <v>239</v>
       </c>
-      <c r="D27" s="38" t="s">
+      <c r="B27" s="40" t="s">
         <v>240</v>
       </c>
-      <c r="E27" s="34" t="s">
+      <c r="D27" s="45" t="s">
         <v>241</v>
       </c>
-      <c r="G27" s="38" t="s">
+      <c r="E27" s="40" t="s">
         <v>242</v>
       </c>
-      <c r="H27" s="34" t="s">
+      <c r="G27" s="45" t="s">
         <v>243</v>
       </c>
+      <c r="H27" s="40" t="s">
+        <v>244</v>
+      </c>
     </row>
     <row r="28" ht="15.0" customHeight="1">
-      <c r="A28" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="B28" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="D28" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="E28" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="G28" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="H28" s="40" t="s">
-        <v>58</v>
+      <c r="A28" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="B28" s="46" t="s">
+        <v>110</v>
+      </c>
+      <c r="D28" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="E28" s="46" t="s">
+        <v>110</v>
+      </c>
+      <c r="G28" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="H28" s="46" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="29" ht="27.75" customHeight="1">
-      <c r="A29" s="43" t="s">
-        <v>244</v>
-      </c>
-      <c r="B29" s="43" t="s">
+      <c r="A29" s="48" t="s">
         <v>245</v>
       </c>
-      <c r="D29" s="43" t="s">
+      <c r="B29" s="48" t="s">
         <v>246</v>
       </c>
-      <c r="E29" s="43" t="s">
+      <c r="D29" s="48" t="s">
         <v>247</v>
       </c>
-      <c r="G29" s="43" t="s">
+      <c r="E29" s="48" t="s">
         <v>248</v>
       </c>
-      <c r="H29" s="43" t="s">
+      <c r="G29" s="48" t="s">
         <v>249</v>
       </c>
+      <c r="H29" s="48" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="30" ht="18.0" customHeight="1">
-      <c r="A30" s="46" t="s">
-        <v>250</v>
-      </c>
-      <c r="B30" s="18"/>
-      <c r="D30" s="46" t="s">
+      <c r="A30" s="50" t="s">
         <v>251</v>
       </c>
-      <c r="E30" s="18"/>
-      <c r="G30" s="46" t="s">
+      <c r="B30" s="16"/>
+      <c r="D30" s="50" t="s">
         <v>252</v>
       </c>
-      <c r="H30" s="18"/>
+      <c r="E30" s="16"/>
+      <c r="G30" s="50" t="s">
+        <v>253</v>
+      </c>
+      <c r="H30" s="16"/>
     </row>
     <row r="31" ht="15.75" customHeight="1"/>
     <row r="32" ht="15.75" customHeight="1"/>
     <row r="33" ht="15.75" customHeight="1"/>
     <row r="34" ht="21.75" customHeight="1">
-      <c r="A34" s="60" t="s">
-        <v>253</v>
-      </c>
-      <c r="B34" s="18"/>
-      <c r="D34" s="61" t="s">
+      <c r="A34" s="61" t="s">
         <v>254</v>
       </c>
-      <c r="E34" s="18"/>
-      <c r="G34" s="62" t="s">
+      <c r="B34" s="16"/>
+      <c r="D34" s="62" t="s">
         <v>255</v>
       </c>
-      <c r="H34" s="18"/>
+      <c r="E34" s="16"/>
+      <c r="G34" s="63" t="s">
+        <v>256</v>
+      </c>
+      <c r="H34" s="16"/>
     </row>
     <row r="35" ht="18.0" customHeight="1">
-      <c r="A35" s="21" t="s">
-        <v>256</v>
-      </c>
-      <c r="B35" s="18"/>
-      <c r="D35" s="21" t="s">
+      <c r="A35" s="24" t="s">
         <v>257</v>
       </c>
-      <c r="E35" s="18"/>
-      <c r="G35" s="51" t="s">
+      <c r="B35" s="16"/>
+      <c r="D35" s="24" t="s">
         <v>258</v>
       </c>
-      <c r="H35" s="18"/>
+      <c r="E35" s="16"/>
+      <c r="G35" s="55" t="s">
+        <v>259</v>
+      </c>
+      <c r="H35" s="16"/>
     </row>
     <row r="36" ht="19.5" customHeight="1">
-      <c r="A36" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="B36" s="27" t="s">
+      <c r="A36" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="D36" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="E36" s="27" t="s">
+      <c r="B36" s="34" t="s">
+        <v>45</v>
+      </c>
+      <c r="D36" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="G36" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="H36" s="27" t="s">
+      <c r="E36" s="34" t="s">
+        <v>45</v>
+      </c>
+      <c r="G36" s="31" t="s">
         <v>35</v>
       </c>
+      <c r="H36" s="34" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="37" ht="42.0" customHeight="1">
-      <c r="A37" s="38" t="s">
-        <v>259</v>
-      </c>
-      <c r="B37" s="34" t="s">
+      <c r="A37" s="45" t="s">
         <v>260</v>
       </c>
-      <c r="D37" s="38" t="s">
+      <c r="B37" s="40" t="s">
         <v>261</v>
       </c>
-      <c r="E37" s="34" t="s">
+      <c r="D37" s="45" t="s">
         <v>262</v>
       </c>
-      <c r="G37" s="38" t="s">
+      <c r="E37" s="40" t="s">
         <v>263</v>
       </c>
-      <c r="H37" s="34" t="s">
+      <c r="G37" s="45" t="s">
         <v>264</v>
       </c>
+      <c r="H37" s="40" t="s">
+        <v>265</v>
+      </c>
     </row>
     <row r="38" ht="15.0" customHeight="1">
-      <c r="A38" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="B38" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="D38" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="E38" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="G38" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="H38" s="40" t="s">
-        <v>58</v>
+      <c r="A38" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="B38" s="46" t="s">
+        <v>110</v>
+      </c>
+      <c r="D38" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="E38" s="46" t="s">
+        <v>110</v>
+      </c>
+      <c r="G38" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="H38" s="46" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="39" ht="27.75" customHeight="1">
-      <c r="A39" s="43" t="s">
-        <v>265</v>
-      </c>
-      <c r="B39" s="43" t="s">
+      <c r="A39" s="48" t="s">
         <v>266</v>
       </c>
-      <c r="D39" s="43" t="s">
+      <c r="B39" s="48" t="s">
         <v>267</v>
       </c>
-      <c r="E39" s="43" t="s">
+      <c r="D39" s="48" t="s">
         <v>268</v>
       </c>
-      <c r="G39" s="43" t="s">
+      <c r="E39" s="48" t="s">
         <v>269</v>
       </c>
-      <c r="H39" s="43" t="s">
-        <v>121</v>
+      <c r="G39" s="48" t="s">
+        <v>270</v>
+      </c>
+      <c r="H39" s="48" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="40" ht="18.0" customHeight="1">
-      <c r="A40" s="46" t="s">
-        <v>270</v>
-      </c>
-      <c r="B40" s="18"/>
-      <c r="D40" s="46" t="s">
+      <c r="A40" s="50" t="s">
         <v>271</v>
       </c>
-      <c r="E40" s="18"/>
-      <c r="G40" s="46" t="s">
+      <c r="B40" s="16"/>
+      <c r="D40" s="50" t="s">
         <v>272</v>
       </c>
-      <c r="H40" s="18"/>
+      <c r="E40" s="16"/>
+      <c r="G40" s="50" t="s">
+        <v>273</v>
+      </c>
+      <c r="H40" s="16"/>
     </row>
     <row r="41" ht="15.75" customHeight="1"/>
     <row r="42" ht="15.75" customHeight="1"/>
     <row r="43" ht="15.75" customHeight="1"/>
     <row r="44" ht="21.75" customHeight="1">
-      <c r="A44" s="63" t="s">
-        <v>273</v>
-      </c>
-      <c r="B44" s="18"/>
-      <c r="D44" s="64" t="s">
+      <c r="A44" s="64" t="s">
         <v>274</v>
       </c>
-      <c r="E44" s="18"/>
-      <c r="G44" s="65" t="s">
+      <c r="B44" s="16"/>
+      <c r="D44" s="65" t="s">
         <v>275</v>
       </c>
-      <c r="H44" s="18"/>
+      <c r="E44" s="16"/>
+      <c r="G44" s="66" t="s">
+        <v>276</v>
+      </c>
+      <c r="H44" s="16"/>
     </row>
     <row r="45" ht="18.0" customHeight="1">
-      <c r="A45" s="21" t="s">
-        <v>276</v>
-      </c>
-      <c r="B45" s="18"/>
-      <c r="D45" s="21" t="s">
-        <v>63</v>
-      </c>
-      <c r="E45" s="18"/>
-      <c r="G45" s="21" t="s">
-        <v>63</v>
-      </c>
-      <c r="H45" s="18"/>
+      <c r="A45" s="24" t="s">
+        <v>277</v>
+      </c>
+      <c r="B45" s="16"/>
+      <c r="D45" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="E45" s="16"/>
+      <c r="G45" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="H45" s="16"/>
     </row>
     <row r="46" ht="19.5" customHeight="1">
-      <c r="A46" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="B46" s="27" t="s">
+      <c r="A46" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="D46" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="E46" s="27" t="s">
+      <c r="B46" s="34" t="s">
+        <v>45</v>
+      </c>
+      <c r="D46" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="G46" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="H46" s="27" t="s">
+      <c r="E46" s="34" t="s">
+        <v>45</v>
+      </c>
+      <c r="G46" s="31" t="s">
         <v>35</v>
       </c>
+      <c r="H46" s="34" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="47" ht="42.0" customHeight="1">
-      <c r="A47" s="38" t="s">
-        <v>277</v>
-      </c>
-      <c r="B47" s="34" t="s">
+      <c r="A47" s="45" t="s">
         <v>278</v>
       </c>
-      <c r="D47" s="38" t="s">
+      <c r="B47" s="40" t="s">
         <v>279</v>
       </c>
-      <c r="E47" s="34" t="s">
+      <c r="D47" s="45" t="s">
         <v>280</v>
       </c>
-      <c r="G47" s="38" t="s">
+      <c r="E47" s="40" t="s">
         <v>281</v>
       </c>
-      <c r="H47" s="34" t="s">
+      <c r="G47" s="45" t="s">
         <v>282</v>
       </c>
+      <c r="H47" s="40" t="s">
+        <v>283</v>
+      </c>
     </row>
     <row r="48" ht="15.0" customHeight="1">
-      <c r="A48" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="B48" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="D48" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="E48" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="G48" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="H48" s="40" t="s">
-        <v>58</v>
+      <c r="A48" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="B48" s="46" t="s">
+        <v>110</v>
+      </c>
+      <c r="D48" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="E48" s="46" t="s">
+        <v>110</v>
+      </c>
+      <c r="G48" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="H48" s="46" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="49" ht="27.75" customHeight="1">
-      <c r="A49" s="43" t="s">
-        <v>283</v>
-      </c>
-      <c r="B49" s="43" t="s">
+      <c r="A49" s="48" t="s">
         <v>284</v>
       </c>
-      <c r="D49" s="43" t="s">
+      <c r="B49" s="48" t="s">
         <v>285</v>
       </c>
-      <c r="E49" s="43" t="s">
+      <c r="D49" s="48" t="s">
         <v>286</v>
       </c>
-      <c r="G49" s="43" t="s">
+      <c r="E49" s="48" t="s">
         <v>287</v>
       </c>
-      <c r="H49" s="43" t="s">
+      <c r="G49" s="48" t="s">
         <v>288</v>
       </c>
+      <c r="H49" s="48" t="s">
+        <v>289</v>
+      </c>
     </row>
     <row r="50" ht="18.0" customHeight="1">
-      <c r="A50" s="46" t="s">
-        <v>289</v>
-      </c>
-      <c r="B50" s="18"/>
-      <c r="D50" s="46" t="s">
+      <c r="A50" s="50" t="s">
         <v>290</v>
       </c>
-      <c r="E50" s="18"/>
-      <c r="G50" s="46" t="s">
+      <c r="B50" s="16"/>
+      <c r="D50" s="50" t="s">
         <v>291</v>
       </c>
-      <c r="H50" s="18"/>
+      <c r="E50" s="16"/>
+      <c r="G50" s="50" t="s">
+        <v>292</v>
+      </c>
+      <c r="H50" s="16"/>
     </row>
     <row r="51" ht="15.75" customHeight="1"/>
     <row r="52" ht="15.75" customHeight="1"/>
     <row r="53" ht="15.75" customHeight="1"/>
     <row r="54" ht="21.75" customHeight="1">
-      <c r="A54" s="66" t="s">
-        <v>292</v>
-      </c>
-      <c r="B54" s="18"/>
-      <c r="D54" s="67" t="s">
+      <c r="A54" s="67" t="s">
         <v>293</v>
       </c>
-      <c r="E54" s="18"/>
-      <c r="G54" s="68" t="s">
+      <c r="B54" s="16"/>
+      <c r="D54" s="68" t="s">
         <v>294</v>
       </c>
-      <c r="H54" s="18"/>
+      <c r="E54" s="16"/>
+      <c r="G54" s="69" t="s">
+        <v>295</v>
+      </c>
+      <c r="H54" s="16"/>
     </row>
     <row r="55" ht="18.0" customHeight="1">
-      <c r="A55" s="21" t="s">
-        <v>295</v>
-      </c>
-      <c r="B55" s="18"/>
-      <c r="D55" s="21" t="s">
+      <c r="A55" s="24" t="s">
         <v>296</v>
       </c>
-      <c r="E55" s="18"/>
-      <c r="G55" s="21" t="s">
-        <v>63</v>
-      </c>
-      <c r="H55" s="18"/>
+      <c r="B55" s="16"/>
+      <c r="D55" s="24" t="s">
+        <v>297</v>
+      </c>
+      <c r="E55" s="16"/>
+      <c r="G55" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="H55" s="16"/>
     </row>
     <row r="56" ht="19.5" customHeight="1">
-      <c r="A56" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="B56" s="27" t="s">
+      <c r="A56" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="D56" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="E56" s="27" t="s">
+      <c r="B56" s="34" t="s">
+        <v>45</v>
+      </c>
+      <c r="D56" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="G56" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="H56" s="27" t="s">
+      <c r="E56" s="34" t="s">
+        <v>45</v>
+      </c>
+      <c r="G56" s="31" t="s">
         <v>35</v>
       </c>
+      <c r="H56" s="34" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="57" ht="42.0" customHeight="1">
-      <c r="A57" s="38" t="s">
-        <v>297</v>
-      </c>
-      <c r="B57" s="34" t="s">
+      <c r="A57" s="45" t="s">
         <v>298</v>
       </c>
-      <c r="D57" s="38" t="s">
-        <v>53</v>
-      </c>
-      <c r="E57" s="34" t="s">
+      <c r="B57" s="40" t="s">
         <v>299</v>
       </c>
-      <c r="G57" s="38" t="s">
+      <c r="D57" s="45" t="s">
+        <v>101</v>
+      </c>
+      <c r="E57" s="40" t="s">
         <v>300</v>
       </c>
-      <c r="H57" s="34" t="s">
+      <c r="G57" s="45" t="s">
         <v>301</v>
       </c>
+      <c r="H57" s="40" t="s">
+        <v>302</v>
+      </c>
     </row>
     <row r="58" ht="15.0" customHeight="1">
-      <c r="A58" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="B58" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="D58" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="E58" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="G58" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="H58" s="40" t="s">
-        <v>58</v>
+      <c r="A58" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="B58" s="46" t="s">
+        <v>110</v>
+      </c>
+      <c r="D58" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="E58" s="46" t="s">
+        <v>110</v>
+      </c>
+      <c r="G58" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="H58" s="46" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="59" ht="27.75" customHeight="1">
-      <c r="A59" s="43" t="s">
-        <v>302</v>
-      </c>
-      <c r="B59" s="43" t="s">
+      <c r="A59" s="48" t="s">
         <v>303</v>
       </c>
-      <c r="D59" s="43" t="s">
+      <c r="B59" s="48" t="s">
         <v>304</v>
       </c>
-      <c r="E59" s="43" t="s">
+      <c r="D59" s="48" t="s">
         <v>305</v>
       </c>
-      <c r="G59" s="43" t="s">
+      <c r="E59" s="48" t="s">
         <v>306</v>
       </c>
-      <c r="H59" s="43" t="s">
+      <c r="G59" s="48" t="s">
         <v>307</v>
       </c>
+      <c r="H59" s="48" t="s">
+        <v>308</v>
+      </c>
     </row>
     <row r="60" ht="18.0" customHeight="1">
-      <c r="A60" s="46" t="s">
-        <v>308</v>
-      </c>
-      <c r="B60" s="18"/>
-      <c r="D60" s="46" t="s">
+      <c r="A60" s="50" t="s">
         <v>309</v>
       </c>
-      <c r="E60" s="18"/>
-      <c r="G60" s="46" t="s">
+      <c r="B60" s="16"/>
+      <c r="D60" s="50" t="s">
         <v>310</v>
       </c>
-      <c r="H60" s="18"/>
+      <c r="E60" s="16"/>
+      <c r="G60" s="50" t="s">
+        <v>311</v>
+      </c>
+      <c r="H60" s="16"/>
     </row>
     <row r="61" ht="15.75" customHeight="1"/>
     <row r="62" ht="15.75" customHeight="1"/>
@@ -4877,11 +4901,11 @@
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
-      <c r="H1" s="4"/>
+      <c r="H1" s="5"/>
     </row>
     <row r="2" ht="19.5" customHeight="1">
-      <c r="A2" s="12" t="s">
-        <v>3</v>
+      <c r="A2" s="11" t="s">
+        <v>5</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -4889,304 +4913,304 @@
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
-      <c r="H2" s="4"/>
+      <c r="H2" s="5"/>
     </row>
     <row r="4" ht="21.75" customHeight="1">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="16"/>
+      <c r="D4" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="18"/>
-      <c r="D4" s="16" t="s">
+      <c r="E4" s="16"/>
+      <c r="G4" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="H4" s="16"/>
+    </row>
+    <row r="5" ht="18.0" customHeight="1">
+      <c r="A5" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="18"/>
-      <c r="G4" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="H4" s="18"/>
-    </row>
-    <row r="5" ht="18.0" customHeight="1">
-      <c r="A5" s="21" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="18"/>
-      <c r="D5" s="21" t="s">
+      <c r="B5" s="16"/>
+      <c r="D5" s="24" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="16"/>
+      <c r="G5" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="18"/>
-      <c r="G5" s="21" t="s">
-        <v>32</v>
-      </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="16"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="B6" s="27" t="s">
+      <c r="A6" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="D6" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="E6" s="27" t="s">
+      <c r="B6" s="34" t="s">
+        <v>45</v>
+      </c>
+      <c r="D6" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="G6" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="H6" s="27" t="s">
+      <c r="E6" s="34" t="s">
+        <v>45</v>
+      </c>
+      <c r="G6" s="31" t="s">
         <v>35</v>
       </c>
+      <c r="H6" s="34" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="7" ht="42.0" customHeight="1">
-      <c r="A7" s="32" t="s">
-        <v>38</v>
-      </c>
-      <c r="B7" s="34" t="s">
+      <c r="A7" s="38" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7" s="40" t="s">
+        <v>57</v>
+      </c>
+      <c r="D7" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="E7" s="40" t="s">
+        <v>95</v>
+      </c>
+      <c r="G7" s="45" t="s">
+        <v>101</v>
+      </c>
+      <c r="H7" s="40" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="8" ht="15.0" customHeight="1">
+      <c r="A8" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="B8" s="46" t="s">
+        <v>110</v>
+      </c>
+      <c r="D8" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="E8" s="46" t="s">
+        <v>110</v>
+      </c>
+      <c r="G8" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="H8" s="46" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="9" ht="27.75" customHeight="1">
+      <c r="A9" s="48" t="s">
+        <v>114</v>
+      </c>
+      <c r="B9" s="48" t="s">
+        <v>130</v>
+      </c>
+      <c r="D9" s="48" t="s">
+        <v>132</v>
+      </c>
+      <c r="E9" s="48" t="s">
+        <v>135</v>
+      </c>
+      <c r="G9" s="48" t="s">
+        <v>139</v>
+      </c>
+      <c r="H9" s="48" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="10" ht="18.0" customHeight="1">
+      <c r="A10" s="50" t="s">
+        <v>149</v>
+      </c>
+      <c r="B10" s="16"/>
+      <c r="D10" s="50" t="s">
+        <v>159</v>
+      </c>
+      <c r="E10" s="16"/>
+      <c r="G10" s="50" t="s">
+        <v>167</v>
+      </c>
+      <c r="H10" s="16"/>
+    </row>
+    <row r="14" ht="21.75" customHeight="1">
+      <c r="A14" s="13" t="s">
+        <v>178</v>
+      </c>
+      <c r="B14" s="16"/>
+      <c r="D14" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="E14" s="16"/>
+      <c r="G14" s="53" t="s">
+        <v>193</v>
+      </c>
+      <c r="H14" s="16"/>
+    </row>
+    <row r="15" ht="18.0" customHeight="1">
+      <c r="A15" s="24" t="s">
+        <v>197</v>
+      </c>
+      <c r="B15" s="16"/>
+      <c r="D15" s="24" t="s">
+        <v>198</v>
+      </c>
+      <c r="E15" s="16"/>
+      <c r="G15" s="55" t="s">
+        <v>199</v>
+      </c>
+      <c r="H15" s="16"/>
+    </row>
+    <row r="16" ht="19.5" customHeight="1">
+      <c r="A16" s="31" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="D7" s="38" t="s">
-        <v>48</v>
-      </c>
-      <c r="E7" s="34" t="s">
-        <v>52</v>
-      </c>
-      <c r="G7" s="38" t="s">
-        <v>53</v>
-      </c>
-      <c r="H7" s="34" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="B8" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="D8" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="E8" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="G8" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="H8" s="40" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" ht="27.75" customHeight="1">
-      <c r="A9" s="43" t="s">
-        <v>60</v>
-      </c>
-      <c r="B9" s="43" t="s">
-        <v>65</v>
-      </c>
-      <c r="D9" s="43" t="s">
-        <v>66</v>
-      </c>
-      <c r="E9" s="43" t="s">
-        <v>67</v>
-      </c>
-      <c r="G9" s="43" t="s">
-        <v>68</v>
-      </c>
-      <c r="H9" s="43" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="10" ht="18.0" customHeight="1">
-      <c r="A10" s="46" t="s">
-        <v>71</v>
-      </c>
-      <c r="B10" s="18"/>
-      <c r="D10" s="46" t="s">
-        <v>77</v>
-      </c>
-      <c r="E10" s="18"/>
-      <c r="G10" s="46" t="s">
-        <v>113</v>
-      </c>
-      <c r="H10" s="18"/>
-    </row>
-    <row r="14" ht="21.75" customHeight="1">
-      <c r="A14" s="16" t="s">
-        <v>114</v>
-      </c>
-      <c r="B14" s="18"/>
-      <c r="D14" s="16" t="s">
-        <v>117</v>
-      </c>
-      <c r="E14" s="18"/>
-      <c r="G14" s="50" t="s">
-        <v>128</v>
-      </c>
-      <c r="H14" s="18"/>
-    </row>
-    <row r="15" ht="18.0" customHeight="1">
-      <c r="A15" s="21" t="s">
-        <v>142</v>
-      </c>
-      <c r="B15" s="18"/>
-      <c r="D15" s="21" t="s">
-        <v>149</v>
-      </c>
-      <c r="E15" s="18"/>
-      <c r="G15" s="51" t="s">
-        <v>157</v>
-      </c>
-      <c r="H15" s="18"/>
-    </row>
-    <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="B16" s="27" t="s">
+      <c r="D16" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="D16" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="E16" s="27" t="s">
+      <c r="E16" s="34" t="s">
+        <v>45</v>
+      </c>
+      <c r="G16" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="G16" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="H16" s="27" t="s">
-        <v>35</v>
+      <c r="H16" s="34" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="17" ht="42.0" customHeight="1">
-      <c r="A17" s="38" t="s">
-        <v>174</v>
-      </c>
-      <c r="B17" s="34" t="s">
-        <v>176</v>
-      </c>
-      <c r="D17" s="38" t="s">
-        <v>178</v>
-      </c>
-      <c r="E17" s="53" t="s">
-        <v>184</v>
-      </c>
-      <c r="G17" s="32" t="s">
-        <v>190</v>
-      </c>
-      <c r="H17" s="53" t="s">
-        <v>192</v>
+      <c r="A17" s="45" t="s">
+        <v>202</v>
+      </c>
+      <c r="B17" s="40" t="s">
+        <v>203</v>
+      </c>
+      <c r="D17" s="45" t="s">
+        <v>205</v>
+      </c>
+      <c r="E17" s="56" t="s">
+        <v>210</v>
+      </c>
+      <c r="G17" s="38" t="s">
+        <v>212</v>
+      </c>
+      <c r="H17" s="56" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="18" ht="15.0" customHeight="1">
-      <c r="A18" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="B18" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="D18" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="E18" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="G18" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="H18" s="40" t="s">
-        <v>58</v>
+      <c r="A18" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="B18" s="46" t="s">
+        <v>110</v>
+      </c>
+      <c r="D18" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="E18" s="46" t="s">
+        <v>110</v>
+      </c>
+      <c r="G18" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="H18" s="46" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="19" ht="27.75" customHeight="1">
-      <c r="A19" s="43" t="s">
-        <v>199</v>
-      </c>
-      <c r="B19" s="43" t="s">
-        <v>201</v>
-      </c>
-      <c r="D19" s="43" t="s">
-        <v>207</v>
-      </c>
-      <c r="E19" s="43" t="s">
-        <v>121</v>
-      </c>
-      <c r="G19" s="43" t="s">
-        <v>121</v>
-      </c>
-      <c r="H19" s="43" t="s">
-        <v>121</v>
+      <c r="A19" s="48" t="s">
+        <v>221</v>
+      </c>
+      <c r="B19" s="48" t="s">
+        <v>222</v>
+      </c>
+      <c r="D19" s="48" t="s">
+        <v>223</v>
+      </c>
+      <c r="E19" s="48" t="s">
+        <v>115</v>
+      </c>
+      <c r="G19" s="48" t="s">
+        <v>115</v>
+      </c>
+      <c r="H19" s="48" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="20" ht="18.0" customHeight="1">
-      <c r="A20" s="46" t="s">
-        <v>208</v>
-      </c>
-      <c r="B20" s="18"/>
-      <c r="D20" s="46" t="s">
-        <v>210</v>
-      </c>
-      <c r="E20" s="18"/>
-      <c r="G20" s="56" t="s">
-        <v>212</v>
-      </c>
-      <c r="H20" s="18"/>
+      <c r="A20" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B20" s="16"/>
+      <c r="D20" s="50" t="s">
+        <v>226</v>
+      </c>
+      <c r="E20" s="16"/>
+      <c r="G20" s="57" t="s">
+        <v>228</v>
+      </c>
+      <c r="H20" s="16"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
     <row r="23" ht="15.75" customHeight="1"/>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="50" t="s">
-        <v>213</v>
-      </c>
-      <c r="B24" s="18"/>
+      <c r="A24" s="53" t="s">
+        <v>230</v>
+      </c>
+      <c r="B24" s="16"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="51" t="s">
-        <v>216</v>
-      </c>
-      <c r="B25" s="18"/>
+      <c r="A25" s="55" t="s">
+        <v>232</v>
+      </c>
+      <c r="B25" s="16"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="B26" s="27" t="s">
+      <c r="A26" s="31" t="s">
         <v>35</v>
       </c>
+      <c r="B26" s="34" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="27" ht="44.25" customHeight="1">
-      <c r="A27" s="32" t="s">
-        <v>221</v>
-      </c>
-      <c r="B27" s="53" t="s">
-        <v>222</v>
+      <c r="A27" s="38" t="s">
+        <v>234</v>
+      </c>
+      <c r="B27" s="56" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="B28" s="40" t="s">
-        <v>58</v>
+      <c r="A28" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="B28" s="46" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="29" ht="27.75" customHeight="1">
-      <c r="A29" s="43" t="s">
-        <v>121</v>
-      </c>
-      <c r="B29" s="43" t="s">
-        <v>121</v>
+      <c r="A29" s="48" t="s">
+        <v>115</v>
+      </c>
+      <c r="B29" s="48" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="B30" s="18"/>
+      <c r="A30" s="57" t="s">
+        <v>237</v>
+      </c>
+      <c r="B30" s="16"/>
     </row>
     <row r="31" ht="15.75" customHeight="1"/>
     <row r="32" ht="15.75" customHeight="1"/>
@@ -6210,438 +6234,438 @@
   </cols>
   <sheetData>
     <row r="1" ht="27.75" customHeight="1">
-      <c r="A1" s="7" t="s">
-        <v>5</v>
+      <c r="A1" s="6" t="s">
+        <v>3</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
-      <c r="E1" s="4"/>
+      <c r="E1" s="5"/>
     </row>
     <row r="2" ht="18.0" customHeight="1">
-      <c r="A2" s="11"/>
+      <c r="A2" s="9"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
-      <c r="E2" s="4"/>
+      <c r="E2" s="5"/>
     </row>
     <row r="3">
-      <c r="B3" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="D3" s="19" t="s">
-        <v>3</v>
+      <c r="B3" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="4" ht="24.0" customHeight="1">
-      <c r="A4" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="C4" s="29" t="s">
-        <v>39</v>
-      </c>
-      <c r="D4" s="29" t="s">
-        <v>40</v>
-      </c>
-      <c r="E4" s="22" t="s">
-        <v>41</v>
+      <c r="A4" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="5" ht="21.75" customHeight="1">
-      <c r="A5" s="33" t="s">
-        <v>42</v>
-      </c>
-      <c r="B5" s="35" t="s">
-        <v>47</v>
-      </c>
-      <c r="C5" s="37" t="s">
-        <v>49</v>
-      </c>
-      <c r="D5" s="39" t="s">
-        <v>51</v>
-      </c>
-      <c r="E5" s="42" t="s">
-        <v>57</v>
+      <c r="A5" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="26" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="28" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="29" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="6" ht="21.75" customHeight="1">
-      <c r="A6" s="44" t="s">
+      <c r="A6" s="32" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="36" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="D6" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="E6" s="39" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" ht="21.75" customHeight="1">
+      <c r="A7" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="B7" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="45" t="s">
+      <c r="C7" s="26" t="s">
+        <v>63</v>
+      </c>
+      <c r="D7" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="E7" s="29" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="8" ht="21.75" customHeight="1">
+      <c r="A8" s="32" t="s">
+        <v>66</v>
+      </c>
+      <c r="B8" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="D8" s="28" t="s">
+        <v>69</v>
+      </c>
+      <c r="E8" s="39" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" ht="21.75" customHeight="1">
+      <c r="A9" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="C6" s="37" t="s">
+      <c r="B9" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="D6" s="39" t="s">
+      <c r="D9" s="28" t="s">
         <v>75</v>
       </c>
-      <c r="E6" s="47" t="s">
+      <c r="E9" s="29" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="7" ht="21.75" customHeight="1">
-      <c r="A7" s="33" t="s">
+    <row r="10" ht="21.75" customHeight="1">
+      <c r="A10" s="32" t="s">
+        <v>77</v>
+      </c>
+      <c r="B10" s="36" t="s">
         <v>78</v>
       </c>
-      <c r="B7" s="35" t="s">
+      <c r="C10" s="26" t="s">
         <v>79</v>
       </c>
-      <c r="C7" s="37" t="s">
+      <c r="D10" s="28" t="s">
         <v>80</v>
       </c>
-      <c r="D7" s="39" t="s">
+      <c r="E10" s="39" t="s">
         <v>81</v>
       </c>
-      <c r="E7" s="42" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="8" ht="21.75" customHeight="1">
-      <c r="A8" s="44" t="s">
+    </row>
+    <row r="11" ht="21.75" customHeight="1">
+      <c r="A11" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="B8" s="45" t="s">
-        <v>47</v>
-      </c>
-      <c r="C8" s="37" t="s">
+      <c r="B11" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="D8" s="39" t="s">
+      <c r="C11" s="26" t="s">
         <v>85</v>
       </c>
-      <c r="E8" s="47" t="s">
+      <c r="D11" s="28" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="9" ht="21.75" customHeight="1">
-      <c r="A9" s="33" t="s">
+      <c r="E11" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="B9" s="35" t="s">
+    </row>
+    <row r="12" ht="21.75" customHeight="1">
+      <c r="A12" s="32" t="s">
         <v>88</v>
       </c>
-      <c r="C9" s="37" t="s">
-        <v>89</v>
-      </c>
-      <c r="D9" s="39" t="s">
-        <v>90</v>
-      </c>
-      <c r="E9" s="42" t="s">
+      <c r="B12" s="36" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="10" ht="21.75" customHeight="1">
-      <c r="A10" s="44" t="s">
-        <v>92</v>
-      </c>
-      <c r="B10" s="45" t="s">
+      <c r="C12" s="26" t="s">
         <v>93</v>
       </c>
-      <c r="C10" s="37" t="s">
-        <v>95</v>
-      </c>
-      <c r="D10" s="39" t="s">
+      <c r="D12" s="28" t="s">
         <v>96</v>
       </c>
-      <c r="E10" s="47" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="11" ht="21.75" customHeight="1">
-      <c r="A11" s="33" t="s">
+      <c r="E12" s="39" t="s">
         <v>99</v>
       </c>
-      <c r="B11" s="35" t="s">
+    </row>
+    <row r="13" ht="21.75" customHeight="1">
+      <c r="A13" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="C11" s="37" t="s">
-        <v>101</v>
-      </c>
-      <c r="D11" s="39" t="s">
-        <v>102</v>
-      </c>
-      <c r="E11" s="42" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="12" ht="21.75" customHeight="1">
-      <c r="A12" s="44" t="s">
+      <c r="B13" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" s="26" t="s">
+        <v>104</v>
+      </c>
+      <c r="D13" s="28" t="s">
         <v>105</v>
       </c>
-      <c r="B12" s="45" t="s">
+      <c r="E13" s="29" t="s">
         <v>106</v>
       </c>
-      <c r="C12" s="37" t="s">
+    </row>
+    <row r="14" ht="21.75" customHeight="1">
+      <c r="A14" s="32" t="s">
         <v>107</v>
       </c>
-      <c r="D12" s="39" t="s">
+      <c r="B14" s="36" t="s">
         <v>108</v>
       </c>
-      <c r="E12" s="47" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="13" ht="21.75" customHeight="1">
-      <c r="A13" s="33" t="s">
+      <c r="C14" s="26" t="s">
+        <v>112</v>
+      </c>
+      <c r="D14" s="28" t="s">
         <v>116</v>
       </c>
-      <c r="B13" s="35" t="s">
-        <v>47</v>
-      </c>
-      <c r="C13" s="37" t="s">
+      <c r="E14" s="39" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="15" ht="21.75" customHeight="1">
+      <c r="A15" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="D13" s="39" t="s">
+      <c r="B15" s="22" t="s">
         <v>119</v>
       </c>
-      <c r="E13" s="42" t="s">
+      <c r="C15" s="26" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="14" ht="21.75" customHeight="1">
-      <c r="A14" s="44" t="s">
+      <c r="D15" s="28" t="s">
         <v>122</v>
       </c>
-      <c r="B14" s="45" t="s">
+      <c r="E15" s="29" t="s">
         <v>123</v>
       </c>
-      <c r="C14" s="37" t="s">
-        <v>124</v>
-      </c>
-      <c r="D14" s="39" t="s">
+    </row>
+    <row r="16" ht="21.75" customHeight="1">
+      <c r="A16" s="32" t="s">
+        <v>125</v>
+      </c>
+      <c r="B16" s="36" t="s">
         <v>126</v>
       </c>
-      <c r="E14" s="47" t="s">
+      <c r="C16" s="26" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="15" ht="21.75" customHeight="1">
-      <c r="A15" s="33" t="s">
-        <v>129</v>
-      </c>
-      <c r="B15" s="35" t="s">
-        <v>131</v>
-      </c>
-      <c r="C15" s="37" t="s">
-        <v>132</v>
-      </c>
-      <c r="D15" s="39" t="s">
+      <c r="D16" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="E16" s="39" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="17" ht="21.75" customHeight="1">
+      <c r="A17" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="E15" s="42" t="s">
+      <c r="B17" s="22" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="16" ht="21.75" customHeight="1">
-      <c r="A16" s="44" t="s">
+      <c r="C17" s="26" t="s">
         <v>136</v>
       </c>
-      <c r="B16" s="45" t="s">
-        <v>137</v>
-      </c>
-      <c r="C16" s="37" t="s">
-        <v>139</v>
-      </c>
-      <c r="D16" s="39" t="s">
+      <c r="D17" s="28" t="s">
+        <v>138</v>
+      </c>
+      <c r="E17" s="29" t="s">
         <v>140</v>
       </c>
-      <c r="E16" s="47" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="17" ht="21.75" customHeight="1">
-      <c r="A17" s="33" t="s">
+    </row>
+    <row r="18" ht="21.75" customHeight="1">
+      <c r="A18" s="32" t="s">
         <v>141</v>
       </c>
-      <c r="B17" s="35" t="s">
+      <c r="B18" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18" s="26" t="s">
         <v>143</v>
       </c>
-      <c r="C17" s="37" t="s">
+      <c r="D18" s="28" t="s">
+        <v>144</v>
+      </c>
+      <c r="E18" s="39" t="s">
         <v>145</v>
       </c>
-      <c r="D17" s="39" t="s">
+    </row>
+    <row r="19" ht="21.75" customHeight="1">
+      <c r="A19" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" s="26" t="s">
         <v>146</v>
       </c>
-      <c r="E17" s="42" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="18" ht="21.75" customHeight="1">
-      <c r="A18" s="44" t="s">
+      <c r="D19" s="28" t="s">
         <v>148</v>
       </c>
-      <c r="B18" s="45" t="s">
-        <v>47</v>
-      </c>
-      <c r="C18" s="37" t="s">
+      <c r="E19" s="29" t="s">
         <v>150</v>
       </c>
-      <c r="D18" s="39" t="s">
+    </row>
+    <row r="20" ht="21.75" customHeight="1">
+      <c r="A20" s="32" t="s">
         <v>151</v>
       </c>
-      <c r="E18" s="47" t="s">
+      <c r="B20" s="36" t="s">
+        <v>152</v>
+      </c>
+      <c r="C20" s="26" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="19" ht="21.75" customHeight="1">
-      <c r="A19" s="33" t="s">
-        <v>110</v>
-      </c>
-      <c r="B19" s="35" t="s">
-        <v>47</v>
-      </c>
-      <c r="C19" s="37" t="s">
+      <c r="D20" s="28" t="s">
         <v>154</v>
       </c>
-      <c r="D19" s="39" t="s">
+      <c r="E20" s="39" t="s">
         <v>155</v>
       </c>
-      <c r="E19" s="42" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="20" ht="21.75" customHeight="1">
-      <c r="A20" s="44" t="s">
+    </row>
+    <row r="21" ht="21.75" customHeight="1">
+      <c r="A21" s="19" t="s">
+        <v>157</v>
+      </c>
+      <c r="B21" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="B20" s="45" t="s">
+      <c r="C21" s="26" t="s">
         <v>160</v>
       </c>
-      <c r="C20" s="37" t="s">
+      <c r="D21" s="28" t="s">
         <v>161</v>
       </c>
-      <c r="D20" s="39" t="s">
+      <c r="E21" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="E20" s="47" t="s">
+    </row>
+    <row r="22" ht="21.75" customHeight="1">
+      <c r="A22" s="32" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="21" ht="21.75" customHeight="1">
-      <c r="A21" s="33" t="s">
+      <c r="B22" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="C22" s="26" t="s">
         <v>164</v>
       </c>
-      <c r="B21" s="35" t="s">
+      <c r="D22" s="28" t="s">
         <v>165</v>
       </c>
-      <c r="C21" s="37" t="s">
+      <c r="E22" s="39" t="s">
         <v>166</v>
       </c>
-      <c r="D21" s="39" t="s">
-        <v>167</v>
-      </c>
-      <c r="E21" s="42" t="s">
+    </row>
+    <row r="23" ht="21.75" customHeight="1">
+      <c r="A23" s="19" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="22" ht="21.75" customHeight="1">
-      <c r="A22" s="44" t="s">
+      <c r="B23" s="22" t="s">
         <v>169</v>
       </c>
-      <c r="B22" s="45" t="s">
-        <v>47</v>
-      </c>
-      <c r="C22" s="37" t="s">
-        <v>171</v>
-      </c>
-      <c r="D22" s="39" t="s">
+      <c r="C23" s="26" t="s">
+        <v>170</v>
+      </c>
+      <c r="D23" s="28" t="s">
         <v>172</v>
       </c>
-      <c r="E22" s="47" t="s">
+      <c r="E23" s="29" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="23" ht="21.75" customHeight="1">
-      <c r="A23" s="33" t="s">
+    <row r="24" ht="21.75" customHeight="1">
+      <c r="A24" s="32" t="s">
+        <v>174</v>
+      </c>
+      <c r="B24" s="36" t="s">
         <v>175</v>
       </c>
-      <c r="B23" s="35" t="s">
+      <c r="C24" s="26" t="s">
+        <v>176</v>
+      </c>
+      <c r="D24" s="28" t="s">
         <v>177</v>
       </c>
-      <c r="C23" s="37" t="s">
+      <c r="E24" s="39" t="s">
         <v>179</v>
       </c>
-      <c r="D23" s="39" t="s">
+    </row>
+    <row r="25" ht="21.75" customHeight="1">
+      <c r="A25" s="19" t="s">
         <v>180</v>
       </c>
-      <c r="E23" s="42" t="s">
+      <c r="B25" s="22" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="24" ht="21.75" customHeight="1">
-      <c r="A24" s="44" t="s">
+      <c r="C25" s="26" t="s">
+        <v>160</v>
+      </c>
+      <c r="D25" s="28" t="s">
         <v>183</v>
       </c>
-      <c r="B24" s="45" t="s">
+      <c r="E25" s="29" t="s">
         <v>185</v>
       </c>
-      <c r="C24" s="37" t="s">
+    </row>
+    <row r="26" ht="21.75" customHeight="1">
+      <c r="A26" s="32" t="s">
         <v>186</v>
       </c>
-      <c r="D24" s="39" t="s">
+      <c r="B26" s="36" t="s">
         <v>187</v>
       </c>
-      <c r="E24" s="47" t="s">
+      <c r="C26" s="26" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="25" ht="21.75" customHeight="1">
-      <c r="A25" s="33" t="s">
+      <c r="D26" s="28" t="s">
         <v>189</v>
       </c>
-      <c r="B25" s="35" t="s">
+      <c r="E26" s="39" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="27" ht="21.75" customHeight="1">
+      <c r="A27" s="19" t="s">
         <v>191</v>
       </c>
-      <c r="C25" s="37" t="s">
-        <v>166</v>
-      </c>
-      <c r="D25" s="39" t="s">
-        <v>194</v>
-      </c>
-      <c r="E25" s="42" t="s">
+      <c r="B27" s="22" t="s">
+        <v>192</v>
+      </c>
+      <c r="C27" s="26" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="26" ht="21.75" customHeight="1">
-      <c r="A26" s="44" t="s">
+      <c r="D27" s="28" t="s">
         <v>196</v>
       </c>
-      <c r="B26" s="45" t="s">
-        <v>197</v>
-      </c>
-      <c r="C26" s="37" t="s">
-        <v>198</v>
-      </c>
-      <c r="D26" s="39" t="s">
-        <v>200</v>
-      </c>
-      <c r="E26" s="47" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="27" ht="21.75" customHeight="1">
-      <c r="A27" s="33" t="s">
-        <v>203</v>
-      </c>
-      <c r="B27" s="35" t="s">
-        <v>204</v>
-      </c>
-      <c r="C27" s="37" t="s">
-        <v>205</v>
-      </c>
-      <c r="D27" s="39" t="s">
-        <v>206</v>
-      </c>
-      <c r="E27" s="42" t="s">
-        <v>105</v>
+      <c r="E27" s="29" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Atualização automática da planilha (2026-09-14)
</commit_message>
<xml_diff>
--- a/times.xlsx
+++ b/times.xlsx
@@ -19,25 +19,82 @@
     <t>GUIA DE ROTAÇÃO &amp; METAGAME - POKEALLIANCE(PKA)</t>
   </si>
   <si>
+    <t>GUIA RÁPIDO</t>
+  </si>
+  <si>
     <t>RECOMENDAÇÃO DE TIME PARA HUNTS!</t>
   </si>
   <si>
     <t>GUIA VISUAL DE HUNT: CARDS - ELEMENTOS</t>
   </si>
   <si>
-    <t>GUIA RÁPIDO</t>
-  </si>
-  <si>
     <t>Requisitos de Entrada e Progressão 2x2x2.</t>
   </si>
   <si>
     <t>https://www.twitch.tv/safnaww</t>
   </si>
   <si>
+    <t>Segue lá!</t>
+  </si>
+  <si>
+    <t>★ METAGROSS</t>
+  </si>
+  <si>
+    <t>📌 REQUISITOS INICIAIS (START DE ROTAÇÃO)</t>
+  </si>
+  <si>
+    <t>★ LUCARIO</t>
+  </si>
+  <si>
+    <t>⚡ UPGRADE: ROTAÇÃO 2x2x2</t>
+  </si>
+  <si>
+    <t>★ GENGAR</t>
+  </si>
+  <si>
+    <t>Nível &amp; Held:</t>
+  </si>
+  <si>
+    <t>Hunt: Steel / Psychic</t>
+  </si>
+  <si>
+    <t>Hunt: Fighting / Steel</t>
+  </si>
+  <si>
     <t>Com algumas exceções, todos os restantes são SHINYS.</t>
   </si>
   <si>
-    <t>Segue lá!</t>
+    <t>Hunt: Ghost / Poison</t>
+  </si>
+  <si>
+    <t>Todos os Pokémon +15 com Atk 4</t>
+  </si>
+  <si>
+    <t>Todos os Pokémon +25 com Atk 5</t>
+  </si>
+  <si>
+    <t>Atalho / Dica:</t>
+  </si>
+  <si>
+    <t>🛡️ LURAR / TANQUE (T1)</t>
+  </si>
+  <si>
+    <t>Runas de Atk no Pokelog ajudam a adiantar a meta</t>
+  </si>
+  <si>
+    <t>Estrelas Mínimas:</t>
+  </si>
+  <si>
+    <t>⚔️ DPS / DANO (SR)</t>
+  </si>
+  <si>
+    <t>Tier 1: 2★ (estrelas)  |  SR: 1★ (estrela)</t>
+  </si>
+  <si>
+    <t>Meta no Dummy:</t>
+  </si>
+  <si>
+    <t>Bater 560k de dano com 3 Pokémon</t>
   </si>
   <si>
     <r>
@@ -61,171 +118,219 @@
     </r>
   </si>
   <si>
-    <t>★ METAGROSS</t>
+    <t>Bater 560k de dano com apenas 2 Pokémon</t>
+  </si>
+  <si>
+    <t>⭐ S.Rapidash, S.Typhlosion, S.Steelix</t>
+  </si>
+  <si>
+    <t>Regra de Prey:</t>
+  </si>
+  <si>
+    <t>Obrigatório Prey de Atk na hunt (já calculada no dummy)</t>
+  </si>
+  <si>
+    <t>Manter sempre Prey de Atk ativa na hunt</t>
   </si>
   <si>
     <t>ELEMENTO / HUNT</t>
   </si>
   <si>
+    <t>💡 POR QUE COMPOSIÇÕES COM 2 A 3 ELEMENTOS SÃO SUPERIORES? (ANTI-MONO)</t>
+  </si>
+  <si>
+    <t>⭐ Arcanine, Houndoom, Pupitar</t>
+  </si>
+  <si>
+    <t>⭐ Hitmontop, Typhlosion, Rapidash</t>
+  </si>
+  <si>
     <t>ALVO (HUNT)</t>
   </si>
   <si>
+    <t>⭐ Arcanine, Machamp, Pupitar</t>
+  </si>
+  <si>
+    <t>⭐ Umbreon, Crawdaunt, Sableye</t>
+  </si>
+  <si>
+    <t>⭐ Houndoom, Hydreigon, Pupitar</t>
+  </si>
+  <si>
+    <t>Nessa planilha não indicaremos pokémons T2 ou T3 para a rotação.</t>
+  </si>
+  <si>
+    <t>⏱️ Cooldown Reduzido por Tier</t>
+  </si>
+  <si>
     <t>🛡️ LURAR (T1)</t>
   </si>
   <si>
+    <t>Outras Opções T1:</t>
+  </si>
+  <si>
     <t>⚔️ DPS (SR)</t>
   </si>
   <si>
     <t>🎨 TIPO SMEARGLE</t>
   </si>
   <si>
+    <t>Outras Opções SR:</t>
+  </si>
+  <si>
+    <t>★ BUG</t>
+  </si>
+  <si>
     <t>Bug</t>
   </si>
   <si>
-    <t>📌 REQUISITOS INICIAIS (START DE ROTAÇÃO)</t>
-  </si>
-  <si>
-    <t>★ LUCARIO</t>
-  </si>
-  <si>
-    <t>★ GENGAR</t>
-  </si>
-  <si>
-    <t>⚡ UPGRADE: ROTAÇÃO 2x2x2</t>
-  </si>
-  <si>
-    <t>Nessa planilha não indicaremos pokémons T2 ou T3 para a rotação.</t>
-  </si>
-  <si>
-    <t>Nível &amp; Held:</t>
-  </si>
-  <si>
     <t>Em breve</t>
   </si>
   <si>
-    <t>★ BUG</t>
-  </si>
-  <si>
-    <t>Hunt: Steel / Psychic</t>
-  </si>
-  <si>
-    <t>Todos os Pokémon +15 com Atk 4</t>
+    <t>Umbreon</t>
+  </si>
+  <si>
+    <t>No PKA, tiers mais altos não dão só dano: reduzem o cooldown das skills, deixando a rotação muito mais rápida.</t>
+  </si>
+  <si>
+    <t>Rapidash, Typhlosion, Magcargo</t>
+  </si>
+  <si>
+    <t>Torterra, Misdreavus</t>
+  </si>
+  <si>
+    <t>Poliwrath, Medicham, Hariyama</t>
+  </si>
+  <si>
+    <t>Infernape, Kangaskhan, Torterra</t>
+  </si>
+  <si>
+    <t>Cacturne, Banette, Dusclops</t>
+  </si>
+  <si>
+    <t>Misdreavus, Dusknoir, Torterra</t>
+  </si>
+  <si>
+    <t>🎨 Smeargle: Fire, Ground, Ghost, Dark</t>
   </si>
   <si>
     <t>★ FAIRY</t>
   </si>
   <si>
-    <t>Rapidash, Typhlosion, Magcargo</t>
+    <t>🎨 Smeargle: Fighting, Fire, Ground</t>
+  </si>
+  <si>
+    <t>📈 Mais Mobs e Brokes / Hora</t>
+  </si>
+  <si>
+    <t>🎨 Smeargle: Dark, Ghost, Ground</t>
+  </si>
+  <si>
+    <t>Rotação mais fluida = mais mobs derrotados/hora, aumentando drasticamente a chance de Shiny/hr e lucro.</t>
+  </si>
+  <si>
+    <t>★ GARDEVOIR</t>
+  </si>
+  <si>
+    <t>⚔️ Hazards Mais Altos</t>
+  </si>
+  <si>
+    <t>★ GYARADOS</t>
   </si>
   <si>
     <t>★ FIRE</t>
   </si>
   <si>
-    <t>Hunt: Fighting / Steel</t>
-  </si>
-  <si>
-    <t>Hunt: Ghost / Poison</t>
-  </si>
-  <si>
-    <t>Todos os Pokémon +25 com Atk 5</t>
-  </si>
-  <si>
-    <t>Atalho / Dica:</t>
+    <t>Mesmo encurtando o número total de hunts, permite solar níveis de Hazard superiores com segurança e eficiência.</t>
+  </si>
+  <si>
+    <t>★ SWAMPERT</t>
+  </si>
+  <si>
+    <t>🏆 Futuro &amp; Escalabilidade (Endgame)</t>
+  </si>
+  <si>
+    <t>Trabalhar com 2 ou 3 elementos abre um catálogo amplo de opções viáveis para evoluir: T1, SR, UR e Lendários.</t>
   </si>
   <si>
     <t>Arcanine, Infernape, Armaldo</t>
   </si>
   <si>
-    <t>Runas de Atk no Pokelog ajudam a adiantar a meta</t>
-  </si>
-  <si>
-    <t>🛡️ LURAR / TANQUE (T1)</t>
-  </si>
-  <si>
     <t>Hunt: Em breve</t>
   </si>
   <si>
+    <t>Hunt: Psychic / Fairy</t>
+  </si>
+  <si>
+    <t>Hunt: Shiny Sylveon (Lendário)</t>
+  </si>
+  <si>
+    <t>Hunt: Water / Flying</t>
+  </si>
+  <si>
     <t>Fire, Rock</t>
   </si>
   <si>
+    <t>Hunt: Magmar (Lendário) / Torkoal (UR)</t>
+  </si>
+  <si>
+    <t>Hunt: Water / Ground</t>
+  </si>
+  <si>
     <t>Fairy</t>
   </si>
   <si>
-    <t>Hunt: Shiny Sylveon (Lendário)</t>
-  </si>
-  <si>
-    <t>Hunt: Magmar (Lendário) / Torkoal (UR)</t>
-  </si>
-  <si>
-    <t>Estrelas Mínimas:</t>
-  </si>
-  <si>
-    <t>Tier 1: 2★ (estrelas)  |  SR: 1★ (estrela)</t>
-  </si>
-  <si>
-    <t>Meta no Dummy:</t>
-  </si>
-  <si>
-    <t>Bater 560k de dano com 3 Pokémon</t>
-  </si>
-  <si>
-    <t>⚔️ DPS / DANO (SR)</t>
-  </si>
-  <si>
     <t>Shiny Sylveon (Lendário)</t>
   </si>
   <si>
-    <t>Bater 560k de dano com apenas 2 Pokémon</t>
-  </si>
-  <si>
-    <t>Regra de Prey:</t>
-  </si>
-  <si>
-    <t>⭐ S.Rapidash, S.Typhlosion, S.Steelix</t>
-  </si>
-  <si>
-    <t>Obrigatório Prey de Atk na hunt (já calculada no dummy)</t>
-  </si>
-  <si>
-    <t>Manter sempre Prey de Atk ativa na hunt</t>
-  </si>
-  <si>
-    <t>💡 POR QUE COMPOSIÇÕES COM 2 A 3 ELEMENTOS SÃO SUPERIORES? (ANTI-MONO)</t>
+    <t>⭐S.Rapidash, S.Typhlosion, S.Magcargo</t>
   </si>
   <si>
     <t>Muk, Tentacruel, Mawile</t>
   </si>
   <si>
+    <t>⭐ Arcanine, Infernape, Armaldo</t>
+  </si>
+  <si>
     <t>Aggron, Skarmory, Toxicroak</t>
   </si>
   <si>
-    <t>⏱️ Cooldown Reduzido por Tier</t>
+    <t>⭐ Muk, Tentacruel, Mawile</t>
   </si>
   <si>
     <t>Poison, Metal</t>
   </si>
   <si>
-    <t>⭐ Arcanine, Houndoom, Pupitar</t>
-  </si>
-  <si>
-    <t>⭐S.Rapidash, S.Typhlosion, S.Magcargo</t>
-  </si>
-  <si>
-    <t>⭐ Arcanine, Infernape, Armaldo</t>
-  </si>
-  <si>
-    <t>⭐ Muk, Tentacruel, Mawile</t>
+    <t>⭐ Mawile, Muk, Tentacruel</t>
+  </si>
+  <si>
+    <t>⭐ Aggron, Skarmory, Toxicroak</t>
+  </si>
+  <si>
+    <t>⭐ Toxicroak, Seviper, Misdreavus</t>
+  </si>
+  <si>
+    <t>⭐ Blastoise, Feraligatr, Omastar</t>
   </si>
   <si>
     <t>Fire</t>
   </si>
   <si>
+    <t>⭐ Ampharos, Luxray, Jolteon</t>
+  </si>
+  <si>
     <t>Magmar (Lendário) / Torkoal (UR)</t>
   </si>
   <si>
+    <t>⭐ Pupitar, Torterra, Kingdra</t>
+  </si>
+  <si>
     <t>Blastoise, Feraligatr, Omastar</t>
   </si>
   <si>
+    <t>⭐ S.Luxray, S.Pachirisu, Smeargle Eletric</t>
+  </si>
+  <si>
     <t>Pupitar, Torterra, Kingdra</t>
   </si>
   <si>
@@ -235,21 +340,21 @@
     <t>Fighting</t>
   </si>
   <si>
-    <t>No PKA, tiers mais altos não dão só dano: reduzem o cooldown das skills, deixando a rotação muito mais rápida.</t>
-  </si>
-  <si>
     <t>Mega Clefable, Pidgeot, Espeon</t>
   </si>
   <si>
     <t>Wobbuffet, Mimikyu, Gliscor</t>
   </si>
   <si>
-    <t>⭐ Hitmontop, Typhlosion, Rapidash</t>
+    <t>⭐Venusaur, Gogoat, Tangrowth</t>
   </si>
   <si>
     <t>Psychic, Flying, Fairy</t>
   </si>
   <si>
+    <t>⭐ S.Tangrowth,S. Gogoat, Smeargle Grass</t>
+  </si>
+  <si>
     <t>Dark</t>
   </si>
   <si>
@@ -271,6 +376,9 @@
     <t>Milotic (UR)</t>
   </si>
   <si>
+    <t>S.Charizard, Kabutops, Golem</t>
+  </si>
+  <si>
     <t>Tangrowth, Ampharos, Venusaur</t>
   </si>
   <si>
@@ -280,70 +388,64 @@
     <t>Grass, Electric</t>
   </si>
   <si>
-    <t>📈 Mais Mobs e Brokes / Hora</t>
+    <t>Metang, Banette, Dusclops, Nidoking</t>
   </si>
   <si>
     <t>Grass</t>
   </si>
   <si>
+    <t>Aggron, Skarmory</t>
+  </si>
+  <si>
     <t>Leafeon (Lendário) / Sceptile (UR)</t>
   </si>
   <si>
+    <t>—</t>
+  </si>
+  <si>
     <t>Typhlosion, Rapidash, Pidgeot</t>
   </si>
   <si>
+    <t>Raichu</t>
+  </si>
+  <si>
     <t>Arcanine, Infernape, Scyther</t>
   </si>
   <si>
+    <t>Metang, Magneton Estrelado</t>
+  </si>
+  <si>
     <t>Poison, Bug, Fire, Fly, Ice</t>
   </si>
   <si>
     <t>Electric</t>
   </si>
   <si>
-    <t>Rotação mais fluida = mais mobs derrotados/hora, aumentando drasticamente a chance de Shiny/hr e lucro.</t>
-  </si>
-  <si>
-    <t>⭐ Aggron, Skarmory, Toxicroak</t>
+    <t>SevIper</t>
   </si>
   <si>
     <t>Electabuzz (Lendário) / Manectric (UR)</t>
   </si>
   <si>
-    <t>⭐ Blastoise, Feraligatr, Omastar</t>
-  </si>
-  <si>
     <t>Steelix, Nidoqueen, Torterra</t>
   </si>
   <si>
-    <t>⭐ Pupitar, Torterra, Kingdra</t>
-  </si>
-  <si>
-    <t>⭐ Arcanine, Machamp, Pupitar</t>
-  </si>
-  <si>
     <t>Torterra, Pupitar, Smeargle</t>
   </si>
   <si>
-    <t>⚔️ Hazards Mais Altos</t>
-  </si>
-  <si>
-    <t>Outras Opções T1:</t>
-  </si>
-  <si>
     <t>Ground</t>
   </si>
   <si>
+    <t>🎨 Smeargle: Poison, Ghost, Metal</t>
+  </si>
+  <si>
     <t>Ghost</t>
   </si>
   <si>
-    <t>⭐ Umbreon, Crawdaunt, Sableye</t>
-  </si>
-  <si>
-    <t>Mesmo encurtando o número total de hunts, permite solar níveis de Hazard superiores com segurança e eficiência.</t>
-  </si>
-  <si>
-    <t>⭐ Houndoom, Hydreigon, Pupitar</t>
+    <t>Vaporeon, Rhyperior, Magcargo</t>
+  </si>
+  <si>
+    <t>Sharpedo</t>
   </si>
   <si>
     <t>Umbreon, Crawdaunt, Dusknoir</t>
@@ -358,36 +460,24 @@
     <t>Ice</t>
   </si>
   <si>
+    <t>🎨 Smeargle: Fire, Rock</t>
+  </si>
+  <si>
     <t>Glaceon (Lendário) / Glalie (UR)</t>
   </si>
   <si>
-    <t>🏆 Futuro &amp; Escalabilidade (Endgame)</t>
-  </si>
-  <si>
-    <t>Outras Opções SR:</t>
-  </si>
-  <si>
-    <t>S.Charizard, Kabutops, Golem</t>
-  </si>
-  <si>
     <t>Typhlosion, Rapidash, Hitmontop</t>
   </si>
   <si>
-    <t>Trabalhar com 2 ou 3 elementos abre um catálogo amplo de opções viáveis para evoluir: T1, SR, UR e Lendários.</t>
-  </si>
-  <si>
-    <t>Umbreon</t>
-  </si>
-  <si>
-    <t>—</t>
-  </si>
-  <si>
     <t>Infernape, Machamp, Skarmory</t>
   </si>
   <si>
     <t>Fighting, Fire, Metal</t>
   </si>
   <si>
+    <t>🎨 Smeargle: Electric</t>
+  </si>
+  <si>
     <t>Poison</t>
   </si>
   <si>
@@ -397,18 +487,15 @@
     <t>Steelix, Espeon, Nidoqueen</t>
   </si>
   <si>
-    <t>Metang, Magneton Estrelado</t>
-  </si>
-  <si>
     <t>Wobbuffet, Mr. Mime, Pupitar</t>
   </si>
   <si>
+    <t>🎨 Smeargle: Poison, Metal</t>
+  </si>
+  <si>
     <t>Ground, Psychic</t>
   </si>
   <si>
-    <t>SevIper</t>
-  </si>
-  <si>
     <t>Normal</t>
   </si>
   <si>
@@ -421,48 +508,30 @@
     <t>Machamp, Kangaskhan, Smeargle</t>
   </si>
   <si>
-    <t>Vaporeon, Rhyperior, Magcargo</t>
-  </si>
-  <si>
-    <t>Torterra, Misdreavus</t>
-  </si>
-  <si>
-    <t>Sharpedo</t>
-  </si>
-  <si>
-    <t>Poliwrath, Medicham, Hariyama</t>
-  </si>
-  <si>
     <t>Rock</t>
   </si>
   <si>
+    <t>🎨 Smeargle: Rock, Water, Ground</t>
+  </si>
+  <si>
     <t>Rampardos (UR)</t>
   </si>
   <si>
-    <t>Infernape, Kangaskhan, Torterra</t>
-  </si>
-  <si>
     <t>Tangrowth, Steelix, Blastoise</t>
   </si>
   <si>
-    <t>🎨 Smeargle: Fire, Rock</t>
-  </si>
-  <si>
     <t>Tangrowth, Machamp, Gogoat</t>
   </si>
   <si>
-    <t>Cacturne, Banette, Dusclops</t>
-  </si>
-  <si>
     <t>Fighting, Ground, Water, Grass</t>
   </si>
   <si>
+    <t>🎨 Smeargle: Grass</t>
+  </si>
+  <si>
     <t>Steel</t>
   </si>
   <si>
-    <t>Misdreavus, Dusknoir, Torterra</t>
-  </si>
-  <si>
     <t>Hitmontop, Rapidash, Typhlosion</t>
   </si>
   <si>
@@ -475,15 +544,9 @@
     <t>Blastoise, Tangrowth, Gogoat</t>
   </si>
   <si>
-    <t>🎨 Smeargle: Poison, Metal</t>
-  </si>
-  <si>
     <t>Tangrowth, Kingdra, Sharpedo</t>
   </si>
   <si>
-    <t>🎨 Smeargle: Fire, Ground, Ghost, Dark</t>
-  </si>
-  <si>
     <t>Water, Ice, Grass</t>
   </si>
   <si>
@@ -493,6 +556,9 @@
     <t>Salamence (UR) / Flygon (Lendário)</t>
   </si>
   <si>
+    <t>★ FIGHTING</t>
+  </si>
+  <si>
     <t>Lapras, Mega Clefable, Jynx</t>
   </si>
   <si>
@@ -502,18 +568,12 @@
     <t>Dragon, Ice, Fairy</t>
   </si>
   <si>
-    <t>🎨 Smeargle: Rock, Water, Ground</t>
-  </si>
-  <si>
     <t>Psychic</t>
   </si>
   <si>
     <t>Alakazam (Lendário)</t>
   </si>
   <si>
-    <t>🎨 Smeargle: Fighting, Fire, Ground</t>
-  </si>
-  <si>
     <t>Umbreon, Crawdaunt, Sableye</t>
   </si>
   <si>
@@ -526,6 +586,9 @@
     <t>Flying</t>
   </si>
   <si>
+    <t>★ SCIZOR</t>
+  </si>
+  <si>
     <t>Ampharos, Magcargo, Lapras</t>
   </si>
   <si>
@@ -535,24 +598,24 @@
     <t>Electric, Ice, Rock</t>
   </si>
   <si>
-    <t>🎨 Smeargle: Dark, Ghost, Ground</t>
-  </si>
-  <si>
     <t>Metagross</t>
   </si>
   <si>
     <t>Steel / Psychic</t>
   </si>
   <si>
+    <t>★ DARK</t>
+  </si>
+  <si>
     <t>Rapidash, Typhlosion, Steelix</t>
   </si>
   <si>
-    <t>★ FIGHTING</t>
-  </si>
-  <si>
     <t>Arcanine, Houndoom, Pupitar</t>
   </si>
   <si>
+    <t>Hunt: Bug</t>
+  </si>
+  <si>
     <t>Fire, Ground, Ghost, Dark</t>
   </si>
   <si>
@@ -562,15 +625,15 @@
     <t>Fighting / Steel</t>
   </si>
   <si>
+    <t>★ WATER</t>
+  </si>
+  <si>
     <t>Hitmontop, Typhlosion, Rapidash</t>
   </si>
   <si>
     <t>Arcanine, Machamp, Pupitar</t>
   </si>
   <si>
-    <t>★ GARDEVOIR</t>
-  </si>
-  <si>
     <t>Fighting, Fire, Ground</t>
   </si>
   <si>
@@ -580,15 +643,9 @@
     <t>Ghost / Poison</t>
   </si>
   <si>
-    <t>★ DARK</t>
-  </si>
-  <si>
     <t>Houndoom, Hydreigon, Pupitar</t>
   </si>
   <si>
-    <t>★ GYARADOS</t>
-  </si>
-  <si>
     <t>Dark, Ghost, Ground</t>
   </si>
   <si>
@@ -610,48 +667,33 @@
     <t>Gyarados</t>
   </si>
   <si>
+    <t>⭐ S.Rapidash, S.Typhlosion, S.Zard</t>
+  </si>
+  <si>
     <t>Water / Flying</t>
   </si>
   <si>
-    <t>★ SWAMPERT</t>
-  </si>
-  <si>
-    <t>★ WATER</t>
-  </si>
-  <si>
     <t>Ampharos, Luxray, Jolteon</t>
   </si>
   <si>
+    <t>⭐S.Arcanine, S.Infernape, Smeargle Fire</t>
+  </si>
+  <si>
     <t>Luxray, Pachirisu, Smeargle Eletric</t>
   </si>
   <si>
-    <t>Hunt: Psychic / Fairy</t>
-  </si>
-  <si>
-    <t>Hunt: Water / Flying</t>
-  </si>
-  <si>
-    <t>Hunt: Water / Ground</t>
-  </si>
-  <si>
     <t>Hunt: Absol (Lendário) / Mightyena (UR)</t>
   </si>
   <si>
     <t>Hunt: Milotic (UR)</t>
   </si>
   <si>
-    <t>⭐ Mawile, Muk, Tentacruel</t>
-  </si>
-  <si>
-    <t>⭐ Toxicroak, Seviper, Misdreavus</t>
+    <t>🎨 Smeargle: Fire</t>
   </si>
   <si>
     <t>⭐ Mega Clefable, Pidgeot, Espeon</t>
   </si>
   <si>
-    <t>⭐ Ampharos, Luxray, Jolteon</t>
-  </si>
-  <si>
     <t>⭐ Wobbuffet, Mimikyu, Gliscor</t>
   </si>
   <si>
@@ -664,18 +706,9 @@
     <t>⭐ Tangrowth, Ampharos, Venusaur</t>
   </si>
   <si>
-    <t>⭐ S.Luxray, S.Pachirisu, Smeargle Eletric</t>
-  </si>
-  <si>
     <t>⭐ Tangrowth, Gogoat, Luxray</t>
   </si>
   <si>
-    <t>⭐Venusaur, Gogoat, Tangrowth</t>
-  </si>
-  <si>
-    <t>⭐ S.Tangrowth,S. Gogoat, Smeargle Grass</t>
-  </si>
-  <si>
     <t>Farfetch'd, Gliscor</t>
   </si>
   <si>
@@ -697,55 +730,22 @@
     <t>🎨 Smeargle: Psychic, Flying, Fairy</t>
   </si>
   <si>
-    <t>Metang, Banette, Dusclops, Nidoking</t>
-  </si>
-  <si>
-    <t>Aggron, Skarmory</t>
-  </si>
-  <si>
-    <t>Raichu</t>
-  </si>
-  <si>
     <t>🎨 Smeargle: Fighting, Fairy, Bug</t>
   </si>
   <si>
-    <t>🎨 Smeargle: Poison, Ghost, Metal</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Electric</t>
-  </si>
-  <si>
     <t>🎨 Smeargle: Grass, Electric</t>
   </si>
   <si>
-    <t>🎨 Smeargle: Grass</t>
-  </si>
-  <si>
     <t>★ GRASS</t>
   </si>
   <si>
-    <t>★ SCIZOR</t>
-  </si>
-  <si>
     <t>★ ELECTRIC</t>
   </si>
   <si>
-    <t>Hunt: Bug</t>
-  </si>
-  <si>
     <t>★ GHOST</t>
   </si>
   <si>
-    <t>⭐ S.Rapidash, S.Typhlosion, S.Zard</t>
-  </si>
-  <si>
-    <t>⭐S.Arcanine, S.Infernape, Smeargle Fire</t>
-  </si>
-  <si>
     <t>Hunt: Leafeon (Lendário) / Sceptile (UR)</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Fire</t>
   </si>
   <si>
     <t>Hunt: Electabuzz (Lendário) / Manectric (UR)</t>
@@ -989,12 +989,6 @@
     </font>
     <font/>
     <font>
-      <b/>
-      <sz val="13.0"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
       <i/>
       <sz val="9.0"/>
       <color rgb="FF94A3B8"/>
@@ -1007,12 +1001,6 @@
     </font>
     <font>
       <i/>
-      <sz val="9.0"/>
-      <color rgb="FFD1D5DB"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <i/>
       <u/>
       <sz val="9.0"/>
       <color rgb="FF0000FF"/>
@@ -1021,6 +1009,12 @@
     <font>
       <u/>
       <color rgb="FF0000FF"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13.0"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Quattrocento Sans"/>
     </font>
     <font>
       <b/>
@@ -1036,26 +1030,8 @@
     </font>
     <font>
       <i/>
-      <u/>
       <sz val="9.0"/>
-      <color rgb="FFE5E7EB"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10.0"/>
-      <color rgb="FF1E293B"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9.0"/>
-      <color rgb="FF334155"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <sz val="9.0"/>
-      <color rgb="FF475569"/>
+      <color rgb="FFD1D5DB"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1067,7 +1043,76 @@
     <font>
       <b/>
       <sz val="9.0"/>
+      <color rgb="FF334155"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9.0"/>
       <color rgb="FF0F172A"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9.0"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <sz val="9.0"/>
+      <color rgb="FF0F172A"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10.0"/>
+      <color rgb="FF1A1A1A"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <i/>
+      <u/>
+      <sz val="9.0"/>
+      <color rgb="FFE5E7EB"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8.0"/>
+      <color rgb="FF4B5563"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9.0"/>
+      <color rgb="FF1E3A8A"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10.0"/>
+      <color rgb="FF1E293B"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <sz val="9.0"/>
+      <color rgb="FF475569"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <sz val="8.0"/>
+      <color rgb="FF4A4A4A"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <sz val="9.0"/>
+      <color rgb="FF1F2937"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8.0"/>
+      <color rgb="FF1E3A8A"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1089,54 +1134,9 @@
       <name val="Quattrocento Sans"/>
     </font>
     <font>
-      <sz val="9.0"/>
-      <color rgb="FF0F172A"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9.0"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10.0"/>
-      <color rgb="FF1A1A1A"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9.0"/>
-      <color rgb="FF1E3A8A"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <sz val="9.0"/>
-      <color rgb="FF1F2937"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="8.0"/>
-      <color rgb="FF4B5563"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <sz val="8.0"/>
-      <color rgb="FF4A4A4A"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
       <b/>
       <sz val="8.0"/>
       <color rgb="FF4A4A4A"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="8.0"/>
-      <color rgb="FF1E3A8A"/>
       <name val="Quattrocento Sans"/>
     </font>
   </fonts>
@@ -1179,8 +1179,74 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF374151"/>
+        <bgColor rgb="FF374151"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFF1F5F9"/>
         <bgColor rgb="FFF1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E7D32"/>
+        <bgColor rgb="FF2E7D32"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC62828"/>
+        <bgColor rgb="FFC62828"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCFCE7"/>
+        <bgColor rgb="FFDCFCE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF3C7"/>
+        <bgColor rgb="FFFEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8F5E9"/>
+        <bgColor rgb="FFE8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEBEE"/>
+        <bgColor rgb="FFFFEBEE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1E40AF"/>
+        <bgColor rgb="FF1E40AF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF0F4F8"/>
+        <bgColor rgb="FFF0F4F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEFF6FF"/>
+        <bgColor rgb="FFEFF6FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF9FAFB"/>
+        <bgColor rgb="FFF9FAFB"/>
       </patternFill>
     </fill>
     <fill>
@@ -1191,14 +1257,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE68D9C"/>
-        <bgColor rgb="FFE68D9C"/>
+        <fgColor rgb="FFEEF2FF"/>
+        <bgColor rgb="FFEEF2FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF374151"/>
-        <bgColor rgb="FF374151"/>
+        <fgColor rgb="FFE68D9C"/>
+        <bgColor rgb="FFE68D9C"/>
       </patternFill>
     </fill>
     <fill>
@@ -1221,74 +1287,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF2E7D32"/>
-        <bgColor rgb="FF2E7D32"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFF8FAFC"/>
         <bgColor rgb="FFF8FAFC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFDCFCE7"/>
-        <bgColor rgb="FFDCFCE7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC62828"/>
-        <bgColor rgb="FFC62828"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFEF3C7"/>
-        <bgColor rgb="FFFEF3C7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1E40AF"/>
-        <bgColor rgb="FF1E40AF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE8F5E9"/>
-        <bgColor rgb="FFE8F5E9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEBEE"/>
-        <bgColor rgb="FFFFEBEE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEFF6FF"/>
-        <bgColor rgb="FFEFF6FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF0F4F8"/>
-        <bgColor rgb="FFF0F4F8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF9FAFB"/>
-        <bgColor rgb="FFF9FAFB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEEF2FF"/>
-        <bgColor rgb="FFEEF2FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -1410,20 +1410,6 @@
       </bottom>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFD1D5DB"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD1D5DB"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD1D5DB"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD1D5DB"/>
-      </bottom>
-    </border>
-    <border>
       <right style="thin">
         <color rgb="FFD1D5DB"/>
       </right>
@@ -1446,6 +1432,20 @@
       </top>
       <bottom style="thin">
         <color rgb="FFCBD5E1"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD1D5DB"/>
       </bottom>
     </border>
     <border>
@@ -1493,192 +1493,192 @@
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="4" fillId="5" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="6" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="7" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="6" fillId="8" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="6" fillId="4" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="9" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="6" fillId="4" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="10" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="6" fillId="11" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="6" fillId="12" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="13" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="6" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="14" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="15" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="7" fillId="13" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="6" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf borderId="7" fillId="16" fontId="18" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="8" fillId="17" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="7" fillId="4" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0"/>
+    <xf borderId="9" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="7" fillId="4" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="7" fillId="18" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="19" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="8" fillId="4" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="20" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="10" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="21" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="22" fontId="25" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="23" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="5" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf borderId="7" fillId="24" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="5" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="7" fillId="4" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="6" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="7" fillId="25" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="6" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="7" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="6" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="3" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="7" fillId="25" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="25" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="14" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="18" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="18" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="20" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="6" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="26" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="4" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="27" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="7" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="8" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="28" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="4" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="29" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="9" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="30" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="10" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="31" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="4" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="5" fillId="11" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="12" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="32" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="13" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="4" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="33" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="4" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="5" fillId="14" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="15" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="34" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="16" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="5" fillId="17" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="7" fillId="18" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="5" fillId="15" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="35" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="19" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="36" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="20" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="5" fillId="15" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="37" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="21" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="8" fillId="22" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="9" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="8" fillId="4" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="10" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="5" fillId="20" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="5" fillId="23" fontId="25" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="5" fillId="24" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="5" fillId="24" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="5" fillId="24" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="25" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="38" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="26" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="39" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="27" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="5" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="28" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="10" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="21" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="25" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="29" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="30" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="31" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="32" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="33" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="34" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="35" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="36" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="37" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="38" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="39" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="40" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="40" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1926,149 +1926,149 @@
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
-      <c r="F2" s="5"/>
+      <c r="F2" s="4"/>
     </row>
     <row r="3" ht="19.5" customHeight="1">
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="5" t="s">
         <v>4</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
-      <c r="F3" s="5"/>
+      <c r="F3" s="4"/>
     </row>
     <row r="4">
-      <c r="B4" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="12" t="s">
+      <c r="B4" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="8" t="s">
-        <v>7</v>
+      <c r="F4" s="10" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="5" ht="24.0" customHeight="1">
-      <c r="B5" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="5"/>
-      <c r="E5" s="18" t="s">
+      <c r="B5" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="E5" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="4"/>
+    </row>
+    <row r="6" ht="24.75" customHeight="1">
+      <c r="B6" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="18" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" ht="24.75" customHeight="1">
+      <c r="B7" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="F5" s="5"/>
-    </row>
-    <row r="6" ht="24.75" customHeight="1">
-      <c r="B6" s="20" t="s">
+      <c r="C7" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="E7" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" s="20" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" ht="24.75" customHeight="1">
+      <c r="B8" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="F6" s="25" t="s">
+      <c r="C8" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8" s="23" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" ht="24.75" customHeight="1">
+      <c r="B9" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="20" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="7" ht="24.75" customHeight="1">
-      <c r="B7" s="20" t="s">
+      <c r="E9" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="30" t="s">
+    </row>
+    <row r="11" ht="24.0" customHeight="1">
+      <c r="B11" s="27" t="s">
         <v>34</v>
-      </c>
-      <c r="E7" s="20" t="s">
-        <v>41</v>
-      </c>
-      <c r="F7" s="30" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="8" ht="24.75" customHeight="1">
-      <c r="B8" s="20" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" s="33" t="s">
-        <v>44</v>
-      </c>
-      <c r="E8" s="20" t="s">
-        <v>43</v>
-      </c>
-      <c r="F8" s="35" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="9" ht="24.75" customHeight="1">
-      <c r="B9" s="20" t="s">
-        <v>48</v>
-      </c>
-      <c r="C9" s="30" t="s">
-        <v>50</v>
-      </c>
-      <c r="E9" s="20" t="s">
-        <v>48</v>
-      </c>
-      <c r="F9" s="30" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="11" ht="24.0" customHeight="1">
-      <c r="B11" s="37" t="s">
-        <v>52</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
-      <c r="F11" s="5"/>
+      <c r="F11" s="4"/>
     </row>
     <row r="12" ht="24.0" customHeight="1">
-      <c r="B12" s="41" t="s">
-        <v>55</v>
-      </c>
-      <c r="C12" s="42"/>
-      <c r="D12" s="43" t="s">
-        <v>67</v>
-      </c>
-      <c r="E12" s="44"/>
-      <c r="F12" s="42"/>
+      <c r="B12" s="32" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="34"/>
+      <c r="D12" s="38" t="s">
+        <v>52</v>
+      </c>
+      <c r="E12" s="40"/>
+      <c r="F12" s="34"/>
     </row>
     <row r="13" ht="24.0" customHeight="1">
-      <c r="B13" s="41" t="s">
-        <v>82</v>
-      </c>
-      <c r="C13" s="42"/>
-      <c r="D13" s="43" t="s">
-        <v>89</v>
-      </c>
-      <c r="E13" s="44"/>
-      <c r="F13" s="42"/>
+      <c r="B13" s="32" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" s="34"/>
+      <c r="D13" s="38" t="s">
+        <v>64</v>
+      </c>
+      <c r="E13" s="40"/>
+      <c r="F13" s="34"/>
     </row>
     <row r="14" ht="24.0" customHeight="1">
-      <c r="B14" s="41" t="s">
-        <v>97</v>
-      </c>
-      <c r="C14" s="42"/>
-      <c r="D14" s="43" t="s">
-        <v>102</v>
-      </c>
-      <c r="E14" s="44"/>
-      <c r="F14" s="42"/>
+      <c r="B14" s="32" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="34"/>
+      <c r="D14" s="38" t="s">
+        <v>69</v>
+      </c>
+      <c r="E14" s="40"/>
+      <c r="F14" s="34"/>
     </row>
     <row r="15" ht="24.0" customHeight="1">
-      <c r="B15" s="41" t="s">
-        <v>109</v>
-      </c>
-      <c r="C15" s="42"/>
-      <c r="D15" s="43" t="s">
-        <v>113</v>
-      </c>
-      <c r="E15" s="44"/>
-      <c r="F15" s="42"/>
+      <c r="B15" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="C15" s="34"/>
+      <c r="D15" s="38" t="s">
+        <v>72</v>
+      </c>
+      <c r="E15" s="40"/>
+      <c r="F15" s="34"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -3094,8 +3094,8 @@
   </cols>
   <sheetData>
     <row r="1" ht="31.5" customHeight="1">
-      <c r="A1" s="4" t="s">
-        <v>2</v>
+      <c r="A1" s="14" t="s">
+        <v>3</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -3103,14 +3103,14 @@
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="8" t="s">
-        <v>6</v>
+      <c r="H1" s="4"/>
+      <c r="I1" s="10" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="2" ht="19.5" customHeight="1">
-      <c r="A2" s="17" t="s">
-        <v>8</v>
+      <c r="A2" s="28" t="s">
+        <v>27</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -3118,379 +3118,379 @@
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="8" t="s">
+      <c r="H2" s="4"/>
+      <c r="I2" s="10" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" ht="21.75" customHeight="1">
+      <c r="A4" s="37" t="s">
+        <v>48</v>
+      </c>
+      <c r="B4" s="12"/>
+      <c r="D4" s="41" t="s">
+        <v>60</v>
+      </c>
+      <c r="E4" s="12"/>
+      <c r="G4" s="43" t="s">
+        <v>68</v>
+      </c>
+      <c r="H4" s="12"/>
+    </row>
+    <row r="5" ht="18.0" customHeight="1">
+      <c r="A5" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="B5" s="12"/>
+      <c r="D5" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="E5" s="12"/>
+      <c r="G5" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="H5" s="12"/>
+    </row>
+    <row r="6" ht="19.5" customHeight="1">
+      <c r="A6" s="19" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="4" ht="21.75" customHeight="1">
-      <c r="A4" s="21" t="s">
+      <c r="B6" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="16"/>
-      <c r="D4" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="E4" s="16"/>
-      <c r="G4" s="27" t="s">
-        <v>28</v>
-      </c>
-      <c r="H4" s="16"/>
-    </row>
-    <row r="5" ht="18.0" customHeight="1">
-      <c r="A5" s="24" t="s">
-        <v>36</v>
-      </c>
-      <c r="B5" s="16"/>
-      <c r="D5" s="24" t="s">
-        <v>39</v>
-      </c>
-      <c r="E5" s="16"/>
-      <c r="G5" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="H5" s="16"/>
-    </row>
-    <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="B6" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="D6" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="E6" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="G6" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="H6" s="34" t="s">
-        <v>45</v>
+      <c r="D6" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="G6" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" s="21" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="7" ht="42.0" customHeight="1">
-      <c r="A7" s="38" t="s">
-        <v>58</v>
-      </c>
-      <c r="B7" s="40" t="s">
-        <v>59</v>
-      </c>
-      <c r="D7" s="45" t="s">
-        <v>60</v>
-      </c>
-      <c r="E7" s="40" t="s">
+      <c r="A7" s="24" t="s">
+        <v>83</v>
+      </c>
+      <c r="B7" s="26" t="s">
+        <v>85</v>
+      </c>
+      <c r="D7" s="29" t="s">
+        <v>87</v>
+      </c>
+      <c r="E7" s="26" t="s">
         <v>90</v>
       </c>
-      <c r="G7" s="45" t="s">
+      <c r="G7" s="29" t="s">
         <v>92</v>
       </c>
-      <c r="H7" s="40" t="s">
-        <v>94</v>
+      <c r="H7" s="26" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="B8" s="46" t="s">
-        <v>110</v>
-      </c>
-      <c r="D8" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="E8" s="46" t="s">
-        <v>110</v>
-      </c>
-      <c r="G8" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="H8" s="46" t="s">
-        <v>110</v>
+      <c r="A8" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" s="31" t="s">
+        <v>47</v>
+      </c>
+      <c r="D8" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="E8" s="31" t="s">
+        <v>47</v>
+      </c>
+      <c r="G8" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="H8" s="31" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="9" ht="27.75" customHeight="1">
-      <c r="A9" s="47" t="s">
-        <v>111</v>
-      </c>
-      <c r="B9" s="48" t="s">
-        <v>115</v>
-      </c>
-      <c r="D9" s="48" t="s">
-        <v>121</v>
-      </c>
-      <c r="E9" s="49" t="s">
-        <v>124</v>
-      </c>
-      <c r="G9" s="48" t="s">
+      <c r="A9" s="52" t="s">
+        <v>114</v>
+      </c>
+      <c r="B9" s="36" t="s">
+        <v>122</v>
+      </c>
+      <c r="D9" s="36" t="s">
+        <v>126</v>
+      </c>
+      <c r="E9" s="53" t="s">
         <v>129</v>
       </c>
-      <c r="H9" s="48" t="s">
-        <v>131</v>
+      <c r="G9" s="36" t="s">
+        <v>136</v>
+      </c>
+      <c r="H9" s="36" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="10" ht="18.0" customHeight="1">
-      <c r="A10" s="50" t="s">
-        <v>137</v>
-      </c>
-      <c r="B10" s="16"/>
-      <c r="D10" s="50" t="s">
-        <v>147</v>
-      </c>
-      <c r="E10" s="16"/>
-      <c r="G10" s="50" t="s">
-        <v>156</v>
-      </c>
-      <c r="H10" s="16"/>
+      <c r="A10" s="39" t="s">
+        <v>142</v>
+      </c>
+      <c r="B10" s="12"/>
+      <c r="D10" s="39" t="s">
+        <v>152</v>
+      </c>
+      <c r="E10" s="12"/>
+      <c r="G10" s="39" t="s">
+        <v>159</v>
+      </c>
+      <c r="H10" s="12"/>
     </row>
     <row r="14" ht="21.75" customHeight="1">
-      <c r="A14" s="51" t="s">
-        <v>171</v>
-      </c>
-      <c r="B14" s="16"/>
-      <c r="D14" s="52" t="s">
-        <v>182</v>
-      </c>
-      <c r="E14" s="16"/>
-      <c r="G14" s="54" t="s">
-        <v>194</v>
-      </c>
-      <c r="H14" s="16"/>
+      <c r="A14" s="55" t="s">
+        <v>174</v>
+      </c>
+      <c r="B14" s="12"/>
+      <c r="D14" s="56" t="s">
+        <v>190</v>
+      </c>
+      <c r="E14" s="12"/>
+      <c r="G14" s="57" t="s">
+        <v>197</v>
+      </c>
+      <c r="H14" s="12"/>
     </row>
     <row r="15" ht="18.0" customHeight="1">
-      <c r="A15" s="24" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15" s="16"/>
-      <c r="D15" s="24" t="s">
-        <v>200</v>
-      </c>
-      <c r="E15" s="16"/>
-      <c r="G15" s="24" t="s">
-        <v>201</v>
-      </c>
-      <c r="H15" s="16"/>
+      <c r="A15" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="B15" s="12"/>
+      <c r="D15" s="16" t="s">
+        <v>216</v>
+      </c>
+      <c r="E15" s="12"/>
+      <c r="G15" s="16" t="s">
+        <v>217</v>
+      </c>
+      <c r="H15" s="12"/>
     </row>
     <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="B16" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="D16" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="E16" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="G16" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="H16" s="34" t="s">
-        <v>45</v>
+      <c r="A16" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="D16" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="E16" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="G16" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="H16" s="21" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="17" ht="42.0" customHeight="1">
-      <c r="A17" s="45" t="s">
-        <v>204</v>
-      </c>
-      <c r="B17" s="40" t="s">
-        <v>206</v>
-      </c>
-      <c r="D17" s="45" t="s">
-        <v>207</v>
-      </c>
-      <c r="E17" s="40" t="s">
-        <v>208</v>
-      </c>
-      <c r="G17" s="45" t="s">
-        <v>209</v>
-      </c>
-      <c r="H17" s="40" t="s">
-        <v>211</v>
+      <c r="A17" s="29" t="s">
+        <v>219</v>
+      </c>
+      <c r="B17" s="26" t="s">
+        <v>220</v>
+      </c>
+      <c r="D17" s="29" t="s">
+        <v>221</v>
+      </c>
+      <c r="E17" s="26" t="s">
+        <v>222</v>
+      </c>
+      <c r="G17" s="29" t="s">
+        <v>223</v>
+      </c>
+      <c r="H17" s="26" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="18" ht="15.0" customHeight="1">
-      <c r="A18" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="B18" s="46" t="s">
-        <v>110</v>
-      </c>
-      <c r="D18" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="E18" s="46" t="s">
-        <v>110</v>
-      </c>
-      <c r="G18" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="H18" s="46" t="s">
-        <v>110</v>
+      <c r="A18" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" s="31" t="s">
+        <v>47</v>
+      </c>
+      <c r="D18" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="E18" s="31" t="s">
+        <v>47</v>
+      </c>
+      <c r="G18" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="H18" s="31" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="19" ht="27.75" customHeight="1">
-      <c r="A19" s="48" t="s">
-        <v>214</v>
-      </c>
-      <c r="B19" s="48" t="s">
-        <v>215</v>
-      </c>
-      <c r="D19" s="48" t="s">
-        <v>216</v>
-      </c>
-      <c r="E19" s="48" t="s">
-        <v>217</v>
-      </c>
-      <c r="G19" s="48" t="s">
-        <v>218</v>
-      </c>
-      <c r="H19" s="48" t="s">
-        <v>219</v>
+      <c r="A19" s="36" t="s">
+        <v>225</v>
+      </c>
+      <c r="B19" s="36" t="s">
+        <v>226</v>
+      </c>
+      <c r="D19" s="36" t="s">
+        <v>227</v>
+      </c>
+      <c r="E19" s="36" t="s">
+        <v>228</v>
+      </c>
+      <c r="G19" s="36" t="s">
+        <v>229</v>
+      </c>
+      <c r="H19" s="36" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="20" ht="18.0" customHeight="1">
-      <c r="A20" s="50" t="s">
-        <v>220</v>
-      </c>
-      <c r="B20" s="16"/>
-      <c r="D20" s="50" t="s">
-        <v>224</v>
-      </c>
-      <c r="E20" s="16"/>
-      <c r="G20" s="50" t="s">
-        <v>227</v>
-      </c>
-      <c r="H20" s="16"/>
+      <c r="A20" s="39" t="s">
+        <v>231</v>
+      </c>
+      <c r="B20" s="12"/>
+      <c r="D20" s="39" t="s">
+        <v>232</v>
+      </c>
+      <c r="E20" s="12"/>
+      <c r="G20" s="39" t="s">
+        <v>233</v>
+      </c>
+      <c r="H20" s="12"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
     <row r="23" ht="15.75" customHeight="1"/>
     <row r="24" ht="21.75" customHeight="1">
       <c r="A24" s="58" t="s">
-        <v>229</v>
-      </c>
-      <c r="B24" s="16"/>
+        <v>234</v>
+      </c>
+      <c r="B24" s="12"/>
       <c r="D24" s="59" t="s">
-        <v>231</v>
-      </c>
-      <c r="E24" s="16"/>
+        <v>235</v>
+      </c>
+      <c r="E24" s="12"/>
       <c r="G24" s="60" t="s">
-        <v>233</v>
-      </c>
-      <c r="H24" s="16"/>
+        <v>236</v>
+      </c>
+      <c r="H24" s="12"/>
     </row>
     <row r="25" ht="18.0" customHeight="1">
-      <c r="A25" s="24" t="s">
-        <v>236</v>
-      </c>
-      <c r="B25" s="16"/>
-      <c r="D25" s="24" t="s">
+      <c r="A25" s="16" t="s">
+        <v>237</v>
+      </c>
+      <c r="B25" s="12"/>
+      <c r="D25" s="16" t="s">
         <v>238</v>
       </c>
-      <c r="E25" s="16"/>
-      <c r="G25" s="24" t="s">
-        <v>36</v>
-      </c>
-      <c r="H25" s="16"/>
+      <c r="E25" s="12"/>
+      <c r="G25" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="H25" s="12"/>
     </row>
     <row r="26" ht="19.5" customHeight="1">
-      <c r="A26" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="B26" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="D26" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="E26" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="G26" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="H26" s="34" t="s">
-        <v>45</v>
+      <c r="A26" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="B26" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="D26" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="E26" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="G26" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="H26" s="21" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="27" ht="42.0" customHeight="1">
-      <c r="A27" s="45" t="s">
+      <c r="A27" s="29" t="s">
         <v>239</v>
       </c>
-      <c r="B27" s="40" t="s">
+      <c r="B27" s="26" t="s">
         <v>240</v>
       </c>
-      <c r="D27" s="45" t="s">
+      <c r="D27" s="29" t="s">
         <v>241</v>
       </c>
-      <c r="E27" s="40" t="s">
+      <c r="E27" s="26" t="s">
         <v>242</v>
       </c>
-      <c r="G27" s="45" t="s">
+      <c r="G27" s="29" t="s">
         <v>243</v>
       </c>
-      <c r="H27" s="40" t="s">
+      <c r="H27" s="26" t="s">
         <v>244</v>
       </c>
     </row>
     <row r="28" ht="15.0" customHeight="1">
-      <c r="A28" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="B28" s="46" t="s">
-        <v>110</v>
-      </c>
-      <c r="D28" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="E28" s="46" t="s">
-        <v>110</v>
-      </c>
-      <c r="G28" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="H28" s="46" t="s">
-        <v>110</v>
+      <c r="A28" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="B28" s="31" t="s">
+        <v>47</v>
+      </c>
+      <c r="D28" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="E28" s="31" t="s">
+        <v>47</v>
+      </c>
+      <c r="G28" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="H28" s="31" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="29" ht="27.75" customHeight="1">
-      <c r="A29" s="48" t="s">
+      <c r="A29" s="36" t="s">
         <v>245</v>
       </c>
-      <c r="B29" s="48" t="s">
+      <c r="B29" s="36" t="s">
         <v>246</v>
       </c>
-      <c r="D29" s="48" t="s">
+      <c r="D29" s="36" t="s">
         <v>247</v>
       </c>
-      <c r="E29" s="48" t="s">
+      <c r="E29" s="36" t="s">
         <v>248</v>
       </c>
-      <c r="G29" s="48" t="s">
+      <c r="G29" s="36" t="s">
         <v>249</v>
       </c>
-      <c r="H29" s="48" t="s">
+      <c r="H29" s="36" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="30" ht="18.0" customHeight="1">
-      <c r="A30" s="50" t="s">
+      <c r="A30" s="39" t="s">
         <v>251</v>
       </c>
-      <c r="B30" s="16"/>
-      <c r="D30" s="50" t="s">
+      <c r="B30" s="12"/>
+      <c r="D30" s="39" t="s">
         <v>252</v>
       </c>
-      <c r="E30" s="16"/>
-      <c r="G30" s="50" t="s">
+      <c r="E30" s="12"/>
+      <c r="G30" s="39" t="s">
         <v>253</v>
       </c>
-      <c r="H30" s="16"/>
+      <c r="H30" s="12"/>
     </row>
     <row r="31" ht="15.75" customHeight="1"/>
     <row r="32" ht="15.75" customHeight="1"/>
@@ -3499,123 +3499,123 @@
       <c r="A34" s="61" t="s">
         <v>254</v>
       </c>
-      <c r="B34" s="16"/>
+      <c r="B34" s="12"/>
       <c r="D34" s="62" t="s">
         <v>255</v>
       </c>
-      <c r="E34" s="16"/>
+      <c r="E34" s="12"/>
       <c r="G34" s="63" t="s">
         <v>256</v>
       </c>
-      <c r="H34" s="16"/>
+      <c r="H34" s="12"/>
     </row>
     <row r="35" ht="18.0" customHeight="1">
-      <c r="A35" s="24" t="s">
+      <c r="A35" s="16" t="s">
         <v>257</v>
       </c>
-      <c r="B35" s="16"/>
-      <c r="D35" s="24" t="s">
+      <c r="B35" s="12"/>
+      <c r="D35" s="16" t="s">
         <v>258</v>
       </c>
-      <c r="E35" s="16"/>
-      <c r="G35" s="55" t="s">
+      <c r="E35" s="12"/>
+      <c r="G35" s="48" t="s">
         <v>259</v>
       </c>
-      <c r="H35" s="16"/>
+      <c r="H35" s="12"/>
     </row>
     <row r="36" ht="19.5" customHeight="1">
-      <c r="A36" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="B36" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="D36" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="E36" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="G36" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="H36" s="34" t="s">
-        <v>45</v>
+      <c r="A36" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="B36" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="D36" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="E36" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="G36" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="H36" s="21" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="37" ht="42.0" customHeight="1">
-      <c r="A37" s="45" t="s">
+      <c r="A37" s="29" t="s">
         <v>260</v>
       </c>
-      <c r="B37" s="40" t="s">
+      <c r="B37" s="26" t="s">
         <v>261</v>
       </c>
-      <c r="D37" s="45" t="s">
+      <c r="D37" s="29" t="s">
         <v>262</v>
       </c>
-      <c r="E37" s="40" t="s">
+      <c r="E37" s="26" t="s">
         <v>263</v>
       </c>
-      <c r="G37" s="45" t="s">
+      <c r="G37" s="29" t="s">
         <v>264</v>
       </c>
-      <c r="H37" s="40" t="s">
+      <c r="H37" s="26" t="s">
         <v>265</v>
       </c>
     </row>
     <row r="38" ht="15.0" customHeight="1">
-      <c r="A38" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="B38" s="46" t="s">
-        <v>110</v>
-      </c>
-      <c r="D38" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="E38" s="46" t="s">
-        <v>110</v>
-      </c>
-      <c r="G38" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="H38" s="46" t="s">
-        <v>110</v>
+      <c r="A38" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="B38" s="31" t="s">
+        <v>47</v>
+      </c>
+      <c r="D38" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="E38" s="31" t="s">
+        <v>47</v>
+      </c>
+      <c r="G38" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="H38" s="31" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="39" ht="27.75" customHeight="1">
-      <c r="A39" s="48" t="s">
+      <c r="A39" s="36" t="s">
         <v>266</v>
       </c>
-      <c r="B39" s="48" t="s">
+      <c r="B39" s="36" t="s">
         <v>267</v>
       </c>
-      <c r="D39" s="48" t="s">
+      <c r="D39" s="36" t="s">
         <v>268</v>
       </c>
-      <c r="E39" s="48" t="s">
+      <c r="E39" s="36" t="s">
         <v>269</v>
       </c>
-      <c r="G39" s="48" t="s">
+      <c r="G39" s="36" t="s">
         <v>270</v>
       </c>
-      <c r="H39" s="48" t="s">
-        <v>115</v>
+      <c r="H39" s="36" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="40" ht="18.0" customHeight="1">
-      <c r="A40" s="50" t="s">
+      <c r="A40" s="39" t="s">
         <v>271</v>
       </c>
-      <c r="B40" s="16"/>
-      <c r="D40" s="50" t="s">
+      <c r="B40" s="12"/>
+      <c r="D40" s="39" t="s">
         <v>272</v>
       </c>
-      <c r="E40" s="16"/>
-      <c r="G40" s="50" t="s">
+      <c r="E40" s="12"/>
+      <c r="G40" s="39" t="s">
         <v>273</v>
       </c>
-      <c r="H40" s="16"/>
+      <c r="H40" s="12"/>
     </row>
     <row r="41" ht="15.75" customHeight="1"/>
     <row r="42" ht="15.75" customHeight="1"/>
@@ -3624,123 +3624,123 @@
       <c r="A44" s="64" t="s">
         <v>274</v>
       </c>
-      <c r="B44" s="16"/>
+      <c r="B44" s="12"/>
       <c r="D44" s="65" t="s">
         <v>275</v>
       </c>
-      <c r="E44" s="16"/>
+      <c r="E44" s="12"/>
       <c r="G44" s="66" t="s">
         <v>276</v>
       </c>
-      <c r="H44" s="16"/>
+      <c r="H44" s="12"/>
     </row>
     <row r="45" ht="18.0" customHeight="1">
-      <c r="A45" s="24" t="s">
+      <c r="A45" s="16" t="s">
         <v>277</v>
       </c>
-      <c r="B45" s="16"/>
-      <c r="D45" s="24" t="s">
-        <v>36</v>
-      </c>
-      <c r="E45" s="16"/>
-      <c r="G45" s="24" t="s">
-        <v>36</v>
-      </c>
-      <c r="H45" s="16"/>
+      <c r="B45" s="12"/>
+      <c r="D45" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="E45" s="12"/>
+      <c r="G45" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="H45" s="12"/>
     </row>
     <row r="46" ht="19.5" customHeight="1">
-      <c r="A46" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="B46" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="D46" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="E46" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="G46" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="H46" s="34" t="s">
-        <v>45</v>
+      <c r="A46" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="B46" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="D46" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="E46" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="G46" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="H46" s="21" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="47" ht="42.0" customHeight="1">
-      <c r="A47" s="45" t="s">
+      <c r="A47" s="29" t="s">
         <v>278</v>
       </c>
-      <c r="B47" s="40" t="s">
+      <c r="B47" s="26" t="s">
         <v>279</v>
       </c>
-      <c r="D47" s="45" t="s">
+      <c r="D47" s="29" t="s">
         <v>280</v>
       </c>
-      <c r="E47" s="40" t="s">
+      <c r="E47" s="26" t="s">
         <v>281</v>
       </c>
-      <c r="G47" s="45" t="s">
+      <c r="G47" s="29" t="s">
         <v>282</v>
       </c>
-      <c r="H47" s="40" t="s">
+      <c r="H47" s="26" t="s">
         <v>283</v>
       </c>
     </row>
     <row r="48" ht="15.0" customHeight="1">
-      <c r="A48" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="B48" s="46" t="s">
-        <v>110</v>
-      </c>
-      <c r="D48" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="E48" s="46" t="s">
-        <v>110</v>
-      </c>
-      <c r="G48" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="H48" s="46" t="s">
-        <v>110</v>
+      <c r="A48" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="B48" s="31" t="s">
+        <v>47</v>
+      </c>
+      <c r="D48" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="E48" s="31" t="s">
+        <v>47</v>
+      </c>
+      <c r="G48" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="H48" s="31" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="49" ht="27.75" customHeight="1">
-      <c r="A49" s="48" t="s">
+      <c r="A49" s="36" t="s">
         <v>284</v>
       </c>
-      <c r="B49" s="48" t="s">
+      <c r="B49" s="36" t="s">
         <v>285</v>
       </c>
-      <c r="D49" s="48" t="s">
+      <c r="D49" s="36" t="s">
         <v>286</v>
       </c>
-      <c r="E49" s="48" t="s">
+      <c r="E49" s="36" t="s">
         <v>287</v>
       </c>
-      <c r="G49" s="48" t="s">
+      <c r="G49" s="36" t="s">
         <v>288</v>
       </c>
-      <c r="H49" s="48" t="s">
+      <c r="H49" s="36" t="s">
         <v>289</v>
       </c>
     </row>
     <row r="50" ht="18.0" customHeight="1">
-      <c r="A50" s="50" t="s">
+      <c r="A50" s="39" t="s">
         <v>290</v>
       </c>
-      <c r="B50" s="16"/>
-      <c r="D50" s="50" t="s">
+      <c r="B50" s="12"/>
+      <c r="D50" s="39" t="s">
         <v>291</v>
       </c>
-      <c r="E50" s="16"/>
-      <c r="G50" s="50" t="s">
+      <c r="E50" s="12"/>
+      <c r="G50" s="39" t="s">
         <v>292</v>
       </c>
-      <c r="H50" s="16"/>
+      <c r="H50" s="12"/>
     </row>
     <row r="51" ht="15.75" customHeight="1"/>
     <row r="52" ht="15.75" customHeight="1"/>
@@ -3749,123 +3749,123 @@
       <c r="A54" s="67" t="s">
         <v>293</v>
       </c>
-      <c r="B54" s="16"/>
+      <c r="B54" s="12"/>
       <c r="D54" s="68" t="s">
         <v>294</v>
       </c>
-      <c r="E54" s="16"/>
+      <c r="E54" s="12"/>
       <c r="G54" s="69" t="s">
         <v>295</v>
       </c>
-      <c r="H54" s="16"/>
+      <c r="H54" s="12"/>
     </row>
     <row r="55" ht="18.0" customHeight="1">
-      <c r="A55" s="24" t="s">
+      <c r="A55" s="16" t="s">
         <v>296</v>
       </c>
-      <c r="B55" s="16"/>
-      <c r="D55" s="24" t="s">
+      <c r="B55" s="12"/>
+      <c r="D55" s="16" t="s">
         <v>297</v>
       </c>
-      <c r="E55" s="16"/>
-      <c r="G55" s="24" t="s">
-        <v>36</v>
-      </c>
-      <c r="H55" s="16"/>
+      <c r="E55" s="12"/>
+      <c r="G55" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="H55" s="12"/>
     </row>
     <row r="56" ht="19.5" customHeight="1">
-      <c r="A56" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="B56" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="D56" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="E56" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="G56" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="H56" s="34" t="s">
-        <v>45</v>
+      <c r="A56" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="B56" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="D56" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="E56" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="G56" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="H56" s="21" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="57" ht="42.0" customHeight="1">
-      <c r="A57" s="45" t="s">
+      <c r="A57" s="29" t="s">
         <v>298</v>
       </c>
-      <c r="B57" s="40" t="s">
+      <c r="B57" s="26" t="s">
         <v>299</v>
       </c>
-      <c r="D57" s="45" t="s">
-        <v>101</v>
-      </c>
-      <c r="E57" s="40" t="s">
+      <c r="D57" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="E57" s="26" t="s">
         <v>300</v>
       </c>
-      <c r="G57" s="45" t="s">
+      <c r="G57" s="29" t="s">
         <v>301</v>
       </c>
-      <c r="H57" s="40" t="s">
+      <c r="H57" s="26" t="s">
         <v>302</v>
       </c>
     </row>
     <row r="58" ht="15.0" customHeight="1">
-      <c r="A58" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="B58" s="46" t="s">
-        <v>110</v>
-      </c>
-      <c r="D58" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="E58" s="46" t="s">
-        <v>110</v>
-      </c>
-      <c r="G58" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="H58" s="46" t="s">
-        <v>110</v>
+      <c r="A58" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="B58" s="31" t="s">
+        <v>47</v>
+      </c>
+      <c r="D58" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="E58" s="31" t="s">
+        <v>47</v>
+      </c>
+      <c r="G58" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="H58" s="31" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="59" ht="27.75" customHeight="1">
-      <c r="A59" s="48" t="s">
+      <c r="A59" s="36" t="s">
         <v>303</v>
       </c>
-      <c r="B59" s="48" t="s">
+      <c r="B59" s="36" t="s">
         <v>304</v>
       </c>
-      <c r="D59" s="48" t="s">
+      <c r="D59" s="36" t="s">
         <v>305</v>
       </c>
-      <c r="E59" s="48" t="s">
+      <c r="E59" s="36" t="s">
         <v>306</v>
       </c>
-      <c r="G59" s="48" t="s">
+      <c r="G59" s="36" t="s">
         <v>307</v>
       </c>
-      <c r="H59" s="48" t="s">
+      <c r="H59" s="36" t="s">
         <v>308</v>
       </c>
     </row>
     <row r="60" ht="18.0" customHeight="1">
-      <c r="A60" s="50" t="s">
+      <c r="A60" s="39" t="s">
         <v>309</v>
       </c>
-      <c r="B60" s="16"/>
-      <c r="D60" s="50" t="s">
+      <c r="B60" s="12"/>
+      <c r="D60" s="39" t="s">
         <v>310</v>
       </c>
-      <c r="E60" s="16"/>
-      <c r="G60" s="50" t="s">
+      <c r="E60" s="12"/>
+      <c r="G60" s="39" t="s">
         <v>311</v>
       </c>
-      <c r="H60" s="16"/>
+      <c r="H60" s="12"/>
     </row>
     <row r="61" ht="15.75" customHeight="1"/>
     <row r="62" ht="15.75" customHeight="1"/>
@@ -4893,7 +4893,7 @@
   <sheetData>
     <row r="1" ht="31.5" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -4901,10 +4901,10 @@
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
-      <c r="H1" s="5"/>
+      <c r="H1" s="4"/>
     </row>
     <row r="2" ht="19.5" customHeight="1">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="7" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="3"/>
@@ -4913,304 +4913,304 @@
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
-      <c r="H2" s="5"/>
+      <c r="H2" s="4"/>
     </row>
     <row r="4" ht="21.75" customHeight="1">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="12"/>
+      <c r="D4" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="16"/>
-      <c r="D4" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" s="16"/>
-      <c r="G4" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="H4" s="16"/>
+      <c r="E4" s="12"/>
+      <c r="G4" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" s="12"/>
     </row>
     <row r="5" ht="18.0" customHeight="1">
-      <c r="A5" s="24" t="s">
-        <v>24</v>
-      </c>
-      <c r="B5" s="16"/>
-      <c r="D5" s="24" t="s">
+      <c r="A5" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="12"/>
+      <c r="D5" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="12"/>
+      <c r="G5" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" s="12"/>
+    </row>
+    <row r="6" ht="19.5" customHeight="1">
+      <c r="A6" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="G6" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" s="21" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" ht="42.0" customHeight="1">
+      <c r="A7" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="16"/>
-      <c r="G5" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="H5" s="16"/>
-    </row>
-    <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="31" t="s">
+      <c r="B7" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="D6" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="E6" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="G6" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="H6" s="34" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="7" ht="42.0" customHeight="1">
-      <c r="A7" s="38" t="s">
-        <v>49</v>
-      </c>
-      <c r="B7" s="40" t="s">
+      <c r="D7" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="G7" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="H7" s="26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" ht="15.0" customHeight="1">
+      <c r="A8" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" s="31" t="s">
+        <v>47</v>
+      </c>
+      <c r="D8" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="E8" s="31" t="s">
+        <v>47</v>
+      </c>
+      <c r="G8" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="H8" s="31" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" ht="27.75" customHeight="1">
+      <c r="A9" s="36" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" s="36" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" s="36" t="s">
+        <v>55</v>
+      </c>
+      <c r="E9" s="36" t="s">
+        <v>56</v>
+      </c>
+      <c r="G9" s="36" t="s">
         <v>57</v>
       </c>
-      <c r="D7" s="45" t="s">
+      <c r="H9" s="36" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10" ht="18.0" customHeight="1">
+      <c r="A10" s="39" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" s="12"/>
+      <c r="D10" s="39" t="s">
+        <v>61</v>
+      </c>
+      <c r="E10" s="12"/>
+      <c r="G10" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="H10" s="12"/>
+    </row>
+    <row r="14" ht="21.75" customHeight="1">
+      <c r="A14" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B14" s="12"/>
+      <c r="D14" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="E14" s="12"/>
+      <c r="G14" s="44" t="s">
         <v>70</v>
       </c>
-      <c r="E7" s="40" t="s">
-        <v>95</v>
-      </c>
-      <c r="G7" s="45" t="s">
-        <v>101</v>
-      </c>
-      <c r="H7" s="40" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="46" t="s">
+      <c r="H14" s="12"/>
+    </row>
+    <row r="15" ht="18.0" customHeight="1">
+      <c r="A15" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="B15" s="12"/>
+      <c r="D15" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="E15" s="12"/>
+      <c r="G15" s="48" t="s">
+        <v>80</v>
+      </c>
+      <c r="H15" s="12"/>
+    </row>
+    <row r="16" ht="19.5" customHeight="1">
+      <c r="A16" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="D16" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="E16" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="G16" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="H16" s="21" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" ht="42.0" customHeight="1">
+      <c r="A17" s="29" t="s">
+        <v>89</v>
+      </c>
+      <c r="B17" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="D17" s="29" t="s">
+        <v>94</v>
+      </c>
+      <c r="E17" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="B8" s="46" t="s">
-        <v>110</v>
-      </c>
-      <c r="D8" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="E8" s="46" t="s">
-        <v>110</v>
-      </c>
-      <c r="G8" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="H8" s="46" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="9" ht="27.75" customHeight="1">
-      <c r="A9" s="48" t="s">
-        <v>114</v>
-      </c>
-      <c r="B9" s="48" t="s">
-        <v>130</v>
-      </c>
-      <c r="D9" s="48" t="s">
-        <v>132</v>
-      </c>
-      <c r="E9" s="48" t="s">
-        <v>135</v>
-      </c>
-      <c r="G9" s="48" t="s">
-        <v>139</v>
-      </c>
-      <c r="H9" s="48" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="10" ht="18.0" customHeight="1">
-      <c r="A10" s="50" t="s">
-        <v>149</v>
-      </c>
-      <c r="B10" s="16"/>
-      <c r="D10" s="50" t="s">
-        <v>159</v>
-      </c>
-      <c r="E10" s="16"/>
-      <c r="G10" s="50" t="s">
-        <v>167</v>
-      </c>
-      <c r="H10" s="16"/>
-    </row>
-    <row r="14" ht="21.75" customHeight="1">
-      <c r="A14" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="B14" s="16"/>
-      <c r="D14" s="13" t="s">
-        <v>184</v>
-      </c>
-      <c r="E14" s="16"/>
-      <c r="G14" s="53" t="s">
-        <v>193</v>
-      </c>
-      <c r="H14" s="16"/>
-    </row>
-    <row r="15" ht="18.0" customHeight="1">
-      <c r="A15" s="24" t="s">
-        <v>197</v>
-      </c>
-      <c r="B15" s="16"/>
-      <c r="D15" s="24" t="s">
-        <v>198</v>
-      </c>
-      <c r="E15" s="16"/>
-      <c r="G15" s="55" t="s">
-        <v>199</v>
-      </c>
-      <c r="H15" s="16"/>
-    </row>
-    <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="B16" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="D16" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="E16" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="G16" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="H16" s="34" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="17" ht="42.0" customHeight="1">
-      <c r="A17" s="45" t="s">
-        <v>202</v>
-      </c>
-      <c r="B17" s="40" t="s">
-        <v>203</v>
-      </c>
-      <c r="D17" s="45" t="s">
-        <v>205</v>
-      </c>
-      <c r="E17" s="56" t="s">
-        <v>210</v>
-      </c>
-      <c r="G17" s="38" t="s">
-        <v>212</v>
-      </c>
-      <c r="H17" s="56" t="s">
-        <v>213</v>
+      <c r="G17" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="H17" s="51" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="18" ht="15.0" customHeight="1">
-      <c r="A18" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="B18" s="46" t="s">
-        <v>110</v>
-      </c>
-      <c r="D18" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="E18" s="46" t="s">
-        <v>110</v>
-      </c>
-      <c r="G18" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="H18" s="46" t="s">
-        <v>110</v>
+      <c r="A18" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" s="31" t="s">
+        <v>47</v>
+      </c>
+      <c r="D18" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="E18" s="31" t="s">
+        <v>47</v>
+      </c>
+      <c r="G18" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="H18" s="31" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="19" ht="27.75" customHeight="1">
-      <c r="A19" s="48" t="s">
-        <v>221</v>
-      </c>
-      <c r="B19" s="48" t="s">
-        <v>222</v>
-      </c>
-      <c r="D19" s="48" t="s">
-        <v>223</v>
-      </c>
-      <c r="E19" s="48" t="s">
-        <v>115</v>
-      </c>
-      <c r="G19" s="48" t="s">
-        <v>115</v>
-      </c>
-      <c r="H19" s="48" t="s">
-        <v>115</v>
+      <c r="A19" s="36" t="s">
+        <v>118</v>
+      </c>
+      <c r="B19" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="D19" s="36" t="s">
+        <v>124</v>
+      </c>
+      <c r="E19" s="36" t="s">
+        <v>122</v>
+      </c>
+      <c r="G19" s="36" t="s">
+        <v>122</v>
+      </c>
+      <c r="H19" s="36" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="20" ht="18.0" customHeight="1">
-      <c r="A20" s="50" t="s">
-        <v>225</v>
-      </c>
-      <c r="B20" s="16"/>
-      <c r="D20" s="50" t="s">
-        <v>226</v>
-      </c>
-      <c r="E20" s="16"/>
-      <c r="G20" s="57" t="s">
-        <v>228</v>
-      </c>
-      <c r="H20" s="16"/>
+      <c r="A20" s="39" t="s">
+        <v>134</v>
+      </c>
+      <c r="B20" s="12"/>
+      <c r="D20" s="39" t="s">
+        <v>147</v>
+      </c>
+      <c r="E20" s="12"/>
+      <c r="G20" s="54" t="s">
+        <v>164</v>
+      </c>
+      <c r="H20" s="12"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
     <row r="23" ht="15.75" customHeight="1"/>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="53" t="s">
-        <v>230</v>
-      </c>
-      <c r="B24" s="16"/>
+      <c r="A24" s="44" t="s">
+        <v>184</v>
+      </c>
+      <c r="B24" s="12"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="55" t="s">
-        <v>232</v>
-      </c>
-      <c r="B25" s="16"/>
+      <c r="A25" s="48" t="s">
+        <v>193</v>
+      </c>
+      <c r="B25" s="12"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="B26" s="34" t="s">
-        <v>45</v>
+      <c r="A26" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="B26" s="21" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="27" ht="44.25" customHeight="1">
-      <c r="A27" s="38" t="s">
-        <v>234</v>
-      </c>
-      <c r="B27" s="56" t="s">
-        <v>235</v>
+      <c r="A27" s="24" t="s">
+        <v>211</v>
+      </c>
+      <c r="B27" s="51" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="B28" s="46" t="s">
-        <v>110</v>
+      <c r="A28" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="B28" s="31" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="29" ht="27.75" customHeight="1">
-      <c r="A29" s="48" t="s">
-        <v>115</v>
-      </c>
-      <c r="B29" s="48" t="s">
-        <v>115</v>
+      <c r="A29" s="36" t="s">
+        <v>122</v>
+      </c>
+      <c r="B29" s="36" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="57" t="s">
-        <v>237</v>
-      </c>
-      <c r="B30" s="16"/>
+      <c r="A30" s="54" t="s">
+        <v>218</v>
+      </c>
+      <c r="B30" s="12"/>
     </row>
     <row r="31" ht="15.75" customHeight="1"/>
     <row r="32" ht="15.75" customHeight="1"/>
@@ -6234,438 +6234,438 @@
   </cols>
   <sheetData>
     <row r="1" ht="27.75" customHeight="1">
-      <c r="A1" s="6" t="s">
-        <v>3</v>
+      <c r="A1" s="9" t="s">
+        <v>1</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
-      <c r="E1" s="5"/>
+      <c r="E1" s="4"/>
     </row>
     <row r="2" ht="18.0" customHeight="1">
-      <c r="A2" s="9"/>
+      <c r="A2" s="15"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
-      <c r="E2" s="5"/>
+      <c r="E2" s="4"/>
     </row>
     <row r="3">
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="8" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" ht="24.0" customHeight="1">
-      <c r="A4" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>14</v>
+      <c r="A4" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" s="30" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="30" t="s">
+        <v>45</v>
+      </c>
+      <c r="E4" s="25" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="5" ht="21.75" customHeight="1">
-      <c r="A5" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="22" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" s="26" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5" s="28" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" s="29" t="s">
-        <v>37</v>
+      <c r="A5" s="33" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="35" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" s="42" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" s="45" t="s">
+        <v>73</v>
+      </c>
+      <c r="E5" s="46" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="6" ht="21.75" customHeight="1">
-      <c r="A6" s="32" t="s">
-        <v>38</v>
-      </c>
-      <c r="B6" s="36" t="s">
-        <v>46</v>
-      </c>
-      <c r="C6" s="26" t="s">
-        <v>53</v>
-      </c>
-      <c r="D6" s="28" t="s">
-        <v>54</v>
-      </c>
-      <c r="E6" s="39" t="s">
-        <v>56</v>
+      <c r="A6" s="47" t="s">
+        <v>81</v>
+      </c>
+      <c r="B6" s="49" t="s">
+        <v>82</v>
+      </c>
+      <c r="C6" s="42" t="s">
+        <v>84</v>
+      </c>
+      <c r="D6" s="45" t="s">
+        <v>86</v>
+      </c>
+      <c r="E6" s="50" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="7" ht="21.75" customHeight="1">
-      <c r="A7" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="B7" s="22" t="s">
-        <v>62</v>
-      </c>
-      <c r="C7" s="26" t="s">
-        <v>63</v>
-      </c>
-      <c r="D7" s="28" t="s">
-        <v>64</v>
-      </c>
-      <c r="E7" s="29" t="s">
-        <v>65</v>
+      <c r="A7" s="33" t="s">
+        <v>93</v>
+      </c>
+      <c r="B7" s="35" t="s">
+        <v>95</v>
+      </c>
+      <c r="C7" s="42" t="s">
+        <v>97</v>
+      </c>
+      <c r="D7" s="45" t="s">
+        <v>99</v>
+      </c>
+      <c r="E7" s="46" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="8" ht="21.75" customHeight="1">
-      <c r="A8" s="32" t="s">
-        <v>66</v>
-      </c>
-      <c r="B8" s="36" t="s">
-        <v>22</v>
-      </c>
-      <c r="C8" s="26" t="s">
-        <v>68</v>
-      </c>
-      <c r="D8" s="28" t="s">
-        <v>69</v>
-      </c>
-      <c r="E8" s="39" t="s">
-        <v>71</v>
+      <c r="A8" s="47" t="s">
+        <v>101</v>
+      </c>
+      <c r="B8" s="49" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" s="42" t="s">
+        <v>102</v>
+      </c>
+      <c r="D8" s="45" t="s">
+        <v>103</v>
+      </c>
+      <c r="E8" s="50" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="9" ht="21.75" customHeight="1">
-      <c r="A9" s="19" t="s">
-        <v>72</v>
-      </c>
-      <c r="B9" s="22" t="s">
-        <v>73</v>
-      </c>
-      <c r="C9" s="26" t="s">
-        <v>74</v>
-      </c>
-      <c r="D9" s="28" t="s">
-        <v>75</v>
-      </c>
-      <c r="E9" s="29" t="s">
-        <v>76</v>
+      <c r="A9" s="33" t="s">
+        <v>107</v>
+      </c>
+      <c r="B9" s="35" t="s">
+        <v>108</v>
+      </c>
+      <c r="C9" s="42" t="s">
+        <v>109</v>
+      </c>
+      <c r="D9" s="45" t="s">
+        <v>110</v>
+      </c>
+      <c r="E9" s="46" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="10" ht="21.75" customHeight="1">
-      <c r="A10" s="32" t="s">
-        <v>77</v>
-      </c>
-      <c r="B10" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="C10" s="26" t="s">
-        <v>79</v>
-      </c>
-      <c r="D10" s="28" t="s">
-        <v>80</v>
-      </c>
-      <c r="E10" s="39" t="s">
-        <v>81</v>
+      <c r="A10" s="47" t="s">
+        <v>112</v>
+      </c>
+      <c r="B10" s="49" t="s">
+        <v>113</v>
+      </c>
+      <c r="C10" s="42" t="s">
+        <v>115</v>
+      </c>
+      <c r="D10" s="45" t="s">
+        <v>116</v>
+      </c>
+      <c r="E10" s="50" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="11" ht="21.75" customHeight="1">
-      <c r="A11" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="B11" s="22" t="s">
-        <v>84</v>
-      </c>
-      <c r="C11" s="26" t="s">
-        <v>85</v>
-      </c>
-      <c r="D11" s="28" t="s">
-        <v>86</v>
-      </c>
-      <c r="E11" s="29" t="s">
-        <v>87</v>
+      <c r="A11" s="33" t="s">
+        <v>119</v>
+      </c>
+      <c r="B11" s="35" t="s">
+        <v>121</v>
+      </c>
+      <c r="C11" s="42" t="s">
+        <v>123</v>
+      </c>
+      <c r="D11" s="45" t="s">
+        <v>125</v>
+      </c>
+      <c r="E11" s="46" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="12" ht="21.75" customHeight="1">
-      <c r="A12" s="32" t="s">
-        <v>88</v>
-      </c>
-      <c r="B12" s="36" t="s">
-        <v>91</v>
-      </c>
-      <c r="C12" s="26" t="s">
-        <v>93</v>
-      </c>
-      <c r="D12" s="28" t="s">
-        <v>96</v>
-      </c>
-      <c r="E12" s="39" t="s">
-        <v>99</v>
+      <c r="A12" s="47" t="s">
+        <v>128</v>
+      </c>
+      <c r="B12" s="49" t="s">
+        <v>130</v>
+      </c>
+      <c r="C12" s="42" t="s">
+        <v>131</v>
+      </c>
+      <c r="D12" s="45" t="s">
+        <v>132</v>
+      </c>
+      <c r="E12" s="50" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="13" ht="21.75" customHeight="1">
-      <c r="A13" s="19" t="s">
-        <v>100</v>
-      </c>
-      <c r="B13" s="22" t="s">
-        <v>22</v>
-      </c>
-      <c r="C13" s="26" t="s">
-        <v>104</v>
-      </c>
-      <c r="D13" s="28" t="s">
-        <v>105</v>
-      </c>
-      <c r="E13" s="29" t="s">
-        <v>106</v>
+      <c r="A13" s="33" t="s">
+        <v>135</v>
+      </c>
+      <c r="B13" s="35" t="s">
+        <v>50</v>
+      </c>
+      <c r="C13" s="42" t="s">
+        <v>138</v>
+      </c>
+      <c r="D13" s="45" t="s">
+        <v>139</v>
+      </c>
+      <c r="E13" s="46" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="14" ht="21.75" customHeight="1">
-      <c r="A14" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="B14" s="36" t="s">
-        <v>108</v>
-      </c>
-      <c r="C14" s="26" t="s">
-        <v>112</v>
-      </c>
-      <c r="D14" s="28" t="s">
-        <v>116</v>
-      </c>
-      <c r="E14" s="39" t="s">
-        <v>117</v>
+      <c r="A14" s="47" t="s">
+        <v>141</v>
+      </c>
+      <c r="B14" s="49" t="s">
+        <v>143</v>
+      </c>
+      <c r="C14" s="42" t="s">
+        <v>144</v>
+      </c>
+      <c r="D14" s="45" t="s">
+        <v>145</v>
+      </c>
+      <c r="E14" s="50" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="15" ht="21.75" customHeight="1">
-      <c r="A15" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="B15" s="22" t="s">
-        <v>119</v>
-      </c>
-      <c r="C15" s="26" t="s">
-        <v>120</v>
-      </c>
-      <c r="D15" s="28" t="s">
-        <v>122</v>
-      </c>
-      <c r="E15" s="29" t="s">
-        <v>123</v>
+      <c r="A15" s="33" t="s">
+        <v>148</v>
+      </c>
+      <c r="B15" s="35" t="s">
+        <v>149</v>
+      </c>
+      <c r="C15" s="42" t="s">
+        <v>150</v>
+      </c>
+      <c r="D15" s="45" t="s">
+        <v>151</v>
+      </c>
+      <c r="E15" s="46" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="16" ht="21.75" customHeight="1">
-      <c r="A16" s="32" t="s">
-        <v>125</v>
-      </c>
-      <c r="B16" s="36" t="s">
-        <v>126</v>
-      </c>
-      <c r="C16" s="26" t="s">
-        <v>127</v>
-      </c>
-      <c r="D16" s="28" t="s">
+      <c r="A16" s="47" t="s">
+        <v>154</v>
+      </c>
+      <c r="B16" s="49" t="s">
+        <v>155</v>
+      </c>
+      <c r="C16" s="42" t="s">
+        <v>156</v>
+      </c>
+      <c r="D16" s="45" t="s">
+        <v>157</v>
+      </c>
+      <c r="E16" s="50" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="17" ht="21.75" customHeight="1">
+      <c r="A17" s="33" t="s">
+        <v>158</v>
+      </c>
+      <c r="B17" s="35" t="s">
+        <v>160</v>
+      </c>
+      <c r="C17" s="42" t="s">
+        <v>161</v>
+      </c>
+      <c r="D17" s="45" t="s">
+        <v>162</v>
+      </c>
+      <c r="E17" s="46" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="18" ht="21.75" customHeight="1">
+      <c r="A18" s="47" t="s">
+        <v>165</v>
+      </c>
+      <c r="B18" s="49" t="s">
+        <v>50</v>
+      </c>
+      <c r="C18" s="42" t="s">
+        <v>166</v>
+      </c>
+      <c r="D18" s="45" t="s">
+        <v>167</v>
+      </c>
+      <c r="E18" s="50" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="19" ht="21.75" customHeight="1">
+      <c r="A19" s="33" t="s">
+        <v>133</v>
+      </c>
+      <c r="B19" s="35" t="s">
+        <v>50</v>
+      </c>
+      <c r="C19" s="42" t="s">
+        <v>169</v>
+      </c>
+      <c r="D19" s="45" t="s">
+        <v>170</v>
+      </c>
+      <c r="E19" s="46" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="20" ht="21.75" customHeight="1">
+      <c r="A20" s="47" t="s">
+        <v>172</v>
+      </c>
+      <c r="B20" s="49" t="s">
+        <v>173</v>
+      </c>
+      <c r="C20" s="42" t="s">
+        <v>175</v>
+      </c>
+      <c r="D20" s="45" t="s">
+        <v>176</v>
+      </c>
+      <c r="E20" s="50" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="21" ht="21.75" customHeight="1">
+      <c r="A21" s="33" t="s">
+        <v>178</v>
+      </c>
+      <c r="B21" s="35" t="s">
+        <v>179</v>
+      </c>
+      <c r="C21" s="42" t="s">
+        <v>180</v>
+      </c>
+      <c r="D21" s="45" t="s">
+        <v>181</v>
+      </c>
+      <c r="E21" s="46" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="22" ht="21.75" customHeight="1">
+      <c r="A22" s="47" t="s">
+        <v>183</v>
+      </c>
+      <c r="B22" s="49" t="s">
+        <v>50</v>
+      </c>
+      <c r="C22" s="42" t="s">
+        <v>185</v>
+      </c>
+      <c r="D22" s="45" t="s">
+        <v>186</v>
+      </c>
+      <c r="E22" s="50" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="23" ht="21.75" customHeight="1">
+      <c r="A23" s="33" t="s">
+        <v>188</v>
+      </c>
+      <c r="B23" s="35" t="s">
+        <v>189</v>
+      </c>
+      <c r="C23" s="42" t="s">
+        <v>191</v>
+      </c>
+      <c r="D23" s="45" t="s">
+        <v>192</v>
+      </c>
+      <c r="E23" s="46" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="24" ht="21.75" customHeight="1">
+      <c r="A24" s="47" t="s">
+        <v>195</v>
+      </c>
+      <c r="B24" s="49" t="s">
+        <v>196</v>
+      </c>
+      <c r="C24" s="42" t="s">
+        <v>198</v>
+      </c>
+      <c r="D24" s="45" t="s">
+        <v>199</v>
+      </c>
+      <c r="E24" s="50" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="25" ht="21.75" customHeight="1">
+      <c r="A25" s="33" t="s">
+        <v>201</v>
+      </c>
+      <c r="B25" s="35" t="s">
+        <v>202</v>
+      </c>
+      <c r="C25" s="42" t="s">
+        <v>180</v>
+      </c>
+      <c r="D25" s="45" t="s">
+        <v>203</v>
+      </c>
+      <c r="E25" s="46" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="26" ht="21.75" customHeight="1">
+      <c r="A26" s="47" t="s">
+        <v>205</v>
+      </c>
+      <c r="B26" s="49" t="s">
+        <v>206</v>
+      </c>
+      <c r="C26" s="42" t="s">
+        <v>207</v>
+      </c>
+      <c r="D26" s="45" t="s">
+        <v>208</v>
+      </c>
+      <c r="E26" s="50" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="27" ht="21.75" customHeight="1">
+      <c r="A27" s="33" t="s">
+        <v>210</v>
+      </c>
+      <c r="B27" s="35" t="s">
+        <v>212</v>
+      </c>
+      <c r="C27" s="42" t="s">
+        <v>213</v>
+      </c>
+      <c r="D27" s="45" t="s">
+        <v>215</v>
+      </c>
+      <c r="E27" s="46" t="s">
         <v>128</v>
-      </c>
-      <c r="E16" s="39" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="17" ht="21.75" customHeight="1">
-      <c r="A17" s="19" t="s">
-        <v>133</v>
-      </c>
-      <c r="B17" s="22" t="s">
-        <v>134</v>
-      </c>
-      <c r="C17" s="26" t="s">
-        <v>136</v>
-      </c>
-      <c r="D17" s="28" t="s">
-        <v>138</v>
-      </c>
-      <c r="E17" s="29" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="18" ht="21.75" customHeight="1">
-      <c r="A18" s="32" t="s">
-        <v>141</v>
-      </c>
-      <c r="B18" s="36" t="s">
-        <v>22</v>
-      </c>
-      <c r="C18" s="26" t="s">
-        <v>143</v>
-      </c>
-      <c r="D18" s="28" t="s">
-        <v>144</v>
-      </c>
-      <c r="E18" s="39" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="19" ht="21.75" customHeight="1">
-      <c r="A19" s="19" t="s">
-        <v>99</v>
-      </c>
-      <c r="B19" s="22" t="s">
-        <v>22</v>
-      </c>
-      <c r="C19" s="26" t="s">
-        <v>146</v>
-      </c>
-      <c r="D19" s="28" t="s">
-        <v>148</v>
-      </c>
-      <c r="E19" s="29" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="20" ht="21.75" customHeight="1">
-      <c r="A20" s="32" t="s">
-        <v>151</v>
-      </c>
-      <c r="B20" s="36" t="s">
-        <v>152</v>
-      </c>
-      <c r="C20" s="26" t="s">
-        <v>153</v>
-      </c>
-      <c r="D20" s="28" t="s">
-        <v>154</v>
-      </c>
-      <c r="E20" s="39" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="21" ht="21.75" customHeight="1">
-      <c r="A21" s="19" t="s">
-        <v>157</v>
-      </c>
-      <c r="B21" s="22" t="s">
-        <v>158</v>
-      </c>
-      <c r="C21" s="26" t="s">
-        <v>160</v>
-      </c>
-      <c r="D21" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="E21" s="29" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="22" ht="21.75" customHeight="1">
-      <c r="A22" s="32" t="s">
-        <v>163</v>
-      </c>
-      <c r="B22" s="36" t="s">
-        <v>22</v>
-      </c>
-      <c r="C22" s="26" t="s">
-        <v>164</v>
-      </c>
-      <c r="D22" s="28" t="s">
-        <v>165</v>
-      </c>
-      <c r="E22" s="39" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="23" ht="21.75" customHeight="1">
-      <c r="A23" s="19" t="s">
-        <v>168</v>
-      </c>
-      <c r="B23" s="22" t="s">
-        <v>169</v>
-      </c>
-      <c r="C23" s="26" t="s">
-        <v>170</v>
-      </c>
-      <c r="D23" s="28" t="s">
-        <v>172</v>
-      </c>
-      <c r="E23" s="29" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="24" ht="21.75" customHeight="1">
-      <c r="A24" s="32" t="s">
-        <v>174</v>
-      </c>
-      <c r="B24" s="36" t="s">
-        <v>175</v>
-      </c>
-      <c r="C24" s="26" t="s">
-        <v>176</v>
-      </c>
-      <c r="D24" s="28" t="s">
-        <v>177</v>
-      </c>
-      <c r="E24" s="39" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="25" ht="21.75" customHeight="1">
-      <c r="A25" s="19" t="s">
-        <v>180</v>
-      </c>
-      <c r="B25" s="22" t="s">
-        <v>181</v>
-      </c>
-      <c r="C25" s="26" t="s">
-        <v>160</v>
-      </c>
-      <c r="D25" s="28" t="s">
-        <v>183</v>
-      </c>
-      <c r="E25" s="29" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="26" ht="21.75" customHeight="1">
-      <c r="A26" s="32" t="s">
-        <v>186</v>
-      </c>
-      <c r="B26" s="36" t="s">
-        <v>187</v>
-      </c>
-      <c r="C26" s="26" t="s">
-        <v>188</v>
-      </c>
-      <c r="D26" s="28" t="s">
-        <v>189</v>
-      </c>
-      <c r="E26" s="39" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="27" ht="21.75" customHeight="1">
-      <c r="A27" s="19" t="s">
-        <v>191</v>
-      </c>
-      <c r="B27" s="22" t="s">
-        <v>192</v>
-      </c>
-      <c r="C27" s="26" t="s">
-        <v>195</v>
-      </c>
-      <c r="D27" s="28" t="s">
-        <v>196</v>
-      </c>
-      <c r="E27" s="29" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Atualização automática da planilha (2026-09-15)
</commit_message>
<xml_diff>
--- a/times.xlsx
+++ b/times.xlsx
@@ -16,12 +16,12 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="312">
   <si>
+    <t>GUIA RÁPIDO</t>
+  </si>
+  <si>
     <t>GUIA DE ROTAÇÃO &amp; METAGAME - POKEALLIANCE(PKA)</t>
   </si>
   <si>
-    <t>GUIA RÁPIDO</t>
-  </si>
-  <si>
     <t>RECOMENDAÇÃO DE TIME PARA HUNTS!</t>
   </si>
   <si>
@@ -31,70 +31,13 @@
     <t>Requisitos de Entrada e Progressão 2x2x2.</t>
   </si>
   <si>
+    <t>Segue lá!</t>
+  </si>
+  <si>
+    <t>Com algumas exceções, todos os restantes são SHINYS.</t>
+  </si>
+  <si>
     <t>https://www.twitch.tv/safnaww</t>
-  </si>
-  <si>
-    <t>Segue lá!</t>
-  </si>
-  <si>
-    <t>★ METAGROSS</t>
-  </si>
-  <si>
-    <t>📌 REQUISITOS INICIAIS (START DE ROTAÇÃO)</t>
-  </si>
-  <si>
-    <t>★ LUCARIO</t>
-  </si>
-  <si>
-    <t>⚡ UPGRADE: ROTAÇÃO 2x2x2</t>
-  </si>
-  <si>
-    <t>★ GENGAR</t>
-  </si>
-  <si>
-    <t>Nível &amp; Held:</t>
-  </si>
-  <si>
-    <t>Hunt: Steel / Psychic</t>
-  </si>
-  <si>
-    <t>Hunt: Fighting / Steel</t>
-  </si>
-  <si>
-    <t>Com algumas exceções, todos os restantes são SHINYS.</t>
-  </si>
-  <si>
-    <t>Hunt: Ghost / Poison</t>
-  </si>
-  <si>
-    <t>Todos os Pokémon +15 com Atk 4</t>
-  </si>
-  <si>
-    <t>Todos os Pokémon +25 com Atk 5</t>
-  </si>
-  <si>
-    <t>Atalho / Dica:</t>
-  </si>
-  <si>
-    <t>🛡️ LURAR / TANQUE (T1)</t>
-  </si>
-  <si>
-    <t>Runas de Atk no Pokelog ajudam a adiantar a meta</t>
-  </si>
-  <si>
-    <t>Estrelas Mínimas:</t>
-  </si>
-  <si>
-    <t>⚔️ DPS / DANO (SR)</t>
-  </si>
-  <si>
-    <t>Tier 1: 2★ (estrelas)  |  SR: 1★ (estrela)</t>
-  </si>
-  <si>
-    <t>Meta no Dummy:</t>
-  </si>
-  <si>
-    <t>Bater 560k de dano com 3 Pokémon</t>
   </si>
   <si>
     <r>
@@ -118,10 +61,160 @@
     </r>
   </si>
   <si>
+    <t>📌 REQUISITOS INICIAIS (START DE ROTAÇÃO)</t>
+  </si>
+  <si>
+    <t>Nessa planilha não indicaremos pokémons T2 ou T3 para a rotação.</t>
+  </si>
+  <si>
+    <t>⚡ UPGRADE: ROTAÇÃO 2x2x2</t>
+  </si>
+  <si>
+    <t>★ BUG</t>
+  </si>
+  <si>
+    <t>ELEMENTO / HUNT</t>
+  </si>
+  <si>
+    <t>Nível &amp; Held:</t>
+  </si>
+  <si>
+    <t>★ METAGROSS</t>
+  </si>
+  <si>
+    <t>Todos os Pokémon +15 com Atk 4</t>
+  </si>
+  <si>
+    <t>ALVO (HUNT)</t>
+  </si>
+  <si>
+    <t>Todos os Pokémon +25 com Atk 5</t>
+  </si>
+  <si>
+    <t>Atalho / Dica:</t>
+  </si>
+  <si>
+    <t>Runas de Atk no Pokelog ajudam a adiantar a meta</t>
+  </si>
+  <si>
+    <t>★ FAIRY</t>
+  </si>
+  <si>
+    <t>★ LUCARIO</t>
+  </si>
+  <si>
+    <t>★ GENGAR</t>
+  </si>
+  <si>
+    <t>★ FIRE</t>
+  </si>
+  <si>
+    <t>Estrelas Mínimas:</t>
+  </si>
+  <si>
+    <t>Tier 1: 2★ (estrelas)  |  SR: 1★ (estrela)</t>
+  </si>
+  <si>
+    <t>Meta no Dummy:</t>
+  </si>
+  <si>
+    <t>Hunt: Steel / Psychic</t>
+  </si>
+  <si>
+    <t>Bater 560k de dano com 3 Pokémon</t>
+  </si>
+  <si>
+    <t>Hunt: Em breve</t>
+  </si>
+  <si>
+    <t>Hunt: Fighting / Steel</t>
+  </si>
+  <si>
+    <t>Hunt: Shiny Sylveon (Lendário)</t>
+  </si>
+  <si>
+    <t>Hunt: Ghost / Poison</t>
+  </si>
+  <si>
+    <t>Hunt: Magmar (Lendário) / Torkoal (UR)</t>
+  </si>
+  <si>
+    <t>🛡️ LURAR / TANQUE (T1)</t>
+  </si>
+  <si>
+    <t>🛡️ LURAR (T1)</t>
+  </si>
+  <si>
+    <t>⚔️ DPS (SR)</t>
+  </si>
+  <si>
+    <t>🎨 TIPO SMEARGLE</t>
+  </si>
+  <si>
+    <t>⚔️ DPS / DANO (SR)</t>
+  </si>
+  <si>
+    <t>Bug</t>
+  </si>
+  <si>
+    <t>Em breve</t>
+  </si>
+  <si>
+    <t>⭐ S.Rapidash, S.Typhlosion, S.Steelix</t>
+  </si>
+  <si>
+    <t>⭐S.Rapidash, S.Typhlosion, S.Magcargo</t>
+  </si>
+  <si>
+    <t>Rapidash, Typhlosion, Magcargo</t>
+  </si>
+  <si>
+    <t>⭐ Arcanine, Infernape, Armaldo</t>
+  </si>
+  <si>
     <t>Bater 560k de dano com apenas 2 Pokémon</t>
   </si>
   <si>
-    <t>⭐ S.Rapidash, S.Typhlosion, S.Steelix</t>
+    <t>Arcanine, Infernape, Armaldo</t>
+  </si>
+  <si>
+    <t>⭐ Arcanine, Houndoom, Pupitar</t>
+  </si>
+  <si>
+    <t>⭐ Muk, Tentacruel, Mawile</t>
+  </si>
+  <si>
+    <t>⭐ Hitmontop, Typhlosion, Rapidash</t>
+  </si>
+  <si>
+    <t>Fire, Rock</t>
+  </si>
+  <si>
+    <t>⭐ Aggron, Skarmory, Toxicroak</t>
+  </si>
+  <si>
+    <t>⭐ Blastoise, Feraligatr, Omastar</t>
+  </si>
+  <si>
+    <t>⭐ Arcanine, Machamp, Pupitar</t>
+  </si>
+  <si>
+    <t>Fairy</t>
+  </si>
+  <si>
+    <t>⭐ Umbreon, Crawdaunt, Sableye</t>
+  </si>
+  <si>
+    <t>⭐ Houndoom, Hydreigon, Pupitar</t>
+  </si>
+  <si>
+    <t>⭐ Pupitar, Torterra, Kingdra</t>
+  </si>
+  <si>
+    <t>Shiny Sylveon (Lendário)</t>
+  </si>
+  <si>
+    <t>Outras Opções T1:</t>
   </si>
   <si>
     <t>Regra de Prey:</t>
@@ -130,643 +223,550 @@
     <t>Obrigatório Prey de Atk na hunt (já calculada no dummy)</t>
   </si>
   <si>
+    <t>Outras Opções SR:</t>
+  </si>
+  <si>
     <t>Manter sempre Prey de Atk ativa na hunt</t>
   </si>
   <si>
-    <t>ELEMENTO / HUNT</t>
+    <t>Umbreon</t>
   </si>
   <si>
     <t>💡 POR QUE COMPOSIÇÕES COM 2 A 3 ELEMENTOS SÃO SUPERIORES? (ANTI-MONO)</t>
   </si>
   <si>
-    <t>⭐ Arcanine, Houndoom, Pupitar</t>
-  </si>
-  <si>
-    <t>⭐ Hitmontop, Typhlosion, Rapidash</t>
-  </si>
-  <si>
-    <t>ALVO (HUNT)</t>
-  </si>
-  <si>
-    <t>⭐ Arcanine, Machamp, Pupitar</t>
-  </si>
-  <si>
-    <t>⭐ Umbreon, Crawdaunt, Sableye</t>
-  </si>
-  <si>
-    <t>⭐ Houndoom, Hydreigon, Pupitar</t>
-  </si>
-  <si>
-    <t>Nessa planilha não indicaremos pokémons T2 ou T3 para a rotação.</t>
+    <t>Muk, Tentacruel, Mawile</t>
+  </si>
+  <si>
+    <t>Aggron, Skarmory, Toxicroak</t>
+  </si>
+  <si>
+    <t>Poison, Metal</t>
   </si>
   <si>
     <t>⏱️ Cooldown Reduzido por Tier</t>
   </si>
   <si>
-    <t>🛡️ LURAR (T1)</t>
-  </si>
-  <si>
-    <t>Outras Opções T1:</t>
-  </si>
-  <si>
-    <t>⚔️ DPS (SR)</t>
-  </si>
-  <si>
-    <t>🎨 TIPO SMEARGLE</t>
-  </si>
-  <si>
-    <t>Outras Opções SR:</t>
-  </si>
-  <si>
-    <t>★ BUG</t>
-  </si>
-  <si>
-    <t>Bug</t>
-  </si>
-  <si>
-    <t>Em breve</t>
-  </si>
-  <si>
-    <t>Umbreon</t>
+    <t>S.Charizard, Kabutops, Golem</t>
+  </si>
+  <si>
+    <t>Fire</t>
+  </si>
+  <si>
+    <t>Magmar (Lendário) / Torkoal (UR)</t>
+  </si>
+  <si>
+    <t>Blastoise, Feraligatr, Omastar</t>
+  </si>
+  <si>
+    <t>Pupitar, Torterra, Kingdra</t>
+  </si>
+  <si>
+    <t>Rock, Water, Ground</t>
+  </si>
+  <si>
+    <t>Fighting</t>
+  </si>
+  <si>
+    <t>Mega Clefable, Pidgeot, Espeon</t>
+  </si>
+  <si>
+    <t>Wobbuffet, Mimikyu, Gliscor</t>
+  </si>
+  <si>
+    <t>Psychic, Flying, Fairy</t>
+  </si>
+  <si>
+    <t>Dark</t>
   </si>
   <si>
     <t>No PKA, tiers mais altos não dão só dano: reduzem o cooldown das skills, deixando a rotação muito mais rápida.</t>
   </si>
   <si>
-    <t>Rapidash, Typhlosion, Magcargo</t>
+    <t>Absol (Lendário) / Mightyena (UR)</t>
+  </si>
+  <si>
+    <t>Hitmontop, Hitmonchan, Poliwrath</t>
+  </si>
+  <si>
+    <t>Machamp, Scyther, Mimikyu</t>
+  </si>
+  <si>
+    <t>Fighting, Fairy, Bug</t>
+  </si>
+  <si>
+    <t>Water</t>
+  </si>
+  <si>
+    <t>Milotic (UR)</t>
+  </si>
+  <si>
+    <t>Tangrowth, Ampharos, Venusaur</t>
+  </si>
+  <si>
+    <t>Tangrowth, Gogoat, Luxray</t>
+  </si>
+  <si>
+    <t>Grass, Electric</t>
+  </si>
+  <si>
+    <t>Grass</t>
+  </si>
+  <si>
+    <t>Leafeon (Lendário) / Sceptile (UR)</t>
+  </si>
+  <si>
+    <t>Typhlosion, Rapidash, Pidgeot</t>
+  </si>
+  <si>
+    <t>Arcanine, Infernape, Scyther</t>
+  </si>
+  <si>
+    <t>Poison, Bug, Fire, Fly, Ice</t>
+  </si>
+  <si>
+    <t>Electric</t>
+  </si>
+  <si>
+    <t>Electabuzz (Lendário) / Manectric (UR)</t>
+  </si>
+  <si>
+    <t>Steelix, Nidoqueen, Torterra</t>
+  </si>
+  <si>
+    <t>Torterra, Pupitar, Smeargle</t>
+  </si>
+  <si>
+    <t>Ground</t>
+  </si>
+  <si>
+    <t>Ghost</t>
+  </si>
+  <si>
+    <t>Umbreon, Crawdaunt, Dusknoir</t>
+  </si>
+  <si>
+    <t>Dusknoir, Houndoom, Hydreigon</t>
+  </si>
+  <si>
+    <t>Dark, Ghost</t>
   </si>
   <si>
     <t>Torterra, Misdreavus</t>
   </si>
   <si>
+    <t>Ice</t>
+  </si>
+  <si>
+    <t>Glaceon (Lendário) / Glalie (UR)</t>
+  </si>
+  <si>
+    <t>Typhlosion, Rapidash, Hitmontop</t>
+  </si>
+  <si>
     <t>Poliwrath, Medicham, Hariyama</t>
   </si>
   <si>
+    <t>Infernape, Machamp, Skarmory</t>
+  </si>
+  <si>
+    <t>Fighting, Fire, Metal</t>
+  </si>
+  <si>
     <t>Infernape, Kangaskhan, Torterra</t>
   </si>
   <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>Poison</t>
+  </si>
+  <si>
+    <t>Garbodor (Lendário) / Swalot (UR)</t>
+  </si>
+  <si>
     <t>Cacturne, Banette, Dusclops</t>
   </si>
   <si>
+    <t>Steelix, Espeon, Nidoqueen</t>
+  </si>
+  <si>
+    <t>Metang, Magneton Estrelado</t>
+  </si>
+  <si>
+    <t>Wobbuffet, Mr. Mime, Pupitar</t>
+  </si>
+  <si>
     <t>Misdreavus, Dusknoir, Torterra</t>
   </si>
   <si>
+    <t>Ground, Psychic</t>
+  </si>
+  <si>
+    <t>Normal</t>
+  </si>
+  <si>
+    <t>SevIper</t>
+  </si>
+  <si>
+    <t>Snorlax (Lendário) / Exploud (UR)</t>
+  </si>
+  <si>
+    <t>Poliwrath, Hitmontop, Medicham</t>
+  </si>
+  <si>
+    <t>Machamp, Kangaskhan, Smeargle</t>
+  </si>
+  <si>
+    <t>Rock</t>
+  </si>
+  <si>
+    <t>Rampardos (UR)</t>
+  </si>
+  <si>
+    <t>Tangrowth, Steelix, Blastoise</t>
+  </si>
+  <si>
+    <t>Tangrowth, Machamp, Gogoat</t>
+  </si>
+  <si>
     <t>🎨 Smeargle: Fire, Ground, Ghost, Dark</t>
   </si>
   <si>
-    <t>★ FAIRY</t>
+    <t>Fighting, Ground, Water, Grass</t>
+  </si>
+  <si>
+    <t>Steel</t>
+  </si>
+  <si>
+    <t>Hitmontop, Rapidash, Typhlosion</t>
+  </si>
+  <si>
+    <t>Arcanine, Machamp, Infernape</t>
+  </si>
+  <si>
+    <t>Ground, Fighting, Fire</t>
+  </si>
+  <si>
+    <t>Blastoise, Tangrowth, Gogoat</t>
+  </si>
+  <si>
+    <t>Tangrowth, Kingdra, Sharpedo</t>
+  </si>
+  <si>
+    <t>Water, Ice, Grass</t>
+  </si>
+  <si>
+    <t>Dragon</t>
+  </si>
+  <si>
+    <t>Salamence (UR) / Flygon (Lendário)</t>
+  </si>
+  <si>
+    <t>Lapras, Mega Clefable, Jynx</t>
+  </si>
+  <si>
+    <t>Vaporeon, Rhyperior, Magcargo</t>
+  </si>
+  <si>
+    <t>Mimikyu, Florges, Walrein</t>
+  </si>
+  <si>
+    <t>Dragon, Ice, Fairy</t>
+  </si>
+  <si>
+    <t>Sharpedo</t>
+  </si>
+  <si>
+    <t>Psychic</t>
+  </si>
+  <si>
+    <t>Alakazam (Lendário)</t>
+  </si>
+  <si>
+    <t>Umbreon, Crawdaunt, Sableye</t>
+  </si>
+  <si>
+    <t>Houndoom, Scyther, Dusknoir</t>
+  </si>
+  <si>
+    <t>Ghost, Dark, Bug</t>
+  </si>
+  <si>
+    <t>🎨 Smeargle: Fire, Rock</t>
+  </si>
+  <si>
+    <t>Flying</t>
+  </si>
+  <si>
+    <t>Ampharos, Magcargo, Lapras</t>
+  </si>
+  <si>
+    <t>Walrein, Luxray, Pachirisu</t>
+  </si>
+  <si>
+    <t>Electric, Ice, Rock</t>
+  </si>
+  <si>
+    <t>Metagross</t>
+  </si>
+  <si>
+    <t>Steel / Psychic</t>
+  </si>
+  <si>
+    <t>Rapidash, Typhlosion, Steelix</t>
+  </si>
+  <si>
+    <t>Arcanine, Houndoom, Pupitar</t>
+  </si>
+  <si>
+    <t>Fire, Ground, Ghost, Dark</t>
+  </si>
+  <si>
+    <t>Lucario</t>
+  </si>
+  <si>
+    <t>Fighting / Steel</t>
+  </si>
+  <si>
+    <t>Hitmontop, Typhlosion, Rapidash</t>
+  </si>
+  <si>
+    <t>Arcanine, Machamp, Pupitar</t>
+  </si>
+  <si>
+    <t>Fighting, Fire, Ground</t>
+  </si>
+  <si>
+    <t>Gengar</t>
+  </si>
+  <si>
+    <t>Ghost / Poison</t>
+  </si>
+  <si>
+    <t>🎨 Smeargle: Poison, Metal</t>
+  </si>
+  <si>
+    <t>Houndoom, Hydreigon, Pupitar</t>
+  </si>
+  <si>
+    <t>Dark, Ghost, Ground</t>
+  </si>
+  <si>
+    <t>Gardevoir</t>
+  </si>
+  <si>
+    <t>Psychic / Fairy</t>
+  </si>
+  <si>
+    <t>Mawile, Muk, Tentacruel</t>
+  </si>
+  <si>
+    <t>Toxicroak, Seviper, Misdreavus</t>
+  </si>
+  <si>
+    <t>🎨 Smeargle: Rock, Water, Ground</t>
+  </si>
+  <si>
+    <t>Poison, Ghost, Metal</t>
+  </si>
+  <si>
+    <t>Gyarados</t>
+  </si>
+  <si>
+    <t>Water / Flying</t>
+  </si>
+  <si>
+    <t>Ampharos, Luxray, Jolteon</t>
   </si>
   <si>
     <t>🎨 Smeargle: Fighting, Fire, Ground</t>
   </si>
   <si>
+    <t>Luxray, Pachirisu, Smeargle Eletric</t>
+  </si>
+  <si>
     <t>📈 Mais Mobs e Brokes / Hora</t>
   </si>
   <si>
+    <t>★ FIGHTING</t>
+  </si>
+  <si>
     <t>🎨 Smeargle: Dark, Ghost, Ground</t>
   </si>
   <si>
     <t>Rotação mais fluida = mais mobs derrotados/hora, aumentando drasticamente a chance de Shiny/hr e lucro.</t>
   </si>
   <si>
+    <t>★ DARK</t>
+  </si>
+  <si>
     <t>★ GARDEVOIR</t>
   </si>
   <si>
     <t>⚔️ Hazards Mais Altos</t>
   </si>
   <si>
+    <t>★ WATER</t>
+  </si>
+  <si>
     <t>★ GYARADOS</t>
   </si>
   <si>
-    <t>★ FIRE</t>
-  </si>
-  <si>
     <t>Mesmo encurtando o número total de hunts, permite solar níveis de Hazard superiores com segurança e eficiência.</t>
   </si>
   <si>
+    <t>Hunt: Absol (Lendário) / Mightyena (UR)</t>
+  </si>
+  <si>
     <t>★ SWAMPERT</t>
   </si>
   <si>
     <t>🏆 Futuro &amp; Escalabilidade (Endgame)</t>
   </si>
   <si>
+    <t>Hunt: Milotic (UR)</t>
+  </si>
+  <si>
     <t>Trabalhar com 2 ou 3 elementos abre um catálogo amplo de opções viáveis para evoluir: T1, SR, UR e Lendários.</t>
   </si>
   <si>
-    <t>Arcanine, Infernape, Armaldo</t>
-  </si>
-  <si>
-    <t>Hunt: Em breve</t>
-  </si>
-  <si>
     <t>Hunt: Psychic / Fairy</t>
   </si>
   <si>
-    <t>Hunt: Shiny Sylveon (Lendário)</t>
+    <t>⭐ Mega Clefable, Pidgeot, Espeon</t>
+  </si>
+  <si>
+    <t>⭐ Wobbuffet, Mimikyu, Gliscor</t>
+  </si>
+  <si>
+    <t>⭐ Hitmontop, Hitmonchan, Poliwrath</t>
   </si>
   <si>
     <t>Hunt: Water / Flying</t>
   </si>
   <si>
-    <t>Fire, Rock</t>
-  </si>
-  <si>
-    <t>Hunt: Magmar (Lendário) / Torkoal (UR)</t>
+    <t>⭐ Machamp, Scyther, Mimikyu</t>
+  </si>
+  <si>
+    <t>⭐ Tangrowth, Ampharos, Venusaur</t>
+  </si>
+  <si>
+    <t>⭐ Tangrowth, Gogoat, Luxray</t>
   </si>
   <si>
     <t>Hunt: Water / Ground</t>
   </si>
   <si>
-    <t>Fairy</t>
-  </si>
-  <si>
-    <t>Shiny Sylveon (Lendário)</t>
-  </si>
-  <si>
-    <t>⭐S.Rapidash, S.Typhlosion, S.Magcargo</t>
-  </si>
-  <si>
-    <t>Muk, Tentacruel, Mawile</t>
-  </si>
-  <si>
-    <t>⭐ Arcanine, Infernape, Armaldo</t>
-  </si>
-  <si>
-    <t>Aggron, Skarmory, Toxicroak</t>
-  </si>
-  <si>
-    <t>⭐ Muk, Tentacruel, Mawile</t>
-  </si>
-  <si>
-    <t>Poison, Metal</t>
+    <t>Farfetch'd, Gliscor</t>
+  </si>
+  <si>
+    <t>Mr. Mime, Florges, Swellow</t>
+  </si>
+  <si>
+    <t>Mega Clefable, Hitmonlee</t>
+  </si>
+  <si>
+    <t>Florges, Kangaskhan, Pinsir</t>
+  </si>
+  <si>
+    <t>Luxray, Gogoat</t>
+  </si>
+  <si>
+    <t>Pachirisu</t>
+  </si>
+  <si>
+    <t>🎨 Smeargle: Psychic, Flying, Fairy</t>
   </si>
   <si>
     <t>⭐ Mawile, Muk, Tentacruel</t>
   </si>
   <si>
-    <t>⭐ Aggron, Skarmory, Toxicroak</t>
+    <t>🎨 Smeargle: Fighting, Fairy, Bug</t>
   </si>
   <si>
     <t>⭐ Toxicroak, Seviper, Misdreavus</t>
   </si>
   <si>
-    <t>⭐ Blastoise, Feraligatr, Omastar</t>
-  </si>
-  <si>
-    <t>Fire</t>
-  </si>
-  <si>
     <t>⭐ Ampharos, Luxray, Jolteon</t>
   </si>
   <si>
-    <t>Magmar (Lendário) / Torkoal (UR)</t>
-  </si>
-  <si>
-    <t>⭐ Pupitar, Torterra, Kingdra</t>
-  </si>
-  <si>
-    <t>Blastoise, Feraligatr, Omastar</t>
-  </si>
-  <si>
     <t>⭐ S.Luxray, S.Pachirisu, Smeargle Eletric</t>
   </si>
   <si>
-    <t>Pupitar, Torterra, Kingdra</t>
-  </si>
-  <si>
-    <t>Rock, Water, Ground</t>
-  </si>
-  <si>
-    <t>Fighting</t>
-  </si>
-  <si>
-    <t>Mega Clefable, Pidgeot, Espeon</t>
-  </si>
-  <si>
-    <t>Wobbuffet, Mimikyu, Gliscor</t>
+    <t>🎨 Smeargle: Grass, Electric</t>
   </si>
   <si>
     <t>⭐Venusaur, Gogoat, Tangrowth</t>
   </si>
   <si>
-    <t>Psychic, Flying, Fairy</t>
-  </si>
-  <si>
     <t>⭐ S.Tangrowth,S. Gogoat, Smeargle Grass</t>
   </si>
   <si>
-    <t>Dark</t>
-  </si>
-  <si>
-    <t>Absol (Lendário) / Mightyena (UR)</t>
-  </si>
-  <si>
-    <t>Hitmontop, Hitmonchan, Poliwrath</t>
-  </si>
-  <si>
-    <t>Machamp, Scyther, Mimikyu</t>
-  </si>
-  <si>
-    <t>Fighting, Fairy, Bug</t>
-  </si>
-  <si>
-    <t>Water</t>
-  </si>
-  <si>
-    <t>Milotic (UR)</t>
-  </si>
-  <si>
-    <t>S.Charizard, Kabutops, Golem</t>
-  </si>
-  <si>
-    <t>Tangrowth, Ampharos, Venusaur</t>
-  </si>
-  <si>
-    <t>Tangrowth, Gogoat, Luxray</t>
-  </si>
-  <si>
-    <t>Grass, Electric</t>
-  </si>
-  <si>
     <t>Metang, Banette, Dusclops, Nidoking</t>
   </si>
   <si>
-    <t>Grass</t>
+    <t>★ GRASS</t>
   </si>
   <si>
     <t>Aggron, Skarmory</t>
   </si>
   <si>
-    <t>Leafeon (Lendário) / Sceptile (UR)</t>
-  </si>
-  <si>
-    <t>—</t>
-  </si>
-  <si>
-    <t>Typhlosion, Rapidash, Pidgeot</t>
-  </si>
-  <si>
     <t>Raichu</t>
   </si>
   <si>
-    <t>Arcanine, Infernape, Scyther</t>
-  </si>
-  <si>
-    <t>Metang, Magneton Estrelado</t>
-  </si>
-  <si>
-    <t>Poison, Bug, Fire, Fly, Ice</t>
-  </si>
-  <si>
-    <t>Electric</t>
-  </si>
-  <si>
-    <t>SevIper</t>
-  </si>
-  <si>
-    <t>Electabuzz (Lendário) / Manectric (UR)</t>
-  </si>
-  <si>
-    <t>Steelix, Nidoqueen, Torterra</t>
-  </si>
-  <si>
-    <t>Torterra, Pupitar, Smeargle</t>
-  </si>
-  <si>
-    <t>Ground</t>
-  </si>
-  <si>
     <t>🎨 Smeargle: Poison, Ghost, Metal</t>
   </si>
   <si>
-    <t>Ghost</t>
-  </si>
-  <si>
-    <t>Vaporeon, Rhyperior, Magcargo</t>
-  </si>
-  <si>
-    <t>Sharpedo</t>
-  </si>
-  <si>
-    <t>Umbreon, Crawdaunt, Dusknoir</t>
-  </si>
-  <si>
-    <t>Dusknoir, Houndoom, Hydreigon</t>
-  </si>
-  <si>
-    <t>Dark, Ghost</t>
-  </si>
-  <si>
-    <t>Ice</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Fire, Rock</t>
-  </si>
-  <si>
-    <t>Glaceon (Lendário) / Glalie (UR)</t>
-  </si>
-  <si>
-    <t>Typhlosion, Rapidash, Hitmontop</t>
-  </si>
-  <si>
-    <t>Infernape, Machamp, Skarmory</t>
-  </si>
-  <si>
-    <t>Fighting, Fire, Metal</t>
-  </si>
-  <si>
     <t>🎨 Smeargle: Electric</t>
   </si>
   <si>
-    <t>Poison</t>
-  </si>
-  <si>
-    <t>Garbodor (Lendário) / Swalot (UR)</t>
-  </si>
-  <si>
-    <t>Steelix, Espeon, Nidoqueen</t>
-  </si>
-  <si>
-    <t>Wobbuffet, Mr. Mime, Pupitar</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Poison, Metal</t>
-  </si>
-  <si>
-    <t>Ground, Psychic</t>
-  </si>
-  <si>
-    <t>Normal</t>
-  </si>
-  <si>
-    <t>Snorlax (Lendário) / Exploud (UR)</t>
-  </si>
-  <si>
-    <t>Poliwrath, Hitmontop, Medicham</t>
-  </si>
-  <si>
-    <t>Machamp, Kangaskhan, Smeargle</t>
-  </si>
-  <si>
-    <t>Rock</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Rock, Water, Ground</t>
-  </si>
-  <si>
-    <t>Rampardos (UR)</t>
-  </si>
-  <si>
-    <t>Tangrowth, Steelix, Blastoise</t>
-  </si>
-  <si>
-    <t>Tangrowth, Machamp, Gogoat</t>
-  </si>
-  <si>
-    <t>Fighting, Ground, Water, Grass</t>
+    <t>★ ELECTRIC</t>
   </si>
   <si>
     <t>🎨 Smeargle: Grass</t>
   </si>
   <si>
-    <t>Steel</t>
-  </si>
-  <si>
-    <t>Hitmontop, Rapidash, Typhlosion</t>
-  </si>
-  <si>
-    <t>Arcanine, Machamp, Infernape</t>
-  </si>
-  <si>
-    <t>Ground, Fighting, Fire</t>
-  </si>
-  <si>
-    <t>Blastoise, Tangrowth, Gogoat</t>
-  </si>
-  <si>
-    <t>Tangrowth, Kingdra, Sharpedo</t>
-  </si>
-  <si>
-    <t>Water, Ice, Grass</t>
-  </si>
-  <si>
-    <t>Dragon</t>
-  </si>
-  <si>
-    <t>Salamence (UR) / Flygon (Lendário)</t>
-  </si>
-  <si>
-    <t>★ FIGHTING</t>
-  </si>
-  <si>
-    <t>Lapras, Mega Clefable, Jynx</t>
-  </si>
-  <si>
-    <t>Mimikyu, Florges, Walrein</t>
-  </si>
-  <si>
-    <t>Dragon, Ice, Fairy</t>
-  </si>
-  <si>
-    <t>Psychic</t>
-  </si>
-  <si>
-    <t>Alakazam (Lendário)</t>
-  </si>
-  <si>
-    <t>Umbreon, Crawdaunt, Sableye</t>
-  </si>
-  <si>
-    <t>Houndoom, Scyther, Dusknoir</t>
-  </si>
-  <si>
-    <t>Ghost, Dark, Bug</t>
-  </si>
-  <si>
-    <t>Flying</t>
+    <t>★ GHOST</t>
+  </si>
+  <si>
+    <t>Hunt: Leafeon (Lendário) / Sceptile (UR)</t>
   </si>
   <si>
     <t>★ SCIZOR</t>
   </si>
   <si>
-    <t>Ampharos, Magcargo, Lapras</t>
-  </si>
-  <si>
-    <t>Walrein, Luxray, Pachirisu</t>
-  </si>
-  <si>
-    <t>Electric, Ice, Rock</t>
-  </si>
-  <si>
-    <t>Metagross</t>
-  </si>
-  <si>
-    <t>Steel / Psychic</t>
-  </si>
-  <si>
-    <t>★ DARK</t>
-  </si>
-  <si>
-    <t>Rapidash, Typhlosion, Steelix</t>
-  </si>
-  <si>
-    <t>Arcanine, Houndoom, Pupitar</t>
+    <t>Hunt: Electabuzz (Lendário) / Manectric (UR)</t>
   </si>
   <si>
     <t>Hunt: Bug</t>
   </si>
   <si>
-    <t>Fire, Ground, Ghost, Dark</t>
-  </si>
-  <si>
-    <t>Lucario</t>
-  </si>
-  <si>
-    <t>Fighting / Steel</t>
-  </si>
-  <si>
-    <t>★ WATER</t>
-  </si>
-  <si>
-    <t>Hitmontop, Typhlosion, Rapidash</t>
-  </si>
-  <si>
-    <t>Arcanine, Machamp, Pupitar</t>
-  </si>
-  <si>
-    <t>Fighting, Fire, Ground</t>
-  </si>
-  <si>
-    <t>Gengar</t>
-  </si>
-  <si>
-    <t>Ghost / Poison</t>
-  </si>
-  <si>
-    <t>Houndoom, Hydreigon, Pupitar</t>
-  </si>
-  <si>
-    <t>Dark, Ghost, Ground</t>
-  </si>
-  <si>
-    <t>Gardevoir</t>
-  </si>
-  <si>
-    <t>Psychic / Fairy</t>
-  </si>
-  <si>
-    <t>Mawile, Muk, Tentacruel</t>
-  </si>
-  <si>
-    <t>Toxicroak, Seviper, Misdreavus</t>
-  </si>
-  <si>
-    <t>Poison, Ghost, Metal</t>
-  </si>
-  <si>
-    <t>Gyarados</t>
-  </si>
-  <si>
     <t>⭐ S.Rapidash, S.Typhlosion, S.Zard</t>
   </si>
   <si>
-    <t>Water / Flying</t>
-  </si>
-  <si>
-    <t>Ampharos, Luxray, Jolteon</t>
+    <t>⭐ Typhlosion, Rapidash, Pidgeot</t>
   </si>
   <si>
     <t>⭐S.Arcanine, S.Infernape, Smeargle Fire</t>
   </si>
   <si>
-    <t>Luxray, Pachirisu, Smeargle Eletric</t>
-  </si>
-  <si>
-    <t>Hunt: Absol (Lendário) / Mightyena (UR)</t>
-  </si>
-  <si>
-    <t>Hunt: Milotic (UR)</t>
+    <t>⭐ Arcanine, Infernape, Scyther</t>
+  </si>
+  <si>
+    <t>⭐ Steelix, Nidoqueen, Torterra</t>
+  </si>
+  <si>
+    <t>⭐ Torterra, Pupitar, Smeargle</t>
+  </si>
+  <si>
+    <t>⭐ Umbreon, Crawdaunt, Dusknoir</t>
+  </si>
+  <si>
+    <t>⭐ Dusknoir, Houndoom, Hydreigon</t>
   </si>
   <si>
     <t>🎨 Smeargle: Fire</t>
-  </si>
-  <si>
-    <t>⭐ Mega Clefable, Pidgeot, Espeon</t>
-  </si>
-  <si>
-    <t>⭐ Wobbuffet, Mimikyu, Gliscor</t>
-  </si>
-  <si>
-    <t>⭐ Hitmontop, Hitmonchan, Poliwrath</t>
-  </si>
-  <si>
-    <t>⭐ Machamp, Scyther, Mimikyu</t>
-  </si>
-  <si>
-    <t>⭐ Tangrowth, Ampharos, Venusaur</t>
-  </si>
-  <si>
-    <t>⭐ Tangrowth, Gogoat, Luxray</t>
-  </si>
-  <si>
-    <t>Farfetch'd, Gliscor</t>
-  </si>
-  <si>
-    <t>Mr. Mime, Florges, Swellow</t>
-  </si>
-  <si>
-    <t>Mega Clefable, Hitmonlee</t>
-  </si>
-  <si>
-    <t>Florges, Kangaskhan, Pinsir</t>
-  </si>
-  <si>
-    <t>Luxray, Gogoat</t>
-  </si>
-  <si>
-    <t>Pachirisu</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Psychic, Flying, Fairy</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Fighting, Fairy, Bug</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Grass, Electric</t>
-  </si>
-  <si>
-    <t>★ GRASS</t>
-  </si>
-  <si>
-    <t>★ ELECTRIC</t>
-  </si>
-  <si>
-    <t>★ GHOST</t>
-  </si>
-  <si>
-    <t>Hunt: Leafeon (Lendário) / Sceptile (UR)</t>
-  </si>
-  <si>
-    <t>Hunt: Electabuzz (Lendário) / Manectric (UR)</t>
-  </si>
-  <si>
-    <t>⭐ Typhlosion, Rapidash, Pidgeot</t>
-  </si>
-  <si>
-    <t>⭐ Arcanine, Infernape, Scyther</t>
-  </si>
-  <si>
-    <t>⭐ Steelix, Nidoqueen, Torterra</t>
-  </si>
-  <si>
-    <t>⭐ Torterra, Pupitar, Smeargle</t>
-  </si>
-  <si>
-    <t>⭐ Umbreon, Crawdaunt, Dusknoir</t>
-  </si>
-  <si>
-    <t>⭐ Dusknoir, Houndoom, Hydreigon</t>
   </si>
   <si>
     <t>Charizard, Lapras, Jynx, Gliscor</t>
@@ -983,11 +983,17 @@
     </font>
     <font>
       <b/>
+      <sz val="13.0"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font/>
+    <font>
+      <b/>
       <sz val="14.0"/>
       <color rgb="FFFFFFFF"/>
       <name val="Quattrocento Sans"/>
     </font>
-    <font/>
     <font>
       <i/>
       <sz val="9.0"/>
@@ -1001,9 +1007,8 @@
     </font>
     <font>
       <i/>
-      <u/>
       <sz val="9.0"/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FFD1D5DB"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1011,15 +1016,10 @@
       <color rgb="FF0000FF"/>
     </font>
     <font>
-      <b/>
-      <sz val="13.0"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11.0"/>
-      <color rgb="FFFFFFFF"/>
+      <i/>
+      <u/>
+      <sz val="9.0"/>
+      <color rgb="FFE5E7EB"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1030,14 +1030,15 @@
     </font>
     <font>
       <i/>
+      <u/>
       <sz val="9.0"/>
-      <color rgb="FFD1D5DB"/>
+      <color rgb="FF0000FF"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
-      <i/>
-      <sz val="9.0"/>
-      <color rgb="FFF3F4F6"/>
+      <b/>
+      <sz val="11.0"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1053,39 +1054,20 @@
       <name val="Quattrocento Sans"/>
     </font>
     <font>
-      <b/>
-      <sz val="9.0"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
       <sz val="9.0"/>
       <color rgb="FF0F172A"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
-      <b/>
-      <sz val="10.0"/>
-      <color rgb="FF1A1A1A"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
       <i/>
-      <u/>
       <sz val="9.0"/>
-      <color rgb="FFE5E7EB"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="8.0"/>
-      <color rgb="FF4B5563"/>
+      <color rgb="FFF3F4F6"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
       <b/>
       <sz val="9.0"/>
-      <color rgb="FF1E3A8A"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1100,19 +1082,9 @@
       <name val="Quattrocento Sans"/>
     </font>
     <font>
-      <sz val="8.0"/>
-      <color rgb="FF4A4A4A"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <sz val="9.0"/>
-      <color rgb="FF1F2937"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
       <b/>
-      <sz val="8.0"/>
-      <color rgb="FF1E3A8A"/>
+      <sz val="10.0"/>
+      <color rgb="FF1A1A1A"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1136,7 +1108,35 @@
     <font>
       <b/>
       <sz val="8.0"/>
+      <color rgb="FF4B5563"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9.0"/>
+      <color rgb="FF1E3A8A"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <sz val="8.0"/>
       <color rgb="FF4A4A4A"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <sz val="9.0"/>
+      <color rgb="FF1F2937"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8.0"/>
+      <color rgb="FF4A4A4A"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8.0"/>
+      <color rgb="FF1E3A8A"/>
       <name val="Quattrocento Sans"/>
     </font>
   </fonts>
@@ -1149,14 +1149,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF1B2A4A"/>
+        <bgColor rgb="FF1B2A4A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF0F172A"/>
         <bgColor rgb="FF0F172A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1B2A4A"/>
-        <bgColor rgb="FF1B2A4A"/>
+        <fgColor rgb="FF334155"/>
+        <bgColor rgb="FF334155"/>
       </patternFill>
     </fill>
     <fill>
@@ -1167,26 +1173,38 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF8DAA34"/>
+        <bgColor rgb="FF8DAA34"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF1F5F9"/>
+        <bgColor rgb="FFF1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF1F4E78"/>
         <bgColor rgb="FF1F4E78"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF334155"/>
-        <bgColor rgb="FF334155"/>
+        <fgColor rgb="FFE68D9C"/>
+        <bgColor rgb="FFE68D9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEA6C2D"/>
+        <bgColor rgb="FFEA6C2D"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF374151"/>
         <bgColor rgb="FF374151"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF1F5F9"/>
-        <bgColor rgb="FFF1F5F9"/>
       </patternFill>
     </fill>
     <fill>
@@ -1209,14 +1227,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFEF3C7"/>
-        <bgColor rgb="FFFEF3C7"/>
+        <fgColor rgb="FFE8F5E9"/>
+        <bgColor rgb="FFE8F5E9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE8F5E9"/>
-        <bgColor rgb="FFE8F5E9"/>
+        <fgColor rgb="FFF0FDF4"/>
+        <bgColor rgb="FFF0FDF4"/>
       </patternFill>
     </fill>
     <fill>
@@ -1227,14 +1245,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1E40AF"/>
-        <bgColor rgb="FF1E40AF"/>
+        <fgColor rgb="FFFEF2F2"/>
+        <bgColor rgb="FFFEF2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8FAFC"/>
+        <bgColor rgb="FFF8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF3C7"/>
+        <bgColor rgb="FFFEF3C7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF0F4F8"/>
         <bgColor rgb="FFF0F4F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1E40AF"/>
+        <bgColor rgb="FF1E40AF"/>
       </patternFill>
     </fill>
     <fill>
@@ -1251,44 +1287,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF8DAA34"/>
-        <bgColor rgb="FF8DAA34"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFEEF2FF"/>
         <bgColor rgb="FFEEF2FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE68D9C"/>
-        <bgColor rgb="FFE68D9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF0FDF4"/>
-        <bgColor rgb="FFF0FDF4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEA6C2D"/>
-        <bgColor rgb="FFEA6C2D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFEF2F2"/>
-        <bgColor rgb="FFFEF2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF8FAFC"/>
-        <bgColor rgb="FFF8FAFC"/>
       </patternFill>
     </fill>
     <fill>
@@ -1410,17 +1410,6 @@
       </bottom>
     </border>
     <border>
-      <right style="thin">
-        <color rgb="FFD1D5DB"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD1D5DB"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD1D5DB"/>
-      </bottom>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FFCBD5E1"/>
       </left>
@@ -1438,6 +1427,17 @@
       <left style="thin">
         <color rgb="FFD1D5DB"/>
       </left>
+      <right style="thin">
+        <color rgb="FFD1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD1D5DB"/>
+      </bottom>
+    </border>
+    <border>
       <right style="thin">
         <color rgb="FFD1D5DB"/>
       </right>
@@ -1489,196 +1489,196 @@
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0"/>
+    <xf borderId="1" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf borderId="1" fillId="4" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="5" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="5" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="6" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="6" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="7" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="6" fillId="4" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="5" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="8" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="9" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="7" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="5" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="10" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="6" fillId="8" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="11" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="6" fillId="4" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="6" fillId="12" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="6" fillId="4" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="13" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="6" fillId="5" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="14" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="7" fillId="9" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="5" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="6" fillId="15" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="6" fillId="16" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="6" fillId="4" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="17" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="7" fillId="10" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="18" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="6" fillId="11" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="15" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="6" fillId="12" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="5" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="6" fillId="19" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="20" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="7" fillId="13" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="21" fontId="23" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="6" fillId="19" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="22" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="6" fillId="19" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="8" fillId="23" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="9" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="6" fillId="24" fontId="25" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="6" fillId="24" fontId="25" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="7" fillId="6" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="8" fillId="5" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="6" fillId="24" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="10" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="25" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="14" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="15" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="26" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="27" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="28" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="8" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="13" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="7" fillId="6" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="11" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="16" fontId="18" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="8" fillId="17" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf borderId="6" fillId="17" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="7" fillId="4" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="29" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="9" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="7" fillId="4" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="30" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="18" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="4" fillId="25" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="19" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="31" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="8" fillId="4" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="20" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="32" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="10" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="21" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="33" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="22" fontId="25" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="23" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="34" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="5" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="7" fillId="24" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="7" fillId="4" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="35" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="25" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="36" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="7" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="7" fillId="25" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="37" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="25" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="38" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="14" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="7" fillId="18" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="7" fillId="18" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="20" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="26" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="39" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="27" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="28" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="29" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="30" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="31" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="32" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="33" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="34" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="35" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="36" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="37" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="38" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="39" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="40" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="40" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1920,155 +1920,155 @@
   </cols>
   <sheetData>
     <row r="2" ht="33.75" customHeight="1">
-      <c r="B2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="4"/>
+      <c r="B2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="3"/>
     </row>
     <row r="3" ht="19.5" customHeight="1">
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="4"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="3"/>
     </row>
     <row r="4">
-      <c r="B4" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="C4" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="8" t="s">
         <v>5</v>
-      </c>
-      <c r="F4" s="10" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="5" ht="24.0" customHeight="1">
       <c r="B5" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="4"/>
+        <v>9</v>
+      </c>
+      <c r="C5" s="3"/>
       <c r="E5" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" s="4"/>
+        <v>11</v>
+      </c>
+      <c r="F5" s="3"/>
     </row>
     <row r="6" ht="24.75" customHeight="1">
-      <c r="B6" s="17" t="s">
-        <v>12</v>
+      <c r="B6" s="16" t="s">
+        <v>14</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>17</v>
-      </c>
-      <c r="E6" s="17" t="s">
-        <v>12</v>
+        <v>16</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>14</v>
       </c>
       <c r="F6" s="18" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="7" ht="24.75" customHeight="1">
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="F7" s="20" t="s">
-        <v>24</v>
+      <c r="C7" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="22" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="8" ht="24.75" customHeight="1">
-      <c r="B8" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="C8" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="E8" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="F8" s="23" t="s">
-        <v>28</v>
+      <c r="B8" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="38" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="9" ht="24.75" customHeight="1">
-      <c r="B9" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="E9" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="F9" s="20" t="s">
-        <v>32</v>
+      <c r="B9" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="F9" s="22" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="11" ht="24.0" customHeight="1">
-      <c r="B11" s="27" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="4"/>
+      <c r="B11" s="41" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="3"/>
     </row>
     <row r="12" ht="24.0" customHeight="1">
-      <c r="B12" s="32" t="s">
-        <v>42</v>
-      </c>
-      <c r="C12" s="34"/>
-      <c r="D12" s="38" t="s">
-        <v>52</v>
-      </c>
-      <c r="E12" s="40"/>
-      <c r="F12" s="34"/>
+      <c r="B12" s="43" t="s">
+        <v>70</v>
+      </c>
+      <c r="C12" s="44"/>
+      <c r="D12" s="47" t="s">
+        <v>82</v>
+      </c>
+      <c r="E12" s="49"/>
+      <c r="F12" s="44"/>
     </row>
     <row r="13" ht="24.0" customHeight="1">
-      <c r="B13" s="32" t="s">
-        <v>62</v>
-      </c>
-      <c r="C13" s="34"/>
-      <c r="D13" s="38" t="s">
-        <v>64</v>
-      </c>
-      <c r="E13" s="40"/>
-      <c r="F13" s="34"/>
+      <c r="B13" s="43" t="s">
+        <v>184</v>
+      </c>
+      <c r="C13" s="44"/>
+      <c r="D13" s="47" t="s">
+        <v>187</v>
+      </c>
+      <c r="E13" s="49"/>
+      <c r="F13" s="44"/>
     </row>
     <row r="14" ht="24.0" customHeight="1">
-      <c r="B14" s="32" t="s">
-        <v>66</v>
-      </c>
-      <c r="C14" s="34"/>
-      <c r="D14" s="38" t="s">
-        <v>69</v>
-      </c>
-      <c r="E14" s="40"/>
-      <c r="F14" s="34"/>
+      <c r="B14" s="43" t="s">
+        <v>190</v>
+      </c>
+      <c r="C14" s="44"/>
+      <c r="D14" s="47" t="s">
+        <v>193</v>
+      </c>
+      <c r="E14" s="49"/>
+      <c r="F14" s="44"/>
     </row>
     <row r="15" ht="24.0" customHeight="1">
-      <c r="B15" s="32" t="s">
-        <v>71</v>
-      </c>
-      <c r="C15" s="34"/>
-      <c r="D15" s="38" t="s">
-        <v>72</v>
-      </c>
-      <c r="E15" s="40"/>
-      <c r="F15" s="34"/>
+      <c r="B15" s="43" t="s">
+        <v>196</v>
+      </c>
+      <c r="C15" s="44"/>
+      <c r="D15" s="47" t="s">
+        <v>198</v>
+      </c>
+      <c r="E15" s="49"/>
+      <c r="F15" s="44"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -3094,403 +3094,403 @@
   </cols>
   <sheetData>
     <row r="1" ht="31.5" customHeight="1">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="10" t="s">
-        <v>15</v>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="8" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="2" ht="19.5" customHeight="1">
-      <c r="A2" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="10" t="s">
-        <v>41</v>
+      <c r="A2" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="8" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="4" ht="21.75" customHeight="1">
-      <c r="A4" s="37" t="s">
-        <v>48</v>
-      </c>
-      <c r="B4" s="12"/>
-      <c r="D4" s="41" t="s">
+      <c r="A4" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="19"/>
+      <c r="D4" s="21" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="19"/>
+      <c r="G4" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4" s="19"/>
+    </row>
+    <row r="5" ht="18.0" customHeight="1">
+      <c r="A5" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="19"/>
+      <c r="D5" s="24" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="19"/>
+      <c r="G5" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" s="19"/>
+    </row>
+    <row r="6" ht="19.5" customHeight="1">
+      <c r="A6" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="G6" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="H6" s="27" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" ht="42.0" customHeight="1">
+      <c r="A7" s="31" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="D7" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="E7" s="33" t="s">
+        <v>52</v>
+      </c>
+      <c r="G7" s="35" t="s">
+        <v>53</v>
+      </c>
+      <c r="H7" s="33" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" ht="15.0" customHeight="1">
+      <c r="A8" s="39" t="s">
         <v>60</v>
       </c>
-      <c r="E4" s="12"/>
-      <c r="G4" s="43" t="s">
-        <v>68</v>
-      </c>
-      <c r="H4" s="12"/>
-    </row>
-    <row r="5" ht="18.0" customHeight="1">
-      <c r="A5" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="B5" s="12"/>
-      <c r="D5" s="16" t="s">
-        <v>76</v>
-      </c>
-      <c r="E5" s="12"/>
-      <c r="G5" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="H5" s="12"/>
-    </row>
-    <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="E6" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="G6" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" s="21" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="7" ht="42.0" customHeight="1">
-      <c r="A7" s="24" t="s">
-        <v>83</v>
-      </c>
-      <c r="B7" s="26" t="s">
-        <v>85</v>
-      </c>
-      <c r="D7" s="29" t="s">
-        <v>87</v>
-      </c>
-      <c r="E7" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="G7" s="29" t="s">
-        <v>92</v>
-      </c>
-      <c r="H7" s="26" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="B8" s="31" t="s">
-        <v>47</v>
-      </c>
-      <c r="D8" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="E8" s="31" t="s">
-        <v>47</v>
-      </c>
-      <c r="G8" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="H8" s="31" t="s">
-        <v>47</v>
+      <c r="B8" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="D8" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="E8" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="G8" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="H8" s="39" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="9" ht="27.75" customHeight="1">
-      <c r="A9" s="52" t="s">
+      <c r="A9" s="46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B9" s="45" t="s">
         <v>114</v>
       </c>
-      <c r="B9" s="36" t="s">
-        <v>122</v>
-      </c>
-      <c r="D9" s="36" t="s">
-        <v>126</v>
-      </c>
-      <c r="E9" s="53" t="s">
-        <v>129</v>
-      </c>
-      <c r="G9" s="36" t="s">
-        <v>136</v>
-      </c>
-      <c r="H9" s="36" t="s">
-        <v>137</v>
+      <c r="D9" s="45" t="s">
+        <v>119</v>
+      </c>
+      <c r="E9" s="48" t="s">
+        <v>124</v>
+      </c>
+      <c r="G9" s="45" t="s">
+        <v>144</v>
+      </c>
+      <c r="H9" s="45" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="10" ht="18.0" customHeight="1">
-      <c r="A10" s="39" t="s">
-        <v>142</v>
-      </c>
-      <c r="B10" s="12"/>
-      <c r="D10" s="39" t="s">
-        <v>152</v>
-      </c>
-      <c r="E10" s="12"/>
-      <c r="G10" s="39" t="s">
-        <v>159</v>
-      </c>
-      <c r="H10" s="12"/>
+      <c r="A10" s="50" t="s">
+        <v>153</v>
+      </c>
+      <c r="B10" s="19"/>
+      <c r="D10" s="50" t="s">
+        <v>170</v>
+      </c>
+      <c r="E10" s="19"/>
+      <c r="G10" s="50" t="s">
+        <v>177</v>
+      </c>
+      <c r="H10" s="19"/>
     </row>
     <row r="14" ht="21.75" customHeight="1">
-      <c r="A14" s="55" t="s">
-        <v>174</v>
-      </c>
-      <c r="B14" s="12"/>
-      <c r="D14" s="56" t="s">
-        <v>190</v>
-      </c>
-      <c r="E14" s="12"/>
-      <c r="G14" s="57" t="s">
+      <c r="A14" s="51" t="s">
+        <v>185</v>
+      </c>
+      <c r="B14" s="19"/>
+      <c r="D14" s="52" t="s">
+        <v>188</v>
+      </c>
+      <c r="E14" s="19"/>
+      <c r="G14" s="53" t="s">
+        <v>191</v>
+      </c>
+      <c r="H14" s="19"/>
+    </row>
+    <row r="15" ht="18.0" customHeight="1">
+      <c r="A15" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" s="19"/>
+      <c r="D15" s="24" t="s">
+        <v>194</v>
+      </c>
+      <c r="E15" s="19"/>
+      <c r="G15" s="24" t="s">
         <v>197</v>
       </c>
-      <c r="H14" s="12"/>
-    </row>
-    <row r="15" ht="18.0" customHeight="1">
-      <c r="A15" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="B15" s="12"/>
-      <c r="D15" s="16" t="s">
+      <c r="H15" s="19"/>
+    </row>
+    <row r="16" ht="19.5" customHeight="1">
+      <c r="A16" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="E16" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="G16" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="H16" s="27" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="17" ht="42.0" customHeight="1">
+      <c r="A17" s="35" t="s">
+        <v>200</v>
+      </c>
+      <c r="B17" s="33" t="s">
+        <v>201</v>
+      </c>
+      <c r="D17" s="35" t="s">
+        <v>202</v>
+      </c>
+      <c r="E17" s="33" t="s">
+        <v>204</v>
+      </c>
+      <c r="G17" s="35" t="s">
+        <v>205</v>
+      </c>
+      <c r="H17" s="33" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="18" ht="15.0" customHeight="1">
+      <c r="A18" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B18" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="D18" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="E18" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="G18" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="H18" s="39" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="19" ht="27.75" customHeight="1">
+      <c r="A19" s="45" t="s">
+        <v>208</v>
+      </c>
+      <c r="B19" s="45" t="s">
+        <v>209</v>
+      </c>
+      <c r="D19" s="45" t="s">
+        <v>210</v>
+      </c>
+      <c r="E19" s="45" t="s">
+        <v>211</v>
+      </c>
+      <c r="G19" s="45" t="s">
+        <v>212</v>
+      </c>
+      <c r="H19" s="45" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="20" ht="18.0" customHeight="1">
+      <c r="A20" s="50" t="s">
+        <v>214</v>
+      </c>
+      <c r="B20" s="19"/>
+      <c r="D20" s="50" t="s">
         <v>216</v>
       </c>
-      <c r="E15" s="12"/>
-      <c r="G15" s="16" t="s">
-        <v>217</v>
-      </c>
-      <c r="H15" s="12"/>
-    </row>
-    <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="D16" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="E16" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="G16" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="H16" s="21" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="17" ht="42.0" customHeight="1">
-      <c r="A17" s="29" t="s">
-        <v>219</v>
-      </c>
-      <c r="B17" s="26" t="s">
+      <c r="E20" s="19"/>
+      <c r="G20" s="50" t="s">
         <v>220</v>
       </c>
-      <c r="D17" s="29" t="s">
-        <v>221</v>
-      </c>
-      <c r="E17" s="26" t="s">
-        <v>222</v>
-      </c>
-      <c r="G17" s="29" t="s">
-        <v>223</v>
-      </c>
-      <c r="H17" s="26" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="18" ht="15.0" customHeight="1">
-      <c r="A18" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="B18" s="31" t="s">
-        <v>47</v>
-      </c>
-      <c r="D18" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="E18" s="31" t="s">
-        <v>47</v>
-      </c>
-      <c r="G18" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="H18" s="31" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="19" ht="27.75" customHeight="1">
-      <c r="A19" s="36" t="s">
-        <v>225</v>
-      </c>
-      <c r="B19" s="36" t="s">
-        <v>226</v>
-      </c>
-      <c r="D19" s="36" t="s">
-        <v>227</v>
-      </c>
-      <c r="E19" s="36" t="s">
-        <v>228</v>
-      </c>
-      <c r="G19" s="36" t="s">
-        <v>229</v>
-      </c>
-      <c r="H19" s="36" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="20" ht="18.0" customHeight="1">
-      <c r="A20" s="39" t="s">
-        <v>231</v>
-      </c>
-      <c r="B20" s="12"/>
-      <c r="D20" s="39" t="s">
-        <v>232</v>
-      </c>
-      <c r="E20" s="12"/>
-      <c r="G20" s="39" t="s">
-        <v>233</v>
-      </c>
-      <c r="H20" s="12"/>
+      <c r="H20" s="19"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
     <row r="23" ht="15.75" customHeight="1"/>
     <row r="24" ht="21.75" customHeight="1">
-      <c r="A24" s="58" t="s">
+      <c r="A24" s="57" t="s">
+        <v>224</v>
+      </c>
+      <c r="B24" s="19"/>
+      <c r="D24" s="58" t="s">
+        <v>229</v>
+      </c>
+      <c r="E24" s="19"/>
+      <c r="G24" s="60" t="s">
+        <v>231</v>
+      </c>
+      <c r="H24" s="19"/>
+    </row>
+    <row r="25" ht="18.0" customHeight="1">
+      <c r="A25" s="24" t="s">
+        <v>232</v>
+      </c>
+      <c r="B25" s="19"/>
+      <c r="D25" s="24" t="s">
         <v>234</v>
       </c>
-      <c r="B24" s="12"/>
-      <c r="D24" s="59" t="s">
-        <v>235</v>
-      </c>
-      <c r="E24" s="12"/>
-      <c r="G24" s="60" t="s">
-        <v>236</v>
-      </c>
-      <c r="H24" s="12"/>
-    </row>
-    <row r="25" ht="18.0" customHeight="1">
-      <c r="A25" s="16" t="s">
+      <c r="E25" s="19"/>
+      <c r="G25" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="H25" s="19"/>
+    </row>
+    <row r="26" ht="19.5" customHeight="1">
+      <c r="A26" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="B26" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="D26" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="E26" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="G26" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="H26" s="27" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="27" ht="42.0" customHeight="1">
+      <c r="A27" s="35" t="s">
         <v>237</v>
       </c>
-      <c r="B25" s="12"/>
-      <c r="D25" s="16" t="s">
-        <v>238</v>
-      </c>
-      <c r="E25" s="12"/>
-      <c r="G25" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="H25" s="12"/>
-    </row>
-    <row r="26" ht="19.5" customHeight="1">
-      <c r="A26" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="B26" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="D26" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="E26" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="G26" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="H26" s="21" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="27" ht="42.0" customHeight="1">
-      <c r="A27" s="29" t="s">
+      <c r="B27" s="33" t="s">
         <v>239</v>
       </c>
-      <c r="B27" s="26" t="s">
+      <c r="D27" s="35" t="s">
         <v>240</v>
       </c>
-      <c r="D27" s="29" t="s">
+      <c r="E27" s="33" t="s">
         <v>241</v>
       </c>
-      <c r="E27" s="26" t="s">
+      <c r="G27" s="35" t="s">
         <v>242</v>
       </c>
-      <c r="G27" s="29" t="s">
+      <c r="H27" s="33" t="s">
         <v>243</v>
       </c>
-      <c r="H27" s="26" t="s">
-        <v>244</v>
-      </c>
     </row>
     <row r="28" ht="15.0" customHeight="1">
-      <c r="A28" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="B28" s="31" t="s">
-        <v>47</v>
-      </c>
-      <c r="D28" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="E28" s="31" t="s">
-        <v>47</v>
-      </c>
-      <c r="G28" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="H28" s="31" t="s">
-        <v>47</v>
+      <c r="A28" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B28" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="D28" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="E28" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="G28" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="H28" s="39" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="29" ht="27.75" customHeight="1">
-      <c r="A29" s="36" t="s">
+      <c r="A29" s="45" t="s">
         <v>245</v>
       </c>
-      <c r="B29" s="36" t="s">
+      <c r="B29" s="45" t="s">
         <v>246</v>
       </c>
-      <c r="D29" s="36" t="s">
+      <c r="D29" s="45" t="s">
         <v>247</v>
       </c>
-      <c r="E29" s="36" t="s">
+      <c r="E29" s="45" t="s">
         <v>248</v>
       </c>
-      <c r="G29" s="36" t="s">
+      <c r="G29" s="45" t="s">
         <v>249</v>
       </c>
-      <c r="H29" s="36" t="s">
+      <c r="H29" s="45" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="30" ht="18.0" customHeight="1">
-      <c r="A30" s="39" t="s">
+      <c r="A30" s="50" t="s">
         <v>251</v>
       </c>
-      <c r="B30" s="12"/>
-      <c r="D30" s="39" t="s">
+      <c r="B30" s="19"/>
+      <c r="D30" s="50" t="s">
         <v>252</v>
       </c>
-      <c r="E30" s="12"/>
-      <c r="G30" s="39" t="s">
+      <c r="E30" s="19"/>
+      <c r="G30" s="50" t="s">
         <v>253</v>
       </c>
-      <c r="H30" s="12"/>
+      <c r="H30" s="19"/>
     </row>
     <row r="31" ht="15.75" customHeight="1"/>
     <row r="32" ht="15.75" customHeight="1"/>
@@ -3499,123 +3499,123 @@
       <c r="A34" s="61" t="s">
         <v>254</v>
       </c>
-      <c r="B34" s="12"/>
+      <c r="B34" s="19"/>
       <c r="D34" s="62" t="s">
         <v>255</v>
       </c>
-      <c r="E34" s="12"/>
+      <c r="E34" s="19"/>
       <c r="G34" s="63" t="s">
         <v>256</v>
       </c>
-      <c r="H34" s="12"/>
+      <c r="H34" s="19"/>
     </row>
     <row r="35" ht="18.0" customHeight="1">
-      <c r="A35" s="16" t="s">
+      <c r="A35" s="24" t="s">
         <v>257</v>
       </c>
-      <c r="B35" s="12"/>
-      <c r="D35" s="16" t="s">
+      <c r="B35" s="19"/>
+      <c r="D35" s="24" t="s">
         <v>258</v>
       </c>
-      <c r="E35" s="12"/>
-      <c r="G35" s="48" t="s">
+      <c r="E35" s="19"/>
+      <c r="G35" s="55" t="s">
         <v>259</v>
       </c>
-      <c r="H35" s="12"/>
+      <c r="H35" s="19"/>
     </row>
     <row r="36" ht="19.5" customHeight="1">
-      <c r="A36" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="B36" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="D36" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="E36" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="G36" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="H36" s="21" t="s">
-        <v>23</v>
+      <c r="A36" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="D36" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="E36" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="G36" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="H36" s="27" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="37" ht="42.0" customHeight="1">
-      <c r="A37" s="29" t="s">
+      <c r="A37" s="35" t="s">
         <v>260</v>
       </c>
-      <c r="B37" s="26" t="s">
+      <c r="B37" s="33" t="s">
         <v>261</v>
       </c>
-      <c r="D37" s="29" t="s">
+      <c r="D37" s="35" t="s">
         <v>262</v>
       </c>
-      <c r="E37" s="26" t="s">
+      <c r="E37" s="33" t="s">
         <v>263</v>
       </c>
-      <c r="G37" s="29" t="s">
+      <c r="G37" s="35" t="s">
         <v>264</v>
       </c>
-      <c r="H37" s="26" t="s">
+      <c r="H37" s="33" t="s">
         <v>265</v>
       </c>
     </row>
     <row r="38" ht="15.0" customHeight="1">
-      <c r="A38" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="B38" s="31" t="s">
-        <v>47</v>
-      </c>
-      <c r="D38" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="E38" s="31" t="s">
-        <v>47</v>
-      </c>
-      <c r="G38" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="H38" s="31" t="s">
-        <v>47</v>
+      <c r="A38" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B38" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="D38" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="E38" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="G38" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="H38" s="39" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="39" ht="27.75" customHeight="1">
-      <c r="A39" s="36" t="s">
+      <c r="A39" s="45" t="s">
         <v>266</v>
       </c>
-      <c r="B39" s="36" t="s">
+      <c r="B39" s="45" t="s">
         <v>267</v>
       </c>
-      <c r="D39" s="36" t="s">
+      <c r="D39" s="45" t="s">
         <v>268</v>
       </c>
-      <c r="E39" s="36" t="s">
+      <c r="E39" s="45" t="s">
         <v>269</v>
       </c>
-      <c r="G39" s="36" t="s">
+      <c r="G39" s="45" t="s">
         <v>270</v>
       </c>
-      <c r="H39" s="36" t="s">
-        <v>122</v>
+      <c r="H39" s="45" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="40" ht="18.0" customHeight="1">
-      <c r="A40" s="39" t="s">
+      <c r="A40" s="50" t="s">
         <v>271</v>
       </c>
-      <c r="B40" s="12"/>
-      <c r="D40" s="39" t="s">
+      <c r="B40" s="19"/>
+      <c r="D40" s="50" t="s">
         <v>272</v>
       </c>
-      <c r="E40" s="12"/>
-      <c r="G40" s="39" t="s">
+      <c r="E40" s="19"/>
+      <c r="G40" s="50" t="s">
         <v>273</v>
       </c>
-      <c r="H40" s="12"/>
+      <c r="H40" s="19"/>
     </row>
     <row r="41" ht="15.75" customHeight="1"/>
     <row r="42" ht="15.75" customHeight="1"/>
@@ -3624,123 +3624,123 @@
       <c r="A44" s="64" t="s">
         <v>274</v>
       </c>
-      <c r="B44" s="12"/>
+      <c r="B44" s="19"/>
       <c r="D44" s="65" t="s">
         <v>275</v>
       </c>
-      <c r="E44" s="12"/>
+      <c r="E44" s="19"/>
       <c r="G44" s="66" t="s">
         <v>276</v>
       </c>
-      <c r="H44" s="12"/>
+      <c r="H44" s="19"/>
     </row>
     <row r="45" ht="18.0" customHeight="1">
-      <c r="A45" s="16" t="s">
+      <c r="A45" s="24" t="s">
         <v>277</v>
       </c>
-      <c r="B45" s="12"/>
-      <c r="D45" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="E45" s="12"/>
-      <c r="G45" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="H45" s="12"/>
+      <c r="B45" s="19"/>
+      <c r="D45" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="E45" s="19"/>
+      <c r="G45" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="H45" s="19"/>
     </row>
     <row r="46" ht="19.5" customHeight="1">
-      <c r="A46" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="B46" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="D46" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="E46" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="G46" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="H46" s="21" t="s">
-        <v>23</v>
+      <c r="A46" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="B46" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="D46" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="E46" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="G46" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="H46" s="27" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="47" ht="42.0" customHeight="1">
-      <c r="A47" s="29" t="s">
+      <c r="A47" s="35" t="s">
         <v>278</v>
       </c>
-      <c r="B47" s="26" t="s">
+      <c r="B47" s="33" t="s">
         <v>279</v>
       </c>
-      <c r="D47" s="29" t="s">
+      <c r="D47" s="35" t="s">
         <v>280</v>
       </c>
-      <c r="E47" s="26" t="s">
+      <c r="E47" s="33" t="s">
         <v>281</v>
       </c>
-      <c r="G47" s="29" t="s">
+      <c r="G47" s="35" t="s">
         <v>282</v>
       </c>
-      <c r="H47" s="26" t="s">
+      <c r="H47" s="33" t="s">
         <v>283</v>
       </c>
     </row>
     <row r="48" ht="15.0" customHeight="1">
-      <c r="A48" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="B48" s="31" t="s">
-        <v>47</v>
-      </c>
-      <c r="D48" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="E48" s="31" t="s">
-        <v>47</v>
-      </c>
-      <c r="G48" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="H48" s="31" t="s">
-        <v>47</v>
+      <c r="A48" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B48" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="D48" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="E48" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="G48" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="H48" s="39" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="49" ht="27.75" customHeight="1">
-      <c r="A49" s="36" t="s">
+      <c r="A49" s="45" t="s">
         <v>284</v>
       </c>
-      <c r="B49" s="36" t="s">
+      <c r="B49" s="45" t="s">
         <v>285</v>
       </c>
-      <c r="D49" s="36" t="s">
+      <c r="D49" s="45" t="s">
         <v>286</v>
       </c>
-      <c r="E49" s="36" t="s">
+      <c r="E49" s="45" t="s">
         <v>287</v>
       </c>
-      <c r="G49" s="36" t="s">
+      <c r="G49" s="45" t="s">
         <v>288</v>
       </c>
-      <c r="H49" s="36" t="s">
+      <c r="H49" s="45" t="s">
         <v>289</v>
       </c>
     </row>
     <row r="50" ht="18.0" customHeight="1">
-      <c r="A50" s="39" t="s">
+      <c r="A50" s="50" t="s">
         <v>290</v>
       </c>
-      <c r="B50" s="12"/>
-      <c r="D50" s="39" t="s">
+      <c r="B50" s="19"/>
+      <c r="D50" s="50" t="s">
         <v>291</v>
       </c>
-      <c r="E50" s="12"/>
-      <c r="G50" s="39" t="s">
+      <c r="E50" s="19"/>
+      <c r="G50" s="50" t="s">
         <v>292</v>
       </c>
-      <c r="H50" s="12"/>
+      <c r="H50" s="19"/>
     </row>
     <row r="51" ht="15.75" customHeight="1"/>
     <row r="52" ht="15.75" customHeight="1"/>
@@ -3749,123 +3749,123 @@
       <c r="A54" s="67" t="s">
         <v>293</v>
       </c>
-      <c r="B54" s="12"/>
+      <c r="B54" s="19"/>
       <c r="D54" s="68" t="s">
         <v>294</v>
       </c>
-      <c r="E54" s="12"/>
+      <c r="E54" s="19"/>
       <c r="G54" s="69" t="s">
         <v>295</v>
       </c>
-      <c r="H54" s="12"/>
+      <c r="H54" s="19"/>
     </row>
     <row r="55" ht="18.0" customHeight="1">
-      <c r="A55" s="16" t="s">
+      <c r="A55" s="24" t="s">
         <v>296</v>
       </c>
-      <c r="B55" s="12"/>
-      <c r="D55" s="16" t="s">
+      <c r="B55" s="19"/>
+      <c r="D55" s="24" t="s">
         <v>297</v>
       </c>
-      <c r="E55" s="12"/>
-      <c r="G55" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="H55" s="12"/>
+      <c r="E55" s="19"/>
+      <c r="G55" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="H55" s="19"/>
     </row>
     <row r="56" ht="19.5" customHeight="1">
-      <c r="A56" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="B56" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="D56" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="E56" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="G56" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="H56" s="21" t="s">
-        <v>23</v>
+      <c r="A56" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="B56" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="D56" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="E56" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="G56" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="H56" s="27" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="57" ht="42.0" customHeight="1">
-      <c r="A57" s="29" t="s">
+      <c r="A57" s="35" t="s">
         <v>298</v>
       </c>
-      <c r="B57" s="26" t="s">
+      <c r="B57" s="33" t="s">
         <v>299</v>
       </c>
-      <c r="D57" s="29" t="s">
-        <v>39</v>
-      </c>
-      <c r="E57" s="26" t="s">
+      <c r="D57" s="35" t="s">
+        <v>56</v>
+      </c>
+      <c r="E57" s="33" t="s">
         <v>300</v>
       </c>
-      <c r="G57" s="29" t="s">
+      <c r="G57" s="35" t="s">
         <v>301</v>
       </c>
-      <c r="H57" s="26" t="s">
+      <c r="H57" s="33" t="s">
         <v>302</v>
       </c>
     </row>
     <row r="58" ht="15.0" customHeight="1">
-      <c r="A58" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="B58" s="31" t="s">
-        <v>47</v>
-      </c>
-      <c r="D58" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="E58" s="31" t="s">
-        <v>47</v>
-      </c>
-      <c r="G58" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="H58" s="31" t="s">
-        <v>47</v>
+      <c r="A58" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B58" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="D58" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="E58" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="G58" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="H58" s="39" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="59" ht="27.75" customHeight="1">
-      <c r="A59" s="36" t="s">
+      <c r="A59" s="45" t="s">
         <v>303</v>
       </c>
-      <c r="B59" s="36" t="s">
+      <c r="B59" s="45" t="s">
         <v>304</v>
       </c>
-      <c r="D59" s="36" t="s">
+      <c r="D59" s="45" t="s">
         <v>305</v>
       </c>
-      <c r="E59" s="36" t="s">
+      <c r="E59" s="45" t="s">
         <v>306</v>
       </c>
-      <c r="G59" s="36" t="s">
+      <c r="G59" s="45" t="s">
         <v>307</v>
       </c>
-      <c r="H59" s="36" t="s">
+      <c r="H59" s="45" t="s">
         <v>308</v>
       </c>
     </row>
     <row r="60" ht="18.0" customHeight="1">
-      <c r="A60" s="39" t="s">
+      <c r="A60" s="50" t="s">
         <v>309</v>
       </c>
-      <c r="B60" s="12"/>
-      <c r="D60" s="39" t="s">
+      <c r="B60" s="19"/>
+      <c r="D60" s="50" t="s">
         <v>310</v>
       </c>
-      <c r="E60" s="12"/>
-      <c r="G60" s="39" t="s">
+      <c r="E60" s="19"/>
+      <c r="G60" s="50" t="s">
         <v>311</v>
       </c>
-      <c r="H60" s="12"/>
+      <c r="H60" s="19"/>
     </row>
     <row r="61" ht="15.75" customHeight="1"/>
     <row r="62" ht="15.75" customHeight="1"/>
@@ -4892,325 +4892,325 @@
   </cols>
   <sheetData>
     <row r="1" ht="31.5" customHeight="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="4"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="3"/>
     </row>
     <row r="2" ht="19.5" customHeight="1">
-      <c r="A2" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="4"/>
+      <c r="A2" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="3"/>
     </row>
     <row r="4" ht="21.75" customHeight="1">
-      <c r="A4" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="12"/>
-      <c r="D4" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4" s="12"/>
-      <c r="G4" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="H4" s="12"/>
+      <c r="A4" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="19"/>
+      <c r="D4" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="19"/>
+      <c r="G4" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="19"/>
     </row>
     <row r="5" ht="18.0" customHeight="1">
-      <c r="A5" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="12"/>
-      <c r="D5" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="12"/>
-      <c r="G5" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="H5" s="12"/>
+      <c r="A5" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="19"/>
+      <c r="D5" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" s="19"/>
+      <c r="G5" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" s="19"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="E6" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="G6" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" s="21" t="s">
-        <v>23</v>
+      <c r="A6" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="G6" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="H6" s="27" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="7" ht="42.0" customHeight="1">
-      <c r="A7" s="24" t="s">
-        <v>29</v>
-      </c>
-      <c r="B7" s="26" t="s">
+      <c r="A7" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" s="33" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="35" t="s">
+        <v>50</v>
+      </c>
+      <c r="E7" s="33" t="s">
+        <v>54</v>
+      </c>
+      <c r="G7" s="35" t="s">
+        <v>56</v>
+      </c>
+      <c r="H7" s="33" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" ht="15.0" customHeight="1">
+      <c r="A8" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B8" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="D8" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="E8" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="G8" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="H8" s="39" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="9" ht="27.75" customHeight="1">
+      <c r="A9" s="45" t="s">
+        <v>65</v>
+      </c>
+      <c r="B9" s="45" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" s="45" t="s">
+        <v>110</v>
+      </c>
+      <c r="E9" s="45" t="s">
+        <v>113</v>
+      </c>
+      <c r="G9" s="45" t="s">
+        <v>117</v>
+      </c>
+      <c r="H9" s="45" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="10" ht="18.0" customHeight="1">
+      <c r="A10" s="50" t="s">
+        <v>132</v>
+      </c>
+      <c r="B10" s="19"/>
+      <c r="D10" s="50" t="s">
+        <v>182</v>
+      </c>
+      <c r="E10" s="19"/>
+      <c r="G10" s="50" t="s">
+        <v>186</v>
+      </c>
+      <c r="H10" s="19"/>
+    </row>
+    <row r="14" ht="21.75" customHeight="1">
+      <c r="A14" s="20" t="s">
+        <v>189</v>
+      </c>
+      <c r="B14" s="19"/>
+      <c r="D14" s="20" t="s">
+        <v>192</v>
+      </c>
+      <c r="E14" s="19"/>
+      <c r="G14" s="54" t="s">
+        <v>195</v>
+      </c>
+      <c r="H14" s="19"/>
+    </row>
+    <row r="15" ht="18.0" customHeight="1">
+      <c r="A15" s="24" t="s">
+        <v>199</v>
+      </c>
+      <c r="B15" s="19"/>
+      <c r="D15" s="24" t="s">
+        <v>203</v>
+      </c>
+      <c r="E15" s="19"/>
+      <c r="G15" s="55" t="s">
+        <v>207</v>
+      </c>
+      <c r="H15" s="19"/>
+    </row>
+    <row r="16" ht="19.5" customHeight="1">
+      <c r="A16" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="D7" s="29" t="s">
-        <v>36</v>
-      </c>
-      <c r="E7" s="26" t="s">
-        <v>38</v>
-      </c>
-      <c r="G7" s="29" t="s">
+      <c r="B16" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="H7" s="26" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="B8" s="31" t="s">
-        <v>47</v>
-      </c>
-      <c r="D8" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="E8" s="31" t="s">
-        <v>47</v>
-      </c>
-      <c r="G8" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="H8" s="31" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="9" ht="27.75" customHeight="1">
-      <c r="A9" s="36" t="s">
-        <v>51</v>
-      </c>
-      <c r="B9" s="36" t="s">
-        <v>54</v>
-      </c>
-      <c r="D9" s="36" t="s">
-        <v>55</v>
-      </c>
-      <c r="E9" s="36" t="s">
-        <v>56</v>
-      </c>
-      <c r="G9" s="36" t="s">
-        <v>57</v>
-      </c>
-      <c r="H9" s="36" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="10" ht="18.0" customHeight="1">
-      <c r="A10" s="39" t="s">
-        <v>59</v>
-      </c>
-      <c r="B10" s="12"/>
-      <c r="D10" s="39" t="s">
-        <v>61</v>
-      </c>
-      <c r="E10" s="12"/>
-      <c r="G10" s="39" t="s">
+      <c r="D16" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="E16" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="G16" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="H16" s="27" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="17" ht="42.0" customHeight="1">
+      <c r="A17" s="35" t="s">
+        <v>215</v>
+      </c>
+      <c r="B17" s="33" t="s">
+        <v>217</v>
+      </c>
+      <c r="D17" s="35" t="s">
+        <v>218</v>
+      </c>
+      <c r="E17" s="56" t="s">
+        <v>219</v>
+      </c>
+      <c r="G17" s="31" t="s">
+        <v>221</v>
+      </c>
+      <c r="H17" s="56" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="18" ht="15.0" customHeight="1">
+      <c r="A18" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B18" s="39" t="s">
         <v>63</v>
       </c>
-      <c r="H10" s="12"/>
-    </row>
-    <row r="14" ht="21.75" customHeight="1">
-      <c r="A14" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="B14" s="12"/>
-      <c r="D14" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="E14" s="12"/>
-      <c r="G14" s="44" t="s">
-        <v>70</v>
-      </c>
-      <c r="H14" s="12"/>
-    </row>
-    <row r="15" ht="18.0" customHeight="1">
-      <c r="A15" s="16" t="s">
-        <v>75</v>
-      </c>
-      <c r="B15" s="12"/>
-      <c r="D15" s="16" t="s">
-        <v>77</v>
-      </c>
-      <c r="E15" s="12"/>
-      <c r="G15" s="48" t="s">
-        <v>80</v>
-      </c>
-      <c r="H15" s="12"/>
-    </row>
-    <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="D16" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="E16" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="G16" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="H16" s="21" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="17" ht="42.0" customHeight="1">
-      <c r="A17" s="29" t="s">
-        <v>89</v>
-      </c>
-      <c r="B17" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="D17" s="29" t="s">
-        <v>94</v>
-      </c>
-      <c r="E17" s="51" t="s">
-        <v>98</v>
-      </c>
-      <c r="G17" s="24" t="s">
-        <v>104</v>
-      </c>
-      <c r="H17" s="51" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="18" ht="15.0" customHeight="1">
-      <c r="A18" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="B18" s="31" t="s">
-        <v>47</v>
-      </c>
-      <c r="D18" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="E18" s="31" t="s">
-        <v>47</v>
-      </c>
-      <c r="G18" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="H18" s="31" t="s">
-        <v>47</v>
+      <c r="D18" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="E18" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="G18" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="H18" s="39" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="19" ht="27.75" customHeight="1">
-      <c r="A19" s="36" t="s">
-        <v>118</v>
-      </c>
-      <c r="B19" s="36" t="s">
-        <v>120</v>
-      </c>
-      <c r="D19" s="36" t="s">
-        <v>124</v>
-      </c>
-      <c r="E19" s="36" t="s">
-        <v>122</v>
-      </c>
-      <c r="G19" s="36" t="s">
-        <v>122</v>
-      </c>
-      <c r="H19" s="36" t="s">
-        <v>122</v>
+      <c r="A19" s="45" t="s">
+        <v>223</v>
+      </c>
+      <c r="B19" s="45" t="s">
+        <v>225</v>
+      </c>
+      <c r="D19" s="45" t="s">
+        <v>226</v>
+      </c>
+      <c r="E19" s="45" t="s">
+        <v>114</v>
+      </c>
+      <c r="G19" s="45" t="s">
+        <v>114</v>
+      </c>
+      <c r="H19" s="45" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="20" ht="18.0" customHeight="1">
-      <c r="A20" s="39" t="s">
-        <v>134</v>
-      </c>
-      <c r="B20" s="12"/>
-      <c r="D20" s="39" t="s">
-        <v>147</v>
-      </c>
-      <c r="E20" s="12"/>
-      <c r="G20" s="54" t="s">
-        <v>164</v>
-      </c>
-      <c r="H20" s="12"/>
+      <c r="A20" s="50" t="s">
+        <v>227</v>
+      </c>
+      <c r="B20" s="19"/>
+      <c r="D20" s="50" t="s">
+        <v>228</v>
+      </c>
+      <c r="E20" s="19"/>
+      <c r="G20" s="59" t="s">
+        <v>230</v>
+      </c>
+      <c r="H20" s="19"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
     <row r="23" ht="15.75" customHeight="1"/>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="44" t="s">
-        <v>184</v>
-      </c>
-      <c r="B24" s="12"/>
+      <c r="A24" s="54" t="s">
+        <v>233</v>
+      </c>
+      <c r="B24" s="19"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="48" t="s">
-        <v>193</v>
-      </c>
-      <c r="B25" s="12"/>
+      <c r="A25" s="55" t="s">
+        <v>235</v>
+      </c>
+      <c r="B25" s="19"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="B26" s="21" t="s">
-        <v>23</v>
+      <c r="A26" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="B26" s="27" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="27" ht="44.25" customHeight="1">
-      <c r="A27" s="24" t="s">
-        <v>211</v>
-      </c>
-      <c r="B27" s="51" t="s">
-        <v>214</v>
+      <c r="A27" s="31" t="s">
+        <v>236</v>
+      </c>
+      <c r="B27" s="56" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="B28" s="31" t="s">
-        <v>47</v>
+      <c r="A28" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B28" s="39" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="29" ht="27.75" customHeight="1">
-      <c r="A29" s="36" t="s">
-        <v>122</v>
-      </c>
-      <c r="B29" s="36" t="s">
-        <v>122</v>
+      <c r="A29" s="45" t="s">
+        <v>114</v>
+      </c>
+      <c r="B29" s="45" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="54" t="s">
-        <v>218</v>
-      </c>
-      <c r="B30" s="12"/>
+      <c r="A30" s="59" t="s">
+        <v>244</v>
+      </c>
+      <c r="B30" s="19"/>
     </row>
     <row r="31" ht="15.75" customHeight="1"/>
     <row r="32" ht="15.75" customHeight="1"/>
@@ -6234,438 +6234,438 @@
   </cols>
   <sheetData>
     <row r="1" ht="27.75" customHeight="1">
-      <c r="A1" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="4"/>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="3"/>
     </row>
     <row r="2" ht="18.0" customHeight="1">
-      <c r="A2" s="15"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="4"/>
+      <c r="A2" s="10"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="3"/>
     </row>
     <row r="3">
-      <c r="B3" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>5</v>
+      <c r="B3" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="4" ht="24.0" customHeight="1">
-      <c r="A4" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="B4" s="30" t="s">
+      <c r="A4" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="30" t="s">
-        <v>43</v>
-      </c>
-      <c r="D4" s="30" t="s">
-        <v>45</v>
-      </c>
-      <c r="E4" s="25" t="s">
-        <v>46</v>
+      <c r="E4" s="17" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="5" ht="21.75" customHeight="1">
-      <c r="A5" s="33" t="s">
-        <v>49</v>
-      </c>
-      <c r="B5" s="35" t="s">
-        <v>50</v>
-      </c>
-      <c r="C5" s="42" t="s">
-        <v>53</v>
-      </c>
-      <c r="D5" s="45" t="s">
+      <c r="A5" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" s="30" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="32" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="34" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" s="36" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" ht="21.75" customHeight="1">
+      <c r="A6" s="37" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" s="40" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="D6" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="E6" s="42" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" ht="21.75" customHeight="1">
+      <c r="A7" s="28" t="s">
+        <v>72</v>
+      </c>
+      <c r="B7" s="30" t="s">
         <v>73</v>
       </c>
-      <c r="E5" s="46" t="s">
+      <c r="C7" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="D7" s="34" t="s">
+        <v>75</v>
+      </c>
+      <c r="E7" s="36" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" ht="21.75" customHeight="1">
+      <c r="A8" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" s="40" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="32" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="6" ht="21.75" customHeight="1">
-      <c r="A6" s="47" t="s">
+      <c r="D8" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="E8" s="42" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="9" ht="21.75" customHeight="1">
+      <c r="A9" s="28" t="s">
         <v>81</v>
       </c>
-      <c r="B6" s="49" t="s">
-        <v>82</v>
-      </c>
-      <c r="C6" s="42" t="s">
+      <c r="B9" s="30" t="s">
+        <v>83</v>
+      </c>
+      <c r="C9" s="32" t="s">
         <v>84</v>
       </c>
-      <c r="D6" s="45" t="s">
+      <c r="D9" s="34" t="s">
+        <v>85</v>
+      </c>
+      <c r="E9" s="36" t="s">
         <v>86</v>
       </c>
-      <c r="E6" s="50" t="s">
+    </row>
+    <row r="10" ht="21.75" customHeight="1">
+      <c r="A10" s="37" t="s">
+        <v>87</v>
+      </c>
+      <c r="B10" s="40" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="7" ht="21.75" customHeight="1">
-      <c r="A7" s="33" t="s">
+      <c r="C10" s="32" t="s">
+        <v>89</v>
+      </c>
+      <c r="D10" s="34" t="s">
+        <v>90</v>
+      </c>
+      <c r="E10" s="42" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="11" ht="21.75" customHeight="1">
+      <c r="A11" s="28" t="s">
+        <v>92</v>
+      </c>
+      <c r="B11" s="30" t="s">
         <v>93</v>
       </c>
-      <c r="B7" s="35" t="s">
+      <c r="C11" s="32" t="s">
+        <v>94</v>
+      </c>
+      <c r="D11" s="34" t="s">
         <v>95</v>
       </c>
-      <c r="C7" s="42" t="s">
+      <c r="E11" s="36" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="12" ht="21.75" customHeight="1">
+      <c r="A12" s="37" t="s">
         <v>97</v>
       </c>
-      <c r="D7" s="45" t="s">
+      <c r="B12" s="40" t="s">
+        <v>98</v>
+      </c>
+      <c r="C12" s="32" t="s">
         <v>99</v>
       </c>
-      <c r="E7" s="46" t="s">
+      <c r="D12" s="34" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="8" ht="21.75" customHeight="1">
-      <c r="A8" s="47" t="s">
+      <c r="E12" s="42" t="s">
         <v>101</v>
       </c>
-      <c r="B8" s="49" t="s">
-        <v>50</v>
-      </c>
-      <c r="C8" s="42" t="s">
+    </row>
+    <row r="13" ht="21.75" customHeight="1">
+      <c r="A13" s="28" t="s">
         <v>102</v>
       </c>
-      <c r="D8" s="45" t="s">
+      <c r="B13" s="30" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" s="32" t="s">
         <v>103</v>
       </c>
-      <c r="E8" s="50" t="s">
+      <c r="D13" s="34" t="s">
+        <v>104</v>
+      </c>
+      <c r="E13" s="36" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="9" ht="21.75" customHeight="1">
-      <c r="A9" s="33" t="s">
+    <row r="14" ht="21.75" customHeight="1">
+      <c r="A14" s="37" t="s">
         <v>107</v>
       </c>
-      <c r="B9" s="35" t="s">
+      <c r="B14" s="40" t="s">
         <v>108</v>
       </c>
-      <c r="C9" s="42" t="s">
+      <c r="C14" s="32" t="s">
         <v>109</v>
       </c>
-      <c r="D9" s="45" t="s">
-        <v>110</v>
-      </c>
-      <c r="E9" s="46" t="s">
+      <c r="D14" s="34" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="10" ht="21.75" customHeight="1">
-      <c r="A10" s="47" t="s">
+      <c r="E14" s="42" t="s">
         <v>112</v>
       </c>
-      <c r="B10" s="49" t="s">
-        <v>113</v>
-      </c>
-      <c r="C10" s="42" t="s">
+    </row>
+    <row r="15" ht="21.75" customHeight="1">
+      <c r="A15" s="28" t="s">
         <v>115</v>
       </c>
-      <c r="D10" s="45" t="s">
+      <c r="B15" s="30" t="s">
         <v>116</v>
       </c>
-      <c r="E10" s="50" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="11" ht="21.75" customHeight="1">
-      <c r="A11" s="33" t="s">
-        <v>119</v>
-      </c>
-      <c r="B11" s="35" t="s">
-        <v>121</v>
-      </c>
-      <c r="C11" s="42" t="s">
+      <c r="C15" s="32" t="s">
+        <v>118</v>
+      </c>
+      <c r="D15" s="34" t="s">
+        <v>120</v>
+      </c>
+      <c r="E15" s="36" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="16" ht="21.75" customHeight="1">
+      <c r="A16" s="37" t="s">
         <v>123</v>
       </c>
-      <c r="D11" s="45" t="s">
+      <c r="B16" s="40" t="s">
         <v>125</v>
       </c>
-      <c r="E11" s="46" t="s">
+      <c r="C16" s="32" t="s">
+        <v>126</v>
+      </c>
+      <c r="D16" s="34" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="12" ht="21.75" customHeight="1">
-      <c r="A12" s="47" t="s">
+      <c r="E16" s="42" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="17" ht="21.75" customHeight="1">
+      <c r="A17" s="28" t="s">
         <v>128</v>
       </c>
-      <c r="B12" s="49" t="s">
+      <c r="B17" s="30" t="s">
+        <v>129</v>
+      </c>
+      <c r="C17" s="32" t="s">
         <v>130</v>
       </c>
-      <c r="C12" s="42" t="s">
+      <c r="D17" s="34" t="s">
         <v>131</v>
       </c>
-      <c r="D12" s="45" t="s">
-        <v>132</v>
-      </c>
-      <c r="E12" s="50" t="s">
+      <c r="E17" s="36" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="13" ht="21.75" customHeight="1">
-      <c r="A13" s="33" t="s">
+    <row r="18" ht="21.75" customHeight="1">
+      <c r="A18" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="B18" s="40" t="s">
+        <v>41</v>
+      </c>
+      <c r="C18" s="32" t="s">
         <v>135</v>
       </c>
-      <c r="B13" s="35" t="s">
-        <v>50</v>
-      </c>
-      <c r="C13" s="42" t="s">
+      <c r="D18" s="34" t="s">
+        <v>136</v>
+      </c>
+      <c r="E18" s="42" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="19" ht="21.75" customHeight="1">
+      <c r="A19" s="28" t="s">
+        <v>101</v>
+      </c>
+      <c r="B19" s="30" t="s">
+        <v>41</v>
+      </c>
+      <c r="C19" s="32" t="s">
         <v>138</v>
       </c>
-      <c r="D13" s="45" t="s">
+      <c r="D19" s="34" t="s">
         <v>139</v>
       </c>
-      <c r="E13" s="46" t="s">
+      <c r="E19" s="36" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="14" ht="21.75" customHeight="1">
-      <c r="A14" s="47" t="s">
+    <row r="20" ht="21.75" customHeight="1">
+      <c r="A20" s="37" t="s">
         <v>141</v>
       </c>
-      <c r="B14" s="49" t="s">
+      <c r="B20" s="40" t="s">
+        <v>142</v>
+      </c>
+      <c r="C20" s="32" t="s">
         <v>143</v>
       </c>
-      <c r="C14" s="42" t="s">
-        <v>144</v>
-      </c>
-      <c r="D14" s="45" t="s">
+      <c r="D20" s="34" t="s">
         <v>145</v>
       </c>
-      <c r="E14" s="50" t="s">
+      <c r="E20" s="42" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="15" ht="21.75" customHeight="1">
-      <c r="A15" s="33" t="s">
+    <row r="21" ht="21.75" customHeight="1">
+      <c r="A21" s="28" t="s">
         <v>148</v>
       </c>
-      <c r="B15" s="35" t="s">
+      <c r="B21" s="30" t="s">
         <v>149</v>
       </c>
-      <c r="C15" s="42" t="s">
+      <c r="C21" s="32" t="s">
         <v>150</v>
       </c>
-      <c r="D15" s="45" t="s">
+      <c r="D21" s="34" t="s">
         <v>151</v>
       </c>
-      <c r="E15" s="46" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="16" ht="21.75" customHeight="1">
-      <c r="A16" s="47" t="s">
+      <c r="E21" s="36" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="22" ht="21.75" customHeight="1">
+      <c r="A22" s="37" t="s">
         <v>154</v>
       </c>
-      <c r="B16" s="49" t="s">
+      <c r="B22" s="40" t="s">
+        <v>41</v>
+      </c>
+      <c r="C22" s="32" t="s">
         <v>155</v>
       </c>
-      <c r="C16" s="42" t="s">
+      <c r="D22" s="34" t="s">
         <v>156</v>
       </c>
-      <c r="D16" s="45" t="s">
+      <c r="E22" s="42" t="s">
         <v>157</v>
       </c>
-      <c r="E16" s="50" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="17" ht="21.75" customHeight="1">
-      <c r="A17" s="33" t="s">
+    </row>
+    <row r="23" ht="21.75" customHeight="1">
+      <c r="A23" s="28" t="s">
         <v>158</v>
       </c>
-      <c r="B17" s="35" t="s">
+      <c r="B23" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="C23" s="32" t="s">
         <v>160</v>
       </c>
-      <c r="C17" s="42" t="s">
+      <c r="D23" s="34" t="s">
         <v>161</v>
       </c>
-      <c r="D17" s="45" t="s">
+      <c r="E23" s="36" t="s">
         <v>162</v>
       </c>
-      <c r="E17" s="46" t="s">
+    </row>
+    <row r="24" ht="21.75" customHeight="1">
+      <c r="A24" s="37" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="18" ht="21.75" customHeight="1">
-      <c r="A18" s="47" t="s">
+      <c r="B24" s="40" t="s">
+        <v>164</v>
+      </c>
+      <c r="C24" s="32" t="s">
         <v>165</v>
       </c>
-      <c r="B18" s="49" t="s">
-        <v>50</v>
-      </c>
-      <c r="C18" s="42" t="s">
+      <c r="D24" s="34" t="s">
         <v>166</v>
       </c>
-      <c r="D18" s="45" t="s">
+      <c r="E24" s="42" t="s">
         <v>167</v>
       </c>
-      <c r="E18" s="50" t="s">
+    </row>
+    <row r="25" ht="21.75" customHeight="1">
+      <c r="A25" s="28" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="19" ht="21.75" customHeight="1">
-      <c r="A19" s="33" t="s">
-        <v>133</v>
-      </c>
-      <c r="B19" s="35" t="s">
-        <v>50</v>
-      </c>
-      <c r="C19" s="42" t="s">
+      <c r="B25" s="30" t="s">
         <v>169</v>
       </c>
-      <c r="D19" s="45" t="s">
-        <v>170</v>
-      </c>
-      <c r="E19" s="46" t="s">
+      <c r="C25" s="32" t="s">
+        <v>150</v>
+      </c>
+      <c r="D25" s="34" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="20" ht="21.75" customHeight="1">
-      <c r="A20" s="47" t="s">
+      <c r="E25" s="36" t="s">
         <v>172</v>
       </c>
-      <c r="B20" s="49" t="s">
+    </row>
+    <row r="26" ht="21.75" customHeight="1">
+      <c r="A26" s="37" t="s">
         <v>173</v>
       </c>
-      <c r="C20" s="42" t="s">
+      <c r="B26" s="40" t="s">
+        <v>174</v>
+      </c>
+      <c r="C26" s="32" t="s">
         <v>175</v>
       </c>
-      <c r="D20" s="45" t="s">
+      <c r="D26" s="34" t="s">
         <v>176</v>
       </c>
-      <c r="E20" s="50" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="21" ht="21.75" customHeight="1">
-      <c r="A21" s="33" t="s">
+      <c r="E26" s="42" t="s">
         <v>178</v>
       </c>
-      <c r="B21" s="35" t="s">
+    </row>
+    <row r="27" ht="21.75" customHeight="1">
+      <c r="A27" s="28" t="s">
         <v>179</v>
       </c>
-      <c r="C21" s="42" t="s">
+      <c r="B27" s="30" t="s">
         <v>180</v>
       </c>
-      <c r="D21" s="45" t="s">
+      <c r="C27" s="32" t="s">
         <v>181</v>
       </c>
-      <c r="E21" s="46" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="22" ht="21.75" customHeight="1">
-      <c r="A22" s="47" t="s">
+      <c r="D27" s="34" t="s">
         <v>183</v>
       </c>
-      <c r="B22" s="49" t="s">
-        <v>50</v>
-      </c>
-      <c r="C22" s="42" t="s">
-        <v>185</v>
-      </c>
-      <c r="D22" s="45" t="s">
-        <v>186</v>
-      </c>
-      <c r="E22" s="50" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="23" ht="21.75" customHeight="1">
-      <c r="A23" s="33" t="s">
-        <v>188</v>
-      </c>
-      <c r="B23" s="35" t="s">
-        <v>189</v>
-      </c>
-      <c r="C23" s="42" t="s">
-        <v>191</v>
-      </c>
-      <c r="D23" s="45" t="s">
-        <v>192</v>
-      </c>
-      <c r="E23" s="46" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="24" ht="21.75" customHeight="1">
-      <c r="A24" s="47" t="s">
-        <v>195</v>
-      </c>
-      <c r="B24" s="49" t="s">
-        <v>196</v>
-      </c>
-      <c r="C24" s="42" t="s">
-        <v>198</v>
-      </c>
-      <c r="D24" s="45" t="s">
-        <v>199</v>
-      </c>
-      <c r="E24" s="50" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="25" ht="21.75" customHeight="1">
-      <c r="A25" s="33" t="s">
-        <v>201</v>
-      </c>
-      <c r="B25" s="35" t="s">
-        <v>202</v>
-      </c>
-      <c r="C25" s="42" t="s">
-        <v>180</v>
-      </c>
-      <c r="D25" s="45" t="s">
-        <v>203</v>
-      </c>
-      <c r="E25" s="46" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="26" ht="21.75" customHeight="1">
-      <c r="A26" s="47" t="s">
-        <v>205</v>
-      </c>
-      <c r="B26" s="49" t="s">
-        <v>206</v>
-      </c>
-      <c r="C26" s="42" t="s">
-        <v>207</v>
-      </c>
-      <c r="D26" s="45" t="s">
-        <v>208</v>
-      </c>
-      <c r="E26" s="50" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="27" ht="21.75" customHeight="1">
-      <c r="A27" s="33" t="s">
-        <v>210</v>
-      </c>
-      <c r="B27" s="35" t="s">
-        <v>212</v>
-      </c>
-      <c r="C27" s="42" t="s">
-        <v>213</v>
-      </c>
-      <c r="D27" s="45" t="s">
-        <v>215</v>
-      </c>
-      <c r="E27" s="46" t="s">
-        <v>128</v>
+      <c r="E27" s="36" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Atualização automática da planilha (2026-09-16)
</commit_message>
<xml_diff>
--- a/times.xlsx
+++ b/times.xlsx
@@ -16,12 +16,12 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="312">
   <si>
+    <t>GUIA DE ROTAÇÃO &amp; METAGAME - POKEALLIANCE(PKA)</t>
+  </si>
+  <si>
     <t>GUIA RÁPIDO</t>
   </si>
   <si>
-    <t>GUIA DE ROTAÇÃO &amp; METAGAME - POKEALLIANCE(PKA)</t>
-  </si>
-  <si>
     <t>RECOMENDAÇÃO DE TIME PARA HUNTS!</t>
   </si>
   <si>
@@ -31,13 +31,13 @@
     <t>Requisitos de Entrada e Progressão 2x2x2.</t>
   </si>
   <si>
+    <t>https://www.twitch.tv/safnaww</t>
+  </si>
+  <si>
     <t>Segue lá!</t>
   </si>
   <si>
     <t>Com algumas exceções, todos os restantes são SHINYS.</t>
-  </si>
-  <si>
-    <t>https://www.twitch.tv/safnaww</t>
   </si>
   <si>
     <r>
@@ -61,577 +61,601 @@
     </r>
   </si>
   <si>
+    <t>ELEMENTO / HUNT</t>
+  </si>
+  <si>
     <t>📌 REQUISITOS INICIAIS (START DE ROTAÇÃO)</t>
   </si>
   <si>
+    <t>ALVO (HUNT)</t>
+  </si>
+  <si>
+    <t>⚡ UPGRADE: ROTAÇÃO 2x2x2</t>
+  </si>
+  <si>
+    <t>🛡️ LURAR (T1)</t>
+  </si>
+  <si>
+    <t>⚔️ DPS (SR)</t>
+  </si>
+  <si>
+    <t>🎨 TIPO SMEARGLE</t>
+  </si>
+  <si>
+    <t>Bug</t>
+  </si>
+  <si>
+    <t>Nível &amp; Held:</t>
+  </si>
+  <si>
+    <t>Todos os Pokémon +15 com Atk 4</t>
+  </si>
+  <si>
+    <t>Em breve</t>
+  </si>
+  <si>
+    <t>Todos os Pokémon +25 com Atk 5</t>
+  </si>
+  <si>
+    <t>★ METAGROSS</t>
+  </si>
+  <si>
+    <t>Atalho / Dica:</t>
+  </si>
+  <si>
+    <t>Runas de Atk no Pokelog ajudam a adiantar a meta</t>
+  </si>
+  <si>
+    <t>Rapidash, Typhlosion, Magcargo</t>
+  </si>
+  <si>
+    <t>Arcanine, Infernape, Armaldo</t>
+  </si>
+  <si>
+    <t>Estrelas Mínimas:</t>
+  </si>
+  <si>
+    <t>Tier 1: 2★ (estrelas)  |  SR: 1★ (estrela)</t>
+  </si>
+  <si>
+    <t>Meta no Dummy:</t>
+  </si>
+  <si>
     <t>Nessa planilha não indicaremos pokémons T2 ou T3 para a rotação.</t>
   </si>
   <si>
-    <t>⚡ UPGRADE: ROTAÇÃO 2x2x2</t>
+    <t>Bater 560k de dano com 3 Pokémon</t>
   </si>
   <si>
     <t>★ BUG</t>
   </si>
   <si>
-    <t>ELEMENTO / HUNT</t>
-  </si>
-  <si>
-    <t>Nível &amp; Held:</t>
-  </si>
-  <si>
-    <t>★ METAGROSS</t>
-  </si>
-  <si>
-    <t>Todos os Pokémon +15 com Atk 4</t>
-  </si>
-  <si>
-    <t>ALVO (HUNT)</t>
-  </si>
-  <si>
-    <t>Todos os Pokémon +25 com Atk 5</t>
-  </si>
-  <si>
-    <t>Atalho / Dica:</t>
-  </si>
-  <si>
-    <t>Runas de Atk no Pokelog ajudam a adiantar a meta</t>
+    <t>Bater 560k de dano com apenas 2 Pokémon</t>
+  </si>
+  <si>
+    <t>Fire, Rock</t>
+  </si>
+  <si>
+    <t>★ LUCARIO</t>
+  </si>
+  <si>
+    <t>Fairy</t>
+  </si>
+  <si>
+    <t>Regra de Prey:</t>
+  </si>
+  <si>
+    <t>★ GENGAR</t>
+  </si>
+  <si>
+    <t>Obrigatório Prey de Atk na hunt (já calculada no dummy)</t>
+  </si>
+  <si>
+    <t>Manter sempre Prey de Atk ativa na hunt</t>
+  </si>
+  <si>
+    <t>💡 POR QUE COMPOSIÇÕES COM 2 A 3 ELEMENTOS SÃO SUPERIORES? (ANTI-MONO)</t>
+  </si>
+  <si>
+    <t>Hunt: Steel / Psychic</t>
   </si>
   <si>
     <t>★ FAIRY</t>
   </si>
   <si>
-    <t>★ LUCARIO</t>
-  </si>
-  <si>
-    <t>★ GENGAR</t>
+    <t>Shiny Sylveon (Lendário)</t>
+  </si>
+  <si>
+    <t>⏱️ Cooldown Reduzido por Tier</t>
+  </si>
+  <si>
+    <t>Hunt: Fighting / Steel</t>
+  </si>
+  <si>
+    <t>Muk, Tentacruel, Mawile</t>
+  </si>
+  <si>
+    <t>Aggron, Skarmory, Toxicroak</t>
+  </si>
+  <si>
+    <t>Poison, Metal</t>
   </si>
   <si>
     <t>★ FIRE</t>
   </si>
   <si>
-    <t>Estrelas Mínimas:</t>
-  </si>
-  <si>
-    <t>Tier 1: 2★ (estrelas)  |  SR: 1★ (estrela)</t>
-  </si>
-  <si>
-    <t>Meta no Dummy:</t>
-  </si>
-  <si>
-    <t>Hunt: Steel / Psychic</t>
-  </si>
-  <si>
-    <t>Bater 560k de dano com 3 Pokémon</t>
+    <t>Hunt: Ghost / Poison</t>
+  </si>
+  <si>
+    <t>Fire</t>
+  </si>
+  <si>
+    <t>Magmar (Lendário) / Torkoal (UR)</t>
+  </si>
+  <si>
+    <t>Blastoise, Feraligatr, Omastar</t>
+  </si>
+  <si>
+    <t>No PKA, tiers mais altos não dão só dano: reduzem o cooldown das skills, deixando a rotação muito mais rápida.</t>
+  </si>
+  <si>
+    <t>Pupitar, Torterra, Kingdra</t>
+  </si>
+  <si>
+    <t>Rock, Water, Ground</t>
+  </si>
+  <si>
+    <t>Fighting</t>
+  </si>
+  <si>
+    <t>🛡️ LURAR / TANQUE (T1)</t>
+  </si>
+  <si>
+    <t>Mega Clefable, Pidgeot, Espeon</t>
+  </si>
+  <si>
+    <t>Wobbuffet, Mimikyu, Gliscor</t>
+  </si>
+  <si>
+    <t>Psychic, Flying, Fairy</t>
+  </si>
+  <si>
+    <t>Dark</t>
+  </si>
+  <si>
+    <t>Absol (Lendário) / Mightyena (UR)</t>
+  </si>
+  <si>
+    <t>Hitmontop, Hitmonchan, Poliwrath</t>
   </si>
   <si>
     <t>Hunt: Em breve</t>
   </si>
   <si>
-    <t>Hunt: Fighting / Steel</t>
+    <t>Machamp, Scyther, Mimikyu</t>
+  </si>
+  <si>
+    <t>Fighting, Fairy, Bug</t>
+  </si>
+  <si>
+    <t>Water</t>
+  </si>
+  <si>
+    <t>Milotic (UR)</t>
+  </si>
+  <si>
+    <t>Tangrowth, Ampharos, Venusaur</t>
+  </si>
+  <si>
+    <t>Tangrowth, Gogoat, Luxray</t>
+  </si>
+  <si>
+    <t>Grass, Electric</t>
+  </si>
+  <si>
+    <t>Grass</t>
+  </si>
+  <si>
+    <t>Leafeon (Lendário) / Sceptile (UR)</t>
+  </si>
+  <si>
+    <t>Typhlosion, Rapidash, Pidgeot</t>
   </si>
   <si>
     <t>Hunt: Shiny Sylveon (Lendário)</t>
   </si>
   <si>
-    <t>Hunt: Ghost / Poison</t>
+    <t>⚔️ DPS / DANO (SR)</t>
+  </si>
+  <si>
+    <t>Arcanine, Infernape, Scyther</t>
+  </si>
+  <si>
+    <t>📈 Mais Mobs e Brokes / Hora</t>
+  </si>
+  <si>
+    <t>Poison, Bug, Fire, Fly, Ice</t>
+  </si>
+  <si>
+    <t>Electric</t>
+  </si>
+  <si>
+    <t>Electabuzz (Lendário) / Manectric (UR)</t>
+  </si>
+  <si>
+    <t>Steelix, Nidoqueen, Torterra</t>
+  </si>
+  <si>
+    <t>Torterra, Pupitar, Smeargle</t>
+  </si>
+  <si>
+    <t>Ground</t>
+  </si>
+  <si>
+    <t>Ghost</t>
+  </si>
+  <si>
+    <t>Rotação mais fluida = mais mobs derrotados/hora, aumentando drasticamente a chance de Shiny/hr e lucro.</t>
+  </si>
+  <si>
+    <t>Umbreon, Crawdaunt, Dusknoir</t>
+  </si>
+  <si>
+    <t>Dusknoir, Houndoom, Hydreigon</t>
   </si>
   <si>
     <t>Hunt: Magmar (Lendário) / Torkoal (UR)</t>
   </si>
   <si>
-    <t>🛡️ LURAR / TANQUE (T1)</t>
-  </si>
-  <si>
-    <t>🛡️ LURAR (T1)</t>
-  </si>
-  <si>
-    <t>⚔️ DPS (SR)</t>
-  </si>
-  <si>
-    <t>🎨 TIPO SMEARGLE</t>
-  </si>
-  <si>
-    <t>⚔️ DPS / DANO (SR)</t>
-  </si>
-  <si>
-    <t>Bug</t>
-  </si>
-  <si>
-    <t>Em breve</t>
+    <t>Dark, Ghost</t>
+  </si>
+  <si>
+    <t>Ice</t>
+  </si>
+  <si>
+    <t>Glaceon (Lendário) / Glalie (UR)</t>
+  </si>
+  <si>
+    <t>Typhlosion, Rapidash, Hitmontop</t>
+  </si>
+  <si>
+    <t>Infernape, Machamp, Skarmory</t>
+  </si>
+  <si>
+    <t>Fighting, Fire, Metal</t>
+  </si>
+  <si>
+    <t>⚔️ Hazards Mais Altos</t>
+  </si>
+  <si>
+    <t>Poison</t>
+  </si>
+  <si>
+    <t>Garbodor (Lendário) / Swalot (UR)</t>
+  </si>
+  <si>
+    <t>Steelix, Espeon, Nidoqueen</t>
+  </si>
+  <si>
+    <t>Wobbuffet, Mr. Mime, Pupitar</t>
+  </si>
+  <si>
+    <t>Ground, Psychic</t>
+  </si>
+  <si>
+    <t>Mesmo encurtando o número total de hunts, permite solar níveis de Hazard superiores com segurança e eficiência.</t>
+  </si>
+  <si>
+    <t>Normal</t>
+  </si>
+  <si>
+    <t>Snorlax (Lendário) / Exploud (UR)</t>
+  </si>
+  <si>
+    <t>Poliwrath, Hitmontop, Medicham</t>
+  </si>
+  <si>
+    <t>Machamp, Kangaskhan, Smeargle</t>
   </si>
   <si>
     <t>⭐ S.Rapidash, S.Typhlosion, S.Steelix</t>
   </si>
   <si>
+    <t>Rock</t>
+  </si>
+  <si>
+    <t>Rampardos (UR)</t>
+  </si>
+  <si>
+    <t>Tangrowth, Steelix, Blastoise</t>
+  </si>
+  <si>
+    <t>Tangrowth, Machamp, Gogoat</t>
+  </si>
+  <si>
+    <t>🏆 Futuro &amp; Escalabilidade (Endgame)</t>
+  </si>
+  <si>
+    <t>Fighting, Ground, Water, Grass</t>
+  </si>
+  <si>
+    <t>Steel</t>
+  </si>
+  <si>
+    <t>Hitmontop, Rapidash, Typhlosion</t>
+  </si>
+  <si>
+    <t>Arcanine, Machamp, Infernape</t>
+  </si>
+  <si>
+    <t>Ground, Fighting, Fire</t>
+  </si>
+  <si>
+    <t>⭐ Arcanine, Houndoom, Pupitar</t>
+  </si>
+  <si>
+    <t>Trabalhar com 2 ou 3 elementos abre um catálogo amplo de opções viáveis para evoluir: T1, SR, UR e Lendários.</t>
+  </si>
+  <si>
+    <t>Blastoise, Tangrowth, Gogoat</t>
+  </si>
+  <si>
+    <t>Tangrowth, Kingdra, Sharpedo</t>
+  </si>
+  <si>
+    <t>Water, Ice, Grass</t>
+  </si>
+  <si>
+    <t>Dragon</t>
+  </si>
+  <si>
+    <t>Salamence (UR) / Flygon (Lendário)</t>
+  </si>
+  <si>
+    <t>Lapras, Mega Clefable, Jynx</t>
+  </si>
+  <si>
+    <t>Mimikyu, Florges, Walrein</t>
+  </si>
+  <si>
+    <t>Dragon, Ice, Fairy</t>
+  </si>
+  <si>
     <t>⭐S.Rapidash, S.Typhlosion, S.Magcargo</t>
   </si>
   <si>
-    <t>Rapidash, Typhlosion, Magcargo</t>
+    <t>⭐ Hitmontop, Typhlosion, Rapidash</t>
+  </si>
+  <si>
+    <t>Psychic</t>
+  </si>
+  <si>
+    <t>Alakazam (Lendário)</t>
+  </si>
+  <si>
+    <t>Umbreon, Crawdaunt, Sableye</t>
+  </si>
+  <si>
+    <t>Houndoom, Scyther, Dusknoir</t>
+  </si>
+  <si>
+    <t>Ghost, Dark, Bug</t>
+  </si>
+  <si>
+    <t>⭐ Arcanine, Machamp, Pupitar</t>
+  </si>
+  <si>
+    <t>Flying</t>
   </si>
   <si>
     <t>⭐ Arcanine, Infernape, Armaldo</t>
   </si>
   <si>
-    <t>Bater 560k de dano com apenas 2 Pokémon</t>
-  </si>
-  <si>
-    <t>Arcanine, Infernape, Armaldo</t>
-  </si>
-  <si>
-    <t>⭐ Arcanine, Houndoom, Pupitar</t>
+    <t>⭐ Umbreon, Crawdaunt, Sableye</t>
+  </si>
+  <si>
+    <t>Ampharos, Magcargo, Lapras</t>
+  </si>
+  <si>
+    <t>Walrein, Luxray, Pachirisu</t>
+  </si>
+  <si>
+    <t>⭐ Houndoom, Hydreigon, Pupitar</t>
+  </si>
+  <si>
+    <t>Electric, Ice, Rock</t>
+  </si>
+  <si>
+    <t>Metagross</t>
   </si>
   <si>
     <t>⭐ Muk, Tentacruel, Mawile</t>
   </si>
   <si>
-    <t>⭐ Hitmontop, Typhlosion, Rapidash</t>
-  </si>
-  <si>
-    <t>Fire, Rock</t>
+    <t>Steel / Psychic</t>
+  </si>
+  <si>
+    <t>Rapidash, Typhlosion, Steelix</t>
+  </si>
+  <si>
+    <t>Outras Opções T1:</t>
+  </si>
+  <si>
+    <t>Arcanine, Houndoom, Pupitar</t>
   </si>
   <si>
     <t>⭐ Aggron, Skarmory, Toxicroak</t>
   </si>
   <si>
+    <t>Fire, Ground, Ghost, Dark</t>
+  </si>
+  <si>
+    <t>Lucario</t>
+  </si>
+  <si>
     <t>⭐ Blastoise, Feraligatr, Omastar</t>
   </si>
   <si>
-    <t>⭐ Arcanine, Machamp, Pupitar</t>
-  </si>
-  <si>
-    <t>Fairy</t>
-  </si>
-  <si>
-    <t>⭐ Umbreon, Crawdaunt, Sableye</t>
-  </si>
-  <si>
-    <t>⭐ Houndoom, Hydreigon, Pupitar</t>
+    <t>Fighting / Steel</t>
+  </si>
+  <si>
+    <t>Hitmontop, Typhlosion, Rapidash</t>
   </si>
   <si>
     <t>⭐ Pupitar, Torterra, Kingdra</t>
   </si>
   <si>
-    <t>Shiny Sylveon (Lendário)</t>
-  </si>
-  <si>
-    <t>Outras Opções T1:</t>
-  </si>
-  <si>
-    <t>Regra de Prey:</t>
-  </si>
-  <si>
-    <t>Obrigatório Prey de Atk na hunt (já calculada no dummy)</t>
+    <t>Arcanine, Machamp, Pupitar</t>
+  </si>
+  <si>
+    <t>Fighting, Fire, Ground</t>
+  </si>
+  <si>
+    <t>Gengar</t>
+  </si>
+  <si>
+    <t>Ghost / Poison</t>
   </si>
   <si>
     <t>Outras Opções SR:</t>
   </si>
   <si>
-    <t>Manter sempre Prey de Atk ativa na hunt</t>
+    <t>Houndoom, Hydreigon, Pupitar</t>
+  </si>
+  <si>
+    <t>Dark, Ghost, Ground</t>
+  </si>
+  <si>
+    <t>Gardevoir</t>
+  </si>
+  <si>
+    <t>Psychic / Fairy</t>
+  </si>
+  <si>
+    <t>Mawile, Muk, Tentacruel</t>
+  </si>
+  <si>
+    <t>Toxicroak, Seviper, Misdreavus</t>
+  </si>
+  <si>
+    <t>Poison, Ghost, Metal</t>
+  </si>
+  <si>
+    <t>Gyarados</t>
   </si>
   <si>
     <t>Umbreon</t>
   </si>
   <si>
-    <t>💡 POR QUE COMPOSIÇÕES COM 2 A 3 ELEMENTOS SÃO SUPERIORES? (ANTI-MONO)</t>
-  </si>
-  <si>
-    <t>Muk, Tentacruel, Mawile</t>
-  </si>
-  <si>
-    <t>Aggron, Skarmory, Toxicroak</t>
-  </si>
-  <si>
-    <t>Poison, Metal</t>
-  </si>
-  <si>
-    <t>⏱️ Cooldown Reduzido por Tier</t>
+    <t>Water / Flying</t>
+  </si>
+  <si>
+    <t>Ampharos, Luxray, Jolteon</t>
+  </si>
+  <si>
+    <t>Luxray, Pachirisu, Smeargle Eletric</t>
   </si>
   <si>
     <t>S.Charizard, Kabutops, Golem</t>
   </si>
   <si>
-    <t>Fire</t>
-  </si>
-  <si>
-    <t>Magmar (Lendário) / Torkoal (UR)</t>
-  </si>
-  <si>
-    <t>Blastoise, Feraligatr, Omastar</t>
-  </si>
-  <si>
-    <t>Pupitar, Torterra, Kingdra</t>
-  </si>
-  <si>
-    <t>Rock, Water, Ground</t>
-  </si>
-  <si>
-    <t>Fighting</t>
-  </si>
-  <si>
-    <t>Mega Clefable, Pidgeot, Espeon</t>
-  </si>
-  <si>
-    <t>Wobbuffet, Mimikyu, Gliscor</t>
-  </si>
-  <si>
-    <t>Psychic, Flying, Fairy</t>
-  </si>
-  <si>
-    <t>Dark</t>
-  </si>
-  <si>
-    <t>No PKA, tiers mais altos não dão só dano: reduzem o cooldown das skills, deixando a rotação muito mais rápida.</t>
-  </si>
-  <si>
-    <t>Absol (Lendário) / Mightyena (UR)</t>
-  </si>
-  <si>
-    <t>Hitmontop, Hitmonchan, Poliwrath</t>
-  </si>
-  <si>
-    <t>Machamp, Scyther, Mimikyu</t>
-  </si>
-  <si>
-    <t>Fighting, Fairy, Bug</t>
-  </si>
-  <si>
-    <t>Water</t>
-  </si>
-  <si>
-    <t>Milotic (UR)</t>
-  </si>
-  <si>
-    <t>Tangrowth, Ampharos, Venusaur</t>
-  </si>
-  <si>
-    <t>Tangrowth, Gogoat, Luxray</t>
-  </si>
-  <si>
-    <t>Grass, Electric</t>
-  </si>
-  <si>
-    <t>Grass</t>
-  </si>
-  <si>
-    <t>Leafeon (Lendário) / Sceptile (UR)</t>
-  </si>
-  <si>
-    <t>Typhlosion, Rapidash, Pidgeot</t>
-  </si>
-  <si>
-    <t>Arcanine, Infernape, Scyther</t>
-  </si>
-  <si>
-    <t>Poison, Bug, Fire, Fly, Ice</t>
-  </si>
-  <si>
-    <t>Electric</t>
-  </si>
-  <si>
-    <t>Electabuzz (Lendário) / Manectric (UR)</t>
-  </si>
-  <si>
-    <t>Steelix, Nidoqueen, Torterra</t>
-  </si>
-  <si>
-    <t>Torterra, Pupitar, Smeargle</t>
-  </si>
-  <si>
-    <t>Ground</t>
-  </si>
-  <si>
-    <t>Ghost</t>
-  </si>
-  <si>
-    <t>Umbreon, Crawdaunt, Dusknoir</t>
-  </si>
-  <si>
-    <t>Dusknoir, Houndoom, Hydreigon</t>
-  </si>
-  <si>
-    <t>Dark, Ghost</t>
-  </si>
-  <si>
     <t>Torterra, Misdreavus</t>
   </si>
   <si>
-    <t>Ice</t>
-  </si>
-  <si>
-    <t>Glaceon (Lendário) / Glalie (UR)</t>
-  </si>
-  <si>
-    <t>Typhlosion, Rapidash, Hitmontop</t>
-  </si>
-  <si>
     <t>Poliwrath, Medicham, Hariyama</t>
   </si>
   <si>
-    <t>Infernape, Machamp, Skarmory</t>
-  </si>
-  <si>
-    <t>Fighting, Fire, Metal</t>
-  </si>
-  <si>
     <t>Infernape, Kangaskhan, Torterra</t>
   </si>
   <si>
+    <t>Cacturne, Banette, Dusclops</t>
+  </si>
+  <si>
+    <t>Misdreavus, Dusknoir, Torterra</t>
+  </si>
+  <si>
+    <t>🎨 Smeargle: Fire, Ground, Ghost, Dark</t>
+  </si>
+  <si>
     <t>—</t>
   </si>
   <si>
-    <t>Poison</t>
-  </si>
-  <si>
-    <t>Garbodor (Lendário) / Swalot (UR)</t>
-  </si>
-  <si>
-    <t>Cacturne, Banette, Dusclops</t>
-  </si>
-  <si>
-    <t>Steelix, Espeon, Nidoqueen</t>
-  </si>
-  <si>
     <t>Metang, Magneton Estrelado</t>
   </si>
   <si>
-    <t>Wobbuffet, Mr. Mime, Pupitar</t>
-  </si>
-  <si>
-    <t>Misdreavus, Dusknoir, Torterra</t>
-  </si>
-  <si>
-    <t>Ground, Psychic</t>
-  </si>
-  <si>
-    <t>Normal</t>
-  </si>
-  <si>
     <t>SevIper</t>
   </si>
   <si>
-    <t>Snorlax (Lendário) / Exploud (UR)</t>
-  </si>
-  <si>
-    <t>Poliwrath, Hitmontop, Medicham</t>
-  </si>
-  <si>
-    <t>Machamp, Kangaskhan, Smeargle</t>
-  </si>
-  <si>
-    <t>Rock</t>
-  </si>
-  <si>
-    <t>Rampardos (UR)</t>
-  </si>
-  <si>
-    <t>Tangrowth, Steelix, Blastoise</t>
-  </si>
-  <si>
-    <t>Tangrowth, Machamp, Gogoat</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Fire, Ground, Ghost, Dark</t>
-  </si>
-  <si>
-    <t>Fighting, Ground, Water, Grass</t>
-  </si>
-  <si>
-    <t>Steel</t>
-  </si>
-  <si>
-    <t>Hitmontop, Rapidash, Typhlosion</t>
-  </si>
-  <si>
-    <t>Arcanine, Machamp, Infernape</t>
-  </si>
-  <si>
-    <t>Ground, Fighting, Fire</t>
-  </si>
-  <si>
-    <t>Blastoise, Tangrowth, Gogoat</t>
-  </si>
-  <si>
-    <t>Tangrowth, Kingdra, Sharpedo</t>
-  </si>
-  <si>
-    <t>Water, Ice, Grass</t>
-  </si>
-  <si>
-    <t>Dragon</t>
-  </si>
-  <si>
-    <t>Salamence (UR) / Flygon (Lendário)</t>
-  </si>
-  <si>
-    <t>Lapras, Mega Clefable, Jynx</t>
+    <t>🎨 Smeargle: Fighting, Fire, Ground</t>
   </si>
   <si>
     <t>Vaporeon, Rhyperior, Magcargo</t>
   </si>
   <si>
-    <t>Mimikyu, Florges, Walrein</t>
-  </si>
-  <si>
-    <t>Dragon, Ice, Fairy</t>
-  </si>
-  <si>
     <t>Sharpedo</t>
   </si>
   <si>
-    <t>Psychic</t>
-  </si>
-  <si>
-    <t>Alakazam (Lendário)</t>
-  </si>
-  <si>
-    <t>Umbreon, Crawdaunt, Sableye</t>
-  </si>
-  <si>
-    <t>Houndoom, Scyther, Dusknoir</t>
-  </si>
-  <si>
-    <t>Ghost, Dark, Bug</t>
+    <t>🎨 Smeargle: Dark, Ghost, Ground</t>
   </si>
   <si>
     <t>🎨 Smeargle: Fire, Rock</t>
   </si>
   <si>
-    <t>Flying</t>
-  </si>
-  <si>
-    <t>Ampharos, Magcargo, Lapras</t>
-  </si>
-  <si>
-    <t>Walrein, Luxray, Pachirisu</t>
-  </si>
-  <si>
-    <t>Electric, Ice, Rock</t>
-  </si>
-  <si>
-    <t>Metagross</t>
-  </si>
-  <si>
-    <t>Steel / Psychic</t>
-  </si>
-  <si>
-    <t>Rapidash, Typhlosion, Steelix</t>
-  </si>
-  <si>
-    <t>Arcanine, Houndoom, Pupitar</t>
-  </si>
-  <si>
-    <t>Fire, Ground, Ghost, Dark</t>
-  </si>
-  <si>
-    <t>Lucario</t>
-  </si>
-  <si>
-    <t>Fighting / Steel</t>
-  </si>
-  <si>
-    <t>Hitmontop, Typhlosion, Rapidash</t>
-  </si>
-  <si>
-    <t>Arcanine, Machamp, Pupitar</t>
-  </si>
-  <si>
-    <t>Fighting, Fire, Ground</t>
-  </si>
-  <si>
-    <t>Gengar</t>
-  </si>
-  <si>
-    <t>Ghost / Poison</t>
-  </si>
-  <si>
     <t>🎨 Smeargle: Poison, Metal</t>
   </si>
   <si>
-    <t>Houndoom, Hydreigon, Pupitar</t>
-  </si>
-  <si>
-    <t>Dark, Ghost, Ground</t>
-  </si>
-  <si>
-    <t>Gardevoir</t>
-  </si>
-  <si>
-    <t>Psychic / Fairy</t>
-  </si>
-  <si>
-    <t>Mawile, Muk, Tentacruel</t>
-  </si>
-  <si>
-    <t>Toxicroak, Seviper, Misdreavus</t>
+    <t>★ GARDEVOIR</t>
   </si>
   <si>
     <t>🎨 Smeargle: Rock, Water, Ground</t>
   </si>
   <si>
-    <t>Poison, Ghost, Metal</t>
-  </si>
-  <si>
-    <t>Gyarados</t>
-  </si>
-  <si>
-    <t>Water / Flying</t>
-  </si>
-  <si>
-    <t>Ampharos, Luxray, Jolteon</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Fighting, Fire, Ground</t>
-  </si>
-  <si>
-    <t>Luxray, Pachirisu, Smeargle Eletric</t>
-  </si>
-  <si>
-    <t>📈 Mais Mobs e Brokes / Hora</t>
+    <t>★ GYARADOS</t>
   </si>
   <si>
     <t>★ FIGHTING</t>
   </si>
   <si>
-    <t>🎨 Smeargle: Dark, Ghost, Ground</t>
-  </si>
-  <si>
-    <t>Rotação mais fluida = mais mobs derrotados/hora, aumentando drasticamente a chance de Shiny/hr e lucro.</t>
+    <t>★ SWAMPERT</t>
   </si>
   <si>
     <t>★ DARK</t>
   </si>
   <si>
-    <t>★ GARDEVOIR</t>
-  </si>
-  <si>
-    <t>⚔️ Hazards Mais Altos</t>
+    <t>Hunt: Psychic / Fairy</t>
+  </si>
+  <si>
+    <t>Hunt: Water / Flying</t>
   </si>
   <si>
     <t>★ WATER</t>
   </si>
   <si>
-    <t>★ GYARADOS</t>
-  </si>
-  <si>
-    <t>Mesmo encurtando o número total de hunts, permite solar níveis de Hazard superiores com segurança e eficiência.</t>
+    <t>Hunt: Water / Ground</t>
   </si>
   <si>
     <t>Hunt: Absol (Lendário) / Mightyena (UR)</t>
   </si>
   <si>
-    <t>★ SWAMPERT</t>
-  </si>
-  <si>
-    <t>🏆 Futuro &amp; Escalabilidade (Endgame)</t>
+    <t>⭐ Mawile, Muk, Tentacruel</t>
   </si>
   <si>
     <t>Hunt: Milotic (UR)</t>
   </si>
   <si>
-    <t>Trabalhar com 2 ou 3 elementos abre um catálogo amplo de opções viáveis para evoluir: T1, SR, UR e Lendários.</t>
-  </si>
-  <si>
-    <t>Hunt: Psychic / Fairy</t>
+    <t>⭐ Toxicroak, Seviper, Misdreavus</t>
+  </si>
+  <si>
+    <t>⭐ Ampharos, Luxray, Jolteon</t>
+  </si>
+  <si>
+    <t>⭐ S.Luxray, S.Pachirisu, Smeargle Eletric</t>
+  </si>
+  <si>
+    <t>⭐Venusaur, Gogoat, Tangrowth</t>
+  </si>
+  <si>
+    <t>⭐ S.Tangrowth,S. Gogoat, Smeargle Grass</t>
   </si>
   <si>
     <t>⭐ Mega Clefable, Pidgeot, Espeon</t>
@@ -643,24 +667,33 @@
     <t>⭐ Hitmontop, Hitmonchan, Poliwrath</t>
   </si>
   <si>
-    <t>Hunt: Water / Flying</t>
+    <t>Metang, Banette, Dusclops, Nidoking</t>
   </si>
   <si>
     <t>⭐ Machamp, Scyther, Mimikyu</t>
   </si>
   <si>
+    <t>Aggron, Skarmory</t>
+  </si>
+  <si>
     <t>⭐ Tangrowth, Ampharos, Venusaur</t>
   </si>
   <si>
+    <t>Raichu</t>
+  </si>
+  <si>
     <t>⭐ Tangrowth, Gogoat, Luxray</t>
   </si>
   <si>
-    <t>Hunt: Water / Ground</t>
+    <t>🎨 Smeargle: Poison, Ghost, Metal</t>
   </si>
   <si>
     <t>Farfetch'd, Gliscor</t>
   </si>
   <si>
+    <t>🎨 Smeargle: Electric</t>
+  </si>
+  <si>
     <t>Mr. Mime, Florges, Swellow</t>
   </si>
   <si>
@@ -679,78 +712,48 @@
     <t>🎨 Smeargle: Psychic, Flying, Fairy</t>
   </si>
   <si>
-    <t>⭐ Mawile, Muk, Tentacruel</t>
+    <t>🎨 Smeargle: Grass</t>
   </si>
   <si>
     <t>🎨 Smeargle: Fighting, Fairy, Bug</t>
   </si>
   <si>
-    <t>⭐ Toxicroak, Seviper, Misdreavus</t>
-  </si>
-  <si>
-    <t>⭐ Ampharos, Luxray, Jolteon</t>
-  </si>
-  <si>
-    <t>⭐ S.Luxray, S.Pachirisu, Smeargle Eletric</t>
+    <t>★ SCIZOR</t>
   </si>
   <si>
     <t>🎨 Smeargle: Grass, Electric</t>
   </si>
   <si>
-    <t>⭐Venusaur, Gogoat, Tangrowth</t>
-  </si>
-  <si>
-    <t>⭐ S.Tangrowth,S. Gogoat, Smeargle Grass</t>
-  </si>
-  <si>
-    <t>Metang, Banette, Dusclops, Nidoking</t>
+    <t>Hunt: Bug</t>
   </si>
   <si>
     <t>★ GRASS</t>
   </si>
   <si>
-    <t>Aggron, Skarmory</t>
-  </si>
-  <si>
-    <t>Raichu</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Poison, Ghost, Metal</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Electric</t>
+    <t>⭐ S.Rapidash, S.Typhlosion, S.Zard</t>
+  </si>
+  <si>
+    <t>⭐S.Arcanine, S.Infernape, Smeargle Fire</t>
+  </si>
+  <si>
+    <t>🎨 Smeargle: Fire</t>
   </si>
   <si>
     <t>★ ELECTRIC</t>
   </si>
   <si>
-    <t>🎨 Smeargle: Grass</t>
-  </si>
-  <si>
     <t>★ GHOST</t>
   </si>
   <si>
     <t>Hunt: Leafeon (Lendário) / Sceptile (UR)</t>
   </si>
   <si>
-    <t>★ SCIZOR</t>
-  </si>
-  <si>
     <t>Hunt: Electabuzz (Lendário) / Manectric (UR)</t>
   </si>
   <si>
-    <t>Hunt: Bug</t>
-  </si>
-  <si>
-    <t>⭐ S.Rapidash, S.Typhlosion, S.Zard</t>
-  </si>
-  <si>
     <t>⭐ Typhlosion, Rapidash, Pidgeot</t>
   </si>
   <si>
-    <t>⭐S.Arcanine, S.Infernape, Smeargle Fire</t>
-  </si>
-  <si>
     <t>⭐ Arcanine, Infernape, Scyther</t>
   </si>
   <si>
@@ -764,9 +767,6 @@
   </si>
   <si>
     <t>⭐ Dusknoir, Houndoom, Hydreigon</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Fire</t>
   </si>
   <si>
     <t>Charizard, Lapras, Jynx, Gliscor</t>
@@ -983,14 +983,14 @@
     </font>
     <font>
       <b/>
-      <sz val="13.0"/>
+      <sz val="14.0"/>
       <color rgb="FFFFFFFF"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font/>
     <font>
       <b/>
-      <sz val="14.0"/>
+      <sz val="13.0"/>
       <color rgb="FFFFFFFF"/>
       <name val="Quattrocento Sans"/>
     </font>
@@ -1016,13 +1016,6 @@
       <color rgb="FF0000FF"/>
     </font>
     <font>
-      <i/>
-      <u/>
-      <sz val="9.0"/>
-      <color rgb="FFE5E7EB"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
       <b/>
       <sz val="10.0"/>
       <color rgb="FFFFFFFF"/>
@@ -1037,14 +1030,14 @@
     </font>
     <font>
       <b/>
-      <sz val="11.0"/>
-      <color rgb="FFFFFFFF"/>
+      <sz val="9.0"/>
+      <color rgb="FF334155"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
       <b/>
-      <sz val="9.0"/>
-      <color rgb="FF334155"/>
+      <sz val="10.0"/>
+      <color rgb="FF1E293B"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1055,42 +1048,31 @@
     </font>
     <font>
       <sz val="9.0"/>
-      <color rgb="FF0F172A"/>
+      <color rgb="FF475569"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
       <i/>
+      <u/>
       <sz val="9.0"/>
-      <color rgb="FFF3F4F6"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9.0"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10.0"/>
-      <color rgb="FF1E293B"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <sz val="9.0"/>
-      <color rgb="FF475569"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10.0"/>
-      <color rgb="FF1A1A1A"/>
+      <color rgb="FFE5E7EB"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
       <b/>
       <sz val="9.0"/>
       <color rgb="FF166534"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <sz val="9.0"/>
+      <color rgb="FF0F172A"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11.0"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1106,9 +1088,9 @@
       <name val="Quattrocento Sans"/>
     </font>
     <font>
-      <b/>
-      <sz val="8.0"/>
-      <color rgb="FF4B5563"/>
+      <i/>
+      <sz val="9.0"/>
+      <color rgb="FFF3F4F6"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1118,17 +1100,29 @@
       <name val="Quattrocento Sans"/>
     </font>
     <font>
-      <sz val="8.0"/>
-      <color rgb="FF4A4A4A"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
       <sz val="9.0"/>
       <color rgb="FF1F2937"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
       <b/>
+      <sz val="9.0"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10.0"/>
+      <color rgb="FF1A1A1A"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8.0"/>
+      <color rgb="FF4B5563"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
       <sz val="8.0"/>
       <color rgb="FF4A4A4A"/>
       <name val="Quattrocento Sans"/>
@@ -1137,6 +1131,12 @@
       <b/>
       <sz val="8.0"/>
       <color rgb="FF1E3A8A"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8.0"/>
+      <color rgb="FF4A4A4A"/>
       <name val="Quattrocento Sans"/>
     </font>
   </fonts>
@@ -1149,14 +1149,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1B2A4A"/>
-        <bgColor rgb="FF1B2A4A"/>
+        <fgColor rgb="FF0F172A"/>
+        <bgColor rgb="FF0F172A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0F172A"/>
-        <bgColor rgb="FF0F172A"/>
+        <fgColor rgb="FF1B2A4A"/>
+        <bgColor rgb="FF1B2A4A"/>
       </patternFill>
     </fill>
     <fill>
@@ -1173,14 +1173,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF8DAA34"/>
-        <bgColor rgb="FF8DAA34"/>
+        <fgColor rgb="FFF1F5F9"/>
+        <bgColor rgb="FFF1F5F9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF1F5F9"/>
-        <bgColor rgb="FFF1F5F9"/>
+        <fgColor rgb="FFF0FDF4"/>
+        <bgColor rgb="FFF0FDF4"/>
       </patternFill>
     </fill>
     <fill>
@@ -1191,20 +1191,62 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFDCFCE7"/>
+        <bgColor rgb="FFDCFCE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF2F2"/>
+        <bgColor rgb="FFFEF2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF3C7"/>
+        <bgColor rgb="FFFEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF8DAA34"/>
+        <bgColor rgb="FF8DAA34"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8FAFC"/>
+        <bgColor rgb="FFF8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1E40AF"/>
+        <bgColor rgb="FF1E40AF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF374151"/>
+        <bgColor rgb="FF374151"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFE68D9C"/>
         <bgColor rgb="FFE68D9C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEA6C2D"/>
-        <bgColor rgb="FFEA6C2D"/>
+        <fgColor rgb="FFEFF6FF"/>
+        <bgColor rgb="FFEFF6FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF374151"/>
-        <bgColor rgb="FF374151"/>
+        <fgColor rgb="FFEA6C2D"/>
+        <bgColor rgb="FFEA6C2D"/>
       </patternFill>
     </fill>
     <fill>
@@ -1221,20 +1263,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFDCFCE7"/>
-        <bgColor rgb="FFDCFCE7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFE8F5E9"/>
         <bgColor rgb="FFE8F5E9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF0FDF4"/>
-        <bgColor rgb="FFF0FDF4"/>
       </patternFill>
     </fill>
     <fill>
@@ -1245,38 +1275,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFEF2F2"/>
-        <bgColor rgb="FFFEF2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF8FAFC"/>
-        <bgColor rgb="FFF8FAFC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFEF3C7"/>
-        <bgColor rgb="FFFEF3C7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFF0F4F8"/>
         <bgColor rgb="FFF0F4F8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1E40AF"/>
-        <bgColor rgb="FF1E40AF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEFF6FF"/>
-        <bgColor rgb="FFEFF6FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -1402,6 +1402,9 @@
       <left style="thin">
         <color rgb="FFD1D5DB"/>
       </left>
+      <right style="thin">
+        <color rgb="FFD1D5DB"/>
+      </right>
       <top style="thin">
         <color rgb="FFD1D5DB"/>
       </top>
@@ -1427,9 +1430,6 @@
       <left style="thin">
         <color rgb="FFD1D5DB"/>
       </left>
-      <right style="thin">
-        <color rgb="FFD1D5DB"/>
-      </right>
       <top style="thin">
         <color rgb="FFD1D5DB"/>
       </top>
@@ -1489,196 +1489,196 @@
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
+    <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
     <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0"/>
     </xf>
+    <xf borderId="1" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="5" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="6" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="5" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="5" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="5" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="6" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="7" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="5" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="6" fillId="8" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="7" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="9" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="10" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="6" fillId="4" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="7" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="5" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="5" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="11" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="7" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="8" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="12" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="9" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="13" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="5" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="14" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="13" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="6" fillId="15" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="6" fillId="16" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="8" fillId="17" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="13" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="9" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="6" fillId="18" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="8" fillId="5" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="4" fillId="10" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="19" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="10" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="20" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="21" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="22" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="21" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="23" fontId="25" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="4" fillId="24" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="24" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="6" fillId="25" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="11" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="24" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="6" fillId="26" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="6" fillId="4" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="8" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="6" fillId="12" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="6" fillId="13" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="6" fillId="5" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="27" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="14" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="6" fillId="5" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="28" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="6" fillId="15" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="15" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="22" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="6" fillId="16" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf borderId="6" fillId="25" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="6" fillId="17" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="6" fillId="18" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="6" fillId="15" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="6" fillId="5" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="29" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="6" fillId="19" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="30" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="20" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="6" fillId="21" fontId="23" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="6" fillId="19" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="31" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="22" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="32" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="6" fillId="19" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="33" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="8" fillId="23" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="9" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="6" fillId="24" fontId="25" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="6" fillId="24" fontId="25" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="8" fillId="5" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="6" fillId="24" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="10" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="25" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="34" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="26" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="35" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="27" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="36" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="28" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="37" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="8" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="11" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="6" fillId="17" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="29" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="38" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="30" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="39" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="25" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="31" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="32" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="33" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="34" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="35" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="36" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="37" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="38" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="39" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="40" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="40" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1920,155 +1920,155 @@
   </cols>
   <sheetData>
     <row r="2" ht="33.75" customHeight="1">
-      <c r="B2" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="3"/>
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="4"/>
     </row>
     <row r="3" ht="19.5" customHeight="1">
       <c r="B3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="4"/>
     </row>
     <row r="4">
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="11" t="s">
-        <v>7</v>
-      </c>
       <c r="E4" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="F4" s="8" t="s">
         <v>5</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="5" ht="24.0" customHeight="1">
       <c r="B5" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="3"/>
+        <v>10</v>
+      </c>
+      <c r="C5" s="4"/>
       <c r="E5" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="3"/>
+        <v>12</v>
+      </c>
+      <c r="F5" s="4"/>
     </row>
     <row r="6" ht="24.75" customHeight="1">
       <c r="B6" s="16" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" ht="24.75" customHeight="1">
       <c r="B7" s="16" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F7" s="22" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" ht="24.75" customHeight="1">
       <c r="B8" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" s="29" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="C8" s="24" t="s">
+        <v>30</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="38" t="s">
-        <v>46</v>
+        <v>28</v>
+      </c>
+      <c r="F8" s="28" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="9" ht="24.75" customHeight="1">
       <c r="B9" s="16" t="s">
-        <v>61</v>
+        <v>36</v>
       </c>
       <c r="C9" s="22" t="s">
-        <v>62</v>
+        <v>38</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>61</v>
+        <v>36</v>
       </c>
       <c r="F9" s="22" t="s">
-        <v>64</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" ht="24.0" customHeight="1">
-      <c r="B11" s="41" t="s">
-        <v>66</v>
-      </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="3"/>
+      <c r="B11" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="4"/>
     </row>
     <row r="12" ht="24.0" customHeight="1">
-      <c r="B12" s="43" t="s">
-        <v>70</v>
-      </c>
-      <c r="C12" s="44"/>
-      <c r="D12" s="47" t="s">
-        <v>82</v>
-      </c>
-      <c r="E12" s="49"/>
-      <c r="F12" s="44"/>
+      <c r="B12" s="35" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" s="37"/>
+      <c r="D12" s="39" t="s">
+        <v>54</v>
+      </c>
+      <c r="E12" s="41"/>
+      <c r="F12" s="37"/>
     </row>
     <row r="13" ht="24.0" customHeight="1">
-      <c r="B13" s="43" t="s">
-        <v>184</v>
-      </c>
-      <c r="C13" s="44"/>
-      <c r="D13" s="47" t="s">
-        <v>187</v>
-      </c>
-      <c r="E13" s="49"/>
-      <c r="F13" s="44"/>
+      <c r="B13" s="35" t="s">
+        <v>79</v>
+      </c>
+      <c r="C13" s="37"/>
+      <c r="D13" s="39" t="s">
+        <v>87</v>
+      </c>
+      <c r="E13" s="41"/>
+      <c r="F13" s="37"/>
     </row>
     <row r="14" ht="24.0" customHeight="1">
-      <c r="B14" s="43" t="s">
-        <v>190</v>
-      </c>
-      <c r="C14" s="44"/>
-      <c r="D14" s="47" t="s">
-        <v>193</v>
-      </c>
-      <c r="E14" s="49"/>
-      <c r="F14" s="44"/>
+      <c r="B14" s="35" t="s">
+        <v>97</v>
+      </c>
+      <c r="C14" s="37"/>
+      <c r="D14" s="39" t="s">
+        <v>103</v>
+      </c>
+      <c r="E14" s="41"/>
+      <c r="F14" s="37"/>
     </row>
     <row r="15" ht="24.0" customHeight="1">
-      <c r="B15" s="43" t="s">
-        <v>196</v>
-      </c>
-      <c r="C15" s="44"/>
-      <c r="D15" s="47" t="s">
-        <v>198</v>
-      </c>
-      <c r="E15" s="49"/>
-      <c r="F15" s="44"/>
+      <c r="B15" s="35" t="s">
+        <v>113</v>
+      </c>
+      <c r="C15" s="37"/>
+      <c r="D15" s="39" t="s">
+        <v>120</v>
+      </c>
+      <c r="E15" s="41"/>
+      <c r="F15" s="37"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -3094,403 +3094,403 @@
   </cols>
   <sheetData>
     <row r="1" ht="31.5" customHeight="1">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="8" t="s">
-        <v>6</v>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="10" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="2" ht="19.5" customHeight="1">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="8" t="s">
-        <v>10</v>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="10" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="4" ht="21.75" customHeight="1">
-      <c r="A4" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="19"/>
-      <c r="D4" s="21" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" s="19"/>
-      <c r="G4" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="H4" s="19"/>
+      <c r="A4" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="26"/>
+      <c r="D4" s="34" t="s">
+        <v>42</v>
+      </c>
+      <c r="E4" s="26"/>
+      <c r="G4" s="38" t="s">
+        <v>49</v>
+      </c>
+      <c r="H4" s="26"/>
     </row>
     <row r="5" ht="18.0" customHeight="1">
-      <c r="A5" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="B5" s="19"/>
-      <c r="D5" s="24" t="s">
-        <v>32</v>
-      </c>
-      <c r="E5" s="19"/>
-      <c r="G5" s="24" t="s">
-        <v>34</v>
-      </c>
-      <c r="H5" s="19"/>
+      <c r="A5" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="B5" s="26"/>
+      <c r="D5" s="33" t="s">
+        <v>76</v>
+      </c>
+      <c r="E5" s="26"/>
+      <c r="G5" s="33" t="s">
+        <v>90</v>
+      </c>
+      <c r="H5" s="26"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="B6" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="D6" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="E6" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="G6" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="H6" s="27" t="s">
-        <v>39</v>
+      <c r="A6" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="B6" s="42" t="s">
+        <v>77</v>
+      </c>
+      <c r="D6" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="E6" s="42" t="s">
+        <v>77</v>
+      </c>
+      <c r="G6" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" s="42" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="7" ht="42.0" customHeight="1">
-      <c r="A7" s="31" t="s">
-        <v>43</v>
-      </c>
-      <c r="B7" s="33" t="s">
-        <v>45</v>
-      </c>
-      <c r="D7" s="35" t="s">
-        <v>49</v>
-      </c>
-      <c r="E7" s="33" t="s">
-        <v>52</v>
-      </c>
-      <c r="G7" s="35" t="s">
-        <v>53</v>
-      </c>
-      <c r="H7" s="33" t="s">
-        <v>58</v>
+      <c r="A7" s="43" t="s">
+        <v>129</v>
+      </c>
+      <c r="B7" s="44" t="s">
+        <v>138</v>
+      </c>
+      <c r="D7" s="45" t="s">
+        <v>145</v>
+      </c>
+      <c r="E7" s="44" t="s">
+        <v>150</v>
+      </c>
+      <c r="G7" s="45" t="s">
+        <v>153</v>
+      </c>
+      <c r="H7" s="44" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="B8" s="39" t="s">
-        <v>63</v>
-      </c>
-      <c r="D8" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="E8" s="39" t="s">
-        <v>63</v>
-      </c>
-      <c r="G8" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="H8" s="39" t="s">
-        <v>63</v>
+      <c r="A8" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="B8" s="46" t="s">
+        <v>161</v>
+      </c>
+      <c r="D8" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="E8" s="46" t="s">
+        <v>161</v>
+      </c>
+      <c r="G8" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="H8" s="46" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="9" ht="27.75" customHeight="1">
-      <c r="A9" s="46" t="s">
-        <v>71</v>
-      </c>
-      <c r="B9" s="45" t="s">
-        <v>114</v>
-      </c>
-      <c r="D9" s="45" t="s">
-        <v>119</v>
-      </c>
-      <c r="E9" s="48" t="s">
-        <v>124</v>
-      </c>
-      <c r="G9" s="45" t="s">
-        <v>144</v>
-      </c>
-      <c r="H9" s="45" t="s">
-        <v>147</v>
+      <c r="A9" s="48" t="s">
+        <v>174</v>
+      </c>
+      <c r="B9" s="47" t="s">
+        <v>181</v>
+      </c>
+      <c r="D9" s="47" t="s">
+        <v>182</v>
+      </c>
+      <c r="E9" s="50" t="s">
+        <v>183</v>
+      </c>
+      <c r="G9" s="47" t="s">
+        <v>185</v>
+      </c>
+      <c r="H9" s="47" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="10" ht="18.0" customHeight="1">
-      <c r="A10" s="50" t="s">
-        <v>153</v>
-      </c>
-      <c r="B10" s="19"/>
-      <c r="D10" s="50" t="s">
-        <v>170</v>
-      </c>
-      <c r="E10" s="19"/>
-      <c r="G10" s="50" t="s">
-        <v>177</v>
-      </c>
-      <c r="H10" s="19"/>
+      <c r="A10" s="49" t="s">
+        <v>188</v>
+      </c>
+      <c r="B10" s="26"/>
+      <c r="D10" s="49" t="s">
+        <v>189</v>
+      </c>
+      <c r="E10" s="26"/>
+      <c r="G10" s="49" t="s">
+        <v>191</v>
+      </c>
+      <c r="H10" s="26"/>
     </row>
     <row r="14" ht="21.75" customHeight="1">
       <c r="A14" s="51" t="s">
-        <v>185</v>
-      </c>
-      <c r="B14" s="19"/>
-      <c r="D14" s="52" t="s">
-        <v>188</v>
-      </c>
-      <c r="E14" s="19"/>
-      <c r="G14" s="53" t="s">
-        <v>191</v>
-      </c>
-      <c r="H14" s="19"/>
+        <v>193</v>
+      </c>
+      <c r="B14" s="26"/>
+      <c r="D14" s="53" t="s">
+        <v>195</v>
+      </c>
+      <c r="E14" s="26"/>
+      <c r="G14" s="54" t="s">
+        <v>198</v>
+      </c>
+      <c r="H14" s="26"/>
     </row>
     <row r="15" ht="18.0" customHeight="1">
-      <c r="A15" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="B15" s="19"/>
-      <c r="D15" s="24" t="s">
-        <v>194</v>
-      </c>
-      <c r="E15" s="19"/>
-      <c r="G15" s="24" t="s">
-        <v>197</v>
-      </c>
-      <c r="H15" s="19"/>
+      <c r="A15" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="B15" s="26"/>
+      <c r="D15" s="33" t="s">
+        <v>200</v>
+      </c>
+      <c r="E15" s="26"/>
+      <c r="G15" s="33" t="s">
+        <v>202</v>
+      </c>
+      <c r="H15" s="26"/>
     </row>
     <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="B16" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="D16" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="E16" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="G16" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="H16" s="27" t="s">
-        <v>39</v>
+      <c r="A16" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="B16" s="42" t="s">
+        <v>77</v>
+      </c>
+      <c r="D16" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="E16" s="42" t="s">
+        <v>77</v>
+      </c>
+      <c r="G16" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="H16" s="42" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="17" ht="42.0" customHeight="1">
-      <c r="A17" s="35" t="s">
-        <v>200</v>
-      </c>
-      <c r="B17" s="33" t="s">
-        <v>201</v>
-      </c>
-      <c r="D17" s="35" t="s">
-        <v>202</v>
-      </c>
-      <c r="E17" s="33" t="s">
-        <v>204</v>
-      </c>
-      <c r="G17" s="35" t="s">
-        <v>205</v>
-      </c>
-      <c r="H17" s="33" t="s">
-        <v>206</v>
+      <c r="A17" s="45" t="s">
+        <v>208</v>
+      </c>
+      <c r="B17" s="44" t="s">
+        <v>209</v>
+      </c>
+      <c r="D17" s="45" t="s">
+        <v>210</v>
+      </c>
+      <c r="E17" s="44" t="s">
+        <v>212</v>
+      </c>
+      <c r="G17" s="45" t="s">
+        <v>214</v>
+      </c>
+      <c r="H17" s="44" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="18" ht="15.0" customHeight="1">
-      <c r="A18" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="B18" s="39" t="s">
-        <v>63</v>
-      </c>
-      <c r="D18" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="E18" s="39" t="s">
-        <v>63</v>
-      </c>
-      <c r="G18" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="H18" s="39" t="s">
-        <v>63</v>
+      <c r="A18" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="B18" s="46" t="s">
+        <v>161</v>
+      </c>
+      <c r="D18" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="E18" s="46" t="s">
+        <v>161</v>
+      </c>
+      <c r="G18" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="H18" s="46" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="19" ht="27.75" customHeight="1">
-      <c r="A19" s="45" t="s">
-        <v>208</v>
-      </c>
-      <c r="B19" s="45" t="s">
-        <v>209</v>
-      </c>
-      <c r="D19" s="45" t="s">
-        <v>210</v>
-      </c>
-      <c r="E19" s="45" t="s">
-        <v>211</v>
-      </c>
-      <c r="G19" s="45" t="s">
-        <v>212</v>
-      </c>
-      <c r="H19" s="45" t="s">
-        <v>213</v>
+      <c r="A19" s="47" t="s">
+        <v>218</v>
+      </c>
+      <c r="B19" s="47" t="s">
+        <v>220</v>
+      </c>
+      <c r="D19" s="47" t="s">
+        <v>221</v>
+      </c>
+      <c r="E19" s="47" t="s">
+        <v>222</v>
+      </c>
+      <c r="G19" s="47" t="s">
+        <v>223</v>
+      </c>
+      <c r="H19" s="47" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="20" ht="18.0" customHeight="1">
-      <c r="A20" s="50" t="s">
-        <v>214</v>
-      </c>
-      <c r="B20" s="19"/>
-      <c r="D20" s="50" t="s">
-        <v>216</v>
-      </c>
-      <c r="E20" s="19"/>
-      <c r="G20" s="50" t="s">
-        <v>220</v>
-      </c>
-      <c r="H20" s="19"/>
+      <c r="A20" s="49" t="s">
+        <v>225</v>
+      </c>
+      <c r="B20" s="26"/>
+      <c r="D20" s="49" t="s">
+        <v>227</v>
+      </c>
+      <c r="E20" s="26"/>
+      <c r="G20" s="49" t="s">
+        <v>229</v>
+      </c>
+      <c r="H20" s="26"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
     <row r="23" ht="15.75" customHeight="1"/>
     <row r="24" ht="21.75" customHeight="1">
-      <c r="A24" s="57" t="s">
-        <v>224</v>
-      </c>
-      <c r="B24" s="19"/>
-      <c r="D24" s="58" t="s">
-        <v>229</v>
-      </c>
-      <c r="E24" s="19"/>
+      <c r="A24" s="58" t="s">
+        <v>231</v>
+      </c>
+      <c r="B24" s="26"/>
+      <c r="D24" s="59" t="s">
+        <v>235</v>
+      </c>
+      <c r="E24" s="26"/>
       <c r="G24" s="60" t="s">
-        <v>231</v>
-      </c>
-      <c r="H24" s="19"/>
+        <v>236</v>
+      </c>
+      <c r="H24" s="26"/>
     </row>
     <row r="25" ht="18.0" customHeight="1">
-      <c r="A25" s="24" t="s">
-        <v>232</v>
-      </c>
-      <c r="B25" s="19"/>
-      <c r="D25" s="24" t="s">
-        <v>234</v>
-      </c>
-      <c r="E25" s="19"/>
-      <c r="G25" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="H25" s="19"/>
+      <c r="A25" s="33" t="s">
+        <v>237</v>
+      </c>
+      <c r="B25" s="26"/>
+      <c r="D25" s="33" t="s">
+        <v>238</v>
+      </c>
+      <c r="E25" s="26"/>
+      <c r="G25" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="H25" s="26"/>
     </row>
     <row r="26" ht="19.5" customHeight="1">
-      <c r="A26" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="B26" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="D26" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="E26" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="G26" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="H26" s="27" t="s">
-        <v>39</v>
+      <c r="A26" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="B26" s="42" t="s">
+        <v>77</v>
+      </c>
+      <c r="D26" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="E26" s="42" t="s">
+        <v>77</v>
+      </c>
+      <c r="G26" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="H26" s="42" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="27" ht="42.0" customHeight="1">
-      <c r="A27" s="35" t="s">
-        <v>237</v>
-      </c>
-      <c r="B27" s="33" t="s">
+      <c r="A27" s="45" t="s">
         <v>239</v>
       </c>
-      <c r="D27" s="35" t="s">
+      <c r="B27" s="44" t="s">
         <v>240</v>
       </c>
-      <c r="E27" s="33" t="s">
+      <c r="D27" s="45" t="s">
         <v>241</v>
       </c>
-      <c r="G27" s="35" t="s">
+      <c r="E27" s="44" t="s">
         <v>242</v>
       </c>
-      <c r="H27" s="33" t="s">
+      <c r="G27" s="45" t="s">
         <v>243</v>
       </c>
+      <c r="H27" s="44" t="s">
+        <v>244</v>
+      </c>
     </row>
     <row r="28" ht="15.0" customHeight="1">
-      <c r="A28" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="B28" s="39" t="s">
-        <v>63</v>
-      </c>
-      <c r="D28" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="E28" s="39" t="s">
-        <v>63</v>
-      </c>
-      <c r="G28" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="H28" s="39" t="s">
-        <v>63</v>
+      <c r="A28" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="B28" s="46" t="s">
+        <v>161</v>
+      </c>
+      <c r="D28" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="E28" s="46" t="s">
+        <v>161</v>
+      </c>
+      <c r="G28" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="H28" s="46" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="29" ht="27.75" customHeight="1">
-      <c r="A29" s="45" t="s">
+      <c r="A29" s="47" t="s">
         <v>245</v>
       </c>
-      <c r="B29" s="45" t="s">
+      <c r="B29" s="47" t="s">
         <v>246</v>
       </c>
-      <c r="D29" s="45" t="s">
+      <c r="D29" s="47" t="s">
         <v>247</v>
       </c>
-      <c r="E29" s="45" t="s">
+      <c r="E29" s="47" t="s">
         <v>248</v>
       </c>
-      <c r="G29" s="45" t="s">
+      <c r="G29" s="47" t="s">
         <v>249</v>
       </c>
-      <c r="H29" s="45" t="s">
+      <c r="H29" s="47" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="30" ht="18.0" customHeight="1">
-      <c r="A30" s="50" t="s">
+      <c r="A30" s="49" t="s">
         <v>251</v>
       </c>
-      <c r="B30" s="19"/>
-      <c r="D30" s="50" t="s">
+      <c r="B30" s="26"/>
+      <c r="D30" s="49" t="s">
         <v>252</v>
       </c>
-      <c r="E30" s="19"/>
-      <c r="G30" s="50" t="s">
+      <c r="E30" s="26"/>
+      <c r="G30" s="49" t="s">
         <v>253</v>
       </c>
-      <c r="H30" s="19"/>
+      <c r="H30" s="26"/>
     </row>
     <row r="31" ht="15.75" customHeight="1"/>
     <row r="32" ht="15.75" customHeight="1"/>
@@ -3499,123 +3499,123 @@
       <c r="A34" s="61" t="s">
         <v>254</v>
       </c>
-      <c r="B34" s="19"/>
+      <c r="B34" s="26"/>
       <c r="D34" s="62" t="s">
         <v>255</v>
       </c>
-      <c r="E34" s="19"/>
+      <c r="E34" s="26"/>
       <c r="G34" s="63" t="s">
         <v>256</v>
       </c>
-      <c r="H34" s="19"/>
+      <c r="H34" s="26"/>
     </row>
     <row r="35" ht="18.0" customHeight="1">
-      <c r="A35" s="24" t="s">
+      <c r="A35" s="33" t="s">
         <v>257</v>
       </c>
-      <c r="B35" s="19"/>
-      <c r="D35" s="24" t="s">
+      <c r="B35" s="26"/>
+      <c r="D35" s="33" t="s">
         <v>258</v>
       </c>
-      <c r="E35" s="19"/>
+      <c r="E35" s="26"/>
       <c r="G35" s="55" t="s">
         <v>259</v>
       </c>
-      <c r="H35" s="19"/>
+      <c r="H35" s="26"/>
     </row>
     <row r="36" ht="19.5" customHeight="1">
-      <c r="A36" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="B36" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="D36" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="E36" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="G36" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="H36" s="27" t="s">
-        <v>39</v>
+      <c r="A36" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36" s="42" t="s">
+        <v>77</v>
+      </c>
+      <c r="D36" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="E36" s="42" t="s">
+        <v>77</v>
+      </c>
+      <c r="G36" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="H36" s="42" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="37" ht="42.0" customHeight="1">
-      <c r="A37" s="35" t="s">
+      <c r="A37" s="45" t="s">
         <v>260</v>
       </c>
-      <c r="B37" s="33" t="s">
+      <c r="B37" s="44" t="s">
         <v>261</v>
       </c>
-      <c r="D37" s="35" t="s">
+      <c r="D37" s="45" t="s">
         <v>262</v>
       </c>
-      <c r="E37" s="33" t="s">
+      <c r="E37" s="44" t="s">
         <v>263</v>
       </c>
-      <c r="G37" s="35" t="s">
+      <c r="G37" s="45" t="s">
         <v>264</v>
       </c>
-      <c r="H37" s="33" t="s">
+      <c r="H37" s="44" t="s">
         <v>265</v>
       </c>
     </row>
     <row r="38" ht="15.0" customHeight="1">
-      <c r="A38" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="B38" s="39" t="s">
-        <v>63</v>
-      </c>
-      <c r="D38" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="E38" s="39" t="s">
-        <v>63</v>
-      </c>
-      <c r="G38" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="H38" s="39" t="s">
-        <v>63</v>
+      <c r="A38" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="B38" s="46" t="s">
+        <v>161</v>
+      </c>
+      <c r="D38" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="E38" s="46" t="s">
+        <v>161</v>
+      </c>
+      <c r="G38" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="H38" s="46" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="39" ht="27.75" customHeight="1">
-      <c r="A39" s="45" t="s">
+      <c r="A39" s="47" t="s">
         <v>266</v>
       </c>
-      <c r="B39" s="45" t="s">
+      <c r="B39" s="47" t="s">
         <v>267</v>
       </c>
-      <c r="D39" s="45" t="s">
+      <c r="D39" s="47" t="s">
         <v>268</v>
       </c>
-      <c r="E39" s="45" t="s">
+      <c r="E39" s="47" t="s">
         <v>269</v>
       </c>
-      <c r="G39" s="45" t="s">
+      <c r="G39" s="47" t="s">
         <v>270</v>
       </c>
-      <c r="H39" s="45" t="s">
-        <v>114</v>
+      <c r="H39" s="47" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="40" ht="18.0" customHeight="1">
-      <c r="A40" s="50" t="s">
+      <c r="A40" s="49" t="s">
         <v>271</v>
       </c>
-      <c r="B40" s="19"/>
-      <c r="D40" s="50" t="s">
+      <c r="B40" s="26"/>
+      <c r="D40" s="49" t="s">
         <v>272</v>
       </c>
-      <c r="E40" s="19"/>
-      <c r="G40" s="50" t="s">
+      <c r="E40" s="26"/>
+      <c r="G40" s="49" t="s">
         <v>273</v>
       </c>
-      <c r="H40" s="19"/>
+      <c r="H40" s="26"/>
     </row>
     <row r="41" ht="15.75" customHeight="1"/>
     <row r="42" ht="15.75" customHeight="1"/>
@@ -3624,123 +3624,123 @@
       <c r="A44" s="64" t="s">
         <v>274</v>
       </c>
-      <c r="B44" s="19"/>
+      <c r="B44" s="26"/>
       <c r="D44" s="65" t="s">
         <v>275</v>
       </c>
-      <c r="E44" s="19"/>
+      <c r="E44" s="26"/>
       <c r="G44" s="66" t="s">
         <v>276</v>
       </c>
-      <c r="H44" s="19"/>
+      <c r="H44" s="26"/>
     </row>
     <row r="45" ht="18.0" customHeight="1">
-      <c r="A45" s="24" t="s">
+      <c r="A45" s="33" t="s">
         <v>277</v>
       </c>
-      <c r="B45" s="19"/>
-      <c r="D45" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="E45" s="19"/>
-      <c r="G45" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="H45" s="19"/>
+      <c r="B45" s="26"/>
+      <c r="D45" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="E45" s="26"/>
+      <c r="G45" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="H45" s="26"/>
     </row>
     <row r="46" ht="19.5" customHeight="1">
-      <c r="A46" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="B46" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="D46" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="E46" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="G46" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="H46" s="27" t="s">
-        <v>39</v>
+      <c r="A46" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="B46" s="42" t="s">
+        <v>77</v>
+      </c>
+      <c r="D46" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="E46" s="42" t="s">
+        <v>77</v>
+      </c>
+      <c r="G46" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="H46" s="42" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="47" ht="42.0" customHeight="1">
-      <c r="A47" s="35" t="s">
+      <c r="A47" s="45" t="s">
         <v>278</v>
       </c>
-      <c r="B47" s="33" t="s">
+      <c r="B47" s="44" t="s">
         <v>279</v>
       </c>
-      <c r="D47" s="35" t="s">
+      <c r="D47" s="45" t="s">
         <v>280</v>
       </c>
-      <c r="E47" s="33" t="s">
+      <c r="E47" s="44" t="s">
         <v>281</v>
       </c>
-      <c r="G47" s="35" t="s">
+      <c r="G47" s="45" t="s">
         <v>282</v>
       </c>
-      <c r="H47" s="33" t="s">
+      <c r="H47" s="44" t="s">
         <v>283</v>
       </c>
     </row>
     <row r="48" ht="15.0" customHeight="1">
-      <c r="A48" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="B48" s="39" t="s">
-        <v>63</v>
-      </c>
-      <c r="D48" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="E48" s="39" t="s">
-        <v>63</v>
-      </c>
-      <c r="G48" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="H48" s="39" t="s">
-        <v>63</v>
+      <c r="A48" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="B48" s="46" t="s">
+        <v>161</v>
+      </c>
+      <c r="D48" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="E48" s="46" t="s">
+        <v>161</v>
+      </c>
+      <c r="G48" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="H48" s="46" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="49" ht="27.75" customHeight="1">
-      <c r="A49" s="45" t="s">
+      <c r="A49" s="47" t="s">
         <v>284</v>
       </c>
-      <c r="B49" s="45" t="s">
+      <c r="B49" s="47" t="s">
         <v>285</v>
       </c>
-      <c r="D49" s="45" t="s">
+      <c r="D49" s="47" t="s">
         <v>286</v>
       </c>
-      <c r="E49" s="45" t="s">
+      <c r="E49" s="47" t="s">
         <v>287</v>
       </c>
-      <c r="G49" s="45" t="s">
+      <c r="G49" s="47" t="s">
         <v>288</v>
       </c>
-      <c r="H49" s="45" t="s">
+      <c r="H49" s="47" t="s">
         <v>289</v>
       </c>
     </row>
     <row r="50" ht="18.0" customHeight="1">
-      <c r="A50" s="50" t="s">
+      <c r="A50" s="49" t="s">
         <v>290</v>
       </c>
-      <c r="B50" s="19"/>
-      <c r="D50" s="50" t="s">
+      <c r="B50" s="26"/>
+      <c r="D50" s="49" t="s">
         <v>291</v>
       </c>
-      <c r="E50" s="19"/>
-      <c r="G50" s="50" t="s">
+      <c r="E50" s="26"/>
+      <c r="G50" s="49" t="s">
         <v>292</v>
       </c>
-      <c r="H50" s="19"/>
+      <c r="H50" s="26"/>
     </row>
     <row r="51" ht="15.75" customHeight="1"/>
     <row r="52" ht="15.75" customHeight="1"/>
@@ -3749,123 +3749,123 @@
       <c r="A54" s="67" t="s">
         <v>293</v>
       </c>
-      <c r="B54" s="19"/>
+      <c r="B54" s="26"/>
       <c r="D54" s="68" t="s">
         <v>294</v>
       </c>
-      <c r="E54" s="19"/>
+      <c r="E54" s="26"/>
       <c r="G54" s="69" t="s">
         <v>295</v>
       </c>
-      <c r="H54" s="19"/>
+      <c r="H54" s="26"/>
     </row>
     <row r="55" ht="18.0" customHeight="1">
-      <c r="A55" s="24" t="s">
+      <c r="A55" s="33" t="s">
         <v>296</v>
       </c>
-      <c r="B55" s="19"/>
-      <c r="D55" s="24" t="s">
+      <c r="B55" s="26"/>
+      <c r="D55" s="33" t="s">
         <v>297</v>
       </c>
-      <c r="E55" s="19"/>
-      <c r="G55" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="H55" s="19"/>
+      <c r="E55" s="26"/>
+      <c r="G55" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="H55" s="26"/>
     </row>
     <row r="56" ht="19.5" customHeight="1">
-      <c r="A56" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="B56" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="D56" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="E56" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="G56" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="H56" s="27" t="s">
-        <v>39</v>
+      <c r="A56" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="B56" s="42" t="s">
+        <v>77</v>
+      </c>
+      <c r="D56" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="E56" s="42" t="s">
+        <v>77</v>
+      </c>
+      <c r="G56" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="H56" s="42" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="57" ht="42.0" customHeight="1">
-      <c r="A57" s="35" t="s">
+      <c r="A57" s="45" t="s">
         <v>298</v>
       </c>
-      <c r="B57" s="33" t="s">
+      <c r="B57" s="44" t="s">
         <v>299</v>
       </c>
-      <c r="D57" s="35" t="s">
-        <v>56</v>
-      </c>
-      <c r="E57" s="33" t="s">
+      <c r="D57" s="45" t="s">
+        <v>139</v>
+      </c>
+      <c r="E57" s="44" t="s">
         <v>300</v>
       </c>
-      <c r="G57" s="35" t="s">
+      <c r="G57" s="45" t="s">
         <v>301</v>
       </c>
-      <c r="H57" s="33" t="s">
+      <c r="H57" s="44" t="s">
         <v>302</v>
       </c>
     </row>
     <row r="58" ht="15.0" customHeight="1">
-      <c r="A58" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="B58" s="39" t="s">
-        <v>63</v>
-      </c>
-      <c r="D58" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="E58" s="39" t="s">
-        <v>63</v>
-      </c>
-      <c r="G58" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="H58" s="39" t="s">
-        <v>63</v>
+      <c r="A58" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="B58" s="46" t="s">
+        <v>161</v>
+      </c>
+      <c r="D58" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="E58" s="46" t="s">
+        <v>161</v>
+      </c>
+      <c r="G58" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="H58" s="46" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="59" ht="27.75" customHeight="1">
-      <c r="A59" s="45" t="s">
+      <c r="A59" s="47" t="s">
         <v>303</v>
       </c>
-      <c r="B59" s="45" t="s">
+      <c r="B59" s="47" t="s">
         <v>304</v>
       </c>
-      <c r="D59" s="45" t="s">
+      <c r="D59" s="47" t="s">
         <v>305</v>
       </c>
-      <c r="E59" s="45" t="s">
+      <c r="E59" s="47" t="s">
         <v>306</v>
       </c>
-      <c r="G59" s="45" t="s">
+      <c r="G59" s="47" t="s">
         <v>307</v>
       </c>
-      <c r="H59" s="45" t="s">
+      <c r="H59" s="47" t="s">
         <v>308</v>
       </c>
     </row>
     <row r="60" ht="18.0" customHeight="1">
-      <c r="A60" s="50" t="s">
+      <c r="A60" s="49" t="s">
         <v>309</v>
       </c>
-      <c r="B60" s="19"/>
-      <c r="D60" s="50" t="s">
+      <c r="B60" s="26"/>
+      <c r="D60" s="49" t="s">
         <v>310</v>
       </c>
-      <c r="E60" s="19"/>
-      <c r="G60" s="50" t="s">
+      <c r="E60" s="26"/>
+      <c r="G60" s="49" t="s">
         <v>311</v>
       </c>
-      <c r="H60" s="19"/>
+      <c r="H60" s="26"/>
     </row>
     <row r="61" ht="15.75" customHeight="1"/>
     <row r="62" ht="15.75" customHeight="1"/>
@@ -4892,325 +4892,325 @@
   </cols>
   <sheetData>
     <row r="1" ht="31.5" customHeight="1">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="3"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="4"/>
     </row>
     <row r="2" ht="19.5" customHeight="1">
-      <c r="A2" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="3"/>
+      <c r="A2" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="4"/>
     </row>
     <row r="4" ht="21.75" customHeight="1">
-      <c r="A4" s="20" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="19"/>
-      <c r="D4" s="20" t="s">
-        <v>22</v>
-      </c>
-      <c r="E4" s="19"/>
-      <c r="G4" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" s="19"/>
+      <c r="A4" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="26"/>
+      <c r="D4" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" s="26"/>
+      <c r="G4" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="H4" s="26"/>
     </row>
     <row r="5" ht="18.0" customHeight="1">
-      <c r="A5" s="24" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" s="19"/>
-      <c r="D5" s="24" t="s">
-        <v>31</v>
-      </c>
-      <c r="E5" s="19"/>
-      <c r="G5" s="24" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" s="19"/>
+      <c r="A5" s="33" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="26"/>
+      <c r="D5" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="E5" s="26"/>
+      <c r="G5" s="33" t="s">
+        <v>50</v>
+      </c>
+      <c r="H5" s="26"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="B6" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="D6" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="E6" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="G6" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="H6" s="27" t="s">
-        <v>39</v>
+      <c r="A6" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="B6" s="42" t="s">
+        <v>77</v>
+      </c>
+      <c r="D6" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="E6" s="42" t="s">
+        <v>77</v>
+      </c>
+      <c r="G6" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" s="42" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="7" ht="42.0" customHeight="1">
-      <c r="A7" s="31" t="s">
-        <v>42</v>
-      </c>
-      <c r="B7" s="33" t="s">
-        <v>48</v>
-      </c>
-      <c r="D7" s="35" t="s">
-        <v>50</v>
-      </c>
-      <c r="E7" s="33" t="s">
-        <v>54</v>
-      </c>
-      <c r="G7" s="35" t="s">
-        <v>56</v>
-      </c>
-      <c r="H7" s="33" t="s">
-        <v>57</v>
+      <c r="A7" s="43" t="s">
+        <v>108</v>
+      </c>
+      <c r="B7" s="44" t="s">
+        <v>119</v>
+      </c>
+      <c r="D7" s="45" t="s">
+        <v>130</v>
+      </c>
+      <c r="E7" s="44" t="s">
+        <v>136</v>
+      </c>
+      <c r="G7" s="45" t="s">
+        <v>139</v>
+      </c>
+      <c r="H7" s="44" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="B8" s="39" t="s">
-        <v>63</v>
-      </c>
-      <c r="D8" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="E8" s="39" t="s">
-        <v>63</v>
-      </c>
-      <c r="G8" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="H8" s="39" t="s">
-        <v>63</v>
+      <c r="A8" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="B8" s="46" t="s">
+        <v>161</v>
+      </c>
+      <c r="D8" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="E8" s="46" t="s">
+        <v>161</v>
+      </c>
+      <c r="G8" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="H8" s="46" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="9" ht="27.75" customHeight="1">
-      <c r="A9" s="45" t="s">
-        <v>65</v>
-      </c>
-      <c r="B9" s="45" t="s">
-        <v>106</v>
-      </c>
-      <c r="D9" s="45" t="s">
-        <v>110</v>
-      </c>
-      <c r="E9" s="45" t="s">
-        <v>113</v>
-      </c>
-      <c r="G9" s="45" t="s">
-        <v>117</v>
-      </c>
-      <c r="H9" s="45" t="s">
-        <v>121</v>
+      <c r="A9" s="47" t="s">
+        <v>170</v>
+      </c>
+      <c r="B9" s="47" t="s">
+        <v>175</v>
+      </c>
+      <c r="D9" s="47" t="s">
+        <v>176</v>
+      </c>
+      <c r="E9" s="47" t="s">
+        <v>177</v>
+      </c>
+      <c r="G9" s="47" t="s">
+        <v>178</v>
+      </c>
+      <c r="H9" s="47" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="10" ht="18.0" customHeight="1">
-      <c r="A10" s="50" t="s">
-        <v>132</v>
-      </c>
-      <c r="B10" s="19"/>
-      <c r="D10" s="50" t="s">
-        <v>182</v>
-      </c>
-      <c r="E10" s="19"/>
-      <c r="G10" s="50" t="s">
-        <v>186</v>
-      </c>
-      <c r="H10" s="19"/>
+      <c r="A10" s="49" t="s">
+        <v>180</v>
+      </c>
+      <c r="B10" s="26"/>
+      <c r="D10" s="49" t="s">
+        <v>184</v>
+      </c>
+      <c r="E10" s="26"/>
+      <c r="G10" s="49" t="s">
+        <v>187</v>
+      </c>
+      <c r="H10" s="26"/>
     </row>
     <row r="14" ht="21.75" customHeight="1">
-      <c r="A14" s="20" t="s">
-        <v>189</v>
-      </c>
-      <c r="B14" s="19"/>
-      <c r="D14" s="20" t="s">
+      <c r="A14" s="23" t="s">
+        <v>190</v>
+      </c>
+      <c r="B14" s="26"/>
+      <c r="D14" s="23" t="s">
         <v>192</v>
       </c>
-      <c r="E14" s="19"/>
-      <c r="G14" s="54" t="s">
-        <v>195</v>
-      </c>
-      <c r="H14" s="19"/>
+      <c r="E14" s="26"/>
+      <c r="G14" s="52" t="s">
+        <v>194</v>
+      </c>
+      <c r="H14" s="26"/>
     </row>
     <row r="15" ht="18.0" customHeight="1">
-      <c r="A15" s="24" t="s">
+      <c r="A15" s="33" t="s">
+        <v>196</v>
+      </c>
+      <c r="B15" s="26"/>
+      <c r="D15" s="33" t="s">
+        <v>197</v>
+      </c>
+      <c r="E15" s="26"/>
+      <c r="G15" s="55" t="s">
         <v>199</v>
       </c>
-      <c r="B15" s="19"/>
-      <c r="D15" s="24" t="s">
+      <c r="H15" s="26"/>
+    </row>
+    <row r="16" ht="19.5" customHeight="1">
+      <c r="A16" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="B16" s="42" t="s">
+        <v>77</v>
+      </c>
+      <c r="D16" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="E16" s="42" t="s">
+        <v>77</v>
+      </c>
+      <c r="G16" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="H16" s="42" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="17" ht="42.0" customHeight="1">
+      <c r="A17" s="45" t="s">
+        <v>201</v>
+      </c>
+      <c r="B17" s="44" t="s">
         <v>203</v>
       </c>
-      <c r="E15" s="19"/>
-      <c r="G15" s="55" t="s">
+      <c r="D17" s="45" t="s">
+        <v>204</v>
+      </c>
+      <c r="E17" s="56" t="s">
+        <v>205</v>
+      </c>
+      <c r="G17" s="43" t="s">
+        <v>206</v>
+      </c>
+      <c r="H17" s="56" t="s">
         <v>207</v>
       </c>
-      <c r="H15" s="19"/>
-    </row>
-    <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="B16" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="D16" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="E16" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="G16" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="H16" s="27" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="17" ht="42.0" customHeight="1">
-      <c r="A17" s="35" t="s">
+    </row>
+    <row r="18" ht="15.0" customHeight="1">
+      <c r="A18" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="B18" s="46" t="s">
+        <v>161</v>
+      </c>
+      <c r="D18" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="E18" s="46" t="s">
+        <v>161</v>
+      </c>
+      <c r="G18" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="H18" s="46" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="19" ht="27.75" customHeight="1">
+      <c r="A19" s="47" t="s">
+        <v>211</v>
+      </c>
+      <c r="B19" s="47" t="s">
+        <v>213</v>
+      </c>
+      <c r="D19" s="47" t="s">
         <v>215</v>
       </c>
-      <c r="B17" s="33" t="s">
+      <c r="E19" s="47" t="s">
+        <v>181</v>
+      </c>
+      <c r="G19" s="47" t="s">
+        <v>181</v>
+      </c>
+      <c r="H19" s="47" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="20" ht="18.0" customHeight="1">
+      <c r="A20" s="49" t="s">
         <v>217</v>
       </c>
-      <c r="D17" s="35" t="s">
-        <v>218</v>
-      </c>
-      <c r="E17" s="56" t="s">
+      <c r="B20" s="26"/>
+      <c r="D20" s="49" t="s">
         <v>219</v>
       </c>
-      <c r="G17" s="31" t="s">
-        <v>221</v>
-      </c>
-      <c r="H17" s="56" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="18" ht="15.0" customHeight="1">
-      <c r="A18" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="B18" s="39" t="s">
-        <v>63</v>
-      </c>
-      <c r="D18" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="E18" s="39" t="s">
-        <v>63</v>
-      </c>
-      <c r="G18" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="H18" s="39" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="19" ht="27.75" customHeight="1">
-      <c r="A19" s="45" t="s">
-        <v>223</v>
-      </c>
-      <c r="B19" s="45" t="s">
-        <v>225</v>
-      </c>
-      <c r="D19" s="45" t="s">
+      <c r="E20" s="26"/>
+      <c r="G20" s="57" t="s">
         <v>226</v>
       </c>
-      <c r="E19" s="45" t="s">
-        <v>114</v>
-      </c>
-      <c r="G19" s="45" t="s">
-        <v>114</v>
-      </c>
-      <c r="H19" s="45" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="20" ht="18.0" customHeight="1">
-      <c r="A20" s="50" t="s">
-        <v>227</v>
-      </c>
-      <c r="B20" s="19"/>
-      <c r="D20" s="50" t="s">
-        <v>228</v>
-      </c>
-      <c r="E20" s="19"/>
-      <c r="G20" s="59" t="s">
-        <v>230</v>
-      </c>
-      <c r="H20" s="19"/>
+      <c r="H20" s="26"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
     <row r="23" ht="15.75" customHeight="1"/>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="54" t="s">
-        <v>233</v>
-      </c>
-      <c r="B24" s="19"/>
+      <c r="A24" s="52" t="s">
+        <v>228</v>
+      </c>
+      <c r="B24" s="26"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="55" t="s">
-        <v>235</v>
-      </c>
-      <c r="B25" s="19"/>
+        <v>230</v>
+      </c>
+      <c r="B25" s="26"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="26" t="s">
-        <v>35</v>
-      </c>
-      <c r="B26" s="27" t="s">
-        <v>39</v>
+      <c r="A26" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="B26" s="42" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="27" ht="44.25" customHeight="1">
-      <c r="A27" s="31" t="s">
-        <v>236</v>
+      <c r="A27" s="43" t="s">
+        <v>232</v>
       </c>
       <c r="B27" s="56" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="B28" s="39" t="s">
-        <v>63</v>
+      <c r="A28" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="B28" s="46" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="29" ht="27.75" customHeight="1">
-      <c r="A29" s="45" t="s">
-        <v>114</v>
-      </c>
-      <c r="B29" s="45" t="s">
-        <v>114</v>
+      <c r="A29" s="47" t="s">
+        <v>181</v>
+      </c>
+      <c r="B29" s="47" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="59" t="s">
-        <v>244</v>
-      </c>
-      <c r="B30" s="19"/>
+      <c r="A30" s="57" t="s">
+        <v>234</v>
+      </c>
+      <c r="B30" s="26"/>
     </row>
     <row r="31" ht="15.75" customHeight="1"/>
     <row r="32" ht="15.75" customHeight="1"/>
@@ -6234,438 +6234,438 @@
   </cols>
   <sheetData>
     <row r="1" ht="27.75" customHeight="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="3"/>
+      <c r="A1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="4"/>
     </row>
     <row r="2" ht="18.0" customHeight="1">
-      <c r="A2" s="10"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="3"/>
+      <c r="A2" s="9"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="4"/>
     </row>
     <row r="3">
       <c r="B3" s="11" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" ht="24.0" customHeight="1">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="25" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="25" t="s">
-        <v>36</v>
-      </c>
-      <c r="D4" s="25" t="s">
-        <v>37</v>
-      </c>
-      <c r="E4" s="17" t="s">
-        <v>38</v>
+      <c r="D4" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="5" ht="21.75" customHeight="1">
-      <c r="A5" s="28" t="s">
-        <v>40</v>
-      </c>
-      <c r="B5" s="30" t="s">
-        <v>41</v>
-      </c>
-      <c r="C5" s="32" t="s">
-        <v>44</v>
-      </c>
-      <c r="D5" s="34" t="s">
+      <c r="A5" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="27" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" ht="21.75" customHeight="1">
+      <c r="A6" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" s="32" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="E5" s="36" t="s">
+      <c r="E6" s="36" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" ht="21.75" customHeight="1">
+      <c r="A7" s="17" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="6" ht="21.75" customHeight="1">
-      <c r="A6" s="37" t="s">
+      <c r="B7" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="B6" s="40" t="s">
+      <c r="E7" s="27" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" ht="21.75" customHeight="1">
+      <c r="A8" s="30" t="s">
+        <v>57</v>
+      </c>
+      <c r="B8" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="C6" s="32" t="s">
+      <c r="D8" s="25" t="s">
+        <v>60</v>
+      </c>
+      <c r="E8" s="36" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" ht="21.75" customHeight="1">
+      <c r="A9" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="E9" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="D6" s="34" t="s">
+    </row>
+    <row r="10" ht="21.75" customHeight="1">
+      <c r="A10" s="30" t="s">
         <v>68</v>
       </c>
-      <c r="E6" s="42" t="s">
+      <c r="B10" s="32" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="7" ht="21.75" customHeight="1">
-      <c r="A7" s="28" t="s">
+      <c r="C10" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="D10" s="25" t="s">
+        <v>71</v>
+      </c>
+      <c r="E10" s="36" t="s">
         <v>72</v>
       </c>
-      <c r="B7" s="30" t="s">
+    </row>
+    <row r="11" ht="21.75" customHeight="1">
+      <c r="A11" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="C7" s="32" t="s">
+      <c r="B11" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="D7" s="34" t="s">
+      <c r="C11" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="E7" s="36" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="8" ht="21.75" customHeight="1">
-      <c r="A8" s="37" t="s">
-        <v>77</v>
-      </c>
-      <c r="B8" s="40" t="s">
-        <v>41</v>
-      </c>
-      <c r="C8" s="32" t="s">
+      <c r="D11" s="25" t="s">
         <v>78</v>
       </c>
-      <c r="D8" s="34" t="s">
-        <v>79</v>
-      </c>
-      <c r="E8" s="42" t="s">
+      <c r="E11" s="27" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="9" ht="21.75" customHeight="1">
-      <c r="A9" s="28" t="s">
+    <row r="12" ht="21.75" customHeight="1">
+      <c r="A12" s="30" t="s">
         <v>81</v>
       </c>
-      <c r="B9" s="30" t="s">
+      <c r="B12" s="32" t="s">
+        <v>82</v>
+      </c>
+      <c r="C12" s="21" t="s">
         <v>83</v>
       </c>
-      <c r="C9" s="32" t="s">
+      <c r="D12" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="D9" s="34" t="s">
+      <c r="E12" s="36" t="s">
         <v>85</v>
       </c>
-      <c r="E9" s="36" t="s">
+    </row>
+    <row r="13" ht="21.75" customHeight="1">
+      <c r="A13" s="17" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="10" ht="21.75" customHeight="1">
-      <c r="A10" s="37" t="s">
-        <v>87</v>
-      </c>
-      <c r="B10" s="40" t="s">
+      <c r="B13" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="21" t="s">
         <v>88</v>
       </c>
-      <c r="C10" s="32" t="s">
+      <c r="D13" s="25" t="s">
         <v>89</v>
       </c>
-      <c r="D10" s="34" t="s">
-        <v>90</v>
-      </c>
-      <c r="E10" s="42" t="s">
+      <c r="E13" s="27" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="11" ht="21.75" customHeight="1">
-      <c r="A11" s="28" t="s">
+    <row r="14" ht="21.75" customHeight="1">
+      <c r="A14" s="30" t="s">
         <v>92</v>
       </c>
-      <c r="B11" s="30" t="s">
+      <c r="B14" s="32" t="s">
         <v>93</v>
       </c>
-      <c r="C11" s="32" t="s">
+      <c r="C14" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="D11" s="34" t="s">
+      <c r="D14" s="25" t="s">
         <v>95</v>
       </c>
-      <c r="E11" s="36" t="s">
+      <c r="E14" s="36" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="12" ht="21.75" customHeight="1">
-      <c r="A12" s="37" t="s">
-        <v>97</v>
-      </c>
-      <c r="B12" s="40" t="s">
+    <row r="15" ht="21.75" customHeight="1">
+      <c r="A15" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="C12" s="32" t="s">
+      <c r="B15" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="D12" s="34" t="s">
+      <c r="C15" s="21" t="s">
         <v>100</v>
       </c>
-      <c r="E12" s="42" t="s">
+      <c r="D15" s="25" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="13" ht="21.75" customHeight="1">
-      <c r="A13" s="28" t="s">
+      <c r="E15" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="B13" s="30" t="s">
-        <v>41</v>
-      </c>
-      <c r="C13" s="32" t="s">
-        <v>103</v>
-      </c>
-      <c r="D13" s="34" t="s">
+    </row>
+    <row r="16" ht="21.75" customHeight="1">
+      <c r="A16" s="30" t="s">
         <v>104</v>
       </c>
-      <c r="E13" s="36" t="s">
+      <c r="B16" s="32" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="14" ht="21.75" customHeight="1">
-      <c r="A14" s="37" t="s">
+      <c r="C16" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="D16" s="25" t="s">
         <v>107</v>
       </c>
-      <c r="B14" s="40" t="s">
-        <v>108</v>
-      </c>
-      <c r="C14" s="32" t="s">
+      <c r="E16" s="36" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17" ht="21.75" customHeight="1">
+      <c r="A17" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="D14" s="34" t="s">
+      <c r="B17" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="C17" s="21" t="s">
         <v>111</v>
       </c>
-      <c r="E14" s="42" t="s">
+      <c r="D17" s="25" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="15" ht="21.75" customHeight="1">
-      <c r="A15" s="28" t="s">
+      <c r="E17" s="27" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="18" ht="21.75" customHeight="1">
+      <c r="A18" s="30" t="s">
         <v>115</v>
       </c>
-      <c r="B15" s="30" t="s">
+      <c r="B18" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="21" t="s">
         <v>116</v>
       </c>
-      <c r="C15" s="32" t="s">
+      <c r="D18" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="E18" s="36" t="s">
         <v>118</v>
       </c>
-      <c r="D15" s="34" t="s">
-        <v>120</v>
-      </c>
-      <c r="E15" s="36" t="s">
+    </row>
+    <row r="19" ht="21.75" customHeight="1">
+      <c r="A19" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="B19" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="C19" s="21" t="s">
+        <v>121</v>
+      </c>
+      <c r="D19" s="25" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="16" ht="21.75" customHeight="1">
-      <c r="A16" s="37" t="s">
+      <c r="E19" s="27" t="s">
         <v>123</v>
       </c>
-      <c r="B16" s="40" t="s">
+    </row>
+    <row r="20" ht="21.75" customHeight="1">
+      <c r="A20" s="30" t="s">
+        <v>124</v>
+      </c>
+      <c r="B20" s="32" t="s">
         <v>125</v>
       </c>
-      <c r="C16" s="32" t="s">
+      <c r="C20" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="D16" s="34" t="s">
+      <c r="D20" s="25" t="s">
         <v>127</v>
       </c>
-      <c r="E16" s="42" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="17" ht="21.75" customHeight="1">
-      <c r="A17" s="28" t="s">
+      <c r="E20" s="36" t="s">
         <v>128</v>
       </c>
-      <c r="B17" s="30" t="s">
-        <v>129</v>
-      </c>
-      <c r="C17" s="32" t="s">
-        <v>130</v>
-      </c>
-      <c r="D17" s="34" t="s">
+    </row>
+    <row r="21" ht="21.75" customHeight="1">
+      <c r="A21" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="E17" s="36" t="s">
+      <c r="B21" s="19" t="s">
+        <v>132</v>
+      </c>
+      <c r="C21" s="21" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="18" ht="21.75" customHeight="1">
-      <c r="A18" s="37" t="s">
+      <c r="D21" s="25" t="s">
         <v>134</v>
       </c>
-      <c r="B18" s="40" t="s">
-        <v>41</v>
-      </c>
-      <c r="C18" s="32" t="s">
+      <c r="E21" s="27" t="s">
         <v>135</v>
       </c>
-      <c r="D18" s="34" t="s">
-        <v>136</v>
-      </c>
-      <c r="E18" s="42" t="s">
+    </row>
+    <row r="22" ht="21.75" customHeight="1">
+      <c r="A22" s="30" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="19" ht="21.75" customHeight="1">
-      <c r="A19" s="28" t="s">
-        <v>101</v>
-      </c>
-      <c r="B19" s="30" t="s">
-        <v>41</v>
-      </c>
-      <c r="C19" s="32" t="s">
-        <v>138</v>
-      </c>
-      <c r="D19" s="34" t="s">
-        <v>139</v>
-      </c>
-      <c r="E19" s="36" t="s">
+      <c r="B22" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="C22" s="21" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="20" ht="21.75" customHeight="1">
-      <c r="A20" s="37" t="s">
+      <c r="D22" s="25" t="s">
         <v>141</v>
       </c>
-      <c r="B20" s="40" t="s">
-        <v>142</v>
-      </c>
-      <c r="C20" s="32" t="s">
+      <c r="E22" s="36" t="s">
         <v>143</v>
       </c>
-      <c r="D20" s="34" t="s">
-        <v>145</v>
-      </c>
-      <c r="E20" s="42" t="s">
+    </row>
+    <row r="23" ht="21.75" customHeight="1">
+      <c r="A23" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="B23" s="19" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="21" ht="21.75" customHeight="1">
-      <c r="A21" s="28" t="s">
-        <v>148</v>
-      </c>
-      <c r="B21" s="30" t="s">
+      <c r="C23" s="21" t="s">
+        <v>147</v>
+      </c>
+      <c r="D23" s="25" t="s">
         <v>149</v>
       </c>
-      <c r="C21" s="32" t="s">
-        <v>150</v>
-      </c>
-      <c r="D21" s="34" t="s">
+      <c r="E23" s="27" t="s">
         <v>151</v>
       </c>
-      <c r="E21" s="36" t="s">
+    </row>
+    <row r="24" ht="21.75" customHeight="1">
+      <c r="A24" s="30" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="22" ht="21.75" customHeight="1">
-      <c r="A22" s="37" t="s">
+      <c r="B24" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="B22" s="40" t="s">
-        <v>41</v>
-      </c>
-      <c r="C22" s="32" t="s">
+      <c r="C24" s="21" t="s">
         <v>155</v>
       </c>
-      <c r="D22" s="34" t="s">
-        <v>156</v>
-      </c>
-      <c r="E22" s="42" t="s">
+      <c r="D24" s="25" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="23" ht="21.75" customHeight="1">
-      <c r="A23" s="28" t="s">
+      <c r="E24" s="36" t="s">
         <v>158</v>
       </c>
-      <c r="B23" s="30" t="s">
+    </row>
+    <row r="25" ht="21.75" customHeight="1">
+      <c r="A25" s="17" t="s">
         <v>159</v>
       </c>
-      <c r="C23" s="32" t="s">
+      <c r="B25" s="19" t="s">
         <v>160</v>
       </c>
-      <c r="D23" s="34" t="s">
-        <v>161</v>
-      </c>
-      <c r="E23" s="36" t="s">
+      <c r="C25" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="D25" s="25" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="24" ht="21.75" customHeight="1">
-      <c r="A24" s="37" t="s">
+      <c r="E25" s="27" t="s">
         <v>163</v>
       </c>
-      <c r="B24" s="40" t="s">
+    </row>
+    <row r="26" ht="21.75" customHeight="1">
+      <c r="A26" s="30" t="s">
         <v>164</v>
       </c>
-      <c r="C24" s="32" t="s">
+      <c r="B26" s="32" t="s">
         <v>165</v>
       </c>
-      <c r="D24" s="34" t="s">
+      <c r="C26" s="21" t="s">
         <v>166</v>
       </c>
-      <c r="E24" s="42" t="s">
+      <c r="D26" s="25" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="25" ht="21.75" customHeight="1">
-      <c r="A25" s="28" t="s">
+      <c r="E26" s="36" t="s">
         <v>168</v>
       </c>
-      <c r="B25" s="30" t="s">
+    </row>
+    <row r="27" ht="21.75" customHeight="1">
+      <c r="A27" s="17" t="s">
         <v>169</v>
       </c>
-      <c r="C25" s="32" t="s">
-        <v>150</v>
-      </c>
-      <c r="D25" s="34" t="s">
+      <c r="B27" s="19" t="s">
         <v>171</v>
       </c>
-      <c r="E25" s="36" t="s">
+      <c r="C27" s="21" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="26" ht="21.75" customHeight="1">
-      <c r="A26" s="37" t="s">
+      <c r="D27" s="25" t="s">
         <v>173</v>
       </c>
-      <c r="B26" s="40" t="s">
-        <v>174</v>
-      </c>
-      <c r="C26" s="32" t="s">
-        <v>175</v>
-      </c>
-      <c r="D26" s="34" t="s">
-        <v>176</v>
-      </c>
-      <c r="E26" s="42" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="27" ht="21.75" customHeight="1">
-      <c r="A27" s="28" t="s">
-        <v>179</v>
-      </c>
-      <c r="B27" s="30" t="s">
-        <v>180</v>
-      </c>
-      <c r="C27" s="32" t="s">
-        <v>181</v>
-      </c>
-      <c r="D27" s="34" t="s">
-        <v>183</v>
-      </c>
-      <c r="E27" s="36" t="s">
-        <v>97</v>
+      <c r="E27" s="27" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Atualização automática da planilha (2026-09-17)
</commit_message>
<xml_diff>
--- a/times.xlsx
+++ b/times.xlsx
@@ -22,22 +22,16 @@
     <t>GUIA RÁPIDO</t>
   </si>
   <si>
+    <t>GUIA VISUAL DE HUNT: CARDS - ELEMENTOS</t>
+  </si>
+  <si>
     <t>RECOMENDAÇÃO DE TIME PARA HUNTS!</t>
   </si>
   <si>
-    <t>GUIA VISUAL DE HUNT: CARDS - ELEMENTOS</t>
-  </si>
-  <si>
-    <t>Requisitos de Entrada e Progressão 2x2x2.</t>
+    <t>Com algumas exceções, todos os restantes são SHINYS.</t>
   </si>
   <si>
     <t>https://www.twitch.tv/safnaww</t>
-  </si>
-  <si>
-    <t>Segue lá!</t>
-  </si>
-  <si>
-    <t>Com algumas exceções, todos os restantes são SHINYS.</t>
   </si>
   <si>
     <r>
@@ -61,588 +55,594 @@
     </r>
   </si>
   <si>
+    <t>Requisitos de Entrada e Progressão 2x2x2.</t>
+  </si>
+  <si>
+    <t>Segue lá!</t>
+  </si>
+  <si>
     <t>ELEMENTO / HUNT</t>
   </si>
   <si>
+    <t>ALVO (HUNT)</t>
+  </si>
+  <si>
+    <t>🛡️ LURAR (T1)</t>
+  </si>
+  <si>
+    <t>⚔️ DPS (SR)</t>
+  </si>
+  <si>
+    <t>🎨 TIPO SMEARGLE</t>
+  </si>
+  <si>
+    <t>Nessa planilha não indicaremos pokémons T2 ou T3 para a rotação.</t>
+  </si>
+  <si>
+    <t>Bug</t>
+  </si>
+  <si>
+    <t>★ BUG</t>
+  </si>
+  <si>
+    <t>Em breve</t>
+  </si>
+  <si>
+    <t>★ METAGROSS</t>
+  </si>
+  <si>
+    <t>Rapidash, Typhlosion, Magcargo</t>
+  </si>
+  <si>
     <t>📌 REQUISITOS INICIAIS (START DE ROTAÇÃO)</t>
   </si>
   <si>
-    <t>ALVO (HUNT)</t>
+    <t>Arcanine, Infernape, Armaldo</t>
+  </si>
+  <si>
+    <t>★ FAIRY</t>
+  </si>
+  <si>
+    <t>★ LUCARIO</t>
+  </si>
+  <si>
+    <t>Fire, Rock</t>
   </si>
   <si>
     <t>⚡ UPGRADE: ROTAÇÃO 2x2x2</t>
   </si>
   <si>
-    <t>🛡️ LURAR (T1)</t>
-  </si>
-  <si>
-    <t>⚔️ DPS (SR)</t>
-  </si>
-  <si>
-    <t>🎨 TIPO SMEARGLE</t>
-  </si>
-  <si>
-    <t>Bug</t>
+    <t>★ GENGAR</t>
+  </si>
+  <si>
+    <t>★ FIRE</t>
+  </si>
+  <si>
+    <t>Fairy</t>
   </si>
   <si>
     <t>Nível &amp; Held:</t>
   </si>
   <si>
+    <t>Shiny Sylveon (Lendário)</t>
+  </si>
+  <si>
+    <t>Hunt: Steel / Psychic</t>
+  </si>
+  <si>
+    <t>Hunt: Em breve</t>
+  </si>
+  <si>
+    <t>Muk, Tentacruel, Mawile</t>
+  </si>
+  <si>
+    <t>Aggron, Skarmory, Toxicroak</t>
+  </si>
+  <si>
     <t>Todos os Pokémon +15 com Atk 4</t>
   </si>
   <si>
-    <t>Em breve</t>
+    <t>Poison, Metal</t>
+  </si>
+  <si>
+    <t>Hunt: Fighting / Steel</t>
+  </si>
+  <si>
+    <t>Hunt: Shiny Sylveon (Lendário)</t>
+  </si>
+  <si>
+    <t>Fire</t>
+  </si>
+  <si>
+    <t>Magmar (Lendário) / Torkoal (UR)</t>
+  </si>
+  <si>
+    <t>Blastoise, Feraligatr, Omastar</t>
+  </si>
+  <si>
+    <t>Pupitar, Torterra, Kingdra</t>
+  </si>
+  <si>
+    <t>Rock, Water, Ground</t>
   </si>
   <si>
     <t>Todos os Pokémon +25 com Atk 5</t>
   </si>
   <si>
-    <t>★ METAGROSS</t>
+    <t>Fighting</t>
+  </si>
+  <si>
+    <t>Hunt: Magmar (Lendário) / Torkoal (UR)</t>
+  </si>
+  <si>
+    <t>Mega Clefable, Pidgeot, Espeon</t>
+  </si>
+  <si>
+    <t>Wobbuffet, Mimikyu, Gliscor</t>
   </si>
   <si>
     <t>Atalho / Dica:</t>
   </si>
   <si>
+    <t>Hunt: Ghost / Poison</t>
+  </si>
+  <si>
+    <t>Psychic, Flying, Fairy</t>
+  </si>
+  <si>
+    <t>Dark</t>
+  </si>
+  <si>
+    <t>Absol (Lendário) / Mightyena (UR)</t>
+  </si>
+  <si>
+    <t>Hitmontop, Hitmonchan, Poliwrath</t>
+  </si>
+  <si>
+    <t>Machamp, Scyther, Mimikyu</t>
+  </si>
+  <si>
+    <t>Fighting, Fairy, Bug</t>
+  </si>
+  <si>
+    <t>Water</t>
+  </si>
+  <si>
     <t>Runas de Atk no Pokelog ajudam a adiantar a meta</t>
   </si>
   <si>
-    <t>Rapidash, Typhlosion, Magcargo</t>
-  </si>
-  <si>
-    <t>Arcanine, Infernape, Armaldo</t>
+    <t>Milotic (UR)</t>
+  </si>
+  <si>
+    <t>Tangrowth, Ampharos, Venusaur</t>
+  </si>
+  <si>
+    <t>Tangrowth, Gogoat, Luxray</t>
+  </si>
+  <si>
+    <t>Grass, Electric</t>
+  </si>
+  <si>
+    <t>🛡️ LURAR / TANQUE (T1)</t>
+  </si>
+  <si>
+    <t>Grass</t>
   </si>
   <si>
     <t>Estrelas Mínimas:</t>
   </si>
   <si>
+    <t>Leafeon (Lendário) / Sceptile (UR)</t>
+  </si>
+  <si>
+    <t>Typhlosion, Rapidash, Pidgeot</t>
+  </si>
+  <si>
+    <t>Arcanine, Infernape, Scyther</t>
+  </si>
+  <si>
     <t>Tier 1: 2★ (estrelas)  |  SR: 1★ (estrela)</t>
   </si>
   <si>
+    <t>Poison, Bug, Fire, Fly, Ice</t>
+  </si>
+  <si>
     <t>Meta no Dummy:</t>
   </si>
   <si>
-    <t>Nessa planilha não indicaremos pokémons T2 ou T3 para a rotação.</t>
+    <t>Electric</t>
+  </si>
+  <si>
+    <t>Electabuzz (Lendário) / Manectric (UR)</t>
+  </si>
+  <si>
+    <t>Steelix, Nidoqueen, Torterra</t>
+  </si>
+  <si>
+    <t>Torterra, Pupitar, Smeargle</t>
+  </si>
+  <si>
+    <t>Ground</t>
+  </si>
+  <si>
+    <t>Ghost</t>
   </si>
   <si>
     <t>Bater 560k de dano com 3 Pokémon</t>
   </si>
   <si>
-    <t>★ BUG</t>
+    <t>⚔️ DPS / DANO (SR)</t>
+  </si>
+  <si>
+    <t>Umbreon, Crawdaunt, Dusknoir</t>
+  </si>
+  <si>
+    <t>Dusknoir, Houndoom, Hydreigon</t>
+  </si>
+  <si>
+    <t>Dark, Ghost</t>
+  </si>
+  <si>
+    <t>Ice</t>
+  </si>
+  <si>
+    <t>Glaceon (Lendário) / Glalie (UR)</t>
+  </si>
+  <si>
+    <t>Typhlosion, Rapidash, Hitmontop</t>
+  </si>
+  <si>
+    <t>Infernape, Machamp, Skarmory</t>
+  </si>
+  <si>
+    <t>Fighting, Fire, Metal</t>
   </si>
   <si>
     <t>Bater 560k de dano com apenas 2 Pokémon</t>
   </si>
   <si>
-    <t>Fire, Rock</t>
-  </si>
-  <si>
-    <t>★ LUCARIO</t>
-  </si>
-  <si>
-    <t>Fairy</t>
+    <t>Poison</t>
+  </si>
+  <si>
+    <t>Garbodor (Lendário) / Swalot (UR)</t>
+  </si>
+  <si>
+    <t>Steelix, Espeon, Nidoqueen</t>
+  </si>
+  <si>
+    <t>Wobbuffet, Mr. Mime, Pupitar</t>
+  </si>
+  <si>
+    <t>Ground, Psychic</t>
+  </si>
+  <si>
+    <t>Normal</t>
+  </si>
+  <si>
+    <t>Snorlax (Lendário) / Exploud (UR)</t>
   </si>
   <si>
     <t>Regra de Prey:</t>
   </si>
   <si>
-    <t>★ GENGAR</t>
+    <t>Poliwrath, Hitmontop, Medicham</t>
+  </si>
+  <si>
+    <t>Machamp, Kangaskhan, Smeargle</t>
   </si>
   <si>
     <t>Obrigatório Prey de Atk na hunt (já calculada no dummy)</t>
   </si>
   <si>
+    <t>⭐S.Rapidash, S.Typhlosion, S.Magcargo</t>
+  </si>
+  <si>
+    <t>Rock</t>
+  </si>
+  <si>
     <t>Manter sempre Prey de Atk ativa na hunt</t>
   </si>
   <si>
+    <t>Rampardos (UR)</t>
+  </si>
+  <si>
+    <t>Tangrowth, Steelix, Blastoise</t>
+  </si>
+  <si>
+    <t>Tangrowth, Machamp, Gogoat</t>
+  </si>
+  <si>
+    <t>Fighting, Ground, Water, Grass</t>
+  </si>
+  <si>
+    <t>Steel</t>
+  </si>
+  <si>
+    <t>⭐ S.Rapidash, S.Typhlosion, S.Steelix</t>
+  </si>
+  <si>
+    <t>Hitmontop, Rapidash, Typhlosion</t>
+  </si>
+  <si>
+    <t>Arcanine, Machamp, Infernape</t>
+  </si>
+  <si>
     <t>💡 POR QUE COMPOSIÇÕES COM 2 A 3 ELEMENTOS SÃO SUPERIORES? (ANTI-MONO)</t>
   </si>
   <si>
-    <t>Hunt: Steel / Psychic</t>
-  </si>
-  <si>
-    <t>★ FAIRY</t>
-  </si>
-  <si>
-    <t>Shiny Sylveon (Lendário)</t>
+    <t>Ground, Fighting, Fire</t>
+  </si>
+  <si>
+    <t>⭐ Arcanine, Infernape, Armaldo</t>
+  </si>
+  <si>
+    <t>Blastoise, Tangrowth, Gogoat</t>
+  </si>
+  <si>
+    <t>Tangrowth, Kingdra, Sharpedo</t>
+  </si>
+  <si>
+    <t>Water, Ice, Grass</t>
+  </si>
+  <si>
+    <t>Dragon</t>
+  </si>
+  <si>
+    <t>Salamence (UR) / Flygon (Lendário)</t>
+  </si>
+  <si>
+    <t>Lapras, Mega Clefable, Jynx</t>
+  </si>
+  <si>
+    <t>⭐ Arcanine, Houndoom, Pupitar</t>
+  </si>
+  <si>
+    <t>⭐ Muk, Tentacruel, Mawile</t>
+  </si>
+  <si>
+    <t>Mimikyu, Florges, Walrein</t>
+  </si>
+  <si>
+    <t>Dragon, Ice, Fairy</t>
+  </si>
+  <si>
+    <t>Psychic</t>
+  </si>
+  <si>
+    <t>Alakazam (Lendário)</t>
+  </si>
+  <si>
+    <t>⭐ Aggron, Skarmory, Toxicroak</t>
+  </si>
+  <si>
+    <t>Umbreon, Crawdaunt, Sableye</t>
+  </si>
+  <si>
+    <t>⭐ Hitmontop, Typhlosion, Rapidash</t>
   </si>
   <si>
     <t>⏱️ Cooldown Reduzido por Tier</t>
   </si>
   <si>
-    <t>Hunt: Fighting / Steel</t>
-  </si>
-  <si>
-    <t>Muk, Tentacruel, Mawile</t>
-  </si>
-  <si>
-    <t>Aggron, Skarmory, Toxicroak</t>
-  </si>
-  <si>
-    <t>Poison, Metal</t>
-  </si>
-  <si>
-    <t>★ FIRE</t>
-  </si>
-  <si>
-    <t>Hunt: Ghost / Poison</t>
-  </si>
-  <si>
-    <t>Fire</t>
-  </si>
-  <si>
-    <t>Magmar (Lendário) / Torkoal (UR)</t>
-  </si>
-  <si>
-    <t>Blastoise, Feraligatr, Omastar</t>
+    <t>⭐ Blastoise, Feraligatr, Omastar</t>
+  </si>
+  <si>
+    <t>Houndoom, Scyther, Dusknoir</t>
+  </si>
+  <si>
+    <t>⭐ Pupitar, Torterra, Kingdra</t>
+  </si>
+  <si>
+    <t>Ghost, Dark, Bug</t>
+  </si>
+  <si>
+    <t>⭐ Arcanine, Machamp, Pupitar</t>
+  </si>
+  <si>
+    <t>Flying</t>
+  </si>
+  <si>
+    <t>⭐ Umbreon, Crawdaunt, Sableye</t>
+  </si>
+  <si>
+    <t>Outras Opções T1:</t>
+  </si>
+  <si>
+    <t>Ampharos, Magcargo, Lapras</t>
+  </si>
+  <si>
+    <t>⭐ Houndoom, Hydreigon, Pupitar</t>
+  </si>
+  <si>
+    <t>Walrein, Luxray, Pachirisu</t>
+  </si>
+  <si>
+    <t>Electric, Ice, Rock</t>
+  </si>
+  <si>
+    <t>Metagross</t>
+  </si>
+  <si>
+    <t>Steel / Psychic</t>
+  </si>
+  <si>
+    <t>Rapidash, Typhlosion, Steelix</t>
+  </si>
+  <si>
+    <t>Arcanine, Houndoom, Pupitar</t>
+  </si>
+  <si>
+    <t>Outras Opções SR:</t>
+  </si>
+  <si>
+    <t>Fire, Ground, Ghost, Dark</t>
+  </si>
+  <si>
+    <t>Lucario</t>
+  </si>
+  <si>
+    <t>Fighting / Steel</t>
+  </si>
+  <si>
+    <t>Hitmontop, Typhlosion, Rapidash</t>
+  </si>
+  <si>
+    <t>Arcanine, Machamp, Pupitar</t>
   </si>
   <si>
     <t>No PKA, tiers mais altos não dão só dano: reduzem o cooldown das skills, deixando a rotação muito mais rápida.</t>
   </si>
   <si>
-    <t>Pupitar, Torterra, Kingdra</t>
-  </si>
-  <si>
-    <t>Rock, Water, Ground</t>
-  </si>
-  <si>
-    <t>Fighting</t>
-  </si>
-  <si>
-    <t>🛡️ LURAR / TANQUE (T1)</t>
-  </si>
-  <si>
-    <t>Mega Clefable, Pidgeot, Espeon</t>
-  </si>
-  <si>
-    <t>Wobbuffet, Mimikyu, Gliscor</t>
-  </si>
-  <si>
-    <t>Psychic, Flying, Fairy</t>
-  </si>
-  <si>
-    <t>Dark</t>
-  </si>
-  <si>
-    <t>Absol (Lendário) / Mightyena (UR)</t>
-  </si>
-  <si>
-    <t>Hitmontop, Hitmonchan, Poliwrath</t>
-  </si>
-  <si>
-    <t>Hunt: Em breve</t>
-  </si>
-  <si>
-    <t>Machamp, Scyther, Mimikyu</t>
-  </si>
-  <si>
-    <t>Fighting, Fairy, Bug</t>
-  </si>
-  <si>
-    <t>Water</t>
-  </si>
-  <si>
-    <t>Milotic (UR)</t>
-  </si>
-  <si>
-    <t>Tangrowth, Ampharos, Venusaur</t>
-  </si>
-  <si>
-    <t>Tangrowth, Gogoat, Luxray</t>
-  </si>
-  <si>
-    <t>Grass, Electric</t>
-  </si>
-  <si>
-    <t>Grass</t>
-  </si>
-  <si>
-    <t>Leafeon (Lendário) / Sceptile (UR)</t>
-  </si>
-  <si>
-    <t>Typhlosion, Rapidash, Pidgeot</t>
-  </si>
-  <si>
-    <t>Hunt: Shiny Sylveon (Lendário)</t>
-  </si>
-  <si>
-    <t>⚔️ DPS / DANO (SR)</t>
-  </si>
-  <si>
-    <t>Arcanine, Infernape, Scyther</t>
+    <t>Fighting, Fire, Ground</t>
+  </si>
+  <si>
+    <t>S.Charizard, Kabutops, Golem</t>
+  </si>
+  <si>
+    <t>Gengar</t>
+  </si>
+  <si>
+    <t>Ghost / Poison</t>
+  </si>
+  <si>
+    <t>Houndoom, Hydreigon, Pupitar</t>
+  </si>
+  <si>
+    <t>Umbreon</t>
+  </si>
+  <si>
+    <t>Dark, Ghost, Ground</t>
+  </si>
+  <si>
+    <t>Gardevoir</t>
+  </si>
+  <si>
+    <t>Psychic / Fairy</t>
+  </si>
+  <si>
+    <t>Mawile, Muk, Tentacruel</t>
+  </si>
+  <si>
+    <t>Toxicroak, Seviper, Misdreavus</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>Poison, Ghost, Metal</t>
+  </si>
+  <si>
+    <t>Gyarados</t>
+  </si>
+  <si>
+    <t>Water / Flying</t>
+  </si>
+  <si>
+    <t>Ampharos, Luxray, Jolteon</t>
+  </si>
+  <si>
+    <t>Luxray, Pachirisu, Smeargle Eletric</t>
+  </si>
+  <si>
+    <t>Torterra, Misdreavus</t>
+  </si>
+  <si>
+    <t>Metang, Magneton Estrelado</t>
+  </si>
+  <si>
+    <t>Poliwrath, Medicham, Hariyama</t>
+  </si>
+  <si>
+    <t>Infernape, Kangaskhan, Torterra</t>
+  </si>
+  <si>
+    <t>Cacturne, Banette, Dusclops</t>
+  </si>
+  <si>
+    <t>Misdreavus, Dusknoir, Torterra</t>
+  </si>
+  <si>
+    <t>SevIper</t>
   </si>
   <si>
     <t>📈 Mais Mobs e Brokes / Hora</t>
   </si>
   <si>
-    <t>Poison, Bug, Fire, Fly, Ice</t>
-  </si>
-  <si>
-    <t>Electric</t>
-  </si>
-  <si>
-    <t>Electabuzz (Lendário) / Manectric (UR)</t>
-  </si>
-  <si>
-    <t>Steelix, Nidoqueen, Torterra</t>
-  </si>
-  <si>
-    <t>Torterra, Pupitar, Smeargle</t>
-  </si>
-  <si>
-    <t>Ground</t>
-  </si>
-  <si>
-    <t>Ghost</t>
+    <t>Vaporeon, Rhyperior, Magcargo</t>
+  </si>
+  <si>
+    <t>Sharpedo</t>
+  </si>
+  <si>
+    <t>🎨 Smeargle: Fire, Ground, Ghost, Dark</t>
   </si>
   <si>
     <t>Rotação mais fluida = mais mobs derrotados/hora, aumentando drasticamente a chance de Shiny/hr e lucro.</t>
   </si>
   <si>
-    <t>Umbreon, Crawdaunt, Dusknoir</t>
-  </si>
-  <si>
-    <t>Dusknoir, Houndoom, Hydreigon</t>
-  </si>
-  <si>
-    <t>Hunt: Magmar (Lendário) / Torkoal (UR)</t>
-  </si>
-  <si>
-    <t>Dark, Ghost</t>
-  </si>
-  <si>
-    <t>Ice</t>
-  </si>
-  <si>
-    <t>Glaceon (Lendário) / Glalie (UR)</t>
-  </si>
-  <si>
-    <t>Typhlosion, Rapidash, Hitmontop</t>
-  </si>
-  <si>
-    <t>Infernape, Machamp, Skarmory</t>
-  </si>
-  <si>
-    <t>Fighting, Fire, Metal</t>
+    <t>🎨 Smeargle: Fighting, Fire, Ground</t>
   </si>
   <si>
     <t>⚔️ Hazards Mais Altos</t>
   </si>
   <si>
-    <t>Poison</t>
-  </si>
-  <si>
-    <t>Garbodor (Lendário) / Swalot (UR)</t>
-  </si>
-  <si>
-    <t>Steelix, Espeon, Nidoqueen</t>
-  </si>
-  <si>
-    <t>Wobbuffet, Mr. Mime, Pupitar</t>
-  </si>
-  <si>
-    <t>Ground, Psychic</t>
+    <t>🎨 Smeargle: Dark, Ghost, Ground</t>
   </si>
   <si>
     <t>Mesmo encurtando o número total de hunts, permite solar níveis de Hazard superiores com segurança e eficiência.</t>
   </si>
   <si>
-    <t>Normal</t>
-  </si>
-  <si>
-    <t>Snorlax (Lendário) / Exploud (UR)</t>
-  </si>
-  <si>
-    <t>Poliwrath, Hitmontop, Medicham</t>
-  </si>
-  <si>
-    <t>Machamp, Kangaskhan, Smeargle</t>
-  </si>
-  <si>
-    <t>⭐ S.Rapidash, S.Typhlosion, S.Steelix</t>
-  </si>
-  <si>
-    <t>Rock</t>
-  </si>
-  <si>
-    <t>Rampardos (UR)</t>
-  </si>
-  <si>
-    <t>Tangrowth, Steelix, Blastoise</t>
-  </si>
-  <si>
-    <t>Tangrowth, Machamp, Gogoat</t>
+    <t>★ GARDEVOIR</t>
   </si>
   <si>
     <t>🏆 Futuro &amp; Escalabilidade (Endgame)</t>
   </si>
   <si>
-    <t>Fighting, Ground, Water, Grass</t>
-  </si>
-  <si>
-    <t>Steel</t>
-  </si>
-  <si>
-    <t>Hitmontop, Rapidash, Typhlosion</t>
-  </si>
-  <si>
-    <t>Arcanine, Machamp, Infernape</t>
-  </si>
-  <si>
-    <t>Ground, Fighting, Fire</t>
-  </si>
-  <si>
-    <t>⭐ Arcanine, Houndoom, Pupitar</t>
+    <t>🎨 Smeargle: Fire, Rock</t>
   </si>
   <si>
     <t>Trabalhar com 2 ou 3 elementos abre um catálogo amplo de opções viáveis para evoluir: T1, SR, UR e Lendários.</t>
   </si>
   <si>
-    <t>Blastoise, Tangrowth, Gogoat</t>
-  </si>
-  <si>
-    <t>Tangrowth, Kingdra, Sharpedo</t>
-  </si>
-  <si>
-    <t>Water, Ice, Grass</t>
-  </si>
-  <si>
-    <t>Dragon</t>
-  </si>
-  <si>
-    <t>Salamence (UR) / Flygon (Lendário)</t>
-  </si>
-  <si>
-    <t>Lapras, Mega Clefable, Jynx</t>
-  </si>
-  <si>
-    <t>Mimikyu, Florges, Walrein</t>
-  </si>
-  <si>
-    <t>Dragon, Ice, Fairy</t>
-  </si>
-  <si>
-    <t>⭐S.Rapidash, S.Typhlosion, S.Magcargo</t>
-  </si>
-  <si>
-    <t>⭐ Hitmontop, Typhlosion, Rapidash</t>
-  </si>
-  <si>
-    <t>Psychic</t>
-  </si>
-  <si>
-    <t>Alakazam (Lendário)</t>
-  </si>
-  <si>
-    <t>Umbreon, Crawdaunt, Sableye</t>
-  </si>
-  <si>
-    <t>Houndoom, Scyther, Dusknoir</t>
-  </si>
-  <si>
-    <t>Ghost, Dark, Bug</t>
-  </si>
-  <si>
-    <t>⭐ Arcanine, Machamp, Pupitar</t>
-  </si>
-  <si>
-    <t>Flying</t>
-  </si>
-  <si>
-    <t>⭐ Arcanine, Infernape, Armaldo</t>
-  </si>
-  <si>
-    <t>⭐ Umbreon, Crawdaunt, Sableye</t>
-  </si>
-  <si>
-    <t>Ampharos, Magcargo, Lapras</t>
-  </si>
-  <si>
-    <t>Walrein, Luxray, Pachirisu</t>
-  </si>
-  <si>
-    <t>⭐ Houndoom, Hydreigon, Pupitar</t>
-  </si>
-  <si>
-    <t>Electric, Ice, Rock</t>
-  </si>
-  <si>
-    <t>Metagross</t>
-  </si>
-  <si>
-    <t>⭐ Muk, Tentacruel, Mawile</t>
-  </si>
-  <si>
-    <t>Steel / Psychic</t>
-  </si>
-  <si>
-    <t>Rapidash, Typhlosion, Steelix</t>
-  </si>
-  <si>
-    <t>Outras Opções T1:</t>
-  </si>
-  <si>
-    <t>Arcanine, Houndoom, Pupitar</t>
-  </si>
-  <si>
-    <t>⭐ Aggron, Skarmory, Toxicroak</t>
-  </si>
-  <si>
-    <t>Fire, Ground, Ghost, Dark</t>
-  </si>
-  <si>
-    <t>Lucario</t>
-  </si>
-  <si>
-    <t>⭐ Blastoise, Feraligatr, Omastar</t>
-  </si>
-  <si>
-    <t>Fighting / Steel</t>
-  </si>
-  <si>
-    <t>Hitmontop, Typhlosion, Rapidash</t>
-  </si>
-  <si>
-    <t>⭐ Pupitar, Torterra, Kingdra</t>
-  </si>
-  <si>
-    <t>Arcanine, Machamp, Pupitar</t>
-  </si>
-  <si>
-    <t>Fighting, Fire, Ground</t>
-  </si>
-  <si>
-    <t>Gengar</t>
-  </si>
-  <si>
-    <t>Ghost / Poison</t>
-  </si>
-  <si>
-    <t>Outras Opções SR:</t>
-  </si>
-  <si>
-    <t>Houndoom, Hydreigon, Pupitar</t>
-  </si>
-  <si>
-    <t>Dark, Ghost, Ground</t>
-  </si>
-  <si>
-    <t>Gardevoir</t>
-  </si>
-  <si>
-    <t>Psychic / Fairy</t>
-  </si>
-  <si>
-    <t>Mawile, Muk, Tentacruel</t>
-  </si>
-  <si>
-    <t>Toxicroak, Seviper, Misdreavus</t>
-  </si>
-  <si>
-    <t>Poison, Ghost, Metal</t>
-  </si>
-  <si>
-    <t>Gyarados</t>
-  </si>
-  <si>
-    <t>Umbreon</t>
-  </si>
-  <si>
-    <t>Water / Flying</t>
-  </si>
-  <si>
-    <t>Ampharos, Luxray, Jolteon</t>
-  </si>
-  <si>
-    <t>Luxray, Pachirisu, Smeargle Eletric</t>
-  </si>
-  <si>
-    <t>S.Charizard, Kabutops, Golem</t>
-  </si>
-  <si>
-    <t>Torterra, Misdreavus</t>
-  </si>
-  <si>
-    <t>Poliwrath, Medicham, Hariyama</t>
-  </si>
-  <si>
-    <t>Infernape, Kangaskhan, Torterra</t>
-  </si>
-  <si>
-    <t>Cacturne, Banette, Dusclops</t>
-  </si>
-  <si>
-    <t>Misdreavus, Dusknoir, Torterra</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Fire, Ground, Ghost, Dark</t>
-  </si>
-  <si>
-    <t>—</t>
-  </si>
-  <si>
-    <t>Metang, Magneton Estrelado</t>
-  </si>
-  <si>
-    <t>SevIper</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Fighting, Fire, Ground</t>
-  </si>
-  <si>
-    <t>Vaporeon, Rhyperior, Magcargo</t>
-  </si>
-  <si>
-    <t>Sharpedo</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Dark, Ghost, Ground</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Fire, Rock</t>
+    <t>★ GYARADOS</t>
   </si>
   <si>
     <t>🎨 Smeargle: Poison, Metal</t>
   </si>
   <si>
-    <t>★ GARDEVOIR</t>
-  </si>
-  <si>
     <t>🎨 Smeargle: Rock, Water, Ground</t>
   </si>
   <si>
-    <t>★ GYARADOS</t>
+    <t>★ SWAMPERT</t>
   </si>
   <si>
     <t>★ FIGHTING</t>
   </si>
   <si>
-    <t>★ SWAMPERT</t>
+    <t>Hunt: Psychic / Fairy</t>
+  </si>
+  <si>
+    <t>Hunt: Water / Flying</t>
   </si>
   <si>
     <t>★ DARK</t>
   </si>
   <si>
-    <t>Hunt: Psychic / Fairy</t>
-  </si>
-  <si>
-    <t>Hunt: Water / Flying</t>
+    <t>Hunt: Water / Ground</t>
   </si>
   <si>
     <t>★ WATER</t>
   </si>
   <si>
-    <t>Hunt: Water / Ground</t>
-  </si>
-  <si>
     <t>Hunt: Absol (Lendário) / Mightyena (UR)</t>
   </si>
   <si>
+    <t>Hunt: Milotic (UR)</t>
+  </si>
+  <si>
     <t>⭐ Mawile, Muk, Tentacruel</t>
   </si>
   <si>
-    <t>Hunt: Milotic (UR)</t>
-  </si>
-  <si>
     <t>⭐ Toxicroak, Seviper, Misdreavus</t>
   </si>
   <si>
@@ -652,82 +652,94 @@
     <t>⭐ S.Luxray, S.Pachirisu, Smeargle Eletric</t>
   </si>
   <si>
+    <t>⭐ Mega Clefable, Pidgeot, Espeon</t>
+  </si>
+  <si>
+    <t>⭐ Wobbuffet, Mimikyu, Gliscor</t>
+  </si>
+  <si>
     <t>⭐Venusaur, Gogoat, Tangrowth</t>
   </si>
   <si>
+    <t>⭐ Hitmontop, Hitmonchan, Poliwrath</t>
+  </si>
+  <si>
+    <t>⭐ Machamp, Scyther, Mimikyu</t>
+  </si>
+  <si>
     <t>⭐ S.Tangrowth,S. Gogoat, Smeargle Grass</t>
   </si>
   <si>
-    <t>⭐ Mega Clefable, Pidgeot, Espeon</t>
-  </si>
-  <si>
-    <t>⭐ Wobbuffet, Mimikyu, Gliscor</t>
-  </si>
-  <si>
-    <t>⭐ Hitmontop, Hitmonchan, Poliwrath</t>
+    <t>⭐ Tangrowth, Ampharos, Venusaur</t>
+  </si>
+  <si>
+    <t>⭐ Tangrowth, Gogoat, Luxray</t>
+  </si>
+  <si>
+    <t>Farfetch'd, Gliscor</t>
+  </si>
+  <si>
+    <t>Mr. Mime, Florges, Swellow</t>
+  </si>
+  <si>
+    <t>Mega Clefable, Hitmonlee</t>
+  </si>
+  <si>
+    <t>Florges, Kangaskhan, Pinsir</t>
+  </si>
+  <si>
+    <t>Luxray, Gogoat</t>
+  </si>
+  <si>
+    <t>Pachirisu</t>
   </si>
   <si>
     <t>Metang, Banette, Dusclops, Nidoking</t>
   </si>
   <si>
-    <t>⭐ Machamp, Scyther, Mimikyu</t>
-  </si>
-  <si>
     <t>Aggron, Skarmory</t>
   </si>
   <si>
-    <t>⭐ Tangrowth, Ampharos, Venusaur</t>
+    <t>🎨 Smeargle: Psychic, Flying, Fairy</t>
   </si>
   <si>
     <t>Raichu</t>
   </si>
   <si>
-    <t>⭐ Tangrowth, Gogoat, Luxray</t>
+    <t>🎨 Smeargle: Fighting, Fairy, Bug</t>
   </si>
   <si>
     <t>🎨 Smeargle: Poison, Ghost, Metal</t>
   </si>
   <si>
-    <t>Farfetch'd, Gliscor</t>
+    <t>🎨 Smeargle: Grass, Electric</t>
   </si>
   <si>
     <t>🎨 Smeargle: Electric</t>
   </si>
   <si>
-    <t>Mr. Mime, Florges, Swellow</t>
-  </si>
-  <si>
-    <t>Mega Clefable, Hitmonlee</t>
-  </si>
-  <si>
-    <t>Florges, Kangaskhan, Pinsir</t>
-  </si>
-  <si>
-    <t>Luxray, Gogoat</t>
-  </si>
-  <si>
-    <t>Pachirisu</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Psychic, Flying, Fairy</t>
+    <t>★ GRASS</t>
   </si>
   <si>
     <t>🎨 Smeargle: Grass</t>
   </si>
   <si>
-    <t>🎨 Smeargle: Fighting, Fairy, Bug</t>
+    <t>★ ELECTRIC</t>
   </si>
   <si>
     <t>★ SCIZOR</t>
   </si>
   <si>
-    <t>🎨 Smeargle: Grass, Electric</t>
+    <t>★ GHOST</t>
   </si>
   <si>
     <t>Hunt: Bug</t>
   </si>
   <si>
-    <t>★ GRASS</t>
+    <t>Hunt: Leafeon (Lendário) / Sceptile (UR)</t>
+  </si>
+  <si>
+    <t>Hunt: Electabuzz (Lendário) / Manectric (UR)</t>
   </si>
   <si>
     <t>⭐ S.Rapidash, S.Typhlosion, S.Zard</t>
@@ -737,18 +749,6 @@
   </si>
   <si>
     <t>🎨 Smeargle: Fire</t>
-  </si>
-  <si>
-    <t>★ ELECTRIC</t>
-  </si>
-  <si>
-    <t>★ GHOST</t>
-  </si>
-  <si>
-    <t>Hunt: Leafeon (Lendário) / Sceptile (UR)</t>
-  </si>
-  <si>
-    <t>Hunt: Electabuzz (Lendário) / Manectric (UR)</t>
   </si>
   <si>
     <t>⭐ Typhlosion, Rapidash, Pidgeot</t>
@@ -983,21 +983,21 @@
     </font>
     <font>
       <b/>
+      <sz val="13.0"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
       <sz val="14.0"/>
       <color rgb="FFFFFFFF"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font/>
     <font>
-      <b/>
-      <sz val="13.0"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
       <i/>
       <sz val="9.0"/>
-      <color rgb="FF94A3B8"/>
+      <color rgb="FFD1D5DB"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1008,7 +1008,7 @@
     <font>
       <i/>
       <sz val="9.0"/>
-      <color rgb="FFD1D5DB"/>
+      <color rgb="FF94A3B8"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1025,13 +1025,14 @@
       <i/>
       <u/>
       <sz val="9.0"/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FFE5E7EB"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
-      <b/>
+      <i/>
+      <u/>
       <sz val="9.0"/>
-      <color rgb="FF334155"/>
+      <color rgb="FF0000FF"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1041,38 +1042,20 @@
       <name val="Quattrocento Sans"/>
     </font>
     <font>
-      <b/>
-      <sz val="9.0"/>
-      <color rgb="FF0F172A"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
       <sz val="9.0"/>
       <color rgb="FF475569"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
-      <i/>
-      <u/>
-      <sz val="9.0"/>
-      <color rgb="FFE5E7EB"/>
+      <b/>
+      <sz val="11.0"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
       <b/>
       <sz val="9.0"/>
       <color rgb="FF166534"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <sz val="9.0"/>
-      <color rgb="FF0F172A"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11.0"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1088,6 +1071,12 @@
       <name val="Quattrocento Sans"/>
     </font>
     <font>
+      <b/>
+      <sz val="9.0"/>
+      <color rgb="FF334155"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
       <i/>
       <sz val="9.0"/>
       <color rgb="FFF3F4F6"/>
@@ -1096,12 +1085,12 @@
     <font>
       <b/>
       <sz val="9.0"/>
-      <color rgb="FF1E3A8A"/>
+      <color rgb="FF0F172A"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
       <sz val="9.0"/>
-      <color rgb="FF1F2937"/>
+      <color rgb="FF0F172A"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1118,6 +1107,12 @@
     </font>
     <font>
       <b/>
+      <sz val="9.0"/>
+      <color rgb="FF1E3A8A"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
       <sz val="8.0"/>
       <color rgb="FF4B5563"/>
       <name val="Quattrocento Sans"/>
@@ -1128,15 +1123,20 @@
       <name val="Quattrocento Sans"/>
     </font>
     <font>
-      <b/>
-      <sz val="8.0"/>
-      <color rgb="FF1E3A8A"/>
+      <sz val="9.0"/>
+      <color rgb="FF1F2937"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
       <b/>
       <sz val="8.0"/>
       <color rgb="FF4A4A4A"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8.0"/>
+      <color rgb="FF1E3A8A"/>
       <name val="Quattrocento Sans"/>
     </font>
   </fonts>
@@ -1149,14 +1149,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0F172A"/>
-        <bgColor rgb="FF0F172A"/>
+        <fgColor rgb="FF1B2A4A"/>
+        <bgColor rgb="FF1B2A4A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1B2A4A"/>
-        <bgColor rgb="FF1B2A4A"/>
+        <fgColor rgb="FF0F172A"/>
+        <bgColor rgb="FF0F172A"/>
       </patternFill>
     </fill>
     <fill>
@@ -1173,8 +1173,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF1F5F9"/>
-        <bgColor rgb="FFF1F5F9"/>
+        <fgColor rgb="FF8DAA34"/>
+        <bgColor rgb="FF8DAA34"/>
       </patternFill>
     </fill>
     <fill>
@@ -1191,26 +1191,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFDCFCE7"/>
-        <bgColor rgb="FFDCFCE7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFEF2F2"/>
         <bgColor rgb="FFFEF2F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFEF3C7"/>
-        <bgColor rgb="FFFEF3C7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF8DAA34"/>
-        <bgColor rgb="FF8DAA34"/>
+        <fgColor rgb="FFE68D9C"/>
+        <bgColor rgb="FFE68D9C"/>
       </patternFill>
     </fill>
     <fill>
@@ -1221,8 +1209,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1E40AF"/>
-        <bgColor rgb="FF1E40AF"/>
+        <fgColor rgb="FFEA6C2D"/>
+        <bgColor rgb="FFEA6C2D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF1F5F9"/>
+        <bgColor rgb="FFF1F5F9"/>
       </patternFill>
     </fill>
     <fill>
@@ -1233,32 +1227,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE68D9C"/>
-        <bgColor rgb="FFE68D9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEFF6FF"/>
-        <bgColor rgb="FFEFF6FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEA6C2D"/>
-        <bgColor rgb="FFEA6C2D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF2E7D32"/>
         <bgColor rgb="FF2E7D32"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFDCFCE7"/>
+        <bgColor rgb="FFDCFCE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFC62828"/>
         <bgColor rgb="FFC62828"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF3C7"/>
+        <bgColor rgb="FFFEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -1271,6 +1259,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFEBEE"/>
         <bgColor rgb="FFFFEBEE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1E40AF"/>
+        <bgColor rgb="FF1E40AF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEFF6FF"/>
+        <bgColor rgb="FFEFF6FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -1414,20 +1414,6 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFCBD5E1"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCBD5E1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCBD5E1"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
         <color rgb="FFD1D5DB"/>
       </left>
       <top style="thin">
@@ -1446,6 +1432,20 @@
       </top>
       <bottom style="thin">
         <color rgb="FFD1D5DB"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCBD5E1"/>
       </bottom>
     </border>
     <border>
@@ -1489,196 +1489,196 @@
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0"/>
+    </xf>
     <xf borderId="4" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="4" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="6" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf borderId="1" fillId="5" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="4" fillId="5" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="5" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="5" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="6" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="7" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="6" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="5" fillId="8" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="9" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="10" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="5" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="11" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="12" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="13" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="11" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="14" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="11" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="5" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="4" fillId="5" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="7" fillId="5" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="15" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="16" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="17" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="18" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="19" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="20" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="21" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="19" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="8" fillId="22" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="23" fontId="24" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="9" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="24" fontId="25" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="8" fillId="5" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="24" fontId="25" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="10" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="24" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="5" fillId="25" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="8" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="7" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="5" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="6" fillId="8" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="26" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="9" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="10" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="7" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="5" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="27" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="11" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="6" fillId="12" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="28" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="13" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="14" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="20" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="5" fillId="29" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="14" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="25" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="30" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="13" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="31" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="6" fillId="15" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="32" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="6" fillId="16" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="33" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="8" fillId="17" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="13" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="34" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="9" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="6" fillId="18" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="35" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="8" fillId="5" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="19" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="10" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="20" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="21" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="22" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="21" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="23" fontId="25" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="4" fillId="24" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="24" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="6" fillId="25" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="36" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="24" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="6" fillId="26" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="37" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="6" fillId="8" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="6" fillId="27" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="38" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="6" fillId="28" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="39" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="6" fillId="15" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="22" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="6" fillId="25" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="6" fillId="29" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="6" fillId="30" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="6" fillId="31" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="6" fillId="32" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="6" fillId="33" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="6" fillId="34" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="6" fillId="35" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="6" fillId="36" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="6" fillId="37" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="6" fillId="38" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="6" fillId="39" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="6" fillId="40" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="40" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1920,7 +1920,7 @@
   </cols>
   <sheetData>
     <row r="2" ht="33.75" customHeight="1">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="8" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="3"/>
@@ -1929,8 +1929,8 @@
       <c r="F2" s="4"/>
     </row>
     <row r="3" ht="19.5" customHeight="1">
-      <c r="B3" s="6" t="s">
-        <v>4</v>
+      <c r="B3" s="9" t="s">
+        <v>7</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -1938,88 +1938,88 @@
       <c r="F3" s="4"/>
     </row>
     <row r="4">
-      <c r="B4" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="11" t="s">
+      <c r="B4" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="10" t="s">
-        <v>6</v>
+      <c r="F4" s="7" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="5" ht="24.0" customHeight="1">
-      <c r="B5" s="13" t="s">
-        <v>10</v>
+      <c r="B5" s="23" t="s">
+        <v>20</v>
       </c>
       <c r="C5" s="4"/>
-      <c r="E5" s="13" t="s">
-        <v>12</v>
+      <c r="E5" s="23" t="s">
+        <v>25</v>
       </c>
       <c r="F5" s="4"/>
     </row>
     <row r="6" ht="24.75" customHeight="1">
-      <c r="B6" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="F6" s="18" t="s">
-        <v>20</v>
+      <c r="B6" s="28" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="32" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" s="28" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="32" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="7" ht="24.75" customHeight="1">
-      <c r="B7" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="C7" s="22" t="s">
-        <v>23</v>
-      </c>
-      <c r="E7" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="F7" s="22" t="s">
-        <v>27</v>
+      <c r="B7" s="28" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="33" t="s">
+        <v>58</v>
+      </c>
+      <c r="E7" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="F7" s="33" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="8" ht="24.75" customHeight="1">
-      <c r="B8" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="F8" s="28" t="s">
-        <v>32</v>
+      <c r="B8" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="C8" s="35" t="s">
+        <v>78</v>
+      </c>
+      <c r="E8" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="F8" s="37" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="9" ht="24.75" customHeight="1">
-      <c r="B9" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="C9" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="E9" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="F9" s="22" t="s">
-        <v>39</v>
+      <c r="B9" s="28" t="s">
+        <v>96</v>
+      </c>
+      <c r="C9" s="33" t="s">
+        <v>99</v>
+      </c>
+      <c r="E9" s="28" t="s">
+        <v>96</v>
+      </c>
+      <c r="F9" s="33" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="11" ht="24.0" customHeight="1">
-      <c r="B11" s="31" t="s">
-        <v>40</v>
+      <c r="B11" s="40" t="s">
+        <v>111</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
@@ -2027,48 +2027,48 @@
       <c r="F11" s="4"/>
     </row>
     <row r="12" ht="24.0" customHeight="1">
-      <c r="B12" s="35" t="s">
-        <v>44</v>
-      </c>
-      <c r="C12" s="37"/>
-      <c r="D12" s="39" t="s">
-        <v>54</v>
-      </c>
-      <c r="E12" s="41"/>
-      <c r="F12" s="37"/>
+      <c r="B12" s="42" t="s">
+        <v>129</v>
+      </c>
+      <c r="C12" s="44"/>
+      <c r="D12" s="46" t="s">
+        <v>152</v>
+      </c>
+      <c r="E12" s="48"/>
+      <c r="F12" s="44"/>
     </row>
     <row r="13" ht="24.0" customHeight="1">
-      <c r="B13" s="35" t="s">
-        <v>79</v>
-      </c>
-      <c r="C13" s="37"/>
-      <c r="D13" s="39" t="s">
-        <v>87</v>
-      </c>
-      <c r="E13" s="41"/>
-      <c r="F13" s="37"/>
+      <c r="B13" s="42" t="s">
+        <v>177</v>
+      </c>
+      <c r="C13" s="44"/>
+      <c r="D13" s="46" t="s">
+        <v>181</v>
+      </c>
+      <c r="E13" s="48"/>
+      <c r="F13" s="44"/>
     </row>
     <row r="14" ht="24.0" customHeight="1">
-      <c r="B14" s="35" t="s">
-        <v>97</v>
-      </c>
-      <c r="C14" s="37"/>
-      <c r="D14" s="39" t="s">
-        <v>103</v>
-      </c>
-      <c r="E14" s="41"/>
-      <c r="F14" s="37"/>
+      <c r="B14" s="42" t="s">
+        <v>183</v>
+      </c>
+      <c r="C14" s="44"/>
+      <c r="D14" s="46" t="s">
+        <v>185</v>
+      </c>
+      <c r="E14" s="48"/>
+      <c r="F14" s="44"/>
     </row>
     <row r="15" ht="24.0" customHeight="1">
-      <c r="B15" s="35" t="s">
-        <v>113</v>
-      </c>
-      <c r="C15" s="37"/>
-      <c r="D15" s="39" t="s">
-        <v>120</v>
-      </c>
-      <c r="E15" s="41"/>
-      <c r="F15" s="37"/>
+      <c r="B15" s="42" t="s">
+        <v>187</v>
+      </c>
+      <c r="C15" s="44"/>
+      <c r="D15" s="46" t="s">
+        <v>189</v>
+      </c>
+      <c r="E15" s="48"/>
+      <c r="F15" s="44"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -3094,8 +3094,8 @@
   </cols>
   <sheetData>
     <row r="1" ht="31.5" customHeight="1">
-      <c r="A1" s="7" t="s">
-        <v>3</v>
+      <c r="A1" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -3104,13 +3104,13 @@
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
       <c r="H1" s="4"/>
-      <c r="I1" s="10" t="s">
-        <v>7</v>
+      <c r="I1" s="7" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="2" ht="19.5" customHeight="1">
-      <c r="A2" s="20" t="s">
-        <v>8</v>
+      <c r="A2" s="14" t="s">
+        <v>6</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -3119,343 +3119,343 @@
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
       <c r="H2" s="4"/>
-      <c r="I2" s="10" t="s">
-        <v>29</v>
+      <c r="I2" s="7" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="4" ht="21.75" customHeight="1">
-      <c r="A4" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="B4" s="26"/>
-      <c r="D4" s="34" t="s">
-        <v>42</v>
-      </c>
-      <c r="E4" s="26"/>
-      <c r="G4" s="38" t="s">
-        <v>49</v>
-      </c>
-      <c r="H4" s="26"/>
+      <c r="A4" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="20"/>
+      <c r="D4" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="20"/>
+      <c r="G4" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" s="20"/>
     </row>
     <row r="5" ht="18.0" customHeight="1">
-      <c r="A5" s="33" t="s">
-        <v>65</v>
-      </c>
-      <c r="B5" s="26"/>
-      <c r="D5" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="E5" s="26"/>
-      <c r="G5" s="33" t="s">
-        <v>90</v>
-      </c>
-      <c r="H5" s="26"/>
+      <c r="A5" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="20"/>
+      <c r="D5" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" s="20"/>
+      <c r="G5" s="30" t="s">
+        <v>46</v>
+      </c>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="B6" s="42" t="s">
-        <v>77</v>
-      </c>
-      <c r="D6" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="E6" s="42" t="s">
-        <v>77</v>
-      </c>
-      <c r="G6" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="H6" s="42" t="s">
-        <v>77</v>
+      <c r="A6" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="D6" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="E6" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="G6" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="H6" s="36" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="7" ht="42.0" customHeight="1">
-      <c r="A7" s="43" t="s">
-        <v>129</v>
-      </c>
-      <c r="B7" s="44" t="s">
-        <v>138</v>
-      </c>
-      <c r="D7" s="45" t="s">
-        <v>145</v>
-      </c>
-      <c r="E7" s="44" t="s">
-        <v>150</v>
-      </c>
-      <c r="G7" s="45" t="s">
-        <v>153</v>
-      </c>
-      <c r="H7" s="44" t="s">
-        <v>156</v>
+      <c r="A7" s="38" t="s">
+        <v>100</v>
+      </c>
+      <c r="B7" s="39" t="s">
+        <v>113</v>
+      </c>
+      <c r="D7" s="41" t="s">
+        <v>121</v>
+      </c>
+      <c r="E7" s="39" t="s">
+        <v>126</v>
+      </c>
+      <c r="G7" s="41" t="s">
+        <v>130</v>
+      </c>
+      <c r="H7" s="39" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="B8" s="46" t="s">
-        <v>161</v>
-      </c>
-      <c r="D8" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="E8" s="46" t="s">
-        <v>161</v>
-      </c>
-      <c r="G8" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="H8" s="46" t="s">
-        <v>161</v>
+      <c r="A8" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="B8" s="43" t="s">
+        <v>146</v>
+      </c>
+      <c r="D8" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="E8" s="43" t="s">
+        <v>146</v>
+      </c>
+      <c r="G8" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="H8" s="43" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="9" ht="27.75" customHeight="1">
-      <c r="A9" s="48" t="s">
-        <v>174</v>
+      <c r="A9" s="45" t="s">
+        <v>154</v>
       </c>
       <c r="B9" s="47" t="s">
-        <v>181</v>
+        <v>164</v>
       </c>
       <c r="D9" s="47" t="s">
-        <v>182</v>
-      </c>
-      <c r="E9" s="50" t="s">
-        <v>183</v>
+        <v>171</v>
+      </c>
+      <c r="E9" s="49" t="s">
+        <v>176</v>
       </c>
       <c r="G9" s="47" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="H9" s="47" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
     </row>
     <row r="10" ht="18.0" customHeight="1">
-      <c r="A10" s="49" t="s">
+      <c r="A10" s="50" t="s">
         <v>188</v>
       </c>
-      <c r="B10" s="26"/>
-      <c r="D10" s="49" t="s">
-        <v>189</v>
-      </c>
-      <c r="E10" s="26"/>
-      <c r="G10" s="49" t="s">
+      <c r="B10" s="20"/>
+      <c r="D10" s="50" t="s">
         <v>191</v>
       </c>
-      <c r="H10" s="26"/>
+      <c r="E10" s="20"/>
+      <c r="G10" s="50" t="s">
+        <v>192</v>
+      </c>
+      <c r="H10" s="20"/>
     </row>
     <row r="14" ht="21.75" customHeight="1">
-      <c r="A14" s="51" t="s">
-        <v>193</v>
-      </c>
-      <c r="B14" s="26"/>
+      <c r="A14" s="52" t="s">
+        <v>194</v>
+      </c>
+      <c r="B14" s="20"/>
       <c r="D14" s="53" t="s">
-        <v>195</v>
-      </c>
-      <c r="E14" s="26"/>
+        <v>197</v>
+      </c>
+      <c r="E14" s="20"/>
       <c r="G14" s="54" t="s">
-        <v>198</v>
-      </c>
-      <c r="H14" s="26"/>
+        <v>199</v>
+      </c>
+      <c r="H14" s="20"/>
     </row>
     <row r="15" ht="18.0" customHeight="1">
-      <c r="A15" s="33" t="s">
-        <v>65</v>
-      </c>
-      <c r="B15" s="26"/>
-      <c r="D15" s="33" t="s">
+      <c r="A15" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="20"/>
+      <c r="D15" s="30" t="s">
         <v>200</v>
       </c>
-      <c r="E15" s="26"/>
-      <c r="G15" s="33" t="s">
-        <v>202</v>
-      </c>
-      <c r="H15" s="26"/>
+      <c r="E15" s="20"/>
+      <c r="G15" s="30" t="s">
+        <v>201</v>
+      </c>
+      <c r="H15" s="20"/>
     </row>
     <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="B16" s="42" t="s">
-        <v>77</v>
-      </c>
-      <c r="D16" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="E16" s="42" t="s">
-        <v>77</v>
-      </c>
-      <c r="G16" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="H16" s="42" t="s">
-        <v>77</v>
+      <c r="A16" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="B16" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="D16" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="E16" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="G16" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="H16" s="36" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="17" ht="42.0" customHeight="1">
-      <c r="A17" s="45" t="s">
-        <v>208</v>
-      </c>
-      <c r="B17" s="44" t="s">
+      <c r="A17" s="41" t="s">
+        <v>206</v>
+      </c>
+      <c r="B17" s="39" t="s">
+        <v>207</v>
+      </c>
+      <c r="D17" s="41" t="s">
         <v>209</v>
       </c>
-      <c r="D17" s="45" t="s">
+      <c r="E17" s="39" t="s">
         <v>210</v>
       </c>
-      <c r="E17" s="44" t="s">
+      <c r="G17" s="41" t="s">
         <v>212</v>
       </c>
-      <c r="G17" s="45" t="s">
-        <v>214</v>
-      </c>
-      <c r="H17" s="44" t="s">
-        <v>216</v>
+      <c r="H17" s="39" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="18" ht="15.0" customHeight="1">
-      <c r="A18" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="B18" s="46" t="s">
-        <v>161</v>
-      </c>
-      <c r="D18" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="E18" s="46" t="s">
-        <v>161</v>
-      </c>
-      <c r="G18" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="H18" s="46" t="s">
-        <v>161</v>
+      <c r="A18" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="B18" s="43" t="s">
+        <v>146</v>
+      </c>
+      <c r="D18" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="E18" s="43" t="s">
+        <v>146</v>
+      </c>
+      <c r="G18" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="H18" s="43" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="19" ht="27.75" customHeight="1">
       <c r="A19" s="47" t="s">
+        <v>214</v>
+      </c>
+      <c r="B19" s="47" t="s">
+        <v>215</v>
+      </c>
+      <c r="D19" s="47" t="s">
+        <v>216</v>
+      </c>
+      <c r="E19" s="47" t="s">
+        <v>217</v>
+      </c>
+      <c r="G19" s="47" t="s">
         <v>218</v>
       </c>
-      <c r="B19" s="47" t="s">
-        <v>220</v>
-      </c>
-      <c r="D19" s="47" t="s">
-        <v>221</v>
-      </c>
-      <c r="E19" s="47" t="s">
+      <c r="H19" s="47" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="20" ht="18.0" customHeight="1">
+      <c r="A20" s="50" t="s">
         <v>222</v>
       </c>
-      <c r="G19" s="47" t="s">
-        <v>223</v>
-      </c>
-      <c r="H19" s="47" t="s">
+      <c r="B20" s="20"/>
+      <c r="D20" s="50" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="20" ht="18.0" customHeight="1">
-      <c r="A20" s="49" t="s">
-        <v>225</v>
-      </c>
-      <c r="B20" s="26"/>
-      <c r="D20" s="49" t="s">
-        <v>227</v>
-      </c>
-      <c r="E20" s="26"/>
-      <c r="G20" s="49" t="s">
-        <v>229</v>
-      </c>
-      <c r="H20" s="26"/>
+      <c r="E20" s="20"/>
+      <c r="G20" s="50" t="s">
+        <v>226</v>
+      </c>
+      <c r="H20" s="20"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
     <row r="23" ht="15.75" customHeight="1"/>
     <row r="24" ht="21.75" customHeight="1">
-      <c r="A24" s="58" t="s">
-        <v>231</v>
-      </c>
-      <c r="B24" s="26"/>
+      <c r="A24" s="57" t="s">
+        <v>228</v>
+      </c>
+      <c r="B24" s="20"/>
       <c r="D24" s="59" t="s">
+        <v>230</v>
+      </c>
+      <c r="E24" s="20"/>
+      <c r="G24" s="60" t="s">
+        <v>232</v>
+      </c>
+      <c r="H24" s="20"/>
+    </row>
+    <row r="25" ht="18.0" customHeight="1">
+      <c r="A25" s="30" t="s">
+        <v>234</v>
+      </c>
+      <c r="B25" s="20"/>
+      <c r="D25" s="30" t="s">
         <v>235</v>
       </c>
-      <c r="E24" s="26"/>
-      <c r="G24" s="60" t="s">
-        <v>236</v>
-      </c>
-      <c r="H24" s="26"/>
-    </row>
-    <row r="25" ht="18.0" customHeight="1">
-      <c r="A25" s="33" t="s">
-        <v>237</v>
-      </c>
-      <c r="B25" s="26"/>
-      <c r="D25" s="33" t="s">
-        <v>238</v>
-      </c>
-      <c r="E25" s="26"/>
-      <c r="G25" s="33" t="s">
-        <v>65</v>
-      </c>
-      <c r="H25" s="26"/>
+      <c r="E25" s="20"/>
+      <c r="G25" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="H25" s="20"/>
     </row>
     <row r="26" ht="19.5" customHeight="1">
-      <c r="A26" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="B26" s="42" t="s">
-        <v>77</v>
-      </c>
-      <c r="D26" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="E26" s="42" t="s">
-        <v>77</v>
-      </c>
-      <c r="G26" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="H26" s="42" t="s">
-        <v>77</v>
+      <c r="A26" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="B26" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="D26" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="E26" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="G26" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="H26" s="36" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="27" ht="42.0" customHeight="1">
-      <c r="A27" s="45" t="s">
+      <c r="A27" s="41" t="s">
         <v>239</v>
       </c>
-      <c r="B27" s="44" t="s">
+      <c r="B27" s="39" t="s">
         <v>240</v>
       </c>
-      <c r="D27" s="45" t="s">
+      <c r="D27" s="41" t="s">
         <v>241</v>
       </c>
-      <c r="E27" s="44" t="s">
+      <c r="E27" s="39" t="s">
         <v>242</v>
       </c>
-      <c r="G27" s="45" t="s">
+      <c r="G27" s="41" t="s">
         <v>243</v>
       </c>
-      <c r="H27" s="44" t="s">
+      <c r="H27" s="39" t="s">
         <v>244</v>
       </c>
     </row>
     <row r="28" ht="15.0" customHeight="1">
-      <c r="A28" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="B28" s="46" t="s">
-        <v>161</v>
-      </c>
-      <c r="D28" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="E28" s="46" t="s">
-        <v>161</v>
-      </c>
-      <c r="G28" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="H28" s="46" t="s">
-        <v>161</v>
+      <c r="A28" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="B28" s="43" t="s">
+        <v>146</v>
+      </c>
+      <c r="D28" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="E28" s="43" t="s">
+        <v>146</v>
+      </c>
+      <c r="G28" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="H28" s="43" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="29" ht="27.75" customHeight="1">
@@ -3479,18 +3479,18 @@
       </c>
     </row>
     <row r="30" ht="18.0" customHeight="1">
-      <c r="A30" s="49" t="s">
+      <c r="A30" s="50" t="s">
         <v>251</v>
       </c>
-      <c r="B30" s="26"/>
-      <c r="D30" s="49" t="s">
+      <c r="B30" s="20"/>
+      <c r="D30" s="50" t="s">
         <v>252</v>
       </c>
-      <c r="E30" s="26"/>
-      <c r="G30" s="49" t="s">
+      <c r="E30" s="20"/>
+      <c r="G30" s="50" t="s">
         <v>253</v>
       </c>
-      <c r="H30" s="26"/>
+      <c r="H30" s="20"/>
     </row>
     <row r="31" ht="15.75" customHeight="1"/>
     <row r="32" ht="15.75" customHeight="1"/>
@@ -3499,88 +3499,88 @@
       <c r="A34" s="61" t="s">
         <v>254</v>
       </c>
-      <c r="B34" s="26"/>
+      <c r="B34" s="20"/>
       <c r="D34" s="62" t="s">
         <v>255</v>
       </c>
-      <c r="E34" s="26"/>
+      <c r="E34" s="20"/>
       <c r="G34" s="63" t="s">
         <v>256</v>
       </c>
-      <c r="H34" s="26"/>
+      <c r="H34" s="20"/>
     </row>
     <row r="35" ht="18.0" customHeight="1">
-      <c r="A35" s="33" t="s">
+      <c r="A35" s="30" t="s">
         <v>257</v>
       </c>
-      <c r="B35" s="26"/>
-      <c r="D35" s="33" t="s">
+      <c r="B35" s="20"/>
+      <c r="D35" s="30" t="s">
         <v>258</v>
       </c>
-      <c r="E35" s="26"/>
+      <c r="E35" s="20"/>
       <c r="G35" s="55" t="s">
         <v>259</v>
       </c>
-      <c r="H35" s="26"/>
+      <c r="H35" s="20"/>
     </row>
     <row r="36" ht="19.5" customHeight="1">
-      <c r="A36" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="B36" s="42" t="s">
-        <v>77</v>
-      </c>
-      <c r="D36" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="E36" s="42" t="s">
-        <v>77</v>
-      </c>
-      <c r="G36" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="H36" s="42" t="s">
-        <v>77</v>
+      <c r="A36" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="B36" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="D36" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="E36" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="G36" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="H36" s="36" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="37" ht="42.0" customHeight="1">
-      <c r="A37" s="45" t="s">
+      <c r="A37" s="41" t="s">
         <v>260</v>
       </c>
-      <c r="B37" s="44" t="s">
+      <c r="B37" s="39" t="s">
         <v>261</v>
       </c>
-      <c r="D37" s="45" t="s">
+      <c r="D37" s="41" t="s">
         <v>262</v>
       </c>
-      <c r="E37" s="44" t="s">
+      <c r="E37" s="39" t="s">
         <v>263</v>
       </c>
-      <c r="G37" s="45" t="s">
+      <c r="G37" s="41" t="s">
         <v>264</v>
       </c>
-      <c r="H37" s="44" t="s">
+      <c r="H37" s="39" t="s">
         <v>265</v>
       </c>
     </row>
     <row r="38" ht="15.0" customHeight="1">
-      <c r="A38" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="B38" s="46" t="s">
-        <v>161</v>
-      </c>
-      <c r="D38" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="E38" s="46" t="s">
-        <v>161</v>
-      </c>
-      <c r="G38" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="H38" s="46" t="s">
-        <v>161</v>
+      <c r="A38" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="B38" s="43" t="s">
+        <v>146</v>
+      </c>
+      <c r="D38" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="E38" s="43" t="s">
+        <v>146</v>
+      </c>
+      <c r="G38" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="H38" s="43" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="39" ht="27.75" customHeight="1">
@@ -3600,22 +3600,22 @@
         <v>270</v>
       </c>
       <c r="H39" s="47" t="s">
-        <v>181</v>
+        <v>164</v>
       </c>
     </row>
     <row r="40" ht="18.0" customHeight="1">
-      <c r="A40" s="49" t="s">
+      <c r="A40" s="50" t="s">
         <v>271</v>
       </c>
-      <c r="B40" s="26"/>
-      <c r="D40" s="49" t="s">
+      <c r="B40" s="20"/>
+      <c r="D40" s="50" t="s">
         <v>272</v>
       </c>
-      <c r="E40" s="26"/>
-      <c r="G40" s="49" t="s">
+      <c r="E40" s="20"/>
+      <c r="G40" s="50" t="s">
         <v>273</v>
       </c>
-      <c r="H40" s="26"/>
+      <c r="H40" s="20"/>
     </row>
     <row r="41" ht="15.75" customHeight="1"/>
     <row r="42" ht="15.75" customHeight="1"/>
@@ -3624,88 +3624,88 @@
       <c r="A44" s="64" t="s">
         <v>274</v>
       </c>
-      <c r="B44" s="26"/>
+      <c r="B44" s="20"/>
       <c r="D44" s="65" t="s">
         <v>275</v>
       </c>
-      <c r="E44" s="26"/>
+      <c r="E44" s="20"/>
       <c r="G44" s="66" t="s">
         <v>276</v>
       </c>
-      <c r="H44" s="26"/>
+      <c r="H44" s="20"/>
     </row>
     <row r="45" ht="18.0" customHeight="1">
-      <c r="A45" s="33" t="s">
+      <c r="A45" s="30" t="s">
         <v>277</v>
       </c>
-      <c r="B45" s="26"/>
-      <c r="D45" s="33" t="s">
-        <v>65</v>
-      </c>
-      <c r="E45" s="26"/>
-      <c r="G45" s="33" t="s">
-        <v>65</v>
-      </c>
-      <c r="H45" s="26"/>
+      <c r="B45" s="20"/>
+      <c r="D45" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="E45" s="20"/>
+      <c r="G45" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="H45" s="20"/>
     </row>
     <row r="46" ht="19.5" customHeight="1">
-      <c r="A46" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="B46" s="42" t="s">
-        <v>77</v>
-      </c>
-      <c r="D46" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="E46" s="42" t="s">
-        <v>77</v>
-      </c>
-      <c r="G46" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="H46" s="42" t="s">
-        <v>77</v>
+      <c r="A46" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="B46" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="D46" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="E46" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="G46" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="H46" s="36" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="47" ht="42.0" customHeight="1">
-      <c r="A47" s="45" t="s">
+      <c r="A47" s="41" t="s">
         <v>278</v>
       </c>
-      <c r="B47" s="44" t="s">
+      <c r="B47" s="39" t="s">
         <v>279</v>
       </c>
-      <c r="D47" s="45" t="s">
+      <c r="D47" s="41" t="s">
         <v>280</v>
       </c>
-      <c r="E47" s="44" t="s">
+      <c r="E47" s="39" t="s">
         <v>281</v>
       </c>
-      <c r="G47" s="45" t="s">
+      <c r="G47" s="41" t="s">
         <v>282</v>
       </c>
-      <c r="H47" s="44" t="s">
+      <c r="H47" s="39" t="s">
         <v>283</v>
       </c>
     </row>
     <row r="48" ht="15.0" customHeight="1">
-      <c r="A48" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="B48" s="46" t="s">
-        <v>161</v>
-      </c>
-      <c r="D48" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="E48" s="46" t="s">
-        <v>161</v>
-      </c>
-      <c r="G48" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="H48" s="46" t="s">
-        <v>161</v>
+      <c r="A48" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="B48" s="43" t="s">
+        <v>146</v>
+      </c>
+      <c r="D48" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="E48" s="43" t="s">
+        <v>146</v>
+      </c>
+      <c r="G48" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="H48" s="43" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="49" ht="27.75" customHeight="1">
@@ -3729,18 +3729,18 @@
       </c>
     </row>
     <row r="50" ht="18.0" customHeight="1">
-      <c r="A50" s="49" t="s">
+      <c r="A50" s="50" t="s">
         <v>290</v>
       </c>
-      <c r="B50" s="26"/>
-      <c r="D50" s="49" t="s">
+      <c r="B50" s="20"/>
+      <c r="D50" s="50" t="s">
         <v>291</v>
       </c>
-      <c r="E50" s="26"/>
-      <c r="G50" s="49" t="s">
+      <c r="E50" s="20"/>
+      <c r="G50" s="50" t="s">
         <v>292</v>
       </c>
-      <c r="H50" s="26"/>
+      <c r="H50" s="20"/>
     </row>
     <row r="51" ht="15.75" customHeight="1"/>
     <row r="52" ht="15.75" customHeight="1"/>
@@ -3749,88 +3749,88 @@
       <c r="A54" s="67" t="s">
         <v>293</v>
       </c>
-      <c r="B54" s="26"/>
+      <c r="B54" s="20"/>
       <c r="D54" s="68" t="s">
         <v>294</v>
       </c>
-      <c r="E54" s="26"/>
+      <c r="E54" s="20"/>
       <c r="G54" s="69" t="s">
         <v>295</v>
       </c>
-      <c r="H54" s="26"/>
+      <c r="H54" s="20"/>
     </row>
     <row r="55" ht="18.0" customHeight="1">
-      <c r="A55" s="33" t="s">
+      <c r="A55" s="30" t="s">
         <v>296</v>
       </c>
-      <c r="B55" s="26"/>
-      <c r="D55" s="33" t="s">
+      <c r="B55" s="20"/>
+      <c r="D55" s="30" t="s">
         <v>297</v>
       </c>
-      <c r="E55" s="26"/>
-      <c r="G55" s="33" t="s">
-        <v>65</v>
-      </c>
-      <c r="H55" s="26"/>
+      <c r="E55" s="20"/>
+      <c r="G55" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="H55" s="20"/>
     </row>
     <row r="56" ht="19.5" customHeight="1">
-      <c r="A56" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="B56" s="42" t="s">
-        <v>77</v>
-      </c>
-      <c r="D56" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="E56" s="42" t="s">
-        <v>77</v>
-      </c>
-      <c r="G56" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="H56" s="42" t="s">
-        <v>77</v>
+      <c r="A56" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="B56" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="D56" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="E56" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="G56" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="H56" s="36" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="57" ht="42.0" customHeight="1">
-      <c r="A57" s="45" t="s">
+      <c r="A57" s="41" t="s">
         <v>298</v>
       </c>
-      <c r="B57" s="44" t="s">
+      <c r="B57" s="39" t="s">
         <v>299</v>
       </c>
-      <c r="D57" s="45" t="s">
-        <v>139</v>
-      </c>
-      <c r="E57" s="44" t="s">
+      <c r="D57" s="41" t="s">
+        <v>136</v>
+      </c>
+      <c r="E57" s="39" t="s">
         <v>300</v>
       </c>
-      <c r="G57" s="45" t="s">
+      <c r="G57" s="41" t="s">
         <v>301</v>
       </c>
-      <c r="H57" s="44" t="s">
+      <c r="H57" s="39" t="s">
         <v>302</v>
       </c>
     </row>
     <row r="58" ht="15.0" customHeight="1">
-      <c r="A58" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="B58" s="46" t="s">
-        <v>161</v>
-      </c>
-      <c r="D58" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="E58" s="46" t="s">
-        <v>161</v>
-      </c>
-      <c r="G58" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="H58" s="46" t="s">
-        <v>161</v>
+      <c r="A58" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="B58" s="43" t="s">
+        <v>146</v>
+      </c>
+      <c r="D58" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="E58" s="43" t="s">
+        <v>146</v>
+      </c>
+      <c r="G58" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="H58" s="43" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="59" ht="27.75" customHeight="1">
@@ -3854,18 +3854,18 @@
       </c>
     </row>
     <row r="60" ht="18.0" customHeight="1">
-      <c r="A60" s="49" t="s">
+      <c r="A60" s="50" t="s">
         <v>309</v>
       </c>
-      <c r="B60" s="26"/>
-      <c r="D60" s="49" t="s">
+      <c r="B60" s="20"/>
+      <c r="D60" s="50" t="s">
         <v>310</v>
       </c>
-      <c r="E60" s="26"/>
-      <c r="G60" s="49" t="s">
+      <c r="E60" s="20"/>
+      <c r="G60" s="50" t="s">
         <v>311</v>
       </c>
-      <c r="H60" s="26"/>
+      <c r="H60" s="20"/>
     </row>
     <row r="61" ht="15.75" customHeight="1"/>
     <row r="62" ht="15.75" customHeight="1"/>
@@ -4892,8 +4892,8 @@
   </cols>
   <sheetData>
     <row r="1" ht="31.5" customHeight="1">
-      <c r="A1" s="2" t="s">
-        <v>2</v>
+      <c r="A1" s="5" t="s">
+        <v>3</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -4916,301 +4916,301 @@
       <c r="H2" s="4"/>
     </row>
     <row r="4" ht="21.75" customHeight="1">
-      <c r="A4" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" s="26"/>
-      <c r="D4" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="E4" s="26"/>
-      <c r="G4" s="23" t="s">
+      <c r="A4" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="20"/>
+      <c r="D4" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="20"/>
+      <c r="G4" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" s="20"/>
+    </row>
+    <row r="5" ht="18.0" customHeight="1">
+      <c r="A5" s="30" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="20"/>
+      <c r="D5" s="30" t="s">
         <v>37</v>
       </c>
-      <c r="H4" s="26"/>
-    </row>
-    <row r="5" ht="18.0" customHeight="1">
-      <c r="A5" s="33" t="s">
-        <v>41</v>
-      </c>
-      <c r="B5" s="26"/>
-      <c r="D5" s="33" t="s">
-        <v>45</v>
-      </c>
-      <c r="E5" s="26"/>
-      <c r="G5" s="33" t="s">
+      <c r="E5" s="20"/>
+      <c r="G5" s="30" t="s">
         <v>50</v>
       </c>
-      <c r="H5" s="26"/>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="B6" s="42" t="s">
-        <v>77</v>
-      </c>
-      <c r="D6" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="E6" s="42" t="s">
-        <v>77</v>
-      </c>
-      <c r="G6" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="H6" s="42" t="s">
-        <v>77</v>
+      <c r="A6" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="D6" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="E6" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="G6" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="H6" s="36" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="7" ht="42.0" customHeight="1">
-      <c r="A7" s="43" t="s">
+      <c r="A7" s="38" t="s">
         <v>108</v>
       </c>
-      <c r="B7" s="44" t="s">
-        <v>119</v>
-      </c>
-      <c r="D7" s="45" t="s">
-        <v>130</v>
-      </c>
-      <c r="E7" s="44" t="s">
+      <c r="B7" s="39" t="s">
+        <v>120</v>
+      </c>
+      <c r="D7" s="41" t="s">
+        <v>128</v>
+      </c>
+      <c r="E7" s="39" t="s">
+        <v>134</v>
+      </c>
+      <c r="G7" s="41" t="s">
         <v>136</v>
       </c>
-      <c r="G7" s="45" t="s">
+      <c r="H7" s="39" t="s">
         <v>139</v>
       </c>
-      <c r="H7" s="44" t="s">
-        <v>142</v>
-      </c>
     </row>
     <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="B8" s="46" t="s">
-        <v>161</v>
-      </c>
-      <c r="D8" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="E8" s="46" t="s">
-        <v>161</v>
-      </c>
-      <c r="G8" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="H8" s="46" t="s">
-        <v>161</v>
+      <c r="A8" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="B8" s="43" t="s">
+        <v>146</v>
+      </c>
+      <c r="D8" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="E8" s="43" t="s">
+        <v>146</v>
+      </c>
+      <c r="G8" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="H8" s="43" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="9" ht="27.75" customHeight="1">
       <c r="A9" s="47" t="s">
+        <v>158</v>
+      </c>
+      <c r="B9" s="47" t="s">
         <v>170</v>
       </c>
-      <c r="B9" s="47" t="s">
+      <c r="D9" s="47" t="s">
+        <v>172</v>
+      </c>
+      <c r="E9" s="47" t="s">
+        <v>173</v>
+      </c>
+      <c r="G9" s="47" t="s">
+        <v>174</v>
+      </c>
+      <c r="H9" s="47" t="s">
         <v>175</v>
       </c>
-      <c r="D9" s="47" t="s">
-        <v>176</v>
-      </c>
-      <c r="E9" s="47" t="s">
-        <v>177</v>
-      </c>
-      <c r="G9" s="47" t="s">
-        <v>178</v>
-      </c>
-      <c r="H9" s="47" t="s">
-        <v>179</v>
-      </c>
     </row>
     <row r="10" ht="18.0" customHeight="1">
-      <c r="A10" s="49" t="s">
+      <c r="A10" s="50" t="s">
         <v>180</v>
       </c>
-      <c r="B10" s="26"/>
-      <c r="D10" s="49" t="s">
+      <c r="B10" s="20"/>
+      <c r="D10" s="50" t="s">
+        <v>182</v>
+      </c>
+      <c r="E10" s="20"/>
+      <c r="G10" s="50" t="s">
         <v>184</v>
       </c>
-      <c r="E10" s="26"/>
-      <c r="G10" s="49" t="s">
-        <v>187</v>
-      </c>
-      <c r="H10" s="26"/>
+      <c r="H10" s="20"/>
     </row>
     <row r="14" ht="21.75" customHeight="1">
-      <c r="A14" s="23" t="s">
+      <c r="A14" s="21" t="s">
+        <v>186</v>
+      </c>
+      <c r="B14" s="20"/>
+      <c r="D14" s="21" t="s">
         <v>190</v>
       </c>
-      <c r="B14" s="26"/>
-      <c r="D14" s="23" t="s">
-        <v>192</v>
-      </c>
-      <c r="E14" s="26"/>
-      <c r="G14" s="52" t="s">
-        <v>194</v>
-      </c>
-      <c r="H14" s="26"/>
+      <c r="E14" s="20"/>
+      <c r="G14" s="51" t="s">
+        <v>193</v>
+      </c>
+      <c r="H14" s="20"/>
     </row>
     <row r="15" ht="18.0" customHeight="1">
-      <c r="A15" s="33" t="s">
+      <c r="A15" s="30" t="s">
+        <v>195</v>
+      </c>
+      <c r="B15" s="20"/>
+      <c r="D15" s="30" t="s">
         <v>196</v>
       </c>
-      <c r="B15" s="26"/>
-      <c r="D15" s="33" t="s">
-        <v>197</v>
-      </c>
-      <c r="E15" s="26"/>
+      <c r="E15" s="20"/>
       <c r="G15" s="55" t="s">
-        <v>199</v>
-      </c>
-      <c r="H15" s="26"/>
+        <v>198</v>
+      </c>
+      <c r="H15" s="20"/>
     </row>
     <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="B16" s="42" t="s">
-        <v>77</v>
-      </c>
-      <c r="D16" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="E16" s="42" t="s">
-        <v>77</v>
-      </c>
-      <c r="G16" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="H16" s="42" t="s">
-        <v>77</v>
+      <c r="A16" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="B16" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="D16" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="E16" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="G16" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="H16" s="36" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="17" ht="42.0" customHeight="1">
-      <c r="A17" s="45" t="s">
-        <v>201</v>
-      </c>
-      <c r="B17" s="44" t="s">
+      <c r="A17" s="41" t="s">
+        <v>202</v>
+      </c>
+      <c r="B17" s="39" t="s">
         <v>203</v>
       </c>
-      <c r="D17" s="45" t="s">
+      <c r="D17" s="41" t="s">
         <v>204</v>
       </c>
       <c r="E17" s="56" t="s">
         <v>205</v>
       </c>
-      <c r="G17" s="43" t="s">
-        <v>206</v>
+      <c r="G17" s="38" t="s">
+        <v>208</v>
       </c>
       <c r="H17" s="56" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
     </row>
     <row r="18" ht="15.0" customHeight="1">
-      <c r="A18" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="B18" s="46" t="s">
-        <v>161</v>
-      </c>
-      <c r="D18" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="E18" s="46" t="s">
-        <v>161</v>
-      </c>
-      <c r="G18" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="H18" s="46" t="s">
-        <v>161</v>
+      <c r="A18" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="B18" s="43" t="s">
+        <v>146</v>
+      </c>
+      <c r="D18" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="E18" s="43" t="s">
+        <v>146</v>
+      </c>
+      <c r="G18" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="H18" s="43" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="19" ht="27.75" customHeight="1">
       <c r="A19" s="47" t="s">
-        <v>211</v>
+        <v>220</v>
       </c>
       <c r="B19" s="47" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="D19" s="47" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="E19" s="47" t="s">
-        <v>181</v>
+        <v>164</v>
       </c>
       <c r="G19" s="47" t="s">
-        <v>181</v>
+        <v>164</v>
       </c>
       <c r="H19" s="47" t="s">
-        <v>181</v>
+        <v>164</v>
       </c>
     </row>
     <row r="20" ht="18.0" customHeight="1">
-      <c r="A20" s="49" t="s">
-        <v>217</v>
-      </c>
-      <c r="B20" s="26"/>
-      <c r="D20" s="49" t="s">
-        <v>219</v>
-      </c>
-      <c r="E20" s="26"/>
-      <c r="G20" s="57" t="s">
-        <v>226</v>
-      </c>
-      <c r="H20" s="26"/>
+      <c r="A20" s="50" t="s">
+        <v>225</v>
+      </c>
+      <c r="B20" s="20"/>
+      <c r="D20" s="50" t="s">
+        <v>227</v>
+      </c>
+      <c r="E20" s="20"/>
+      <c r="G20" s="58" t="s">
+        <v>229</v>
+      </c>
+      <c r="H20" s="20"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
     <row r="23" ht="15.75" customHeight="1"/>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="52" t="s">
-        <v>228</v>
-      </c>
-      <c r="B24" s="26"/>
+      <c r="A24" s="51" t="s">
+        <v>231</v>
+      </c>
+      <c r="B24" s="20"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="55" t="s">
-        <v>230</v>
-      </c>
-      <c r="B25" s="26"/>
+        <v>233</v>
+      </c>
+      <c r="B25" s="20"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="B26" s="42" t="s">
-        <v>77</v>
+      <c r="A26" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="B26" s="36" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="27" ht="44.25" customHeight="1">
-      <c r="A27" s="43" t="s">
-        <v>232</v>
+      <c r="A27" s="38" t="s">
+        <v>236</v>
       </c>
       <c r="B27" s="56" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="46" t="s">
-        <v>148</v>
-      </c>
-      <c r="B28" s="46" t="s">
-        <v>161</v>
+      <c r="A28" s="43" t="s">
+        <v>137</v>
+      </c>
+      <c r="B28" s="43" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="29" ht="27.75" customHeight="1">
       <c r="A29" s="47" t="s">
-        <v>181</v>
+        <v>164</v>
       </c>
       <c r="B29" s="47" t="s">
-        <v>181</v>
+        <v>164</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="57" t="s">
-        <v>234</v>
-      </c>
-      <c r="B30" s="26"/>
+      <c r="A30" s="58" t="s">
+        <v>238</v>
+      </c>
+      <c r="B30" s="20"/>
     </row>
     <row r="31" ht="15.75" customHeight="1"/>
     <row r="32" ht="15.75" customHeight="1"/>
@@ -6234,7 +6234,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="27.75" customHeight="1">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="3"/>
@@ -6243,20 +6243,20 @@
       <c r="E1" s="4"/>
     </row>
     <row r="2" ht="18.0" customHeight="1">
-      <c r="A2" s="9"/>
+      <c r="A2" s="6"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="4"/>
     </row>
     <row r="3">
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="D3" s="10" t="s">
         <v>5</v>
       </c>
     </row>
@@ -6264,408 +6264,408 @@
       <c r="A4" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="D4" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="12" t="s">
+    </row>
+    <row r="5" ht="21.75" customHeight="1">
+      <c r="A5" s="16" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="5" ht="21.75" customHeight="1">
-      <c r="A5" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="21" t="s">
+      <c r="D5" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="E5" s="27" t="s">
+    </row>
+    <row r="6" ht="21.75" customHeight="1">
+      <c r="A6" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="29" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="19" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="6" ht="21.75" customHeight="1">
-      <c r="A6" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="B6" s="32" t="s">
+      <c r="D6" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="31" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" ht="21.75" customHeight="1">
+      <c r="A7" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="C6" s="21" t="s">
-        <v>46</v>
-      </c>
-      <c r="D6" s="25" t="s">
+    </row>
+    <row r="8" ht="21.75" customHeight="1">
+      <c r="A8" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="B8" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="E6" s="36" t="s">
+      <c r="D8" s="22" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="7" ht="21.75" customHeight="1">
-      <c r="A7" s="17" t="s">
+      <c r="E8" s="31" t="s">
         <v>51</v>
       </c>
-      <c r="B7" s="19" t="s">
+    </row>
+    <row r="9" ht="21.75" customHeight="1">
+      <c r="A9" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="B9" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="D7" s="25" t="s">
+      <c r="C9" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="E7" s="27" t="s">
+      <c r="E9" s="25" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="8" ht="21.75" customHeight="1">
-      <c r="A8" s="30" t="s">
+    <row r="10" ht="21.75" customHeight="1">
+      <c r="A10" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="B8" s="32" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="21" t="s">
+      <c r="B10" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="D8" s="25" t="s">
+      <c r="C10" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="E8" s="36" t="s">
+      <c r="D10" s="22" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="9" ht="21.75" customHeight="1">
-      <c r="A9" s="17" t="s">
+      <c r="E10" s="31" t="s">
         <v>62</v>
       </c>
-      <c r="B9" s="19" t="s">
-        <v>63</v>
-      </c>
-      <c r="C9" s="21" t="s">
+    </row>
+    <row r="11" ht="21.75" customHeight="1">
+      <c r="A11" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="D9" s="25" t="s">
+      <c r="B11" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="E9" s="27" t="s">
+      <c r="C11" s="19" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="10" ht="21.75" customHeight="1">
-      <c r="A10" s="30" t="s">
+      <c r="D11" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="B10" s="32" t="s">
-        <v>69</v>
-      </c>
-      <c r="C10" s="21" t="s">
+      <c r="E11" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="D10" s="25" t="s">
-        <v>71</v>
-      </c>
-      <c r="E10" s="36" t="s">
+    </row>
+    <row r="12" ht="21.75" customHeight="1">
+      <c r="A12" s="26" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="11" ht="21.75" customHeight="1">
-      <c r="A11" s="17" t="s">
+      <c r="B12" s="29" t="s">
         <v>73</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="C12" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="D12" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="D11" s="25" t="s">
-        <v>78</v>
-      </c>
-      <c r="E11" s="27" t="s">
+      <c r="E12" s="31" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="13" ht="21.75" customHeight="1">
+      <c r="A13" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="19" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="12" ht="21.75" customHeight="1">
-      <c r="A12" s="30" t="s">
+      <c r="D13" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="B12" s="32" t="s">
+      <c r="E13" s="25" t="s">
         <v>82</v>
       </c>
-      <c r="C12" s="21" t="s">
+    </row>
+    <row r="14" ht="21.75" customHeight="1">
+      <c r="A14" s="26" t="s">
         <v>83</v>
       </c>
-      <c r="D12" s="25" t="s">
+      <c r="B14" s="29" t="s">
         <v>84</v>
       </c>
-      <c r="E12" s="36" t="s">
+      <c r="C14" s="19" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="13" ht="21.75" customHeight="1">
-      <c r="A13" s="17" t="s">
+      <c r="D14" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="B13" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13" s="21" t="s">
-        <v>88</v>
-      </c>
-      <c r="D13" s="25" t="s">
+      <c r="E14" s="31" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" ht="21.75" customHeight="1">
+      <c r="A15" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="E13" s="27" t="s">
+      <c r="B15" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="C15" s="19" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="14" ht="21.75" customHeight="1">
-      <c r="A14" s="30" t="s">
+      <c r="D15" s="22" t="s">
         <v>92</v>
       </c>
-      <c r="B14" s="32" t="s">
+      <c r="E15" s="25" t="s">
         <v>93</v>
       </c>
-      <c r="C14" s="21" t="s">
+    </row>
+    <row r="16" ht="21.75" customHeight="1">
+      <c r="A16" s="26" t="s">
         <v>94</v>
       </c>
-      <c r="D14" s="25" t="s">
+      <c r="B16" s="29" t="s">
         <v>95</v>
       </c>
-      <c r="E14" s="36" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="15" ht="21.75" customHeight="1">
-      <c r="A15" s="17" t="s">
+      <c r="C16" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="D16" s="22" t="s">
         <v>98</v>
       </c>
-      <c r="B15" s="19" t="s">
-        <v>99</v>
-      </c>
-      <c r="C15" s="21" t="s">
-        <v>100</v>
-      </c>
-      <c r="D15" s="25" t="s">
+      <c r="E16" s="31" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="17" ht="21.75" customHeight="1">
+      <c r="A17" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="E15" s="27" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="16" ht="21.75" customHeight="1">
-      <c r="A16" s="30" t="s">
+      <c r="B17" s="17" t="s">
+        <v>103</v>
+      </c>
+      <c r="C17" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="B16" s="32" t="s">
+      <c r="D17" s="22" t="s">
         <v>105</v>
       </c>
-      <c r="C16" s="21" t="s">
+      <c r="E17" s="25" t="s">
         <v>106</v>
       </c>
-      <c r="D16" s="25" t="s">
+    </row>
+    <row r="18" ht="21.75" customHeight="1">
+      <c r="A18" s="26" t="s">
         <v>107</v>
       </c>
-      <c r="E16" s="36" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="17" ht="21.75" customHeight="1">
-      <c r="A17" s="17" t="s">
+      <c r="B18" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="D18" s="22" t="s">
         <v>110</v>
       </c>
-      <c r="C17" s="21" t="s">
-        <v>111</v>
-      </c>
-      <c r="D17" s="25" t="s">
+      <c r="E18" s="31" t="s">
         <v>112</v>
       </c>
-      <c r="E17" s="27" t="s">
+    </row>
+    <row r="19" ht="21.75" customHeight="1">
+      <c r="A19" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="B19" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" s="19" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="18" ht="21.75" customHeight="1">
-      <c r="A18" s="30" t="s">
+      <c r="D19" s="22" t="s">
         <v>115</v>
       </c>
-      <c r="B18" s="32" t="s">
-        <v>19</v>
-      </c>
-      <c r="C18" s="21" t="s">
+      <c r="E19" s="25" t="s">
         <v>116</v>
       </c>
-      <c r="D18" s="25" t="s">
+    </row>
+    <row r="20" ht="21.75" customHeight="1">
+      <c r="A20" s="26" t="s">
         <v>117</v>
       </c>
-      <c r="E18" s="36" t="s">
+      <c r="B20" s="29" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="19" ht="21.75" customHeight="1">
-      <c r="A19" s="17" t="s">
-        <v>85</v>
-      </c>
-      <c r="B19" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="C19" s="21" t="s">
-        <v>121</v>
-      </c>
-      <c r="D19" s="25" t="s">
+      <c r="C20" s="19" t="s">
+        <v>119</v>
+      </c>
+      <c r="D20" s="22" t="s">
         <v>122</v>
       </c>
-      <c r="E19" s="27" t="s">
+      <c r="E20" s="31" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="20" ht="21.75" customHeight="1">
-      <c r="A20" s="30" t="s">
+    <row r="21" ht="21.75" customHeight="1">
+      <c r="A21" s="16" t="s">
         <v>124</v>
       </c>
-      <c r="B20" s="32" t="s">
+      <c r="B21" s="17" t="s">
         <v>125</v>
       </c>
-      <c r="C20" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="D20" s="25" t="s">
+      <c r="C21" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="E20" s="36" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="21" ht="21.75" customHeight="1">
-      <c r="A21" s="17" t="s">
+      <c r="D21" s="22" t="s">
         <v>131</v>
       </c>
-      <c r="B21" s="19" t="s">
-        <v>132</v>
-      </c>
-      <c r="C21" s="21" t="s">
+      <c r="E21" s="25" t="s">
         <v>133</v>
       </c>
-      <c r="D21" s="25" t="s">
-        <v>134</v>
-      </c>
-      <c r="E21" s="27" t="s">
+    </row>
+    <row r="22" ht="21.75" customHeight="1">
+      <c r="A22" s="26" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="22" ht="21.75" customHeight="1">
-      <c r="A22" s="30" t="s">
-        <v>137</v>
-      </c>
-      <c r="B22" s="32" t="s">
-        <v>19</v>
-      </c>
-      <c r="C22" s="21" t="s">
+      <c r="B22" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" s="19" t="s">
+        <v>138</v>
+      </c>
+      <c r="D22" s="22" t="s">
         <v>140</v>
       </c>
-      <c r="D22" s="25" t="s">
+      <c r="E22" s="31" t="s">
         <v>141</v>
       </c>
-      <c r="E22" s="36" t="s">
+    </row>
+    <row r="23" ht="21.75" customHeight="1">
+      <c r="A23" s="16" t="s">
+        <v>142</v>
+      </c>
+      <c r="B23" s="17" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="23" ht="21.75" customHeight="1">
-      <c r="A23" s="17" t="s">
+      <c r="C23" s="19" t="s">
         <v>144</v>
       </c>
-      <c r="B23" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="C23" s="21" t="s">
+      <c r="D23" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="E23" s="25" t="s">
         <v>147</v>
       </c>
-      <c r="D23" s="25" t="s">
+    </row>
+    <row r="24" ht="21.75" customHeight="1">
+      <c r="A24" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="B24" s="29" t="s">
         <v>149</v>
       </c>
-      <c r="E23" s="27" t="s">
+      <c r="C24" s="19" t="s">
+        <v>150</v>
+      </c>
+      <c r="D24" s="22" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="24" ht="21.75" customHeight="1">
-      <c r="A24" s="30" t="s">
-        <v>152</v>
-      </c>
-      <c r="B24" s="32" t="s">
-        <v>154</v>
-      </c>
-      <c r="C24" s="21" t="s">
+      <c r="E24" s="31" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="25" ht="21.75" customHeight="1">
+      <c r="A25" s="16" t="s">
         <v>155</v>
       </c>
-      <c r="D24" s="25" t="s">
+      <c r="B25" s="17" t="s">
+        <v>156</v>
+      </c>
+      <c r="C25" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="D25" s="22" t="s">
         <v>157</v>
       </c>
-      <c r="E24" s="36" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="25" ht="21.75" customHeight="1">
-      <c r="A25" s="17" t="s">
+      <c r="E25" s="25" t="s">
         <v>159</v>
       </c>
-      <c r="B25" s="19" t="s">
+    </row>
+    <row r="26" ht="21.75" customHeight="1">
+      <c r="A26" s="26" t="s">
         <v>160</v>
       </c>
-      <c r="C25" s="21" t="s">
-        <v>133</v>
-      </c>
-      <c r="D25" s="25" t="s">
+      <c r="B26" s="29" t="s">
+        <v>161</v>
+      </c>
+      <c r="C26" s="19" t="s">
         <v>162</v>
       </c>
-      <c r="E25" s="27" t="s">
+      <c r="D26" s="22" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="26" ht="21.75" customHeight="1">
-      <c r="A26" s="30" t="s">
-        <v>164</v>
-      </c>
-      <c r="B26" s="32" t="s">
+      <c r="E26" s="31" t="s">
         <v>165</v>
       </c>
-      <c r="C26" s="21" t="s">
+    </row>
+    <row r="27" ht="21.75" customHeight="1">
+      <c r="A27" s="16" t="s">
         <v>166</v>
       </c>
-      <c r="D26" s="25" t="s">
+      <c r="B27" s="17" t="s">
         <v>167</v>
       </c>
-      <c r="E26" s="36" t="s">
+      <c r="C27" s="19" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="27" ht="21.75" customHeight="1">
-      <c r="A27" s="17" t="s">
+      <c r="D27" s="22" t="s">
         <v>169</v>
       </c>
-      <c r="B27" s="19" t="s">
-        <v>171</v>
-      </c>
-      <c r="C27" s="21" t="s">
-        <v>172</v>
-      </c>
-      <c r="D27" s="25" t="s">
-        <v>173</v>
-      </c>
-      <c r="E27" s="27" t="s">
-        <v>81</v>
+      <c r="E27" s="25" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Atualização automática da planilha (2026-09-18)
</commit_message>
<xml_diff>
--- a/times.xlsx
+++ b/times.xlsx
@@ -19,19 +19,25 @@
     <t>GUIA DE ROTAÇÃO &amp; METAGAME - POKEALLIANCE(PKA)</t>
   </si>
   <si>
+    <t>RECOMENDAÇÃO DE TIME PARA HUNTS!</t>
+  </si>
+  <si>
     <t>GUIA RÁPIDO</t>
   </si>
   <si>
     <t>GUIA VISUAL DE HUNT: CARDS - ELEMENTOS</t>
   </si>
   <si>
-    <t>RECOMENDAÇÃO DE TIME PARA HUNTS!</t>
+    <t>Requisitos de Entrada e Progressão 2x2x2.</t>
+  </si>
+  <si>
+    <t>Segue lá!</t>
+  </si>
+  <si>
+    <t>https://www.twitch.tv/safnaww</t>
   </si>
   <si>
     <t>Com algumas exceções, todos os restantes são SHINYS.</t>
-  </si>
-  <si>
-    <t>https://www.twitch.tv/safnaww</t>
   </si>
   <si>
     <r>
@@ -55,18 +61,84 @@
     </r>
   </si>
   <si>
-    <t>Requisitos de Entrada e Progressão 2x2x2.</t>
-  </si>
-  <si>
-    <t>Segue lá!</t>
+    <t>📌 REQUISITOS INICIAIS (START DE ROTAÇÃO)</t>
+  </si>
+  <si>
+    <t>⚡ UPGRADE: ROTAÇÃO 2x2x2</t>
+  </si>
+  <si>
+    <t>★ METAGROSS</t>
+  </si>
+  <si>
+    <t>Nível &amp; Held:</t>
+  </si>
+  <si>
+    <t>Todos os Pokémon +15 com Atk 4</t>
+  </si>
+  <si>
+    <t>Nessa planilha não indicaremos pokémons T2 ou T3 para a rotação.</t>
+  </si>
+  <si>
+    <t>Todos os Pokémon +25 com Atk 5</t>
+  </si>
+  <si>
+    <t>★ LUCARIO</t>
+  </si>
+  <si>
+    <t>Atalho / Dica:</t>
+  </si>
+  <si>
+    <t>Runas de Atk no Pokelog ajudam a adiantar a meta</t>
+  </si>
+  <si>
+    <t>★ GENGAR</t>
+  </si>
+  <si>
+    <t>★ BUG</t>
+  </si>
+  <si>
+    <t>Estrelas Mínimas:</t>
+  </si>
+  <si>
+    <t>Tier 1: 2★ (estrelas)  |  SR: 1★ (estrela)</t>
+  </si>
+  <si>
+    <t>Meta no Dummy:</t>
+  </si>
+  <si>
+    <t>Bater 560k de dano com 3 Pokémon</t>
+  </si>
+  <si>
+    <t>Hunt: Steel / Psychic</t>
   </si>
   <si>
     <t>ELEMENTO / HUNT</t>
   </si>
   <si>
+    <t>★ FAIRY</t>
+  </si>
+  <si>
+    <t>Bater 560k de dano com apenas 2 Pokémon</t>
+  </si>
+  <si>
     <t>ALVO (HUNT)</t>
   </si>
   <si>
+    <t>Regra de Prey:</t>
+  </si>
+  <si>
+    <t>Obrigatório Prey de Atk na hunt (já calculada no dummy)</t>
+  </si>
+  <si>
+    <t>Manter sempre Prey de Atk ativa na hunt</t>
+  </si>
+  <si>
+    <t>Hunt: Fighting / Steel</t>
+  </si>
+  <si>
+    <t>💡 POR QUE COMPOSIÇÕES COM 2 A 3 ELEMENTOS SÃO SUPERIORES? (ANTI-MONO)</t>
+  </si>
+  <si>
     <t>🛡️ LURAR (T1)</t>
   </si>
   <si>
@@ -76,61 +148,61 @@
     <t>🎨 TIPO SMEARGLE</t>
   </si>
   <si>
-    <t>Nessa planilha não indicaremos pokémons T2 ou T3 para a rotação.</t>
+    <t>Hunt: Ghost / Poison</t>
   </si>
   <si>
     <t>Bug</t>
   </si>
   <si>
-    <t>★ BUG</t>
+    <t>★ FIRE</t>
   </si>
   <si>
     <t>Em breve</t>
   </si>
   <si>
-    <t>★ METAGROSS</t>
-  </si>
-  <si>
     <t>Rapidash, Typhlosion, Magcargo</t>
   </si>
   <si>
-    <t>📌 REQUISITOS INICIAIS (START DE ROTAÇÃO)</t>
+    <t>⏱️ Cooldown Reduzido por Tier</t>
+  </si>
+  <si>
+    <t>Hunt: Em breve</t>
   </si>
   <si>
     <t>Arcanine, Infernape, Armaldo</t>
   </si>
   <si>
-    <t>★ FAIRY</t>
-  </si>
-  <si>
-    <t>★ LUCARIO</t>
+    <t>🛡️ LURAR / TANQUE (T1)</t>
+  </si>
+  <si>
+    <t>Hunt: Shiny Sylveon (Lendário)</t>
   </si>
   <si>
     <t>Fire, Rock</t>
   </si>
   <si>
-    <t>⚡ UPGRADE: ROTAÇÃO 2x2x2</t>
-  </si>
-  <si>
-    <t>★ GENGAR</t>
-  </si>
-  <si>
-    <t>★ FIRE</t>
+    <t>No PKA, tiers mais altos não dão só dano: reduzem o cooldown das skills, deixando a rotação muito mais rápida.</t>
+  </si>
+  <si>
+    <t>Hunt: Magmar (Lendário) / Torkoal (UR)</t>
+  </si>
+  <si>
+    <t>⚔️ DPS / DANO (SR)</t>
   </si>
   <si>
     <t>Fairy</t>
   </si>
   <si>
-    <t>Nível &amp; Held:</t>
+    <t>📈 Mais Mobs e Brokes / Hora</t>
   </si>
   <si>
     <t>Shiny Sylveon (Lendário)</t>
   </si>
   <si>
-    <t>Hunt: Steel / Psychic</t>
-  </si>
-  <si>
-    <t>Hunt: Em breve</t>
+    <t>⭐ S.Rapidash, S.Typhlosion, S.Steelix</t>
+  </si>
+  <si>
+    <t>Rotação mais fluida = mais mobs derrotados/hora, aumentando drasticamente a chance de Shiny/hr e lucro.</t>
   </si>
   <si>
     <t>Muk, Tentacruel, Mawile</t>
@@ -139,16 +211,19 @@
     <t>Aggron, Skarmory, Toxicroak</t>
   </si>
   <si>
-    <t>Todos os Pokémon +15 com Atk 4</t>
-  </si>
-  <si>
     <t>Poison, Metal</t>
   </si>
   <si>
-    <t>Hunt: Fighting / Steel</t>
-  </si>
-  <si>
-    <t>Hunt: Shiny Sylveon (Lendário)</t>
+    <t>⭐ Arcanine, Houndoom, Pupitar</t>
+  </si>
+  <si>
+    <t>⭐S.Rapidash, S.Typhlosion, S.Magcargo</t>
+  </si>
+  <si>
+    <t>⚔️ Hazards Mais Altos</t>
+  </si>
+  <si>
+    <t>⭐ Arcanine, Infernape, Armaldo</t>
   </si>
   <si>
     <t>Fire</t>
@@ -160,39 +235,63 @@
     <t>Blastoise, Feraligatr, Omastar</t>
   </si>
   <si>
+    <t>⭐ Hitmontop, Typhlosion, Rapidash</t>
+  </si>
+  <si>
+    <t>Mesmo encurtando o número total de hunts, permite solar níveis de Hazard superiores com segurança e eficiência.</t>
+  </si>
+  <si>
     <t>Pupitar, Torterra, Kingdra</t>
   </si>
   <si>
+    <t>⭐ Muk, Tentacruel, Mawile</t>
+  </si>
+  <si>
     <t>Rock, Water, Ground</t>
   </si>
   <si>
-    <t>Todos os Pokémon +25 com Atk 5</t>
+    <t>⭐ Arcanine, Machamp, Pupitar</t>
+  </si>
+  <si>
+    <t>⭐ Aggron, Skarmory, Toxicroak</t>
   </si>
   <si>
     <t>Fighting</t>
   </si>
   <si>
-    <t>Hunt: Magmar (Lendário) / Torkoal (UR)</t>
+    <t>⭐ Umbreon, Crawdaunt, Sableye</t>
+  </si>
+  <si>
+    <t>⭐ Blastoise, Feraligatr, Omastar</t>
+  </si>
+  <si>
+    <t>⭐ Houndoom, Hydreigon, Pupitar</t>
   </si>
   <si>
     <t>Mega Clefable, Pidgeot, Espeon</t>
   </si>
   <si>
+    <t>🏆 Futuro &amp; Escalabilidade (Endgame)</t>
+  </si>
+  <si>
+    <t>⭐ Pupitar, Torterra, Kingdra</t>
+  </si>
+  <si>
     <t>Wobbuffet, Mimikyu, Gliscor</t>
   </si>
   <si>
-    <t>Atalho / Dica:</t>
-  </si>
-  <si>
-    <t>Hunt: Ghost / Poison</t>
-  </si>
-  <si>
     <t>Psychic, Flying, Fairy</t>
   </si>
   <si>
+    <t>Outras Opções T1:</t>
+  </si>
+  <si>
     <t>Dark</t>
   </si>
   <si>
+    <t>Trabalhar com 2 ou 3 elementos abre um catálogo amplo de opções viáveis para evoluir: T1, SR, UR e Lendários.</t>
+  </si>
+  <si>
     <t>Absol (Lendário) / Mightyena (UR)</t>
   </si>
   <si>
@@ -205,12 +304,12 @@
     <t>Fighting, Fairy, Bug</t>
   </si>
   <si>
+    <t>Outras Opções SR:</t>
+  </si>
+  <si>
     <t>Water</t>
   </si>
   <si>
-    <t>Runas de Atk no Pokelog ajudam a adiantar a meta</t>
-  </si>
-  <si>
     <t>Milotic (UR)</t>
   </si>
   <si>
@@ -223,15 +322,12 @@
     <t>Grass, Electric</t>
   </si>
   <si>
-    <t>🛡️ LURAR / TANQUE (T1)</t>
+    <t>Umbreon</t>
   </si>
   <si>
     <t>Grass</t>
   </si>
   <si>
-    <t>Estrelas Mínimas:</t>
-  </si>
-  <si>
     <t>Leafeon (Lendário) / Sceptile (UR)</t>
   </si>
   <si>
@@ -241,13 +337,10 @@
     <t>Arcanine, Infernape, Scyther</t>
   </si>
   <si>
-    <t>Tier 1: 2★ (estrelas)  |  SR: 1★ (estrela)</t>
-  </si>
-  <si>
     <t>Poison, Bug, Fire, Fly, Ice</t>
   </si>
   <si>
-    <t>Meta no Dummy:</t>
+    <t>S.Charizard, Kabutops, Golem</t>
   </si>
   <si>
     <t>Electric</t>
@@ -256,30 +349,42 @@
     <t>Electabuzz (Lendário) / Manectric (UR)</t>
   </si>
   <si>
+    <t>Torterra, Misdreavus</t>
+  </si>
+  <si>
     <t>Steelix, Nidoqueen, Torterra</t>
   </si>
   <si>
+    <t>Poliwrath, Medicham, Hariyama</t>
+  </si>
+  <si>
     <t>Torterra, Pupitar, Smeargle</t>
   </si>
   <si>
+    <t>Infernape, Kangaskhan, Torterra</t>
+  </si>
+  <si>
     <t>Ground</t>
   </si>
   <si>
+    <t>Cacturne, Banette, Dusclops</t>
+  </si>
+  <si>
+    <t>Misdreavus, Dusknoir, Torterra</t>
+  </si>
+  <si>
     <t>Ghost</t>
   </si>
   <si>
-    <t>Bater 560k de dano com 3 Pokémon</t>
-  </si>
-  <si>
-    <t>⚔️ DPS / DANO (SR)</t>
-  </si>
-  <si>
     <t>Umbreon, Crawdaunt, Dusknoir</t>
   </si>
   <si>
     <t>Dusknoir, Houndoom, Hydreigon</t>
   </si>
   <si>
+    <t>🎨 Smeargle: Fire, Ground, Ghost, Dark</t>
+  </si>
+  <si>
     <t>Dark, Ghost</t>
   </si>
   <si>
@@ -289,21 +394,30 @@
     <t>Glaceon (Lendário) / Glalie (UR)</t>
   </si>
   <si>
+    <t>—</t>
+  </si>
+  <si>
     <t>Typhlosion, Rapidash, Hitmontop</t>
   </si>
   <si>
     <t>Infernape, Machamp, Skarmory</t>
   </si>
   <si>
+    <t>Metang, Magneton Estrelado</t>
+  </si>
+  <si>
     <t>Fighting, Fire, Metal</t>
   </si>
   <si>
-    <t>Bater 560k de dano com apenas 2 Pokémon</t>
+    <t>🎨 Smeargle: Fighting, Fire, Ground</t>
   </si>
   <si>
     <t>Poison</t>
   </si>
   <si>
+    <t>SevIper</t>
+  </si>
+  <si>
     <t>Garbodor (Lendário) / Swalot (UR)</t>
   </si>
   <si>
@@ -316,36 +430,39 @@
     <t>Ground, Psychic</t>
   </si>
   <si>
+    <t>🎨 Smeargle: Dark, Ghost, Ground</t>
+  </si>
+  <si>
+    <t>Vaporeon, Rhyperior, Magcargo</t>
+  </si>
+  <si>
+    <t>Sharpedo</t>
+  </si>
+  <si>
     <t>Normal</t>
   </si>
   <si>
     <t>Snorlax (Lendário) / Exploud (UR)</t>
   </si>
   <si>
-    <t>Regra de Prey:</t>
-  </si>
-  <si>
     <t>Poliwrath, Hitmontop, Medicham</t>
   </si>
   <si>
     <t>Machamp, Kangaskhan, Smeargle</t>
   </si>
   <si>
-    <t>Obrigatório Prey de Atk na hunt (já calculada no dummy)</t>
-  </si>
-  <si>
-    <t>⭐S.Rapidash, S.Typhlosion, S.Magcargo</t>
+    <t>🎨 Smeargle: Fire, Rock</t>
   </si>
   <si>
     <t>Rock</t>
   </si>
   <si>
-    <t>Manter sempre Prey de Atk ativa na hunt</t>
-  </si>
-  <si>
     <t>Rampardos (UR)</t>
   </si>
   <si>
+    <t>★ GARDEVOIR</t>
+  </si>
+  <si>
     <t>Tangrowth, Steelix, Blastoise</t>
   </si>
   <si>
@@ -355,10 +472,13 @@
     <t>Fighting, Ground, Water, Grass</t>
   </si>
   <si>
+    <t>🎨 Smeargle: Poison, Metal</t>
+  </si>
+  <si>
     <t>Steel</t>
   </si>
   <si>
-    <t>⭐ S.Rapidash, S.Typhlosion, S.Steelix</t>
+    <t>★ GYARADOS</t>
   </si>
   <si>
     <t>Hitmontop, Rapidash, Typhlosion</t>
@@ -367,13 +487,13 @@
     <t>Arcanine, Machamp, Infernape</t>
   </si>
   <si>
-    <t>💡 POR QUE COMPOSIÇÕES COM 2 A 3 ELEMENTOS SÃO SUPERIORES? (ANTI-MONO)</t>
-  </si>
-  <si>
     <t>Ground, Fighting, Fire</t>
   </si>
   <si>
-    <t>⭐ Arcanine, Infernape, Armaldo</t>
+    <t>🎨 Smeargle: Rock, Water, Ground</t>
+  </si>
+  <si>
+    <t>★ SWAMPERT</t>
   </si>
   <si>
     <t>Blastoise, Tangrowth, Gogoat</t>
@@ -394,72 +514,54 @@
     <t>Lapras, Mega Clefable, Jynx</t>
   </si>
   <si>
-    <t>⭐ Arcanine, Houndoom, Pupitar</t>
-  </si>
-  <si>
-    <t>⭐ Muk, Tentacruel, Mawile</t>
-  </si>
-  <si>
     <t>Mimikyu, Florges, Walrein</t>
   </si>
   <si>
+    <t>Hunt: Psychic / Fairy</t>
+  </si>
+  <si>
     <t>Dragon, Ice, Fairy</t>
   </si>
   <si>
+    <t>★ FIGHTING</t>
+  </si>
+  <si>
     <t>Psychic</t>
   </si>
   <si>
     <t>Alakazam (Lendário)</t>
   </si>
   <si>
-    <t>⭐ Aggron, Skarmory, Toxicroak</t>
-  </si>
-  <si>
     <t>Umbreon, Crawdaunt, Sableye</t>
   </si>
   <si>
-    <t>⭐ Hitmontop, Typhlosion, Rapidash</t>
-  </si>
-  <si>
-    <t>⏱️ Cooldown Reduzido por Tier</t>
-  </si>
-  <si>
-    <t>⭐ Blastoise, Feraligatr, Omastar</t>
-  </si>
-  <si>
     <t>Houndoom, Scyther, Dusknoir</t>
   </si>
   <si>
-    <t>⭐ Pupitar, Torterra, Kingdra</t>
+    <t>Hunt: Water / Flying</t>
   </si>
   <si>
     <t>Ghost, Dark, Bug</t>
   </si>
   <si>
-    <t>⭐ Arcanine, Machamp, Pupitar</t>
-  </si>
-  <si>
     <t>Flying</t>
   </si>
   <si>
-    <t>⭐ Umbreon, Crawdaunt, Sableye</t>
-  </si>
-  <si>
-    <t>Outras Opções T1:</t>
-  </si>
-  <si>
     <t>Ampharos, Magcargo, Lapras</t>
   </si>
   <si>
-    <t>⭐ Houndoom, Hydreigon, Pupitar</t>
-  </si>
-  <si>
     <t>Walrein, Luxray, Pachirisu</t>
   </si>
   <si>
+    <t>Hunt: Water / Ground</t>
+  </si>
+  <si>
     <t>Electric, Ice, Rock</t>
   </si>
   <si>
+    <t>★ DARK</t>
+  </si>
+  <si>
     <t>Metagross</t>
   </si>
   <si>
@@ -472,9 +574,6 @@
     <t>Arcanine, Houndoom, Pupitar</t>
   </si>
   <si>
-    <t>Outras Opções SR:</t>
-  </si>
-  <si>
     <t>Fire, Ground, Ghost, Dark</t>
   </si>
   <si>
@@ -487,28 +586,34 @@
     <t>Hitmontop, Typhlosion, Rapidash</t>
   </si>
   <si>
+    <t>★ WATER</t>
+  </si>
+  <si>
     <t>Arcanine, Machamp, Pupitar</t>
   </si>
   <si>
-    <t>No PKA, tiers mais altos não dão só dano: reduzem o cooldown das skills, deixando a rotação muito mais rápida.</t>
-  </si>
-  <si>
     <t>Fighting, Fire, Ground</t>
   </si>
   <si>
-    <t>S.Charizard, Kabutops, Golem</t>
-  </si>
-  <si>
     <t>Gengar</t>
   </si>
   <si>
+    <t>⭐ Mawile, Muk, Tentacruel</t>
+  </si>
+  <si>
     <t>Ghost / Poison</t>
   </si>
   <si>
+    <t>⭐ Toxicroak, Seviper, Misdreavus</t>
+  </si>
+  <si>
+    <t>⭐ Ampharos, Luxray, Jolteon</t>
+  </si>
+  <si>
     <t>Houndoom, Hydreigon, Pupitar</t>
   </si>
   <si>
-    <t>Umbreon</t>
+    <t>⭐ S.Luxray, S.Pachirisu, Smeargle Eletric</t>
   </si>
   <si>
     <t>Dark, Ghost, Ground</t>
@@ -517,24 +622,33 @@
     <t>Gardevoir</t>
   </si>
   <si>
+    <t>⭐Venusaur, Gogoat, Tangrowth</t>
+  </si>
+  <si>
     <t>Psychic / Fairy</t>
   </si>
   <si>
+    <t>⭐ S.Tangrowth,S. Gogoat, Smeargle Grass</t>
+  </si>
+  <si>
     <t>Mawile, Muk, Tentacruel</t>
   </si>
   <si>
+    <t>Hunt: Absol (Lendário) / Mightyena (UR)</t>
+  </si>
+  <si>
     <t>Toxicroak, Seviper, Misdreavus</t>
   </si>
   <si>
-    <t>—</t>
-  </si>
-  <si>
     <t>Poison, Ghost, Metal</t>
   </si>
   <si>
     <t>Gyarados</t>
   </si>
   <si>
+    <t>Hunt: Milotic (UR)</t>
+  </si>
+  <si>
     <t>Water / Flying</t>
   </si>
   <si>
@@ -544,112 +658,19 @@
     <t>Luxray, Pachirisu, Smeargle Eletric</t>
   </si>
   <si>
-    <t>Torterra, Misdreavus</t>
-  </si>
-  <si>
-    <t>Metang, Magneton Estrelado</t>
-  </si>
-  <si>
-    <t>Poliwrath, Medicham, Hariyama</t>
-  </si>
-  <si>
-    <t>Infernape, Kangaskhan, Torterra</t>
-  </si>
-  <si>
-    <t>Cacturne, Banette, Dusclops</t>
-  </si>
-  <si>
-    <t>Misdreavus, Dusknoir, Torterra</t>
-  </si>
-  <si>
-    <t>SevIper</t>
-  </si>
-  <si>
-    <t>📈 Mais Mobs e Brokes / Hora</t>
-  </si>
-  <si>
-    <t>Vaporeon, Rhyperior, Magcargo</t>
-  </si>
-  <si>
-    <t>Sharpedo</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Fire, Ground, Ghost, Dark</t>
-  </si>
-  <si>
-    <t>Rotação mais fluida = mais mobs derrotados/hora, aumentando drasticamente a chance de Shiny/hr e lucro.</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Fighting, Fire, Ground</t>
-  </si>
-  <si>
-    <t>⚔️ Hazards Mais Altos</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Dark, Ghost, Ground</t>
-  </si>
-  <si>
-    <t>Mesmo encurtando o número total de hunts, permite solar níveis de Hazard superiores com segurança e eficiência.</t>
-  </si>
-  <si>
-    <t>★ GARDEVOIR</t>
-  </si>
-  <si>
-    <t>🏆 Futuro &amp; Escalabilidade (Endgame)</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Fire, Rock</t>
-  </si>
-  <si>
-    <t>Trabalhar com 2 ou 3 elementos abre um catálogo amplo de opções viáveis para evoluir: T1, SR, UR e Lendários.</t>
-  </si>
-  <si>
-    <t>★ GYARADOS</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Poison, Metal</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Rock, Water, Ground</t>
-  </si>
-  <si>
-    <t>★ SWAMPERT</t>
-  </si>
-  <si>
-    <t>★ FIGHTING</t>
-  </si>
-  <si>
-    <t>Hunt: Psychic / Fairy</t>
-  </si>
-  <si>
-    <t>Hunt: Water / Flying</t>
-  </si>
-  <si>
-    <t>★ DARK</t>
-  </si>
-  <si>
-    <t>Hunt: Water / Ground</t>
-  </si>
-  <si>
-    <t>★ WATER</t>
-  </si>
-  <si>
-    <t>Hunt: Absol (Lendário) / Mightyena (UR)</t>
-  </si>
-  <si>
-    <t>Hunt: Milotic (UR)</t>
-  </si>
-  <si>
-    <t>⭐ Mawile, Muk, Tentacruel</t>
-  </si>
-  <si>
-    <t>⭐ Toxicroak, Seviper, Misdreavus</t>
-  </si>
-  <si>
-    <t>⭐ Ampharos, Luxray, Jolteon</t>
-  </si>
-  <si>
-    <t>⭐ S.Luxray, S.Pachirisu, Smeargle Eletric</t>
+    <t>Metang, Banette, Dusclops, Nidoking</t>
+  </si>
+  <si>
+    <t>Aggron, Skarmory</t>
+  </si>
+  <si>
+    <t>Raichu</t>
+  </si>
+  <si>
+    <t>🎨 Smeargle: Poison, Ghost, Metal</t>
+  </si>
+  <si>
+    <t>🎨 Smeargle: Electric</t>
   </si>
   <si>
     <t>⭐ Mega Clefable, Pidgeot, Espeon</t>
@@ -658,24 +679,24 @@
     <t>⭐ Wobbuffet, Mimikyu, Gliscor</t>
   </si>
   <si>
-    <t>⭐Venusaur, Gogoat, Tangrowth</t>
-  </si>
-  <si>
     <t>⭐ Hitmontop, Hitmonchan, Poliwrath</t>
   </si>
   <si>
     <t>⭐ Machamp, Scyther, Mimikyu</t>
   </si>
   <si>
-    <t>⭐ S.Tangrowth,S. Gogoat, Smeargle Grass</t>
-  </si>
-  <si>
     <t>⭐ Tangrowth, Ampharos, Venusaur</t>
   </si>
   <si>
+    <t>🎨 Smeargle: Grass</t>
+  </si>
+  <si>
     <t>⭐ Tangrowth, Gogoat, Luxray</t>
   </si>
   <si>
+    <t>★ SCIZOR</t>
+  </si>
+  <si>
     <t>Farfetch'd, Gliscor</t>
   </si>
   <si>
@@ -694,61 +715,40 @@
     <t>Pachirisu</t>
   </si>
   <si>
-    <t>Metang, Banette, Dusclops, Nidoking</t>
-  </si>
-  <si>
-    <t>Aggron, Skarmory</t>
+    <t>Hunt: Bug</t>
   </si>
   <si>
     <t>🎨 Smeargle: Psychic, Flying, Fairy</t>
   </si>
   <si>
-    <t>Raichu</t>
-  </si>
-  <si>
     <t>🎨 Smeargle: Fighting, Fairy, Bug</t>
   </si>
   <si>
-    <t>🎨 Smeargle: Poison, Ghost, Metal</t>
+    <t>⭐ S.Rapidash, S.Typhlosion, S.Zard</t>
   </si>
   <si>
     <t>🎨 Smeargle: Grass, Electric</t>
   </si>
   <si>
-    <t>🎨 Smeargle: Electric</t>
+    <t>⭐S.Arcanine, S.Infernape, Smeargle Fire</t>
   </si>
   <si>
     <t>★ GRASS</t>
   </si>
   <si>
-    <t>🎨 Smeargle: Grass</t>
+    <t>🎨 Smeargle: Fire</t>
   </si>
   <si>
     <t>★ ELECTRIC</t>
   </si>
   <si>
-    <t>★ SCIZOR</t>
-  </si>
-  <si>
     <t>★ GHOST</t>
   </si>
   <si>
-    <t>Hunt: Bug</t>
-  </si>
-  <si>
     <t>Hunt: Leafeon (Lendário) / Sceptile (UR)</t>
   </si>
   <si>
     <t>Hunt: Electabuzz (Lendário) / Manectric (UR)</t>
-  </si>
-  <si>
-    <t>⭐ S.Rapidash, S.Typhlosion, S.Zard</t>
-  </si>
-  <si>
-    <t>⭐S.Arcanine, S.Infernape, Smeargle Fire</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Fire</t>
   </si>
   <si>
     <t>⭐ Typhlosion, Rapidash, Pidgeot</t>
@@ -983,12 +983,6 @@
     </font>
     <font>
       <b/>
-      <sz val="13.0"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
       <sz val="14.0"/>
       <color rgb="FFFFFFFF"/>
       <name val="Quattrocento Sans"/>
@@ -997,7 +991,7 @@
     <font>
       <i/>
       <sz val="9.0"/>
-      <color rgb="FFD1D5DB"/>
+      <color rgb="FF94A3B8"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1006,9 +1000,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
-      <sz val="9.0"/>
-      <color rgb="FF94A3B8"/>
+      <b/>
+      <sz val="13.0"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1016,9 +1010,28 @@
       <color rgb="FF0000FF"/>
     </font>
     <font>
+      <i/>
+      <sz val="9.0"/>
+      <color rgb="FFD1D5DB"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <i/>
+      <u/>
+      <sz val="9.0"/>
+      <color rgb="FF0000FF"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
       <b/>
       <sz val="10.0"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9.0"/>
+      <color rgb="FF334155"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1029,10 +1042,26 @@
       <name val="Quattrocento Sans"/>
     </font>
     <font>
+      <b/>
+      <sz val="11.0"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9.0"/>
+      <color rgb="FF0F172A"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <sz val="9.0"/>
+      <color rgb="FF0F172A"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
       <i/>
-      <u/>
       <sz val="9.0"/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FFF3F4F6"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1048,14 +1077,14 @@
     </font>
     <font>
       <b/>
-      <sz val="11.0"/>
-      <color rgb="FFFFFFFF"/>
+      <sz val="9.0"/>
+      <color rgb="FF166534"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
       <b/>
       <sz val="9.0"/>
-      <color rgb="FF166534"/>
+      <color rgb="FF1E3A8A"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1067,48 +1096,24 @@
     <font>
       <b/>
       <sz val="9.0"/>
-      <color rgb="FF1E40AF"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
       <b/>
       <sz val="9.0"/>
-      <color rgb="FF334155"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="9.0"/>
-      <color rgb="FFF3F4F6"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9.0"/>
-      <color rgb="FF0F172A"/>
+      <color rgb="FF1E40AF"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
       <sz val="9.0"/>
-      <color rgb="FF0F172A"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9.0"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF1F2937"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
       <b/>
       <sz val="10.0"/>
       <color rgb="FF1A1A1A"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9.0"/>
-      <color rgb="FF1E3A8A"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1123,20 +1128,15 @@
       <name val="Quattrocento Sans"/>
     </font>
     <font>
-      <sz val="9.0"/>
-      <color rgb="FF1F2937"/>
+      <b/>
+      <sz val="8.0"/>
+      <color rgb="FF1E3A8A"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
       <b/>
       <sz val="8.0"/>
       <color rgb="FF4A4A4A"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="8.0"/>
-      <color rgb="FF1E3A8A"/>
       <name val="Quattrocento Sans"/>
     </font>
   </fonts>
@@ -1149,14 +1149,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF0F172A"/>
+        <bgColor rgb="FF0F172A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF1B2A4A"/>
         <bgColor rgb="FF1B2A4A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0F172A"/>
-        <bgColor rgb="FF0F172A"/>
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -1167,8 +1173,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <fgColor rgb="FFF1F5F9"/>
+        <bgColor rgb="FFF1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+        <bgColor rgb="FF1F4E78"/>
       </patternFill>
     </fill>
     <fill>
@@ -1179,14 +1191,50 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFDCFCE7"/>
+        <bgColor rgb="FFDCFCE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF3C7"/>
+        <bgColor rgb="FFFEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF374151"/>
+        <bgColor rgb="FF374151"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE68D9C"/>
+        <bgColor rgb="FFE68D9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1E40AF"/>
+        <bgColor rgb="FF1E40AF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEA6C2D"/>
+        <bgColor rgb="FFEA6C2D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFF0FDF4"/>
         <bgColor rgb="FFF0FDF4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E78"/>
-        <bgColor rgb="FF1F4E78"/>
+        <fgColor rgb="FFEFF6FF"/>
+        <bgColor rgb="FFEFF6FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -1197,44 +1245,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE68D9C"/>
-        <bgColor rgb="FFE68D9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF8FAFC"/>
-        <bgColor rgb="FFF8FAFC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEA6C2D"/>
-        <bgColor rgb="FFEA6C2D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF1F5F9"/>
-        <bgColor rgb="FFF1F5F9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF374151"/>
-        <bgColor rgb="FF374151"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF2E7D32"/>
         <bgColor rgb="FF2E7D32"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFDCFCE7"/>
-        <bgColor rgb="FFDCFCE7"/>
       </patternFill>
     </fill>
     <fill>
@@ -1245,8 +1257,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFEF3C7"/>
-        <bgColor rgb="FFFEF3C7"/>
+        <fgColor rgb="FFF8FAFC"/>
+        <bgColor rgb="FFF8FAFC"/>
       </patternFill>
     </fill>
     <fill>
@@ -1259,18 +1271,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFEBEE"/>
         <bgColor rgb="FFFFEBEE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1E40AF"/>
-        <bgColor rgb="FF1E40AF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEFF6FF"/>
-        <bgColor rgb="FFEFF6FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -1400,16 +1400,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFD1D5DB"/>
+        <color rgb="FFCBD5E1"/>
       </left>
       <right style="thin">
-        <color rgb="FFD1D5DB"/>
+        <color rgb="FFCBD5E1"/>
       </right>
       <top style="thin">
-        <color rgb="FFD1D5DB"/>
+        <color rgb="FFCBD5E1"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFD1D5DB"/>
+        <color rgb="FFCBD5E1"/>
       </bottom>
     </border>
     <border>
@@ -1436,16 +1436,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFCBD5E1"/>
+        <color rgb="FFD1D5DB"/>
       </left>
       <right style="thin">
-        <color rgb="FFCBD5E1"/>
+        <color rgb="FFD1D5DB"/>
       </right>
       <top style="thin">
-        <color rgb="FFCBD5E1"/>
+        <color rgb="FFD1D5DB"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFCBD5E1"/>
+        <color rgb="FFD1D5DB"/>
       </bottom>
     </border>
     <border>
@@ -1489,196 +1489,196 @@
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="5" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="6" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="7" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="4" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="6" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="4" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="5" fillId="8" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="9" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="5" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="10" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="5" fillId="11" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="5" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="12" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="13" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="4" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="14" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="4" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="15" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="8" fillId="16" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="17" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="9" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="7" fillId="18" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="4" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="8" fillId="4" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="19" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="10" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="7" fillId="20" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="20" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="21" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="20" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="22" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="21" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="23" fontId="25" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="7" fillId="24" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="24" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="5" fillId="25" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="24" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="5" fillId="7" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="26" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="11" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="5" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="27" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="5" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="28" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="6" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="7" fillId="22" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="5" fillId="25" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="29" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="7" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="6" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="5" fillId="8" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="30" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="9" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="31" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="10" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="32" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="5" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="33" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="11" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="34" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="12" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="35" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="13" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="11" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="36" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="14" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="37" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="11" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="38" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="5" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="7" fillId="5" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="15" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="7" fillId="16" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="17" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="7" fillId="18" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="19" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="20" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="21" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="39" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="19" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="8" fillId="22" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="23" fontId="24" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="9" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="24" fontId="25" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="8" fillId="5" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="24" fontId="25" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="10" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="24" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="5" fillId="25" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="8" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="26" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="27" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="28" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="14" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="20" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="5" fillId="29" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="25" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="30" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="31" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="32" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="33" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="34" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="35" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="36" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="37" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="38" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="39" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="40" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="40" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1920,155 +1920,155 @@
   </cols>
   <sheetData>
     <row r="2" ht="33.75" customHeight="1">
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="4"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="3"/>
     </row>
     <row r="3" ht="19.5" customHeight="1">
-      <c r="B3" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="4"/>
+      <c r="B3" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="3"/>
     </row>
     <row r="4">
-      <c r="B4" s="11" t="s">
-        <v>8</v>
+      <c r="B4" s="7" t="s">
+        <v>5</v>
       </c>
       <c r="C4" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>8</v>
-      </c>
     </row>
     <row r="5" ht="24.0" customHeight="1">
-      <c r="B5" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="4"/>
-      <c r="E5" s="23" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" s="4"/>
+      <c r="B5" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="3"/>
+      <c r="E5" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="3"/>
     </row>
     <row r="6" ht="24.75" customHeight="1">
-      <c r="B6" s="28" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" s="32" t="s">
-        <v>35</v>
-      </c>
-      <c r="E6" s="28" t="s">
-        <v>29</v>
-      </c>
-      <c r="F6" s="32" t="s">
-        <v>44</v>
+      <c r="B6" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="7" ht="24.75" customHeight="1">
-      <c r="B7" s="28" t="s">
+      <c r="B7" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" s="19" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" ht="24.75" customHeight="1">
+      <c r="B8" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" s="23" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" ht="24.75" customHeight="1">
+      <c r="B9" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="19" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" ht="24.0" customHeight="1">
+      <c r="B11" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="3"/>
+    </row>
+    <row r="12" ht="24.0" customHeight="1">
+      <c r="B12" s="32" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" s="34"/>
+      <c r="D12" s="37" t="s">
         <v>49</v>
       </c>
-      <c r="C7" s="33" t="s">
-        <v>58</v>
-      </c>
-      <c r="E7" s="28" t="s">
-        <v>65</v>
-      </c>
-      <c r="F7" s="33" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="8" ht="24.75" customHeight="1">
-      <c r="B8" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="C8" s="35" t="s">
-        <v>78</v>
-      </c>
-      <c r="E8" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="F8" s="37" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="9" ht="24.75" customHeight="1">
-      <c r="B9" s="28" t="s">
-        <v>96</v>
-      </c>
-      <c r="C9" s="33" t="s">
-        <v>99</v>
-      </c>
-      <c r="E9" s="28" t="s">
-        <v>96</v>
-      </c>
-      <c r="F9" s="33" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="11" ht="24.0" customHeight="1">
-      <c r="B11" s="40" t="s">
-        <v>111</v>
-      </c>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="4"/>
-    </row>
-    <row r="12" ht="24.0" customHeight="1">
-      <c r="B12" s="42" t="s">
-        <v>129</v>
-      </c>
-      <c r="C12" s="44"/>
-      <c r="D12" s="46" t="s">
-        <v>152</v>
-      </c>
-      <c r="E12" s="48"/>
-      <c r="F12" s="44"/>
+      <c r="E12" s="39"/>
+      <c r="F12" s="34"/>
     </row>
     <row r="13" ht="24.0" customHeight="1">
-      <c r="B13" s="42" t="s">
-        <v>177</v>
-      </c>
-      <c r="C13" s="44"/>
-      <c r="D13" s="46" t="s">
-        <v>181</v>
-      </c>
-      <c r="E13" s="48"/>
-      <c r="F13" s="44"/>
+      <c r="B13" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="C13" s="34"/>
+      <c r="D13" s="37" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" s="39"/>
+      <c r="F13" s="34"/>
     </row>
     <row r="14" ht="24.0" customHeight="1">
-      <c r="B14" s="42" t="s">
-        <v>183</v>
-      </c>
-      <c r="C14" s="44"/>
-      <c r="D14" s="46" t="s">
-        <v>185</v>
-      </c>
-      <c r="E14" s="48"/>
-      <c r="F14" s="44"/>
+      <c r="B14" s="32" t="s">
+        <v>62</v>
+      </c>
+      <c r="C14" s="34"/>
+      <c r="D14" s="37" t="s">
+        <v>68</v>
+      </c>
+      <c r="E14" s="39"/>
+      <c r="F14" s="34"/>
     </row>
     <row r="15" ht="24.0" customHeight="1">
-      <c r="B15" s="42" t="s">
-        <v>187</v>
-      </c>
-      <c r="C15" s="44"/>
-      <c r="D15" s="46" t="s">
-        <v>189</v>
-      </c>
-      <c r="E15" s="48"/>
-      <c r="F15" s="44"/>
+      <c r="B15" s="32" t="s">
+        <v>79</v>
+      </c>
+      <c r="C15" s="34"/>
+      <c r="D15" s="37" t="s">
+        <v>85</v>
+      </c>
+      <c r="E15" s="39"/>
+      <c r="F15" s="34"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -3094,368 +3094,368 @@
   </cols>
   <sheetData>
     <row r="1" ht="31.5" customHeight="1">
-      <c r="A1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="7" t="s">
-        <v>4</v>
+      <c r="A1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="9" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="2" ht="19.5" customHeight="1">
-      <c r="A2" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="7" t="s">
+      <c r="A2" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="9" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="4" ht="21.75" customHeight="1">
-      <c r="A4" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="20"/>
-      <c r="D4" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="E4" s="20"/>
-      <c r="G4" s="27" t="s">
+      <c r="A4" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="18"/>
+      <c r="D4" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="H4" s="20"/>
+      <c r="E4" s="18"/>
+      <c r="G4" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="H4" s="18"/>
     </row>
     <row r="5" ht="18.0" customHeight="1">
-      <c r="A5" s="30" t="s">
-        <v>32</v>
-      </c>
-      <c r="B5" s="20"/>
-      <c r="D5" s="30" t="s">
-        <v>38</v>
-      </c>
-      <c r="E5" s="20"/>
-      <c r="G5" s="30" t="s">
+      <c r="A5" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" s="18"/>
+      <c r="D5" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" s="18"/>
+      <c r="G5" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="H5" s="18"/>
+    </row>
+    <row r="6" ht="19.5" customHeight="1">
+      <c r="A6" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="H5" s="20"/>
-    </row>
-    <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="34" t="s">
+      <c r="B6" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="E6" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="G6" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="H6" s="38" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7" ht="42.0" customHeight="1">
+      <c r="A7" s="42" t="s">
+        <v>61</v>
+      </c>
+      <c r="B7" s="44" t="s">
         <v>63</v>
       </c>
-      <c r="B6" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="D6" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="E6" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="G6" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="H6" s="36" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="7" ht="42.0" customHeight="1">
-      <c r="A7" s="38" t="s">
-        <v>100</v>
-      </c>
-      <c r="B7" s="39" t="s">
-        <v>113</v>
-      </c>
-      <c r="D7" s="41" t="s">
-        <v>121</v>
-      </c>
-      <c r="E7" s="39" t="s">
-        <v>126</v>
-      </c>
-      <c r="G7" s="41" t="s">
-        <v>130</v>
-      </c>
-      <c r="H7" s="39" t="s">
-        <v>132</v>
+      <c r="D7" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="E7" s="44" t="s">
+        <v>73</v>
+      </c>
+      <c r="G7" s="45" t="s">
+        <v>76</v>
+      </c>
+      <c r="H7" s="44" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="B8" s="43" t="s">
+      <c r="A8" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="B8" s="46" t="s">
+        <v>90</v>
+      </c>
+      <c r="D8" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="E8" s="46" t="s">
+        <v>90</v>
+      </c>
+      <c r="G8" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="H8" s="46" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="9" ht="27.75" customHeight="1">
+      <c r="A9" s="48" t="s">
+        <v>102</v>
+      </c>
+      <c r="B9" s="47" t="s">
+        <v>120</v>
+      </c>
+      <c r="D9" s="47" t="s">
+        <v>123</v>
+      </c>
+      <c r="E9" s="50" t="s">
+        <v>127</v>
+      </c>
+      <c r="G9" s="47" t="s">
+        <v>133</v>
+      </c>
+      <c r="H9" s="47" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="10" ht="18.0" customHeight="1">
+      <c r="A10" s="49" t="s">
+        <v>139</v>
+      </c>
+      <c r="B10" s="18"/>
+      <c r="D10" s="49" t="s">
         <v>146</v>
       </c>
-      <c r="D8" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="E8" s="43" t="s">
-        <v>146</v>
-      </c>
-      <c r="G8" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="H8" s="43" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="9" ht="27.75" customHeight="1">
-      <c r="A9" s="45" t="s">
-        <v>154</v>
-      </c>
-      <c r="B9" s="47" t="s">
-        <v>164</v>
-      </c>
-      <c r="D9" s="47" t="s">
-        <v>171</v>
-      </c>
-      <c r="E9" s="49" t="s">
-        <v>176</v>
-      </c>
-      <c r="G9" s="47" t="s">
-        <v>178</v>
-      </c>
-      <c r="H9" s="47" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="10" ht="18.0" customHeight="1">
-      <c r="A10" s="50" t="s">
-        <v>188</v>
-      </c>
-      <c r="B10" s="20"/>
-      <c r="D10" s="50" t="s">
-        <v>191</v>
-      </c>
-      <c r="E10" s="20"/>
-      <c r="G10" s="50" t="s">
-        <v>192</v>
-      </c>
-      <c r="H10" s="20"/>
+      <c r="E10" s="18"/>
+      <c r="G10" s="49" t="s">
+        <v>152</v>
+      </c>
+      <c r="H10" s="18"/>
     </row>
     <row r="14" ht="21.75" customHeight="1">
       <c r="A14" s="52" t="s">
-        <v>194</v>
-      </c>
-      <c r="B14" s="20"/>
-      <c r="D14" s="53" t="s">
-        <v>197</v>
-      </c>
-      <c r="E14" s="20"/>
-      <c r="G14" s="54" t="s">
-        <v>199</v>
-      </c>
-      <c r="H14" s="20"/>
+        <v>163</v>
+      </c>
+      <c r="B14" s="18"/>
+      <c r="D14" s="54" t="s">
+        <v>175</v>
+      </c>
+      <c r="E14" s="18"/>
+      <c r="G14" s="55" t="s">
+        <v>184</v>
+      </c>
+      <c r="H14" s="18"/>
     </row>
     <row r="15" ht="18.0" customHeight="1">
-      <c r="A15" s="30" t="s">
-        <v>32</v>
-      </c>
-      <c r="B15" s="20"/>
-      <c r="D15" s="30" t="s">
+      <c r="A15" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B15" s="18"/>
+      <c r="D15" s="24" t="s">
         <v>200</v>
       </c>
-      <c r="E15" s="20"/>
-      <c r="G15" s="30" t="s">
-        <v>201</v>
-      </c>
-      <c r="H15" s="20"/>
+      <c r="E15" s="18"/>
+      <c r="G15" s="24" t="s">
+        <v>204</v>
+      </c>
+      <c r="H15" s="18"/>
     </row>
     <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="B16" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="D16" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="E16" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="G16" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="H16" s="36" t="s">
-        <v>79</v>
+      <c r="A16" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="B16" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="D16" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="E16" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="G16" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="H16" s="38" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="17" ht="42.0" customHeight="1">
-      <c r="A17" s="41" t="s">
-        <v>206</v>
-      </c>
-      <c r="B17" s="39" t="s">
-        <v>207</v>
-      </c>
-      <c r="D17" s="41" t="s">
-        <v>209</v>
-      </c>
-      <c r="E17" s="39" t="s">
-        <v>210</v>
-      </c>
-      <c r="G17" s="41" t="s">
-        <v>212</v>
-      </c>
-      <c r="H17" s="39" t="s">
+      <c r="A17" s="45" t="s">
         <v>213</v>
       </c>
+      <c r="B17" s="44" t="s">
+        <v>214</v>
+      </c>
+      <c r="D17" s="45" t="s">
+        <v>215</v>
+      </c>
+      <c r="E17" s="44" t="s">
+        <v>216</v>
+      </c>
+      <c r="G17" s="45" t="s">
+        <v>217</v>
+      </c>
+      <c r="H17" s="44" t="s">
+        <v>219</v>
+      </c>
     </row>
     <row r="18" ht="15.0" customHeight="1">
-      <c r="A18" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="B18" s="43" t="s">
-        <v>146</v>
-      </c>
-      <c r="D18" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="E18" s="43" t="s">
-        <v>146</v>
-      </c>
-      <c r="G18" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="H18" s="43" t="s">
-        <v>146</v>
+      <c r="A18" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="B18" s="46" t="s">
+        <v>90</v>
+      </c>
+      <c r="D18" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="E18" s="46" t="s">
+        <v>90</v>
+      </c>
+      <c r="G18" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="H18" s="46" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="19" ht="27.75" customHeight="1">
       <c r="A19" s="47" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
       <c r="B19" s="47" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="D19" s="47" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="E19" s="47" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="G19" s="47" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="H19" s="47" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
     </row>
     <row r="20" ht="18.0" customHeight="1">
-      <c r="A20" s="50" t="s">
-        <v>222</v>
-      </c>
-      <c r="B20" s="20"/>
-      <c r="D20" s="50" t="s">
-        <v>224</v>
-      </c>
-      <c r="E20" s="20"/>
-      <c r="G20" s="50" t="s">
-        <v>226</v>
-      </c>
-      <c r="H20" s="20"/>
+      <c r="A20" s="49" t="s">
+        <v>228</v>
+      </c>
+      <c r="B20" s="18"/>
+      <c r="D20" s="49" t="s">
+        <v>229</v>
+      </c>
+      <c r="E20" s="18"/>
+      <c r="G20" s="49" t="s">
+        <v>231</v>
+      </c>
+      <c r="H20" s="18"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
     <row r="23" ht="15.75" customHeight="1"/>
     <row r="24" ht="21.75" customHeight="1">
-      <c r="A24" s="57" t="s">
-        <v>228</v>
-      </c>
-      <c r="B24" s="20"/>
+      <c r="A24" s="58" t="s">
+        <v>233</v>
+      </c>
+      <c r="B24" s="18"/>
       <c r="D24" s="59" t="s">
-        <v>230</v>
-      </c>
-      <c r="E24" s="20"/>
+        <v>235</v>
+      </c>
+      <c r="E24" s="18"/>
       <c r="G24" s="60" t="s">
-        <v>232</v>
-      </c>
-      <c r="H24" s="20"/>
+        <v>236</v>
+      </c>
+      <c r="H24" s="18"/>
     </row>
     <row r="25" ht="18.0" customHeight="1">
-      <c r="A25" s="30" t="s">
-        <v>234</v>
-      </c>
-      <c r="B25" s="20"/>
-      <c r="D25" s="30" t="s">
-        <v>235</v>
-      </c>
-      <c r="E25" s="20"/>
-      <c r="G25" s="30" t="s">
-        <v>32</v>
-      </c>
-      <c r="H25" s="20"/>
+      <c r="A25" s="24" t="s">
+        <v>237</v>
+      </c>
+      <c r="B25" s="18"/>
+      <c r="D25" s="24" t="s">
+        <v>238</v>
+      </c>
+      <c r="E25" s="18"/>
+      <c r="G25" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="H25" s="18"/>
     </row>
     <row r="26" ht="19.5" customHeight="1">
-      <c r="A26" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="B26" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="D26" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="E26" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="G26" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="H26" s="36" t="s">
-        <v>79</v>
+      <c r="A26" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="D26" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="E26" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="G26" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="H26" s="38" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="27" ht="42.0" customHeight="1">
-      <c r="A27" s="41" t="s">
+      <c r="A27" s="45" t="s">
         <v>239</v>
       </c>
-      <c r="B27" s="39" t="s">
+      <c r="B27" s="44" t="s">
         <v>240</v>
       </c>
-      <c r="D27" s="41" t="s">
+      <c r="D27" s="45" t="s">
         <v>241</v>
       </c>
-      <c r="E27" s="39" t="s">
+      <c r="E27" s="44" t="s">
         <v>242</v>
       </c>
-      <c r="G27" s="41" t="s">
+      <c r="G27" s="45" t="s">
         <v>243</v>
       </c>
-      <c r="H27" s="39" t="s">
+      <c r="H27" s="44" t="s">
         <v>244</v>
       </c>
     </row>
     <row r="28" ht="15.0" customHeight="1">
-      <c r="A28" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="B28" s="43" t="s">
-        <v>146</v>
-      </c>
-      <c r="D28" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="E28" s="43" t="s">
-        <v>146</v>
-      </c>
-      <c r="G28" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="H28" s="43" t="s">
-        <v>146</v>
+      <c r="A28" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="B28" s="46" t="s">
+        <v>90</v>
+      </c>
+      <c r="D28" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="E28" s="46" t="s">
+        <v>90</v>
+      </c>
+      <c r="G28" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="H28" s="46" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="29" ht="27.75" customHeight="1">
@@ -3479,18 +3479,18 @@
       </c>
     </row>
     <row r="30" ht="18.0" customHeight="1">
-      <c r="A30" s="50" t="s">
+      <c r="A30" s="49" t="s">
         <v>251</v>
       </c>
-      <c r="B30" s="20"/>
-      <c r="D30" s="50" t="s">
+      <c r="B30" s="18"/>
+      <c r="D30" s="49" t="s">
         <v>252</v>
       </c>
-      <c r="E30" s="20"/>
-      <c r="G30" s="50" t="s">
+      <c r="E30" s="18"/>
+      <c r="G30" s="49" t="s">
         <v>253</v>
       </c>
-      <c r="H30" s="20"/>
+      <c r="H30" s="18"/>
     </row>
     <row r="31" ht="15.75" customHeight="1"/>
     <row r="32" ht="15.75" customHeight="1"/>
@@ -3499,88 +3499,88 @@
       <c r="A34" s="61" t="s">
         <v>254</v>
       </c>
-      <c r="B34" s="20"/>
+      <c r="B34" s="18"/>
       <c r="D34" s="62" t="s">
         <v>255</v>
       </c>
-      <c r="E34" s="20"/>
+      <c r="E34" s="18"/>
       <c r="G34" s="63" t="s">
         <v>256</v>
       </c>
-      <c r="H34" s="20"/>
+      <c r="H34" s="18"/>
     </row>
     <row r="35" ht="18.0" customHeight="1">
-      <c r="A35" s="30" t="s">
+      <c r="A35" s="24" t="s">
         <v>257</v>
       </c>
-      <c r="B35" s="20"/>
-      <c r="D35" s="30" t="s">
+      <c r="B35" s="18"/>
+      <c r="D35" s="24" t="s">
         <v>258</v>
       </c>
-      <c r="E35" s="20"/>
-      <c r="G35" s="55" t="s">
+      <c r="E35" s="18"/>
+      <c r="G35" s="53" t="s">
         <v>259</v>
       </c>
-      <c r="H35" s="20"/>
+      <c r="H35" s="18"/>
     </row>
     <row r="36" ht="19.5" customHeight="1">
-      <c r="A36" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="B36" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="D36" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="E36" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="G36" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="H36" s="36" t="s">
-        <v>79</v>
+      <c r="A36" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="B36" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="D36" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="E36" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="G36" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="H36" s="38" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="37" ht="42.0" customHeight="1">
-      <c r="A37" s="41" t="s">
+      <c r="A37" s="45" t="s">
         <v>260</v>
       </c>
-      <c r="B37" s="39" t="s">
+      <c r="B37" s="44" t="s">
         <v>261</v>
       </c>
-      <c r="D37" s="41" t="s">
+      <c r="D37" s="45" t="s">
         <v>262</v>
       </c>
-      <c r="E37" s="39" t="s">
+      <c r="E37" s="44" t="s">
         <v>263</v>
       </c>
-      <c r="G37" s="41" t="s">
+      <c r="G37" s="45" t="s">
         <v>264</v>
       </c>
-      <c r="H37" s="39" t="s">
+      <c r="H37" s="44" t="s">
         <v>265</v>
       </c>
     </row>
     <row r="38" ht="15.0" customHeight="1">
-      <c r="A38" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="B38" s="43" t="s">
-        <v>146</v>
-      </c>
-      <c r="D38" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="E38" s="43" t="s">
-        <v>146</v>
-      </c>
-      <c r="G38" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="H38" s="43" t="s">
-        <v>146</v>
+      <c r="A38" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="B38" s="46" t="s">
+        <v>90</v>
+      </c>
+      <c r="D38" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="E38" s="46" t="s">
+        <v>90</v>
+      </c>
+      <c r="G38" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="H38" s="46" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="39" ht="27.75" customHeight="1">
@@ -3600,22 +3600,22 @@
         <v>270</v>
       </c>
       <c r="H39" s="47" t="s">
-        <v>164</v>
+        <v>120</v>
       </c>
     </row>
     <row r="40" ht="18.0" customHeight="1">
-      <c r="A40" s="50" t="s">
+      <c r="A40" s="49" t="s">
         <v>271</v>
       </c>
-      <c r="B40" s="20"/>
-      <c r="D40" s="50" t="s">
+      <c r="B40" s="18"/>
+      <c r="D40" s="49" t="s">
         <v>272</v>
       </c>
-      <c r="E40" s="20"/>
-      <c r="G40" s="50" t="s">
+      <c r="E40" s="18"/>
+      <c r="G40" s="49" t="s">
         <v>273</v>
       </c>
-      <c r="H40" s="20"/>
+      <c r="H40" s="18"/>
     </row>
     <row r="41" ht="15.75" customHeight="1"/>
     <row r="42" ht="15.75" customHeight="1"/>
@@ -3624,88 +3624,88 @@
       <c r="A44" s="64" t="s">
         <v>274</v>
       </c>
-      <c r="B44" s="20"/>
+      <c r="B44" s="18"/>
       <c r="D44" s="65" t="s">
         <v>275</v>
       </c>
-      <c r="E44" s="20"/>
+      <c r="E44" s="18"/>
       <c r="G44" s="66" t="s">
         <v>276</v>
       </c>
-      <c r="H44" s="20"/>
+      <c r="H44" s="18"/>
     </row>
     <row r="45" ht="18.0" customHeight="1">
-      <c r="A45" s="30" t="s">
+      <c r="A45" s="24" t="s">
         <v>277</v>
       </c>
-      <c r="B45" s="20"/>
-      <c r="D45" s="30" t="s">
-        <v>32</v>
-      </c>
-      <c r="E45" s="20"/>
-      <c r="G45" s="30" t="s">
-        <v>32</v>
-      </c>
-      <c r="H45" s="20"/>
+      <c r="B45" s="18"/>
+      <c r="D45" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="E45" s="18"/>
+      <c r="G45" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="H45" s="18"/>
     </row>
     <row r="46" ht="19.5" customHeight="1">
-      <c r="A46" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="B46" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="D46" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="E46" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="G46" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="H46" s="36" t="s">
-        <v>79</v>
+      <c r="A46" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="B46" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="D46" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="E46" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="G46" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="H46" s="38" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="47" ht="42.0" customHeight="1">
-      <c r="A47" s="41" t="s">
+      <c r="A47" s="45" t="s">
         <v>278</v>
       </c>
-      <c r="B47" s="39" t="s">
+      <c r="B47" s="44" t="s">
         <v>279</v>
       </c>
-      <c r="D47" s="41" t="s">
+      <c r="D47" s="45" t="s">
         <v>280</v>
       </c>
-      <c r="E47" s="39" t="s">
+      <c r="E47" s="44" t="s">
         <v>281</v>
       </c>
-      <c r="G47" s="41" t="s">
+      <c r="G47" s="45" t="s">
         <v>282</v>
       </c>
-      <c r="H47" s="39" t="s">
+      <c r="H47" s="44" t="s">
         <v>283</v>
       </c>
     </row>
     <row r="48" ht="15.0" customHeight="1">
-      <c r="A48" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="B48" s="43" t="s">
-        <v>146</v>
-      </c>
-      <c r="D48" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="E48" s="43" t="s">
-        <v>146</v>
-      </c>
-      <c r="G48" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="H48" s="43" t="s">
-        <v>146</v>
+      <c r="A48" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="B48" s="46" t="s">
+        <v>90</v>
+      </c>
+      <c r="D48" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="E48" s="46" t="s">
+        <v>90</v>
+      </c>
+      <c r="G48" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="H48" s="46" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="49" ht="27.75" customHeight="1">
@@ -3729,18 +3729,18 @@
       </c>
     </row>
     <row r="50" ht="18.0" customHeight="1">
-      <c r="A50" s="50" t="s">
+      <c r="A50" s="49" t="s">
         <v>290</v>
       </c>
-      <c r="B50" s="20"/>
-      <c r="D50" s="50" t="s">
+      <c r="B50" s="18"/>
+      <c r="D50" s="49" t="s">
         <v>291</v>
       </c>
-      <c r="E50" s="20"/>
-      <c r="G50" s="50" t="s">
+      <c r="E50" s="18"/>
+      <c r="G50" s="49" t="s">
         <v>292</v>
       </c>
-      <c r="H50" s="20"/>
+      <c r="H50" s="18"/>
     </row>
     <row r="51" ht="15.75" customHeight="1"/>
     <row r="52" ht="15.75" customHeight="1"/>
@@ -3749,88 +3749,88 @@
       <c r="A54" s="67" t="s">
         <v>293</v>
       </c>
-      <c r="B54" s="20"/>
+      <c r="B54" s="18"/>
       <c r="D54" s="68" t="s">
         <v>294</v>
       </c>
-      <c r="E54" s="20"/>
+      <c r="E54" s="18"/>
       <c r="G54" s="69" t="s">
         <v>295</v>
       </c>
-      <c r="H54" s="20"/>
+      <c r="H54" s="18"/>
     </row>
     <row r="55" ht="18.0" customHeight="1">
-      <c r="A55" s="30" t="s">
+      <c r="A55" s="24" t="s">
         <v>296</v>
       </c>
-      <c r="B55" s="20"/>
-      <c r="D55" s="30" t="s">
+      <c r="B55" s="18"/>
+      <c r="D55" s="24" t="s">
         <v>297</v>
       </c>
-      <c r="E55" s="20"/>
-      <c r="G55" s="30" t="s">
-        <v>32</v>
-      </c>
-      <c r="H55" s="20"/>
+      <c r="E55" s="18"/>
+      <c r="G55" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="H55" s="18"/>
     </row>
     <row r="56" ht="19.5" customHeight="1">
-      <c r="A56" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="B56" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="D56" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="E56" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="G56" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="H56" s="36" t="s">
-        <v>79</v>
+      <c r="A56" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="B56" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="D56" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="E56" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="G56" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="H56" s="38" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="57" ht="42.0" customHeight="1">
-      <c r="A57" s="41" t="s">
+      <c r="A57" s="45" t="s">
         <v>298</v>
       </c>
-      <c r="B57" s="39" t="s">
+      <c r="B57" s="44" t="s">
         <v>299</v>
       </c>
-      <c r="D57" s="41" t="s">
-        <v>136</v>
-      </c>
-      <c r="E57" s="39" t="s">
+      <c r="D57" s="45" t="s">
+        <v>75</v>
+      </c>
+      <c r="E57" s="44" t="s">
         <v>300</v>
       </c>
-      <c r="G57" s="41" t="s">
+      <c r="G57" s="45" t="s">
         <v>301</v>
       </c>
-      <c r="H57" s="39" t="s">
+      <c r="H57" s="44" t="s">
         <v>302</v>
       </c>
     </row>
     <row r="58" ht="15.0" customHeight="1">
-      <c r="A58" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="B58" s="43" t="s">
-        <v>146</v>
-      </c>
-      <c r="D58" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="E58" s="43" t="s">
-        <v>146</v>
-      </c>
-      <c r="G58" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="H58" s="43" t="s">
-        <v>146</v>
+      <c r="A58" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="B58" s="46" t="s">
+        <v>90</v>
+      </c>
+      <c r="D58" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="E58" s="46" t="s">
+        <v>90</v>
+      </c>
+      <c r="G58" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="H58" s="46" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="59" ht="27.75" customHeight="1">
@@ -3854,18 +3854,18 @@
       </c>
     </row>
     <row r="60" ht="18.0" customHeight="1">
-      <c r="A60" s="50" t="s">
+      <c r="A60" s="49" t="s">
         <v>309</v>
       </c>
-      <c r="B60" s="20"/>
-      <c r="D60" s="50" t="s">
+      <c r="B60" s="18"/>
+      <c r="D60" s="49" t="s">
         <v>310</v>
       </c>
-      <c r="E60" s="20"/>
-      <c r="G60" s="50" t="s">
+      <c r="E60" s="18"/>
+      <c r="G60" s="49" t="s">
         <v>311</v>
       </c>
-      <c r="H60" s="20"/>
+      <c r="H60" s="18"/>
     </row>
     <row r="61" ht="15.75" customHeight="1"/>
     <row r="62" ht="15.75" customHeight="1"/>
@@ -4892,325 +4892,325 @@
   </cols>
   <sheetData>
     <row r="1" ht="31.5" customHeight="1">
-      <c r="A1" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="4"/>
+      <c r="A1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="3"/>
     </row>
     <row r="2" ht="19.5" customHeight="1">
-      <c r="A2" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="4"/>
+      <c r="A2" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="3"/>
     </row>
     <row r="4" ht="21.75" customHeight="1">
-      <c r="A4" s="21" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="20"/>
-      <c r="D4" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" s="20"/>
-      <c r="G4" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="H4" s="20"/>
+      <c r="A4" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="18"/>
+      <c r="D4" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="18"/>
+      <c r="G4" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" s="18"/>
     </row>
     <row r="5" ht="18.0" customHeight="1">
-      <c r="A5" s="30" t="s">
-        <v>31</v>
-      </c>
-      <c r="B5" s="20"/>
-      <c r="D5" s="30" t="s">
-        <v>37</v>
-      </c>
-      <c r="E5" s="20"/>
-      <c r="G5" s="30" t="s">
-        <v>50</v>
-      </c>
-      <c r="H5" s="20"/>
+      <c r="A5" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="18"/>
+      <c r="D5" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="18"/>
+      <c r="G5" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="H5" s="18"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="B6" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="D6" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="E6" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="G6" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="H6" s="36" t="s">
-        <v>79</v>
+      <c r="A6" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="E6" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="G6" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="H6" s="38" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="7" ht="42.0" customHeight="1">
-      <c r="A7" s="38" t="s">
-        <v>108</v>
-      </c>
-      <c r="B7" s="39" t="s">
-        <v>120</v>
-      </c>
-      <c r="D7" s="41" t="s">
-        <v>128</v>
-      </c>
-      <c r="E7" s="39" t="s">
-        <v>134</v>
-      </c>
-      <c r="G7" s="41" t="s">
-        <v>136</v>
-      </c>
-      <c r="H7" s="39" t="s">
-        <v>139</v>
+      <c r="A7" s="42" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" s="44" t="s">
+        <v>60</v>
+      </c>
+      <c r="D7" s="45" t="s">
+        <v>67</v>
+      </c>
+      <c r="E7" s="44" t="s">
+        <v>72</v>
+      </c>
+      <c r="G7" s="45" t="s">
+        <v>75</v>
+      </c>
+      <c r="H7" s="44" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="B8" s="43" t="s">
-        <v>146</v>
-      </c>
-      <c r="D8" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="E8" s="43" t="s">
-        <v>146</v>
-      </c>
-      <c r="G8" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="H8" s="43" t="s">
-        <v>146</v>
+      <c r="A8" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="B8" s="46" t="s">
+        <v>90</v>
+      </c>
+      <c r="D8" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="E8" s="46" t="s">
+        <v>90</v>
+      </c>
+      <c r="G8" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="H8" s="46" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="9" ht="27.75" customHeight="1">
       <c r="A9" s="47" t="s">
-        <v>158</v>
+        <v>96</v>
       </c>
       <c r="B9" s="47" t="s">
-        <v>170</v>
+        <v>105</v>
       </c>
       <c r="D9" s="47" t="s">
-        <v>172</v>
+        <v>107</v>
       </c>
       <c r="E9" s="47" t="s">
+        <v>109</v>
+      </c>
+      <c r="G9" s="47" t="s">
+        <v>111</v>
+      </c>
+      <c r="H9" s="47" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="10" ht="18.0" customHeight="1">
+      <c r="A10" s="49" t="s">
+        <v>116</v>
+      </c>
+      <c r="B10" s="18"/>
+      <c r="D10" s="49" t="s">
+        <v>125</v>
+      </c>
+      <c r="E10" s="18"/>
+      <c r="G10" s="49" t="s">
+        <v>132</v>
+      </c>
+      <c r="H10" s="18"/>
+    </row>
+    <row r="14" ht="21.75" customHeight="1">
+      <c r="A14" s="16" t="s">
+        <v>142</v>
+      </c>
+      <c r="B14" s="18"/>
+      <c r="D14" s="16" t="s">
+        <v>148</v>
+      </c>
+      <c r="E14" s="18"/>
+      <c r="G14" s="51" t="s">
+        <v>153</v>
+      </c>
+      <c r="H14" s="18"/>
+    </row>
+    <row r="15" ht="18.0" customHeight="1">
+      <c r="A15" s="24" t="s">
+        <v>161</v>
+      </c>
+      <c r="B15" s="18"/>
+      <c r="D15" s="24" t="s">
+        <v>168</v>
+      </c>
+      <c r="E15" s="18"/>
+      <c r="G15" s="53" t="s">
         <v>173</v>
       </c>
-      <c r="G9" s="47" t="s">
-        <v>174</v>
-      </c>
-      <c r="H9" s="47" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="10" ht="18.0" customHeight="1">
-      <c r="A10" s="50" t="s">
-        <v>180</v>
-      </c>
-      <c r="B10" s="20"/>
-      <c r="D10" s="50" t="s">
-        <v>182</v>
-      </c>
-      <c r="E10" s="20"/>
-      <c r="G10" s="50" t="s">
-        <v>184</v>
-      </c>
-      <c r="H10" s="20"/>
-    </row>
-    <row r="14" ht="21.75" customHeight="1">
-      <c r="A14" s="21" t="s">
-        <v>186</v>
-      </c>
-      <c r="B14" s="20"/>
-      <c r="D14" s="21" t="s">
+      <c r="H15" s="18"/>
+    </row>
+    <row r="16" ht="19.5" customHeight="1">
+      <c r="A16" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="B16" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="D16" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="E16" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="G16" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="H16" s="38" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="17" ht="42.0" customHeight="1">
+      <c r="A17" s="45" t="s">
+        <v>188</v>
+      </c>
+      <c r="B17" s="44" t="s">
         <v>190</v>
       </c>
-      <c r="E14" s="20"/>
-      <c r="G14" s="51" t="s">
+      <c r="D17" s="45" t="s">
+        <v>191</v>
+      </c>
+      <c r="E17" s="56" t="s">
         <v>193</v>
       </c>
-      <c r="H14" s="20"/>
-    </row>
-    <row r="15" ht="18.0" customHeight="1">
-      <c r="A15" s="30" t="s">
-        <v>195</v>
-      </c>
-      <c r="B15" s="20"/>
-      <c r="D15" s="30" t="s">
+      <c r="G17" s="42" t="s">
         <v>196</v>
       </c>
-      <c r="E15" s="20"/>
-      <c r="G15" s="55" t="s">
+      <c r="H17" s="56" t="s">
         <v>198</v>
       </c>
-      <c r="H15" s="20"/>
-    </row>
-    <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="B16" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="D16" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="E16" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="G16" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="H16" s="36" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="17" ht="42.0" customHeight="1">
-      <c r="A17" s="41" t="s">
-        <v>202</v>
-      </c>
-      <c r="B17" s="39" t="s">
-        <v>203</v>
-      </c>
-      <c r="D17" s="41" t="s">
-        <v>204</v>
-      </c>
-      <c r="E17" s="56" t="s">
-        <v>205</v>
-      </c>
-      <c r="G17" s="38" t="s">
-        <v>208</v>
-      </c>
-      <c r="H17" s="56" t="s">
-        <v>211</v>
-      </c>
     </row>
     <row r="18" ht="15.0" customHeight="1">
-      <c r="A18" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="B18" s="43" t="s">
-        <v>146</v>
-      </c>
-      <c r="D18" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="E18" s="43" t="s">
-        <v>146</v>
-      </c>
-      <c r="G18" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="H18" s="43" t="s">
-        <v>146</v>
+      <c r="A18" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="B18" s="46" t="s">
+        <v>90</v>
+      </c>
+      <c r="D18" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="E18" s="46" t="s">
+        <v>90</v>
+      </c>
+      <c r="G18" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="H18" s="46" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="19" ht="27.75" customHeight="1">
       <c r="A19" s="47" t="s">
-        <v>220</v>
+        <v>208</v>
       </c>
       <c r="B19" s="47" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="D19" s="47" t="s">
-        <v>223</v>
+        <v>210</v>
       </c>
       <c r="E19" s="47" t="s">
-        <v>164</v>
+        <v>120</v>
       </c>
       <c r="G19" s="47" t="s">
-        <v>164</v>
+        <v>120</v>
       </c>
       <c r="H19" s="47" t="s">
-        <v>164</v>
+        <v>120</v>
       </c>
     </row>
     <row r="20" ht="18.0" customHeight="1">
-      <c r="A20" s="50" t="s">
-        <v>225</v>
-      </c>
-      <c r="B20" s="20"/>
-      <c r="D20" s="50" t="s">
-        <v>227</v>
-      </c>
-      <c r="E20" s="20"/>
-      <c r="G20" s="58" t="s">
-        <v>229</v>
-      </c>
-      <c r="H20" s="20"/>
+      <c r="A20" s="49" t="s">
+        <v>211</v>
+      </c>
+      <c r="B20" s="18"/>
+      <c r="D20" s="49" t="s">
+        <v>212</v>
+      </c>
+      <c r="E20" s="18"/>
+      <c r="G20" s="57" t="s">
+        <v>218</v>
+      </c>
+      <c r="H20" s="18"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
     <row r="23" ht="15.75" customHeight="1"/>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="51" t="s">
-        <v>231</v>
-      </c>
-      <c r="B24" s="20"/>
+        <v>220</v>
+      </c>
+      <c r="B24" s="18"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="55" t="s">
-        <v>233</v>
-      </c>
-      <c r="B25" s="20"/>
+      <c r="A25" s="53" t="s">
+        <v>227</v>
+      </c>
+      <c r="B25" s="18"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="B26" s="36" t="s">
-        <v>79</v>
+      <c r="A26" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26" s="38" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="27" ht="44.25" customHeight="1">
-      <c r="A27" s="38" t="s">
-        <v>236</v>
+      <c r="A27" s="42" t="s">
+        <v>230</v>
       </c>
       <c r="B27" s="56" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="B28" s="43" t="s">
-        <v>146</v>
+      <c r="A28" s="46" t="s">
+        <v>83</v>
+      </c>
+      <c r="B28" s="46" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="29" ht="27.75" customHeight="1">
       <c r="A29" s="47" t="s">
-        <v>164</v>
+        <v>120</v>
       </c>
       <c r="B29" s="47" t="s">
-        <v>164</v>
+        <v>120</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="58" t="s">
-        <v>238</v>
-      </c>
-      <c r="B30" s="20"/>
+      <c r="A30" s="57" t="s">
+        <v>234</v>
+      </c>
+      <c r="B30" s="18"/>
     </row>
     <row r="31" ht="15.75" customHeight="1"/>
     <row r="32" ht="15.75" customHeight="1"/>
@@ -6234,438 +6234,438 @@
   </cols>
   <sheetData>
     <row r="1" ht="27.75" customHeight="1">
-      <c r="A1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="4"/>
+      <c r="A1" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="3"/>
     </row>
     <row r="2" ht="18.0" customHeight="1">
-      <c r="A2" s="6"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="4"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="3"/>
     </row>
     <row r="3">
       <c r="B3" s="10" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" ht="24.0" customHeight="1">
-      <c r="A4" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="12" t="s">
-        <v>13</v>
+      <c r="A4" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="25" t="s">
+        <v>35</v>
+      </c>
+      <c r="D4" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="E4" s="22" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="5" ht="21.75" customHeight="1">
-      <c r="A5" s="16" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="22" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" s="25" t="s">
-        <v>24</v>
+      <c r="A5" s="28" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="30" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="E5" s="36" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="6" ht="21.75" customHeight="1">
-      <c r="A6" s="26" t="s">
-        <v>28</v>
-      </c>
-      <c r="B6" s="29" t="s">
-        <v>30</v>
-      </c>
-      <c r="C6" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="D6" s="22" t="s">
-        <v>34</v>
-      </c>
-      <c r="E6" s="31" t="s">
-        <v>36</v>
+      <c r="A6" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="B6" s="41" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6" s="33" t="s">
+        <v>58</v>
+      </c>
+      <c r="E6" s="43" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="7" ht="21.75" customHeight="1">
-      <c r="A7" s="16" t="s">
-        <v>39</v>
-      </c>
-      <c r="B7" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="C7" s="19" t="s">
+      <c r="A7" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="B7" s="30" t="s">
+        <v>65</v>
+      </c>
+      <c r="C7" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="D7" s="33" t="s">
+        <v>69</v>
+      </c>
+      <c r="E7" s="36" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="8" ht="21.75" customHeight="1">
+      <c r="A8" s="40" t="s">
+        <v>74</v>
+      </c>
+      <c r="B8" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="D7" s="22" t="s">
-        <v>42</v>
-      </c>
-      <c r="E7" s="25" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="8" ht="21.75" customHeight="1">
-      <c r="A8" s="26" t="s">
-        <v>45</v>
-      </c>
-      <c r="B8" s="29" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="D8" s="22" t="s">
-        <v>48</v>
-      </c>
-      <c r="E8" s="31" t="s">
-        <v>51</v>
+      <c r="C8" s="31" t="s">
+        <v>78</v>
+      </c>
+      <c r="D8" s="33" t="s">
+        <v>81</v>
+      </c>
+      <c r="E8" s="43" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="9" ht="21.75" customHeight="1">
-      <c r="A9" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="B9" s="17" t="s">
-        <v>53</v>
-      </c>
-      <c r="C9" s="19" t="s">
-        <v>54</v>
-      </c>
-      <c r="D9" s="22" t="s">
-        <v>55</v>
-      </c>
-      <c r="E9" s="25" t="s">
-        <v>56</v>
+      <c r="A9" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="B9" s="30" t="s">
+        <v>86</v>
+      </c>
+      <c r="C9" s="31" t="s">
+        <v>87</v>
+      </c>
+      <c r="D9" s="33" t="s">
+        <v>88</v>
+      </c>
+      <c r="E9" s="36" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="10" ht="21.75" customHeight="1">
-      <c r="A10" s="26" t="s">
-        <v>57</v>
-      </c>
-      <c r="B10" s="29" t="s">
-        <v>59</v>
-      </c>
-      <c r="C10" s="19" t="s">
-        <v>60</v>
-      </c>
-      <c r="D10" s="22" t="s">
-        <v>61</v>
-      </c>
-      <c r="E10" s="31" t="s">
-        <v>62</v>
+      <c r="A10" s="40" t="s">
+        <v>91</v>
+      </c>
+      <c r="B10" s="41" t="s">
+        <v>92</v>
+      </c>
+      <c r="C10" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="D10" s="33" t="s">
+        <v>94</v>
+      </c>
+      <c r="E10" s="43" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="11" ht="21.75" customHeight="1">
-      <c r="A11" s="16" t="s">
-        <v>64</v>
-      </c>
-      <c r="B11" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="C11" s="19" t="s">
-        <v>67</v>
-      </c>
-      <c r="D11" s="22" t="s">
-        <v>68</v>
-      </c>
-      <c r="E11" s="25" t="s">
-        <v>70</v>
+      <c r="A11" s="28" t="s">
+        <v>97</v>
+      </c>
+      <c r="B11" s="30" t="s">
+        <v>98</v>
+      </c>
+      <c r="C11" s="31" t="s">
+        <v>99</v>
+      </c>
+      <c r="D11" s="33" t="s">
+        <v>100</v>
+      </c>
+      <c r="E11" s="36" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="12" ht="21.75" customHeight="1">
-      <c r="A12" s="26" t="s">
-        <v>72</v>
-      </c>
-      <c r="B12" s="29" t="s">
-        <v>73</v>
-      </c>
-      <c r="C12" s="19" t="s">
+      <c r="A12" s="40" t="s">
+        <v>103</v>
+      </c>
+      <c r="B12" s="41" t="s">
+        <v>104</v>
+      </c>
+      <c r="C12" s="31" t="s">
+        <v>106</v>
+      </c>
+      <c r="D12" s="33" t="s">
+        <v>108</v>
+      </c>
+      <c r="E12" s="43" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="13" ht="21.75" customHeight="1">
+      <c r="A13" s="28" t="s">
+        <v>113</v>
+      </c>
+      <c r="B13" s="30" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" s="31" t="s">
+        <v>114</v>
+      </c>
+      <c r="D13" s="33" t="s">
+        <v>115</v>
+      </c>
+      <c r="E13" s="36" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="14" ht="21.75" customHeight="1">
+      <c r="A14" s="40" t="s">
+        <v>118</v>
+      </c>
+      <c r="B14" s="41" t="s">
+        <v>119</v>
+      </c>
+      <c r="C14" s="31" t="s">
+        <v>121</v>
+      </c>
+      <c r="D14" s="33" t="s">
+        <v>122</v>
+      </c>
+      <c r="E14" s="43" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="15" ht="21.75" customHeight="1">
+      <c r="A15" s="28" t="s">
+        <v>126</v>
+      </c>
+      <c r="B15" s="30" t="s">
+        <v>128</v>
+      </c>
+      <c r="C15" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="D15" s="33" t="s">
+        <v>130</v>
+      </c>
+      <c r="E15" s="36" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="16" ht="21.75" customHeight="1">
+      <c r="A16" s="40" t="s">
+        <v>135</v>
+      </c>
+      <c r="B16" s="41" t="s">
+        <v>136</v>
+      </c>
+      <c r="C16" s="31" t="s">
+        <v>137</v>
+      </c>
+      <c r="D16" s="33" t="s">
+        <v>138</v>
+      </c>
+      <c r="E16" s="43" t="s">
         <v>74</v>
       </c>
-      <c r="D12" s="22" t="s">
-        <v>75</v>
-      </c>
-      <c r="E12" s="31" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="13" ht="21.75" customHeight="1">
-      <c r="A13" s="16" t="s">
-        <v>77</v>
-      </c>
-      <c r="B13" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="19" t="s">
-        <v>80</v>
-      </c>
-      <c r="D13" s="22" t="s">
-        <v>81</v>
-      </c>
-      <c r="E13" s="25" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="14" ht="21.75" customHeight="1">
-      <c r="A14" s="26" t="s">
-        <v>83</v>
-      </c>
-      <c r="B14" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="C14" s="19" t="s">
-        <v>85</v>
-      </c>
-      <c r="D14" s="22" t="s">
-        <v>86</v>
-      </c>
-      <c r="E14" s="31" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="15" ht="21.75" customHeight="1">
-      <c r="A15" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="B15" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="C15" s="19" t="s">
-        <v>91</v>
-      </c>
-      <c r="D15" s="22" t="s">
-        <v>92</v>
-      </c>
-      <c r="E15" s="25" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="16" ht="21.75" customHeight="1">
-      <c r="A16" s="26" t="s">
-        <v>94</v>
-      </c>
-      <c r="B16" s="29" t="s">
-        <v>95</v>
-      </c>
-      <c r="C16" s="19" t="s">
-        <v>97</v>
-      </c>
-      <c r="D16" s="22" t="s">
-        <v>98</v>
-      </c>
-      <c r="E16" s="31" t="s">
-        <v>45</v>
-      </c>
     </row>
     <row r="17" ht="21.75" customHeight="1">
-      <c r="A17" s="16" t="s">
-        <v>101</v>
-      </c>
-      <c r="B17" s="17" t="s">
+      <c r="A17" s="28" t="s">
+        <v>140</v>
+      </c>
+      <c r="B17" s="30" t="s">
+        <v>141</v>
+      </c>
+      <c r="C17" s="31" t="s">
+        <v>143</v>
+      </c>
+      <c r="D17" s="33" t="s">
+        <v>144</v>
+      </c>
+      <c r="E17" s="36" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="18" ht="21.75" customHeight="1">
+      <c r="A18" s="40" t="s">
+        <v>147</v>
+      </c>
+      <c r="B18" s="41" t="s">
+        <v>41</v>
+      </c>
+      <c r="C18" s="31" t="s">
+        <v>149</v>
+      </c>
+      <c r="D18" s="33" t="s">
+        <v>150</v>
+      </c>
+      <c r="E18" s="43" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="19" ht="21.75" customHeight="1">
+      <c r="A19" s="28" t="s">
+        <v>110</v>
+      </c>
+      <c r="B19" s="30" t="s">
+        <v>41</v>
+      </c>
+      <c r="C19" s="31" t="s">
+        <v>154</v>
+      </c>
+      <c r="D19" s="33" t="s">
+        <v>155</v>
+      </c>
+      <c r="E19" s="36" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="20" ht="21.75" customHeight="1">
+      <c r="A20" s="40" t="s">
+        <v>157</v>
+      </c>
+      <c r="B20" s="41" t="s">
+        <v>158</v>
+      </c>
+      <c r="C20" s="31" t="s">
+        <v>159</v>
+      </c>
+      <c r="D20" s="33" t="s">
+        <v>160</v>
+      </c>
+      <c r="E20" s="43" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="21" ht="21.75" customHeight="1">
+      <c r="A21" s="28" t="s">
+        <v>164</v>
+      </c>
+      <c r="B21" s="30" t="s">
+        <v>165</v>
+      </c>
+      <c r="C21" s="31" t="s">
+        <v>166</v>
+      </c>
+      <c r="D21" s="33" t="s">
+        <v>167</v>
+      </c>
+      <c r="E21" s="36" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="22" ht="21.75" customHeight="1">
+      <c r="A22" s="40" t="s">
+        <v>170</v>
+      </c>
+      <c r="B22" s="41" t="s">
+        <v>41</v>
+      </c>
+      <c r="C22" s="31" t="s">
+        <v>171</v>
+      </c>
+      <c r="D22" s="33" t="s">
+        <v>172</v>
+      </c>
+      <c r="E22" s="43" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="23" ht="21.75" customHeight="1">
+      <c r="A23" s="28" t="s">
+        <v>176</v>
+      </c>
+      <c r="B23" s="30" t="s">
+        <v>177</v>
+      </c>
+      <c r="C23" s="31" t="s">
+        <v>178</v>
+      </c>
+      <c r="D23" s="33" t="s">
+        <v>179</v>
+      </c>
+      <c r="E23" s="36" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="24" ht="21.75" customHeight="1">
+      <c r="A24" s="40" t="s">
+        <v>181</v>
+      </c>
+      <c r="B24" s="41" t="s">
+        <v>182</v>
+      </c>
+      <c r="C24" s="31" t="s">
+        <v>183</v>
+      </c>
+      <c r="D24" s="33" t="s">
+        <v>185</v>
+      </c>
+      <c r="E24" s="43" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="25" ht="21.75" customHeight="1">
+      <c r="A25" s="28" t="s">
+        <v>187</v>
+      </c>
+      <c r="B25" s="30" t="s">
+        <v>189</v>
+      </c>
+      <c r="C25" s="31" t="s">
+        <v>166</v>
+      </c>
+      <c r="D25" s="33" t="s">
+        <v>192</v>
+      </c>
+      <c r="E25" s="36" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="26" ht="21.75" customHeight="1">
+      <c r="A26" s="40" t="s">
+        <v>195</v>
+      </c>
+      <c r="B26" s="41" t="s">
+        <v>197</v>
+      </c>
+      <c r="C26" s="31" t="s">
+        <v>199</v>
+      </c>
+      <c r="D26" s="33" t="s">
+        <v>201</v>
+      </c>
+      <c r="E26" s="43" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="27" ht="21.75" customHeight="1">
+      <c r="A27" s="28" t="s">
+        <v>203</v>
+      </c>
+      <c r="B27" s="30" t="s">
+        <v>205</v>
+      </c>
+      <c r="C27" s="31" t="s">
+        <v>206</v>
+      </c>
+      <c r="D27" s="33" t="s">
+        <v>207</v>
+      </c>
+      <c r="E27" s="36" t="s">
         <v>103</v>
-      </c>
-      <c r="C17" s="19" t="s">
-        <v>104</v>
-      </c>
-      <c r="D17" s="22" t="s">
-        <v>105</v>
-      </c>
-      <c r="E17" s="25" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="18" ht="21.75" customHeight="1">
-      <c r="A18" s="26" t="s">
-        <v>107</v>
-      </c>
-      <c r="B18" s="29" t="s">
-        <v>17</v>
-      </c>
-      <c r="C18" s="19" t="s">
-        <v>109</v>
-      </c>
-      <c r="D18" s="22" t="s">
-        <v>110</v>
-      </c>
-      <c r="E18" s="31" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="19" ht="21.75" customHeight="1">
-      <c r="A19" s="16" t="s">
-        <v>76</v>
-      </c>
-      <c r="B19" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="C19" s="19" t="s">
-        <v>114</v>
-      </c>
-      <c r="D19" s="22" t="s">
-        <v>115</v>
-      </c>
-      <c r="E19" s="25" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="20" ht="21.75" customHeight="1">
-      <c r="A20" s="26" t="s">
-        <v>117</v>
-      </c>
-      <c r="B20" s="29" t="s">
-        <v>118</v>
-      </c>
-      <c r="C20" s="19" t="s">
-        <v>119</v>
-      </c>
-      <c r="D20" s="22" t="s">
-        <v>122</v>
-      </c>
-      <c r="E20" s="31" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="21" ht="21.75" customHeight="1">
-      <c r="A21" s="16" t="s">
-        <v>124</v>
-      </c>
-      <c r="B21" s="17" t="s">
-        <v>125</v>
-      </c>
-      <c r="C21" s="19" t="s">
-        <v>127</v>
-      </c>
-      <c r="D21" s="22" t="s">
-        <v>131</v>
-      </c>
-      <c r="E21" s="25" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="22" ht="21.75" customHeight="1">
-      <c r="A22" s="26" t="s">
-        <v>135</v>
-      </c>
-      <c r="B22" s="29" t="s">
-        <v>17</v>
-      </c>
-      <c r="C22" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="D22" s="22" t="s">
-        <v>140</v>
-      </c>
-      <c r="E22" s="31" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="23" ht="21.75" customHeight="1">
-      <c r="A23" s="16" t="s">
-        <v>142</v>
-      </c>
-      <c r="B23" s="17" t="s">
-        <v>143</v>
-      </c>
-      <c r="C23" s="19" t="s">
-        <v>144</v>
-      </c>
-      <c r="D23" s="22" t="s">
-        <v>145</v>
-      </c>
-      <c r="E23" s="25" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="24" ht="21.75" customHeight="1">
-      <c r="A24" s="26" t="s">
-        <v>148</v>
-      </c>
-      <c r="B24" s="29" t="s">
-        <v>149</v>
-      </c>
-      <c r="C24" s="19" t="s">
-        <v>150</v>
-      </c>
-      <c r="D24" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="E24" s="31" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="25" ht="21.75" customHeight="1">
-      <c r="A25" s="16" t="s">
-        <v>155</v>
-      </c>
-      <c r="B25" s="17" t="s">
-        <v>156</v>
-      </c>
-      <c r="C25" s="19" t="s">
-        <v>127</v>
-      </c>
-      <c r="D25" s="22" t="s">
-        <v>157</v>
-      </c>
-      <c r="E25" s="25" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="26" ht="21.75" customHeight="1">
-      <c r="A26" s="26" t="s">
-        <v>160</v>
-      </c>
-      <c r="B26" s="29" t="s">
-        <v>161</v>
-      </c>
-      <c r="C26" s="19" t="s">
-        <v>162</v>
-      </c>
-      <c r="D26" s="22" t="s">
-        <v>163</v>
-      </c>
-      <c r="E26" s="31" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="27" ht="21.75" customHeight="1">
-      <c r="A27" s="16" t="s">
-        <v>166</v>
-      </c>
-      <c r="B27" s="17" t="s">
-        <v>167</v>
-      </c>
-      <c r="C27" s="19" t="s">
-        <v>168</v>
-      </c>
-      <c r="D27" s="22" t="s">
-        <v>169</v>
-      </c>
-      <c r="E27" s="25" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Atualização automática da planilha (2026-09-19)
</commit_message>
<xml_diff>
--- a/times.xlsx
+++ b/times.xlsx
@@ -16,25 +16,25 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="312">
   <si>
+    <t>GUIA RÁPIDO</t>
+  </si>
+  <si>
     <t>GUIA DE ROTAÇÃO &amp; METAGAME - POKEALLIANCE(PKA)</t>
   </si>
   <si>
     <t>RECOMENDAÇÃO DE TIME PARA HUNTS!</t>
   </si>
   <si>
-    <t>GUIA RÁPIDO</t>
-  </si>
-  <si>
     <t>GUIA VISUAL DE HUNT: CARDS - ELEMENTOS</t>
   </si>
   <si>
     <t>Requisitos de Entrada e Progressão 2x2x2.</t>
   </si>
   <si>
+    <t>https://www.twitch.tv/safnaww</t>
+  </si>
+  <si>
     <t>Segue lá!</t>
-  </si>
-  <si>
-    <t>https://www.twitch.tv/safnaww</t>
   </si>
   <si>
     <t>Com algumas exceções, todos os restantes são SHINYS.</t>
@@ -64,25 +64,43 @@
     <t>📌 REQUISITOS INICIAIS (START DE ROTAÇÃO)</t>
   </si>
   <si>
+    <t>★ METAGROSS</t>
+  </si>
+  <si>
     <t>⚡ UPGRADE: ROTAÇÃO 2x2x2</t>
   </si>
   <si>
-    <t>★ METAGROSS</t>
+    <t>Nessa planilha não indicaremos pokémons T2 ou T3 para a rotação.</t>
+  </si>
+  <si>
+    <t>★ LUCARIO</t>
+  </si>
+  <si>
+    <t>★ BUG</t>
   </si>
   <si>
     <t>Nível &amp; Held:</t>
   </si>
   <si>
+    <t>ELEMENTO / HUNT</t>
+  </si>
+  <si>
+    <t>★ GENGAR</t>
+  </si>
+  <si>
+    <t>Hunt: Steel / Psychic</t>
+  </si>
+  <si>
     <t>Todos os Pokémon +15 com Atk 4</t>
   </si>
   <si>
-    <t>Nessa planilha não indicaremos pokémons T2 ou T3 para a rotação.</t>
+    <t>ALVO (HUNT)</t>
   </si>
   <si>
     <t>Todos os Pokémon +25 com Atk 5</t>
   </si>
   <si>
-    <t>★ LUCARIO</t>
+    <t>Hunt: Fighting / Steel</t>
   </si>
   <si>
     <t>Atalho / Dica:</t>
@@ -91,10 +109,22 @@
     <t>Runas de Atk no Pokelog ajudam a adiantar a meta</t>
   </si>
   <si>
-    <t>★ GENGAR</t>
-  </si>
-  <si>
-    <t>★ BUG</t>
+    <t>🛡️ LURAR (T1)</t>
+  </si>
+  <si>
+    <t>Hunt: Ghost / Poison</t>
+  </si>
+  <si>
+    <t>⚔️ DPS (SR)</t>
+  </si>
+  <si>
+    <t>🎨 TIPO SMEARGLE</t>
+  </si>
+  <si>
+    <t>🛡️ LURAR / TANQUE (T1)</t>
+  </si>
+  <si>
+    <t>Bug</t>
   </si>
   <si>
     <t>Estrelas Mínimas:</t>
@@ -106,22 +136,25 @@
     <t>Meta no Dummy:</t>
   </si>
   <si>
+    <t>⚔️ DPS / DANO (SR)</t>
+  </si>
+  <si>
     <t>Bater 560k de dano com 3 Pokémon</t>
   </si>
   <si>
-    <t>Hunt: Steel / Psychic</t>
-  </si>
-  <si>
-    <t>ELEMENTO / HUNT</t>
-  </si>
-  <si>
     <t>★ FAIRY</t>
   </si>
   <si>
     <t>Bater 560k de dano com apenas 2 Pokémon</t>
   </si>
   <si>
-    <t>ALVO (HUNT)</t>
+    <t>★ FIRE</t>
+  </si>
+  <si>
+    <t>Hunt: Em breve</t>
+  </si>
+  <si>
+    <t>Em breve</t>
   </si>
   <si>
     <t>Regra de Prey:</t>
@@ -130,100 +163,154 @@
     <t>Obrigatório Prey de Atk na hunt (já calculada no dummy)</t>
   </si>
   <si>
+    <t>Hunt: Shiny Sylveon (Lendário)</t>
+  </si>
+  <si>
     <t>Manter sempre Prey de Atk ativa na hunt</t>
   </si>
   <si>
-    <t>Hunt: Fighting / Steel</t>
+    <t>Hunt: Magmar (Lendário) / Torkoal (UR)</t>
   </si>
   <si>
     <t>💡 POR QUE COMPOSIÇÕES COM 2 A 3 ELEMENTOS SÃO SUPERIORES? (ANTI-MONO)</t>
   </si>
   <si>
-    <t>🛡️ LURAR (T1)</t>
-  </si>
-  <si>
-    <t>⚔️ DPS (SR)</t>
-  </si>
-  <si>
-    <t>🎨 TIPO SMEARGLE</t>
-  </si>
-  <si>
-    <t>Hunt: Ghost / Poison</t>
-  </si>
-  <si>
-    <t>Bug</t>
-  </si>
-  <si>
-    <t>★ FIRE</t>
-  </si>
-  <si>
-    <t>Em breve</t>
-  </si>
-  <si>
     <t>Rapidash, Typhlosion, Magcargo</t>
   </si>
   <si>
+    <t>Arcanine, Infernape, Armaldo</t>
+  </si>
+  <si>
+    <t>⭐ S.Rapidash, S.Typhlosion, S.Steelix</t>
+  </si>
+  <si>
+    <t>⭐S.Rapidash, S.Typhlosion, S.Magcargo</t>
+  </si>
+  <si>
+    <t>Fire, Rock</t>
+  </si>
+  <si>
     <t>⏱️ Cooldown Reduzido por Tier</t>
   </si>
   <si>
-    <t>Hunt: Em breve</t>
-  </si>
-  <si>
-    <t>Arcanine, Infernape, Armaldo</t>
-  </si>
-  <si>
-    <t>🛡️ LURAR / TANQUE (T1)</t>
-  </si>
-  <si>
-    <t>Hunt: Shiny Sylveon (Lendário)</t>
-  </si>
-  <si>
-    <t>Fire, Rock</t>
+    <t>⭐ Arcanine, Houndoom, Pupitar</t>
+  </si>
+  <si>
+    <t>⭐ Arcanine, Infernape, Armaldo</t>
+  </si>
+  <si>
+    <t>⭐ Muk, Tentacruel, Mawile</t>
+  </si>
+  <si>
+    <t>⭐ Hitmontop, Typhlosion, Rapidash</t>
+  </si>
+  <si>
+    <t>⭐ Aggron, Skarmory, Toxicroak</t>
+  </si>
+  <si>
+    <t>⭐ Arcanine, Machamp, Pupitar</t>
+  </si>
+  <si>
+    <t>⭐ Blastoise, Feraligatr, Omastar</t>
+  </si>
+  <si>
+    <t>⭐ Umbreon, Crawdaunt, Sableye</t>
+  </si>
+  <si>
+    <t>⭐ Pupitar, Torterra, Kingdra</t>
+  </si>
+  <si>
+    <t>⭐ Houndoom, Hydreigon, Pupitar</t>
+  </si>
+  <si>
+    <t>Outras Opções T1:</t>
+  </si>
+  <si>
+    <t>Outras Opções SR:</t>
+  </si>
+  <si>
+    <t>Fairy</t>
+  </si>
+  <si>
+    <t>S.Charizard, Kabutops, Golem</t>
   </si>
   <si>
     <t>No PKA, tiers mais altos não dão só dano: reduzem o cooldown das skills, deixando a rotação muito mais rápida.</t>
   </si>
   <si>
-    <t>Hunt: Magmar (Lendário) / Torkoal (UR)</t>
-  </si>
-  <si>
-    <t>⚔️ DPS / DANO (SR)</t>
-  </si>
-  <si>
-    <t>Fairy</t>
+    <t>Umbreon</t>
+  </si>
+  <si>
+    <t>Shiny Sylveon (Lendário)</t>
   </si>
   <si>
     <t>📈 Mais Mobs e Brokes / Hora</t>
   </si>
   <si>
-    <t>Shiny Sylveon (Lendário)</t>
-  </si>
-  <si>
-    <t>⭐ S.Rapidash, S.Typhlosion, S.Steelix</t>
+    <t>—</t>
   </si>
   <si>
     <t>Rotação mais fluida = mais mobs derrotados/hora, aumentando drasticamente a chance de Shiny/hr e lucro.</t>
   </si>
   <si>
+    <t>Metang, Magneton Estrelado</t>
+  </si>
+  <si>
+    <t>SevIper</t>
+  </si>
+  <si>
+    <t>Torterra, Misdreavus</t>
+  </si>
+  <si>
+    <t>Poliwrath, Medicham, Hariyama</t>
+  </si>
+  <si>
+    <t>Infernape, Kangaskhan, Torterra</t>
+  </si>
+  <si>
+    <t>Vaporeon, Rhyperior, Magcargo</t>
+  </si>
+  <si>
+    <t>Sharpedo</t>
+  </si>
+  <si>
+    <t>Cacturne, Banette, Dusclops</t>
+  </si>
+  <si>
+    <t>⚔️ Hazards Mais Altos</t>
+  </si>
+  <si>
+    <t>Misdreavus, Dusknoir, Torterra</t>
+  </si>
+  <si>
+    <t>🎨 Smeargle: Fire, Rock</t>
+  </si>
+  <si>
     <t>Muk, Tentacruel, Mawile</t>
   </si>
   <si>
+    <t>Mesmo encurtando o número total de hunts, permite solar níveis de Hazard superiores com segurança e eficiência.</t>
+  </si>
+  <si>
+    <t>🎨 Smeargle: Fire, Ground, Ghost, Dark</t>
+  </si>
+  <si>
     <t>Aggron, Skarmory, Toxicroak</t>
   </si>
   <si>
+    <t>🎨 Smeargle: Poison, Metal</t>
+  </si>
+  <si>
     <t>Poison, Metal</t>
   </si>
   <si>
-    <t>⭐ Arcanine, Houndoom, Pupitar</t>
-  </si>
-  <si>
-    <t>⭐S.Rapidash, S.Typhlosion, S.Magcargo</t>
-  </si>
-  <si>
-    <t>⚔️ Hazards Mais Altos</t>
-  </si>
-  <si>
-    <t>⭐ Arcanine, Infernape, Armaldo</t>
+    <t>🏆 Futuro &amp; Escalabilidade (Endgame)</t>
+  </si>
+  <si>
+    <t>🎨 Smeargle: Fighting, Fire, Ground</t>
+  </si>
+  <si>
+    <t>🎨 Smeargle: Rock, Water, Ground</t>
   </si>
   <si>
     <t>Fire</t>
@@ -232,64 +319,40 @@
     <t>Magmar (Lendário) / Torkoal (UR)</t>
   </si>
   <si>
+    <t>Trabalhar com 2 ou 3 elementos abre um catálogo amplo de opções viáveis para evoluir: T1, SR, UR e Lendários.</t>
+  </si>
+  <si>
     <t>Blastoise, Feraligatr, Omastar</t>
   </si>
   <si>
-    <t>⭐ Hitmontop, Typhlosion, Rapidash</t>
-  </si>
-  <si>
-    <t>Mesmo encurtando o número total de hunts, permite solar níveis de Hazard superiores com segurança e eficiência.</t>
-  </si>
-  <si>
     <t>Pupitar, Torterra, Kingdra</t>
   </si>
   <si>
-    <t>⭐ Muk, Tentacruel, Mawile</t>
-  </si>
-  <si>
     <t>Rock, Water, Ground</t>
   </si>
   <si>
-    <t>⭐ Arcanine, Machamp, Pupitar</t>
-  </si>
-  <si>
-    <t>⭐ Aggron, Skarmory, Toxicroak</t>
+    <t>★ FIGHTING</t>
+  </si>
+  <si>
+    <t>🎨 Smeargle: Dark, Ghost, Ground</t>
   </si>
   <si>
     <t>Fighting</t>
   </si>
   <si>
-    <t>⭐ Umbreon, Crawdaunt, Sableye</t>
-  </si>
-  <si>
-    <t>⭐ Blastoise, Feraligatr, Omastar</t>
-  </si>
-  <si>
-    <t>⭐ Houndoom, Hydreigon, Pupitar</t>
-  </si>
-  <si>
     <t>Mega Clefable, Pidgeot, Espeon</t>
   </si>
   <si>
-    <t>🏆 Futuro &amp; Escalabilidade (Endgame)</t>
-  </si>
-  <si>
-    <t>⭐ Pupitar, Torterra, Kingdra</t>
-  </si>
-  <si>
     <t>Wobbuffet, Mimikyu, Gliscor</t>
   </si>
   <si>
     <t>Psychic, Flying, Fairy</t>
   </si>
   <si>
-    <t>Outras Opções T1:</t>
-  </si>
-  <si>
     <t>Dark</t>
   </si>
   <si>
-    <t>Trabalhar com 2 ou 3 elementos abre um catálogo amplo de opções viáveis para evoluir: T1, SR, UR e Lendários.</t>
+    <t>★ DARK</t>
   </si>
   <si>
     <t>Absol (Lendário) / Mightyena (UR)</t>
@@ -298,15 +361,15 @@
     <t>Hitmontop, Hitmonchan, Poliwrath</t>
   </si>
   <si>
+    <t>★ GARDEVOIR</t>
+  </si>
+  <si>
     <t>Machamp, Scyther, Mimikyu</t>
   </si>
   <si>
     <t>Fighting, Fairy, Bug</t>
   </si>
   <si>
-    <t>Outras Opções SR:</t>
-  </si>
-  <si>
     <t>Water</t>
   </si>
   <si>
@@ -316,15 +379,18 @@
     <t>Tangrowth, Ampharos, Venusaur</t>
   </si>
   <si>
+    <t>★ GYARADOS</t>
+  </si>
+  <si>
+    <t>★ WATER</t>
+  </si>
+  <si>
     <t>Tangrowth, Gogoat, Luxray</t>
   </si>
   <si>
     <t>Grass, Electric</t>
   </si>
   <si>
-    <t>Umbreon</t>
-  </si>
-  <si>
     <t>Grass</t>
   </si>
   <si>
@@ -340,7 +406,7 @@
     <t>Poison, Bug, Fire, Fly, Ice</t>
   </si>
   <si>
-    <t>S.Charizard, Kabutops, Golem</t>
+    <t>★ SWAMPERT</t>
   </si>
   <si>
     <t>Electric</t>
@@ -349,42 +415,33 @@
     <t>Electabuzz (Lendário) / Manectric (UR)</t>
   </si>
   <si>
-    <t>Torterra, Misdreavus</t>
-  </si>
-  <si>
     <t>Steelix, Nidoqueen, Torterra</t>
   </si>
   <si>
-    <t>Poliwrath, Medicham, Hariyama</t>
-  </si>
-  <si>
     <t>Torterra, Pupitar, Smeargle</t>
   </si>
   <si>
-    <t>Infernape, Kangaskhan, Torterra</t>
+    <t>Hunt: Absol (Lendário) / Mightyena (UR)</t>
   </si>
   <si>
     <t>Ground</t>
   </si>
   <si>
-    <t>Cacturne, Banette, Dusclops</t>
-  </si>
-  <si>
-    <t>Misdreavus, Dusknoir, Torterra</t>
-  </si>
-  <si>
     <t>Ghost</t>
   </si>
   <si>
+    <t>Hunt: Milotic (UR)</t>
+  </si>
+  <si>
+    <t>Hunt: Psychic / Fairy</t>
+  </si>
+  <si>
     <t>Umbreon, Crawdaunt, Dusknoir</t>
   </si>
   <si>
     <t>Dusknoir, Houndoom, Hydreigon</t>
   </si>
   <si>
-    <t>🎨 Smeargle: Fire, Ground, Ghost, Dark</t>
-  </si>
-  <si>
     <t>Dark, Ghost</t>
   </si>
   <si>
@@ -394,7 +451,7 @@
     <t>Glaceon (Lendário) / Glalie (UR)</t>
   </si>
   <si>
-    <t>—</t>
+    <t>Hunt: Water / Flying</t>
   </si>
   <si>
     <t>Typhlosion, Rapidash, Hitmontop</t>
@@ -403,40 +460,43 @@
     <t>Infernape, Machamp, Skarmory</t>
   </si>
   <si>
-    <t>Metang, Magneton Estrelado</t>
-  </si>
-  <si>
     <t>Fighting, Fire, Metal</t>
   </si>
   <si>
-    <t>🎨 Smeargle: Fighting, Fire, Ground</t>
+    <t>⭐ Mega Clefable, Pidgeot, Espeon</t>
   </si>
   <si>
     <t>Poison</t>
   </si>
   <si>
-    <t>SevIper</t>
+    <t>⭐ Wobbuffet, Mimikyu, Gliscor</t>
   </si>
   <si>
     <t>Garbodor (Lendário) / Swalot (UR)</t>
   </si>
   <si>
+    <t>⭐ Hitmontop, Hitmonchan, Poliwrath</t>
+  </si>
+  <si>
     <t>Steelix, Espeon, Nidoqueen</t>
   </si>
   <si>
+    <t>⭐ Machamp, Scyther, Mimikyu</t>
+  </si>
+  <si>
+    <t>Hunt: Water / Ground</t>
+  </si>
+  <si>
     <t>Wobbuffet, Mr. Mime, Pupitar</t>
   </si>
   <si>
+    <t>⭐ Tangrowth, Ampharos, Venusaur</t>
+  </si>
+  <si>
     <t>Ground, Psychic</t>
   </si>
   <si>
-    <t>🎨 Smeargle: Dark, Ghost, Ground</t>
-  </si>
-  <si>
-    <t>Vaporeon, Rhyperior, Magcargo</t>
-  </si>
-  <si>
-    <t>Sharpedo</t>
+    <t>⭐ Tangrowth, Gogoat, Luxray</t>
   </si>
   <si>
     <t>Normal</t>
@@ -451,49 +511,67 @@
     <t>Machamp, Kangaskhan, Smeargle</t>
   </si>
   <si>
-    <t>🎨 Smeargle: Fire, Rock</t>
+    <t>Farfetch'd, Gliscor</t>
+  </si>
+  <si>
+    <t>Mr. Mime, Florges, Swellow</t>
+  </si>
+  <si>
+    <t>Mega Clefable, Hitmonlee</t>
   </si>
   <si>
     <t>Rock</t>
   </si>
   <si>
+    <t>Florges, Kangaskhan, Pinsir</t>
+  </si>
+  <si>
     <t>Rampardos (UR)</t>
   </si>
   <si>
-    <t>★ GARDEVOIR</t>
+    <t>Luxray, Gogoat</t>
   </si>
   <si>
     <t>Tangrowth, Steelix, Blastoise</t>
   </si>
   <si>
+    <t>Pachirisu</t>
+  </si>
+  <si>
     <t>Tangrowth, Machamp, Gogoat</t>
   </si>
   <si>
     <t>Fighting, Ground, Water, Grass</t>
   </si>
   <si>
-    <t>🎨 Smeargle: Poison, Metal</t>
+    <t>🎨 Smeargle: Psychic, Flying, Fairy</t>
   </si>
   <si>
     <t>Steel</t>
   </si>
   <si>
-    <t>★ GYARADOS</t>
+    <t>⭐ Mawile, Muk, Tentacruel</t>
+  </si>
+  <si>
+    <t>🎨 Smeargle: Fighting, Fairy, Bug</t>
   </si>
   <si>
     <t>Hitmontop, Rapidash, Typhlosion</t>
   </si>
   <si>
+    <t>⭐ Toxicroak, Seviper, Misdreavus</t>
+  </si>
+  <si>
     <t>Arcanine, Machamp, Infernape</t>
   </si>
   <si>
+    <t>⭐ Ampharos, Luxray, Jolteon</t>
+  </si>
+  <si>
     <t>Ground, Fighting, Fire</t>
   </si>
   <si>
-    <t>🎨 Smeargle: Rock, Water, Ground</t>
-  </si>
-  <si>
-    <t>★ SWAMPERT</t>
+    <t>🎨 Smeargle: Grass, Electric</t>
   </si>
   <si>
     <t>Blastoise, Tangrowth, Gogoat</t>
@@ -505,9 +583,15 @@
     <t>Water, Ice, Grass</t>
   </si>
   <si>
+    <t>⭐ S.Luxray, S.Pachirisu, Smeargle Eletric</t>
+  </si>
+  <si>
     <t>Dragon</t>
   </si>
   <si>
+    <t>★ GRASS</t>
+  </si>
+  <si>
     <t>Salamence (UR) / Flygon (Lendário)</t>
   </si>
   <si>
@@ -517,18 +601,21 @@
     <t>Mimikyu, Florges, Walrein</t>
   </si>
   <si>
-    <t>Hunt: Psychic / Fairy</t>
+    <t>⭐Venusaur, Gogoat, Tangrowth</t>
   </si>
   <si>
     <t>Dragon, Ice, Fairy</t>
   </si>
   <si>
-    <t>★ FIGHTING</t>
+    <t>⭐ S.Tangrowth,S. Gogoat, Smeargle Grass</t>
   </si>
   <si>
     <t>Psychic</t>
   </si>
   <si>
+    <t>★ ELECTRIC</t>
+  </si>
+  <si>
     <t>Alakazam (Lendário)</t>
   </si>
   <si>
@@ -538,28 +625,31 @@
     <t>Houndoom, Scyther, Dusknoir</t>
   </si>
   <si>
-    <t>Hunt: Water / Flying</t>
-  </si>
-  <si>
     <t>Ghost, Dark, Bug</t>
   </si>
   <si>
     <t>Flying</t>
   </si>
   <si>
+    <t>★ GHOST</t>
+  </si>
+  <si>
     <t>Ampharos, Magcargo, Lapras</t>
   </si>
   <si>
     <t>Walrein, Luxray, Pachirisu</t>
   </si>
   <si>
-    <t>Hunt: Water / Ground</t>
+    <t>Metang, Banette, Dusclops, Nidoking</t>
   </si>
   <si>
     <t>Electric, Ice, Rock</t>
   </si>
   <si>
-    <t>★ DARK</t>
+    <t>Aggron, Skarmory</t>
+  </si>
+  <si>
+    <t>Raichu</t>
   </si>
   <si>
     <t>Metagross</t>
@@ -568,6 +658,9 @@
     <t>Steel / Psychic</t>
   </si>
   <si>
+    <t>Hunt: Leafeon (Lendário) / Sceptile (UR)</t>
+  </si>
+  <si>
     <t>Rapidash, Typhlosion, Steelix</t>
   </si>
   <si>
@@ -577,6 +670,12 @@
     <t>Fire, Ground, Ghost, Dark</t>
   </si>
   <si>
+    <t>Hunt: Electabuzz (Lendário) / Manectric (UR)</t>
+  </si>
+  <si>
+    <t>🎨 Smeargle: Poison, Ghost, Metal</t>
+  </si>
+  <si>
     <t>Lucario</t>
   </si>
   <si>
@@ -586,69 +685,66 @@
     <t>Hitmontop, Typhlosion, Rapidash</t>
   </si>
   <si>
-    <t>★ WATER</t>
-  </si>
-  <si>
     <t>Arcanine, Machamp, Pupitar</t>
   </si>
   <si>
     <t>Fighting, Fire, Ground</t>
   </si>
   <si>
+    <t>🎨 Smeargle: Electric</t>
+  </si>
+  <si>
     <t>Gengar</t>
   </si>
   <si>
-    <t>⭐ Mawile, Muk, Tentacruel</t>
-  </si>
-  <si>
     <t>Ghost / Poison</t>
   </si>
   <si>
-    <t>⭐ Toxicroak, Seviper, Misdreavus</t>
-  </si>
-  <si>
-    <t>⭐ Ampharos, Luxray, Jolteon</t>
-  </si>
-  <si>
     <t>Houndoom, Hydreigon, Pupitar</t>
   </si>
   <si>
-    <t>⭐ S.Luxray, S.Pachirisu, Smeargle Eletric</t>
-  </si>
-  <si>
     <t>Dark, Ghost, Ground</t>
   </si>
   <si>
+    <t>⭐ Typhlosion, Rapidash, Pidgeot</t>
+  </si>
+  <si>
     <t>Gardevoir</t>
   </si>
   <si>
-    <t>⭐Venusaur, Gogoat, Tangrowth</t>
+    <t>⭐ Arcanine, Infernape, Scyther</t>
   </si>
   <si>
     <t>Psychic / Fairy</t>
   </si>
   <si>
-    <t>⭐ S.Tangrowth,S. Gogoat, Smeargle Grass</t>
+    <t>🎨 Smeargle: Grass</t>
+  </si>
+  <si>
+    <t>⭐ Steelix, Nidoqueen, Torterra</t>
   </si>
   <si>
     <t>Mawile, Muk, Tentacruel</t>
   </si>
   <si>
-    <t>Hunt: Absol (Lendário) / Mightyena (UR)</t>
+    <t>⭐ Torterra, Pupitar, Smeargle</t>
   </si>
   <si>
     <t>Toxicroak, Seviper, Misdreavus</t>
   </si>
   <si>
+    <t>⭐ Umbreon, Crawdaunt, Dusknoir</t>
+  </si>
+  <si>
     <t>Poison, Ghost, Metal</t>
   </si>
   <si>
+    <t>⭐ Dusknoir, Houndoom, Hydreigon</t>
+  </si>
+  <si>
     <t>Gyarados</t>
   </si>
   <si>
-    <t>Hunt: Milotic (UR)</t>
-  </si>
-  <si>
     <t>Water / Flying</t>
   </si>
   <si>
@@ -658,145 +754,49 @@
     <t>Luxray, Pachirisu, Smeargle Eletric</t>
   </si>
   <si>
-    <t>Metang, Banette, Dusclops, Nidoking</t>
-  </si>
-  <si>
-    <t>Aggron, Skarmory</t>
-  </si>
-  <si>
-    <t>Raichu</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Poison, Ghost, Metal</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Electric</t>
-  </si>
-  <si>
-    <t>⭐ Mega Clefable, Pidgeot, Espeon</t>
-  </si>
-  <si>
-    <t>⭐ Wobbuffet, Mimikyu, Gliscor</t>
-  </si>
-  <si>
-    <t>⭐ Hitmontop, Hitmonchan, Poliwrath</t>
-  </si>
-  <si>
-    <t>⭐ Machamp, Scyther, Mimikyu</t>
-  </si>
-  <si>
-    <t>⭐ Tangrowth, Ampharos, Venusaur</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Grass</t>
-  </si>
-  <si>
-    <t>⭐ Tangrowth, Gogoat, Luxray</t>
-  </si>
-  <si>
     <t>★ SCIZOR</t>
   </si>
   <si>
-    <t>Farfetch'd, Gliscor</t>
-  </si>
-  <si>
-    <t>Mr. Mime, Florges, Swellow</t>
-  </si>
-  <si>
-    <t>Mega Clefable, Hitmonlee</t>
-  </si>
-  <si>
-    <t>Florges, Kangaskhan, Pinsir</t>
-  </si>
-  <si>
-    <t>Luxray, Gogoat</t>
-  </si>
-  <si>
-    <t>Pachirisu</t>
+    <t>Charizard, Lapras, Jynx, Gliscor</t>
+  </si>
+  <si>
+    <t>Gliscor, Swellow, Walrein, Toxicroak</t>
+  </si>
+  <si>
+    <t>Marowak, Whiscash, Claydol</t>
+  </si>
+  <si>
+    <t>Marowak</t>
+  </si>
+  <si>
+    <t>Dusclops, Sableye, Cacturne</t>
+  </si>
+  <si>
+    <t>Misdreavus</t>
   </si>
   <si>
     <t>Hunt: Bug</t>
   </si>
   <si>
-    <t>🎨 Smeargle: Psychic, Flying, Fairy</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Fighting, Fairy, Bug</t>
+    <t>🎨 Smeargle: Poison, Bug, Fire, Fly, Ice</t>
+  </si>
+  <si>
+    <t>🎨 Smeargle: Ground</t>
+  </si>
+  <si>
+    <t>🎨 Smeargle: Dark, Ghost</t>
   </si>
   <si>
     <t>⭐ S.Rapidash, S.Typhlosion, S.Zard</t>
   </si>
   <si>
-    <t>🎨 Smeargle: Grass, Electric</t>
-  </si>
-  <si>
     <t>⭐S.Arcanine, S.Infernape, Smeargle Fire</t>
   </si>
   <si>
-    <t>★ GRASS</t>
+    <t>★ ICE</t>
   </si>
   <si>
     <t>🎨 Smeargle: Fire</t>
-  </si>
-  <si>
-    <t>★ ELECTRIC</t>
-  </si>
-  <si>
-    <t>★ GHOST</t>
-  </si>
-  <si>
-    <t>Hunt: Leafeon (Lendário) / Sceptile (UR)</t>
-  </si>
-  <si>
-    <t>Hunt: Electabuzz (Lendário) / Manectric (UR)</t>
-  </si>
-  <si>
-    <t>⭐ Typhlosion, Rapidash, Pidgeot</t>
-  </si>
-  <si>
-    <t>⭐ Arcanine, Infernape, Scyther</t>
-  </si>
-  <si>
-    <t>⭐ Steelix, Nidoqueen, Torterra</t>
-  </si>
-  <si>
-    <t>⭐ Torterra, Pupitar, Smeargle</t>
-  </si>
-  <si>
-    <t>⭐ Umbreon, Crawdaunt, Dusknoir</t>
-  </si>
-  <si>
-    <t>⭐ Dusknoir, Houndoom, Hydreigon</t>
-  </si>
-  <si>
-    <t>Charizard, Lapras, Jynx, Gliscor</t>
-  </si>
-  <si>
-    <t>Gliscor, Swellow, Walrein, Toxicroak</t>
-  </si>
-  <si>
-    <t>Marowak, Whiscash, Claydol</t>
-  </si>
-  <si>
-    <t>Marowak</t>
-  </si>
-  <si>
-    <t>Dusclops, Sableye, Cacturne</t>
-  </si>
-  <si>
-    <t>Misdreavus</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Poison, Bug, Fire, Fly, Ice</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Ground</t>
-  </si>
-  <si>
-    <t>🎨 Smeargle: Dark, Ghost</t>
-  </si>
-  <si>
-    <t>★ ICE</t>
   </si>
   <si>
     <t>★ POISON</t>
@@ -980,6 +980,12 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13.0"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Quattrocento Sans"/>
     </font>
     <font>
       <b/>
@@ -1000,9 +1006,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="13.0"/>
-      <color rgb="FFFFFFFF"/>
+      <i/>
+      <sz val="9.0"/>
+      <color rgb="FFD1D5DB"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1011,27 +1017,9 @@
     </font>
     <font>
       <i/>
-      <sz val="9.0"/>
-      <color rgb="FFD1D5DB"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <i/>
       <u/>
       <sz val="9.0"/>
       <color rgb="FF0000FF"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10.0"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9.0"/>
-      <color rgb="FF334155"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1043,8 +1031,20 @@
     </font>
     <font>
       <b/>
+      <sz val="10.0"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11.0"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9.0"/>
+      <color rgb="FF334155"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1054,14 +1054,20 @@
       <name val="Quattrocento Sans"/>
     </font>
     <font>
+      <i/>
+      <sz val="9.0"/>
+      <color rgb="FFF3F4F6"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
       <sz val="9.0"/>
       <color rgb="FF0F172A"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
-      <i/>
+      <b/>
       <sz val="9.0"/>
-      <color rgb="FFF3F4F6"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1084,30 +1090,7 @@
     <font>
       <b/>
       <sz val="9.0"/>
-      <color rgb="FF1E3A8A"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9.0"/>
       <color rgb="FF991B1B"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9.0"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9.0"/>
-      <color rgb="FF1E40AF"/>
-      <name val="Quattrocento Sans"/>
-    </font>
-    <font>
-      <sz val="9.0"/>
-      <color rgb="FF1F2937"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1118,8 +1101,25 @@
     </font>
     <font>
       <b/>
+      <sz val="9.0"/>
+      <color rgb="FF1E40AF"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
       <sz val="8.0"/>
       <color rgb="FF4B5563"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9.0"/>
+      <color rgb="FF1E3A8A"/>
+      <name val="Quattrocento Sans"/>
+    </font>
+    <font>
+      <sz val="9.0"/>
+      <color rgb="FF1F2937"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
@@ -1130,13 +1130,13 @@
     <font>
       <b/>
       <sz val="8.0"/>
-      <color rgb="FF1E3A8A"/>
+      <color rgb="FF4A4A4A"/>
       <name val="Quattrocento Sans"/>
     </font>
     <font>
       <b/>
       <sz val="8.0"/>
-      <color rgb="FF4A4A4A"/>
+      <color rgb="FF1E3A8A"/>
       <name val="Quattrocento Sans"/>
     </font>
   </fonts>
@@ -1149,14 +1149,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0F172A"/>
-        <bgColor rgb="FF0F172A"/>
+        <fgColor rgb="FF1B2A4A"/>
+        <bgColor rgb="FF1B2A4A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1B2A4A"/>
-        <bgColor rgb="FF1B2A4A"/>
+        <fgColor rgb="FF0F172A"/>
+        <bgColor rgb="FF0F172A"/>
       </patternFill>
     </fill>
     <fill>
@@ -1173,14 +1173,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+        <bgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFF1F5F9"/>
         <bgColor rgb="FFF1F5F9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E78"/>
-        <bgColor rgb="FF1F4E78"/>
+        <fgColor rgb="FF374151"/>
+        <bgColor rgb="FF374151"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E7D32"/>
+        <bgColor rgb="FF2E7D32"/>
       </patternFill>
     </fill>
     <fill>
@@ -1197,20 +1209,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFE68D9C"/>
+        <bgColor rgb="FFE68D9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEA6C2D"/>
+        <bgColor rgb="FFEA6C2D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFEF3C7"/>
         <bgColor rgb="FFFEF3C7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF374151"/>
-        <bgColor rgb="FF374151"/>
+        <fgColor rgb="FFC62828"/>
+        <bgColor rgb="FFC62828"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE68D9C"/>
-        <bgColor rgb="FFE68D9C"/>
+        <fgColor rgb="FFF0FDF4"/>
+        <bgColor rgb="FFF0FDF4"/>
       </patternFill>
     </fill>
     <fill>
@@ -1221,44 +1245,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEA6C2D"/>
-        <bgColor rgb="FFEA6C2D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF0FDF4"/>
-        <bgColor rgb="FFF0FDF4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEFF6FF"/>
-        <bgColor rgb="FFEFF6FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFEF2F2"/>
         <bgColor rgb="FFFEF2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF2E7D32"/>
-        <bgColor rgb="FF2E7D32"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC62828"/>
-        <bgColor rgb="FFC62828"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF8FAFC"/>
-        <bgColor rgb="FFF8FAFC"/>
       </patternFill>
     </fill>
     <fill>
@@ -1277,6 +1265,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF0F4F8"/>
         <bgColor rgb="FFF0F4F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEFF6FF"/>
+        <bgColor rgb="FFEFF6FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8FAFC"/>
+        <bgColor rgb="FFF8FAFC"/>
       </patternFill>
     </fill>
     <fill>
@@ -1400,20 +1400,6 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFCBD5E1"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCBD5E1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCBD5E1"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
         <color rgb="FFD1D5DB"/>
       </left>
       <top style="thin">
@@ -1432,6 +1418,20 @@
       </top>
       <bottom style="thin">
         <color rgb="FFD1D5DB"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCBD5E1"/>
       </bottom>
     </border>
     <border>
@@ -1489,196 +1489,196 @@
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="1" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="5" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="6" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="6" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="6" fillId="7" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="7" fillId="5" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="6" fillId="4" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="8" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="5" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="7" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="4" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="9" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="10" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="4" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="11" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="6" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="4" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="5" fillId="8" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="9" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="7" fillId="5" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="10" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="5" fillId="11" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="7" fillId="5" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="12" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="13" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="7" fillId="4" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="14" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="12" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="7" fillId="4" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="15" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="13" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="6" fillId="14" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="15" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="8" fillId="16" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="7" fillId="4" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="16" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="17" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="17" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="18" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="9" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="7" fillId="18" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf borderId="7" fillId="19" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="20" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="19" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="7" fillId="4" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="8" fillId="4" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="7" fillId="21" fontId="23" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="8" fillId="22" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="9" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="7" fillId="23" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="8" fillId="4" fontId="25" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="7" fillId="19" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf borderId="10" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="7" fillId="20" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="7" fillId="20" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="7" fillId="21" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="10" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="7" fillId="24" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="7" fillId="20" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="7" fillId="22" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="7" fillId="21" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="7" fillId="23" fontId="25" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="7" fillId="24" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="7" fillId="24" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="7" fillId="24" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="5" fillId="25" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="7" fillId="23" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="24" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="25" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="23" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="26" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="27" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="28" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="6" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="8" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="7" fillId="20" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="5" fillId="7" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="29" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="30" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="31" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="4" fillId="25" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="26" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="32" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="11" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="27" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="33" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="28" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="34" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="7" fillId="22" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="5" fillId="25" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="29" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="35" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="30" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="36" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="31" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="37" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="32" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="38" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="33" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="39" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="34" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="35" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="36" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="37" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="38" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="39" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="40" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="40" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1920,155 +1920,155 @@
   </cols>
   <sheetData>
     <row r="2" ht="33.75" customHeight="1">
-      <c r="B2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="3"/>
+      <c r="B2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="5"/>
     </row>
     <row r="3" ht="19.5" customHeight="1">
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="3"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="5"/>
     </row>
     <row r="4">
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="E4" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="F4" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="5" ht="24.0" customHeight="1">
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="3"/>
-      <c r="E5" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" s="3"/>
+      <c r="C5" s="5"/>
+      <c r="E5" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="5"/>
     </row>
     <row r="6" ht="24.75" customHeight="1">
-      <c r="B6" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="17" t="s">
+      <c r="B6" s="17" t="s">
         <v>15</v>
       </c>
+      <c r="C6" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="19" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="7" ht="24.75" customHeight="1">
-      <c r="B7" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="F7" s="19" t="s">
-        <v>22</v>
+      <c r="B7" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" s="22" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="8" ht="24.75" customHeight="1">
-      <c r="B8" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="C8" s="21" t="s">
-        <v>24</v>
-      </c>
-      <c r="E8" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="F8" s="23" t="s">
-        <v>28</v>
+      <c r="B8" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="25" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="F8" s="29" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="9" ht="24.75" customHeight="1">
-      <c r="B9" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="E9" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="F9" s="19" t="s">
-        <v>32</v>
+      <c r="B9" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="E9" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" s="22" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="11" ht="24.0" customHeight="1">
-      <c r="B11" s="27" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="3"/>
+      <c r="B11" s="33" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="5"/>
     </row>
     <row r="12" ht="24.0" customHeight="1">
-      <c r="B12" s="32" t="s">
-        <v>43</v>
-      </c>
-      <c r="C12" s="34"/>
-      <c r="D12" s="37" t="s">
-        <v>49</v>
-      </c>
-      <c r="E12" s="39"/>
-      <c r="F12" s="34"/>
+      <c r="B12" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="C12" s="41"/>
+      <c r="D12" s="43" t="s">
+        <v>67</v>
+      </c>
+      <c r="E12" s="44"/>
+      <c r="F12" s="41"/>
     </row>
     <row r="13" ht="24.0" customHeight="1">
-      <c r="B13" s="32" t="s">
-        <v>53</v>
-      </c>
-      <c r="C13" s="34"/>
-      <c r="D13" s="37" t="s">
-        <v>56</v>
-      </c>
-      <c r="E13" s="39"/>
-      <c r="F13" s="34"/>
+      <c r="B13" s="40" t="s">
+        <v>70</v>
+      </c>
+      <c r="C13" s="41"/>
+      <c r="D13" s="43" t="s">
+        <v>72</v>
+      </c>
+      <c r="E13" s="44"/>
+      <c r="F13" s="41"/>
     </row>
     <row r="14" ht="24.0" customHeight="1">
-      <c r="B14" s="32" t="s">
-        <v>62</v>
-      </c>
-      <c r="C14" s="34"/>
-      <c r="D14" s="37" t="s">
-        <v>68</v>
-      </c>
-      <c r="E14" s="39"/>
-      <c r="F14" s="34"/>
+      <c r="B14" s="40" t="s">
+        <v>81</v>
+      </c>
+      <c r="C14" s="41"/>
+      <c r="D14" s="43" t="s">
+        <v>85</v>
+      </c>
+      <c r="E14" s="44"/>
+      <c r="F14" s="41"/>
     </row>
     <row r="15" ht="24.0" customHeight="1">
-      <c r="B15" s="32" t="s">
-        <v>79</v>
-      </c>
-      <c r="C15" s="34"/>
-      <c r="D15" s="37" t="s">
-        <v>85</v>
-      </c>
-      <c r="E15" s="39"/>
-      <c r="F15" s="34"/>
+      <c r="B15" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="C15" s="41"/>
+      <c r="D15" s="43" t="s">
+        <v>95</v>
+      </c>
+      <c r="E15" s="44"/>
+      <c r="F15" s="41"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -3097,525 +3097,525 @@
       <c r="A1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="3"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="5"/>
       <c r="I1" s="9" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" ht="19.5" customHeight="1">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="3"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="5"/>
       <c r="I2" s="9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" ht="21.75" customHeight="1">
+      <c r="A4" s="24" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" ht="21.75" customHeight="1">
-      <c r="A4" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="18"/>
+      <c r="B4" s="16"/>
       <c r="D4" s="26" t="s">
-        <v>27</v>
-      </c>
-      <c r="E4" s="18"/>
-      <c r="G4" s="29" t="s">
-        <v>40</v>
-      </c>
-      <c r="H4" s="18"/>
+        <v>36</v>
+      </c>
+      <c r="E4" s="16"/>
+      <c r="G4" s="28" t="s">
+        <v>38</v>
+      </c>
+      <c r="H4" s="16"/>
     </row>
     <row r="5" ht="18.0" customHeight="1">
-      <c r="A5" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="B5" s="18"/>
-      <c r="D5" s="24" t="s">
-        <v>47</v>
-      </c>
-      <c r="E5" s="18"/>
-      <c r="G5" s="24" t="s">
+      <c r="A5" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="16"/>
+      <c r="D5" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="E5" s="16"/>
+      <c r="G5" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="H5" s="16"/>
+    </row>
+    <row r="6" ht="19.5" customHeight="1">
+      <c r="A6" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="H6" s="30" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" ht="42.0" customHeight="1">
+      <c r="A7" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="H5" s="18"/>
-    </row>
-    <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="B6" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="D6" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="E6" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="G6" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="H6" s="38" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="7" ht="42.0" customHeight="1">
-      <c r="A7" s="42" t="s">
+      <c r="B7" s="36" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" s="37" t="s">
+        <v>55</v>
+      </c>
+      <c r="E7" s="36" t="s">
+        <v>57</v>
+      </c>
+      <c r="G7" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="H7" s="36" t="s">
         <v>61</v>
       </c>
-      <c r="B7" s="44" t="s">
+    </row>
+    <row r="8" ht="15.0" customHeight="1">
+      <c r="A8" s="39" t="s">
         <v>63</v>
       </c>
-      <c r="D7" s="45" t="s">
-        <v>70</v>
-      </c>
-      <c r="E7" s="44" t="s">
+      <c r="B8" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="D8" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="E8" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="G8" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="H8" s="39" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9" ht="27.75" customHeight="1">
+      <c r="A9" s="45" t="s">
+        <v>66</v>
+      </c>
+      <c r="B9" s="46" t="s">
+        <v>71</v>
+      </c>
+      <c r="D9" s="46" t="s">
         <v>73</v>
       </c>
-      <c r="G7" s="45" t="s">
-        <v>76</v>
-      </c>
-      <c r="H7" s="44" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="B8" s="46" t="s">
-        <v>90</v>
-      </c>
-      <c r="D8" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="E8" s="46" t="s">
-        <v>90</v>
-      </c>
-      <c r="G8" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="H8" s="46" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="9" ht="27.75" customHeight="1">
-      <c r="A9" s="48" t="s">
-        <v>102</v>
-      </c>
-      <c r="B9" s="47" t="s">
-        <v>120</v>
-      </c>
-      <c r="D9" s="47" t="s">
-        <v>123</v>
-      </c>
-      <c r="E9" s="50" t="s">
-        <v>127</v>
-      </c>
-      <c r="G9" s="47" t="s">
-        <v>133</v>
-      </c>
-      <c r="H9" s="47" t="s">
-        <v>134</v>
+      <c r="E9" s="47" t="s">
+        <v>74</v>
+      </c>
+      <c r="G9" s="46" t="s">
+        <v>78</v>
+      </c>
+      <c r="H9" s="46" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="10" ht="18.0" customHeight="1">
       <c r="A10" s="49" t="s">
-        <v>139</v>
-      </c>
-      <c r="B10" s="18"/>
+        <v>83</v>
+      </c>
+      <c r="B10" s="16"/>
       <c r="D10" s="49" t="s">
-        <v>146</v>
-      </c>
-      <c r="E10" s="18"/>
+        <v>88</v>
+      </c>
+      <c r="E10" s="16"/>
       <c r="G10" s="49" t="s">
+        <v>92</v>
+      </c>
+      <c r="H10" s="16"/>
+    </row>
+    <row r="14" ht="21.75" customHeight="1">
+      <c r="A14" s="51" t="s">
+        <v>99</v>
+      </c>
+      <c r="B14" s="16"/>
+      <c r="D14" s="52" t="s">
+        <v>106</v>
+      </c>
+      <c r="E14" s="16"/>
+      <c r="G14" s="53" t="s">
+        <v>116</v>
+      </c>
+      <c r="H14" s="16"/>
+    </row>
+    <row r="15" ht="18.0" customHeight="1">
+      <c r="A15" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="16"/>
+      <c r="D15" s="20" t="s">
+        <v>129</v>
+      </c>
+      <c r="E15" s="16"/>
+      <c r="G15" s="20" t="s">
+        <v>132</v>
+      </c>
+      <c r="H15" s="16"/>
+    </row>
+    <row r="16" ht="19.5" customHeight="1">
+      <c r="A16" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="E16" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="G16" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="H16" s="30" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" ht="42.0" customHeight="1">
+      <c r="A17" s="37" t="s">
+        <v>143</v>
+      </c>
+      <c r="B17" s="36" t="s">
+        <v>145</v>
+      </c>
+      <c r="D17" s="37" t="s">
+        <v>147</v>
+      </c>
+      <c r="E17" s="36" t="s">
+        <v>149</v>
+      </c>
+      <c r="G17" s="37" t="s">
         <v>152</v>
       </c>
-      <c r="H10" s="18"/>
-    </row>
-    <row r="14" ht="21.75" customHeight="1">
-      <c r="A14" s="52" t="s">
+      <c r="H17" s="36" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="18" ht="15.0" customHeight="1">
+      <c r="A18" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="B18" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="D18" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="E18" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="G18" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="H18" s="39" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="19" ht="27.75" customHeight="1">
+      <c r="A19" s="46" t="s">
+        <v>159</v>
+      </c>
+      <c r="B19" s="46" t="s">
+        <v>160</v>
+      </c>
+      <c r="D19" s="46" t="s">
+        <v>161</v>
+      </c>
+      <c r="E19" s="46" t="s">
         <v>163</v>
       </c>
-      <c r="B14" s="18"/>
-      <c r="D14" s="54" t="s">
-        <v>175</v>
-      </c>
-      <c r="E14" s="18"/>
-      <c r="G14" s="55" t="s">
-        <v>184</v>
-      </c>
-      <c r="H14" s="18"/>
-    </row>
-    <row r="15" ht="18.0" customHeight="1">
-      <c r="A15" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="B15" s="18"/>
-      <c r="D15" s="24" t="s">
-        <v>200</v>
-      </c>
-      <c r="E15" s="18"/>
-      <c r="G15" s="24" t="s">
-        <v>204</v>
-      </c>
-      <c r="H15" s="18"/>
-    </row>
-    <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="B16" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="D16" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="E16" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="G16" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="H16" s="38" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="17" ht="42.0" customHeight="1">
-      <c r="A17" s="45" t="s">
-        <v>213</v>
-      </c>
-      <c r="B17" s="44" t="s">
-        <v>214</v>
-      </c>
-      <c r="D17" s="45" t="s">
-        <v>215</v>
-      </c>
-      <c r="E17" s="44" t="s">
-        <v>216</v>
-      </c>
-      <c r="G17" s="45" t="s">
-        <v>217</v>
-      </c>
-      <c r="H17" s="44" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="18" ht="15.0" customHeight="1">
-      <c r="A18" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="B18" s="46" t="s">
-        <v>90</v>
-      </c>
-      <c r="D18" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="E18" s="46" t="s">
-        <v>90</v>
-      </c>
-      <c r="G18" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="H18" s="46" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="19" ht="27.75" customHeight="1">
-      <c r="A19" s="47" t="s">
-        <v>221</v>
-      </c>
-      <c r="B19" s="47" t="s">
-        <v>222</v>
-      </c>
-      <c r="D19" s="47" t="s">
-        <v>223</v>
-      </c>
-      <c r="E19" s="47" t="s">
-        <v>224</v>
-      </c>
-      <c r="G19" s="47" t="s">
-        <v>225</v>
-      </c>
-      <c r="H19" s="47" t="s">
-        <v>226</v>
+      <c r="G19" s="46" t="s">
+        <v>165</v>
+      </c>
+      <c r="H19" s="46" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="20" ht="18.0" customHeight="1">
       <c r="A20" s="49" t="s">
-        <v>228</v>
-      </c>
-      <c r="B20" s="18"/>
+        <v>170</v>
+      </c>
+      <c r="B20" s="16"/>
       <c r="D20" s="49" t="s">
-        <v>229</v>
-      </c>
-      <c r="E20" s="18"/>
+        <v>173</v>
+      </c>
+      <c r="E20" s="16"/>
       <c r="G20" s="49" t="s">
-        <v>231</v>
-      </c>
-      <c r="H20" s="18"/>
+        <v>179</v>
+      </c>
+      <c r="H20" s="16"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
     <row r="23" ht="15.75" customHeight="1"/>
     <row r="24" ht="21.75" customHeight="1">
-      <c r="A24" s="58" t="s">
+      <c r="A24" s="57" t="s">
+        <v>185</v>
+      </c>
+      <c r="B24" s="16"/>
+      <c r="D24" s="58" t="s">
+        <v>193</v>
+      </c>
+      <c r="E24" s="16"/>
+      <c r="G24" s="59" t="s">
+        <v>199</v>
+      </c>
+      <c r="H24" s="16"/>
+    </row>
+    <row r="25" ht="18.0" customHeight="1">
+      <c r="A25" s="20" t="s">
+        <v>208</v>
+      </c>
+      <c r="B25" s="16"/>
+      <c r="D25" s="20" t="s">
+        <v>212</v>
+      </c>
+      <c r="E25" s="16"/>
+      <c r="G25" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="H25" s="16"/>
+    </row>
+    <row r="26" ht="19.5" customHeight="1">
+      <c r="A26" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B26" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="D26" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="E26" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="G26" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="H26" s="30" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="27" ht="42.0" customHeight="1">
+      <c r="A27" s="37" t="s">
+        <v>224</v>
+      </c>
+      <c r="B27" s="36" t="s">
+        <v>226</v>
+      </c>
+      <c r="D27" s="37" t="s">
+        <v>229</v>
+      </c>
+      <c r="E27" s="36" t="s">
+        <v>231</v>
+      </c>
+      <c r="G27" s="37" t="s">
         <v>233</v>
       </c>
-      <c r="B24" s="18"/>
-      <c r="D24" s="59" t="s">
+      <c r="H27" s="36" t="s">
         <v>235</v>
       </c>
-      <c r="E24" s="18"/>
-      <c r="G24" s="60" t="s">
-        <v>236</v>
-      </c>
-      <c r="H24" s="18"/>
-    </row>
-    <row r="25" ht="18.0" customHeight="1">
-      <c r="A25" s="24" t="s">
-        <v>237</v>
-      </c>
-      <c r="B25" s="18"/>
-      <c r="D25" s="24" t="s">
-        <v>238</v>
-      </c>
-      <c r="E25" s="18"/>
-      <c r="G25" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="H25" s="18"/>
-    </row>
-    <row r="26" ht="19.5" customHeight="1">
-      <c r="A26" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="B26" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="D26" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="E26" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="G26" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="H26" s="38" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="27" ht="42.0" customHeight="1">
-      <c r="A27" s="45" t="s">
-        <v>239</v>
-      </c>
-      <c r="B27" s="44" t="s">
-        <v>240</v>
-      </c>
-      <c r="D27" s="45" t="s">
+    </row>
+    <row r="28" ht="15.0" customHeight="1">
+      <c r="A28" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="B28" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="D28" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="E28" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="G28" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="H28" s="39" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="29" ht="27.75" customHeight="1">
+      <c r="A29" s="46" t="s">
         <v>241</v>
       </c>
-      <c r="E27" s="44" t="s">
+      <c r="B29" s="46" t="s">
         <v>242</v>
       </c>
-      <c r="G27" s="45" t="s">
+      <c r="D29" s="46" t="s">
         <v>243</v>
       </c>
-      <c r="H27" s="44" t="s">
+      <c r="E29" s="46" t="s">
         <v>244</v>
       </c>
-    </row>
-    <row r="28" ht="15.0" customHeight="1">
-      <c r="A28" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="B28" s="46" t="s">
-        <v>90</v>
-      </c>
-      <c r="D28" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="E28" s="46" t="s">
-        <v>90</v>
-      </c>
-      <c r="G28" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="H28" s="46" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="29" ht="27.75" customHeight="1">
-      <c r="A29" s="47" t="s">
+      <c r="G29" s="46" t="s">
         <v>245</v>
       </c>
-      <c r="B29" s="47" t="s">
+      <c r="H29" s="46" t="s">
         <v>246</v>
-      </c>
-      <c r="D29" s="47" t="s">
-        <v>247</v>
-      </c>
-      <c r="E29" s="47" t="s">
-        <v>248</v>
-      </c>
-      <c r="G29" s="47" t="s">
-        <v>249</v>
-      </c>
-      <c r="H29" s="47" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="30" ht="18.0" customHeight="1">
       <c r="A30" s="49" t="s">
-        <v>251</v>
-      </c>
-      <c r="B30" s="18"/>
+        <v>248</v>
+      </c>
+      <c r="B30" s="16"/>
       <c r="D30" s="49" t="s">
-        <v>252</v>
-      </c>
-      <c r="E30" s="18"/>
+        <v>249</v>
+      </c>
+      <c r="E30" s="16"/>
       <c r="G30" s="49" t="s">
-        <v>253</v>
-      </c>
-      <c r="H30" s="18"/>
+        <v>250</v>
+      </c>
+      <c r="H30" s="16"/>
     </row>
     <row r="31" ht="15.75" customHeight="1"/>
     <row r="32" ht="15.75" customHeight="1"/>
     <row r="33" ht="15.75" customHeight="1"/>
     <row r="34" ht="21.75" customHeight="1">
       <c r="A34" s="61" t="s">
-        <v>254</v>
-      </c>
-      <c r="B34" s="18"/>
+        <v>253</v>
+      </c>
+      <c r="B34" s="16"/>
       <c r="D34" s="62" t="s">
         <v>255</v>
       </c>
-      <c r="E34" s="18"/>
+      <c r="E34" s="16"/>
       <c r="G34" s="63" t="s">
         <v>256</v>
       </c>
-      <c r="H34" s="18"/>
+      <c r="H34" s="16"/>
     </row>
     <row r="35" ht="18.0" customHeight="1">
-      <c r="A35" s="24" t="s">
+      <c r="A35" s="20" t="s">
         <v>257</v>
       </c>
-      <c r="B35" s="18"/>
-      <c r="D35" s="24" t="s">
+      <c r="B35" s="16"/>
+      <c r="D35" s="20" t="s">
         <v>258</v>
       </c>
-      <c r="E35" s="18"/>
-      <c r="G35" s="53" t="s">
+      <c r="E35" s="16"/>
+      <c r="G35" s="55" t="s">
         <v>259</v>
       </c>
-      <c r="H35" s="18"/>
+      <c r="H35" s="16"/>
     </row>
     <row r="36" ht="19.5" customHeight="1">
-      <c r="A36" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="B36" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="D36" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="E36" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="G36" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="H36" s="38" t="s">
-        <v>51</v>
+      <c r="A36" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B36" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="D36" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="E36" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="G36" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="H36" s="30" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="37" ht="42.0" customHeight="1">
-      <c r="A37" s="45" t="s">
+      <c r="A37" s="37" t="s">
         <v>260</v>
       </c>
-      <c r="B37" s="44" t="s">
+      <c r="B37" s="36" t="s">
         <v>261</v>
       </c>
-      <c r="D37" s="45" t="s">
+      <c r="D37" s="37" t="s">
         <v>262</v>
       </c>
-      <c r="E37" s="44" t="s">
+      <c r="E37" s="36" t="s">
         <v>263</v>
       </c>
-      <c r="G37" s="45" t="s">
+      <c r="G37" s="37" t="s">
         <v>264</v>
       </c>
-      <c r="H37" s="44" t="s">
+      <c r="H37" s="36" t="s">
         <v>265</v>
       </c>
     </row>
     <row r="38" ht="15.0" customHeight="1">
-      <c r="A38" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="B38" s="46" t="s">
-        <v>90</v>
-      </c>
-      <c r="D38" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="E38" s="46" t="s">
-        <v>90</v>
-      </c>
-      <c r="G38" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="H38" s="46" t="s">
-        <v>90</v>
+      <c r="A38" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="B38" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="D38" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="E38" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="G38" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="H38" s="39" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="39" ht="27.75" customHeight="1">
-      <c r="A39" s="47" t="s">
+      <c r="A39" s="46" t="s">
         <v>266</v>
       </c>
-      <c r="B39" s="47" t="s">
+      <c r="B39" s="46" t="s">
         <v>267</v>
       </c>
-      <c r="D39" s="47" t="s">
+      <c r="D39" s="46" t="s">
         <v>268</v>
       </c>
-      <c r="E39" s="47" t="s">
+      <c r="E39" s="46" t="s">
         <v>269</v>
       </c>
-      <c r="G39" s="47" t="s">
+      <c r="G39" s="46" t="s">
         <v>270</v>
       </c>
-      <c r="H39" s="47" t="s">
-        <v>120</v>
+      <c r="H39" s="46" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="40" ht="18.0" customHeight="1">
       <c r="A40" s="49" t="s">
         <v>271</v>
       </c>
-      <c r="B40" s="18"/>
+      <c r="B40" s="16"/>
       <c r="D40" s="49" t="s">
         <v>272</v>
       </c>
-      <c r="E40" s="18"/>
+      <c r="E40" s="16"/>
       <c r="G40" s="49" t="s">
         <v>273</v>
       </c>
-      <c r="H40" s="18"/>
+      <c r="H40" s="16"/>
     </row>
     <row r="41" ht="15.75" customHeight="1"/>
     <row r="42" ht="15.75" customHeight="1"/>
@@ -3624,107 +3624,107 @@
       <c r="A44" s="64" t="s">
         <v>274</v>
       </c>
-      <c r="B44" s="18"/>
+      <c r="B44" s="16"/>
       <c r="D44" s="65" t="s">
         <v>275</v>
       </c>
-      <c r="E44" s="18"/>
+      <c r="E44" s="16"/>
       <c r="G44" s="66" t="s">
         <v>276</v>
       </c>
-      <c r="H44" s="18"/>
+      <c r="H44" s="16"/>
     </row>
     <row r="45" ht="18.0" customHeight="1">
-      <c r="A45" s="24" t="s">
+      <c r="A45" s="20" t="s">
         <v>277</v>
       </c>
-      <c r="B45" s="18"/>
-      <c r="D45" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="E45" s="18"/>
-      <c r="G45" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="H45" s="18"/>
+      <c r="B45" s="16"/>
+      <c r="D45" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="E45" s="16"/>
+      <c r="G45" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="H45" s="16"/>
     </row>
     <row r="46" ht="19.5" customHeight="1">
-      <c r="A46" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="B46" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="D46" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="E46" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="G46" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="H46" s="38" t="s">
-        <v>51</v>
+      <c r="A46" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B46" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="D46" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="E46" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="G46" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="H46" s="30" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="47" ht="42.0" customHeight="1">
-      <c r="A47" s="45" t="s">
+      <c r="A47" s="37" t="s">
         <v>278</v>
       </c>
-      <c r="B47" s="44" t="s">
+      <c r="B47" s="36" t="s">
         <v>279</v>
       </c>
-      <c r="D47" s="45" t="s">
+      <c r="D47" s="37" t="s">
         <v>280</v>
       </c>
-      <c r="E47" s="44" t="s">
+      <c r="E47" s="36" t="s">
         <v>281</v>
       </c>
-      <c r="G47" s="45" t="s">
+      <c r="G47" s="37" t="s">
         <v>282</v>
       </c>
-      <c r="H47" s="44" t="s">
+      <c r="H47" s="36" t="s">
         <v>283</v>
       </c>
     </row>
     <row r="48" ht="15.0" customHeight="1">
-      <c r="A48" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="B48" s="46" t="s">
-        <v>90</v>
-      </c>
-      <c r="D48" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="E48" s="46" t="s">
-        <v>90</v>
-      </c>
-      <c r="G48" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="H48" s="46" t="s">
-        <v>90</v>
+      <c r="A48" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="B48" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="D48" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="E48" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="G48" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="H48" s="39" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="49" ht="27.75" customHeight="1">
-      <c r="A49" s="47" t="s">
+      <c r="A49" s="46" t="s">
         <v>284</v>
       </c>
-      <c r="B49" s="47" t="s">
+      <c r="B49" s="46" t="s">
         <v>285</v>
       </c>
-      <c r="D49" s="47" t="s">
+      <c r="D49" s="46" t="s">
         <v>286</v>
       </c>
-      <c r="E49" s="47" t="s">
+      <c r="E49" s="46" t="s">
         <v>287</v>
       </c>
-      <c r="G49" s="47" t="s">
+      <c r="G49" s="46" t="s">
         <v>288</v>
       </c>
-      <c r="H49" s="47" t="s">
+      <c r="H49" s="46" t="s">
         <v>289</v>
       </c>
     </row>
@@ -3732,15 +3732,15 @@
       <c r="A50" s="49" t="s">
         <v>290</v>
       </c>
-      <c r="B50" s="18"/>
+      <c r="B50" s="16"/>
       <c r="D50" s="49" t="s">
         <v>291</v>
       </c>
-      <c r="E50" s="18"/>
+      <c r="E50" s="16"/>
       <c r="G50" s="49" t="s">
         <v>292</v>
       </c>
-      <c r="H50" s="18"/>
+      <c r="H50" s="16"/>
     </row>
     <row r="51" ht="15.75" customHeight="1"/>
     <row r="52" ht="15.75" customHeight="1"/>
@@ -3749,107 +3749,107 @@
       <c r="A54" s="67" t="s">
         <v>293</v>
       </c>
-      <c r="B54" s="18"/>
+      <c r="B54" s="16"/>
       <c r="D54" s="68" t="s">
         <v>294</v>
       </c>
-      <c r="E54" s="18"/>
+      <c r="E54" s="16"/>
       <c r="G54" s="69" t="s">
         <v>295</v>
       </c>
-      <c r="H54" s="18"/>
+      <c r="H54" s="16"/>
     </row>
     <row r="55" ht="18.0" customHeight="1">
-      <c r="A55" s="24" t="s">
+      <c r="A55" s="20" t="s">
         <v>296</v>
       </c>
-      <c r="B55" s="18"/>
-      <c r="D55" s="24" t="s">
+      <c r="B55" s="16"/>
+      <c r="D55" s="20" t="s">
         <v>297</v>
       </c>
-      <c r="E55" s="18"/>
-      <c r="G55" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="H55" s="18"/>
+      <c r="E55" s="16"/>
+      <c r="G55" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="H55" s="16"/>
     </row>
     <row r="56" ht="19.5" customHeight="1">
-      <c r="A56" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="B56" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="D56" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="E56" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="G56" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="H56" s="38" t="s">
-        <v>51</v>
+      <c r="A56" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B56" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="D56" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="E56" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="G56" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="H56" s="30" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="57" ht="42.0" customHeight="1">
-      <c r="A57" s="45" t="s">
+      <c r="A57" s="37" t="s">
         <v>298</v>
       </c>
-      <c r="B57" s="44" t="s">
+      <c r="B57" s="36" t="s">
         <v>299</v>
       </c>
-      <c r="D57" s="45" t="s">
-        <v>75</v>
-      </c>
-      <c r="E57" s="44" t="s">
+      <c r="D57" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="E57" s="36" t="s">
         <v>300</v>
       </c>
-      <c r="G57" s="45" t="s">
+      <c r="G57" s="37" t="s">
         <v>301</v>
       </c>
-      <c r="H57" s="44" t="s">
+      <c r="H57" s="36" t="s">
         <v>302</v>
       </c>
     </row>
     <row r="58" ht="15.0" customHeight="1">
-      <c r="A58" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="B58" s="46" t="s">
-        <v>90</v>
-      </c>
-      <c r="D58" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="E58" s="46" t="s">
-        <v>90</v>
-      </c>
-      <c r="G58" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="H58" s="46" t="s">
-        <v>90</v>
+      <c r="A58" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="B58" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="D58" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="E58" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="G58" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="H58" s="39" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="59" ht="27.75" customHeight="1">
-      <c r="A59" s="47" t="s">
+      <c r="A59" s="46" t="s">
         <v>303</v>
       </c>
-      <c r="B59" s="47" t="s">
+      <c r="B59" s="46" t="s">
         <v>304</v>
       </c>
-      <c r="D59" s="47" t="s">
+      <c r="D59" s="46" t="s">
         <v>305</v>
       </c>
-      <c r="E59" s="47" t="s">
+      <c r="E59" s="46" t="s">
         <v>306</v>
       </c>
-      <c r="G59" s="47" t="s">
+      <c r="G59" s="46" t="s">
         <v>307</v>
       </c>
-      <c r="H59" s="47" t="s">
+      <c r="H59" s="46" t="s">
         <v>308</v>
       </c>
     </row>
@@ -3857,15 +3857,15 @@
       <c r="A60" s="49" t="s">
         <v>309</v>
       </c>
-      <c r="B60" s="18"/>
+      <c r="B60" s="16"/>
       <c r="D60" s="49" t="s">
         <v>310</v>
       </c>
-      <c r="E60" s="18"/>
+      <c r="E60" s="16"/>
       <c r="G60" s="49" t="s">
         <v>311</v>
       </c>
-      <c r="H60" s="18"/>
+      <c r="H60" s="16"/>
     </row>
     <row r="61" ht="15.75" customHeight="1"/>
     <row r="62" ht="15.75" customHeight="1"/>
@@ -4892,325 +4892,325 @@
   </cols>
   <sheetData>
     <row r="1" ht="31.5" customHeight="1">
-      <c r="A1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="3"/>
+      <c r="A1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="5"/>
     </row>
     <row r="2" ht="19.5" customHeight="1">
       <c r="A2" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="3"/>
+        <v>5</v>
+      </c>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="5"/>
     </row>
     <row r="4" ht="21.75" customHeight="1">
-      <c r="A4" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="18"/>
-      <c r="D4" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="18"/>
-      <c r="G4" s="16" t="s">
-        <v>19</v>
-      </c>
-      <c r="H4" s="18"/>
+      <c r="A4" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="16"/>
+      <c r="D4" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="16"/>
+      <c r="G4" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="16"/>
     </row>
     <row r="5" ht="18.0" customHeight="1">
-      <c r="A5" s="24" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" s="18"/>
-      <c r="D5" s="24" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" s="18"/>
-      <c r="G5" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="H5" s="18"/>
+      <c r="A5" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="16"/>
+      <c r="D5" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="16"/>
+      <c r="G5" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="H5" s="16"/>
     </row>
     <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="B6" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="D6" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="E6" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="G6" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="H6" s="38" t="s">
-        <v>51</v>
+      <c r="A6" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="H6" s="30" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="7" ht="42.0" customHeight="1">
-      <c r="A7" s="42" t="s">
-        <v>55</v>
-      </c>
-      <c r="B7" s="44" t="s">
+      <c r="A7" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7" s="36" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" s="37" t="s">
+        <v>56</v>
+      </c>
+      <c r="E7" s="36" t="s">
+        <v>58</v>
+      </c>
+      <c r="G7" s="37" t="s">
         <v>60</v>
       </c>
-      <c r="D7" s="45" t="s">
-        <v>67</v>
-      </c>
-      <c r="E7" s="44" t="s">
-        <v>72</v>
-      </c>
-      <c r="G7" s="45" t="s">
+      <c r="H7" s="36" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="8" ht="15.0" customHeight="1">
+      <c r="A8" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="B8" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="D8" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="E8" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="G8" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="H8" s="39" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9" ht="27.75" customHeight="1">
+      <c r="A9" s="46" t="s">
+        <v>68</v>
+      </c>
+      <c r="B9" s="46" t="s">
         <v>75</v>
       </c>
-      <c r="H7" s="44" t="s">
+      <c r="D9" s="46" t="s">
+        <v>76</v>
+      </c>
+      <c r="E9" s="46" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="B8" s="46" t="s">
-        <v>90</v>
-      </c>
-      <c r="D8" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="E8" s="46" t="s">
-        <v>90</v>
-      </c>
-      <c r="G8" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="H8" s="46" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="9" ht="27.75" customHeight="1">
-      <c r="A9" s="47" t="s">
-        <v>96</v>
-      </c>
-      <c r="B9" s="47" t="s">
-        <v>105</v>
-      </c>
-      <c r="D9" s="47" t="s">
-        <v>107</v>
-      </c>
-      <c r="E9" s="47" t="s">
-        <v>109</v>
-      </c>
-      <c r="G9" s="47" t="s">
-        <v>111</v>
-      </c>
-      <c r="H9" s="47" t="s">
-        <v>112</v>
+      <c r="G9" s="46" t="s">
+        <v>80</v>
+      </c>
+      <c r="H9" s="46" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="10" ht="18.0" customHeight="1">
       <c r="A10" s="49" t="s">
-        <v>116</v>
-      </c>
-      <c r="B10" s="18"/>
+        <v>86</v>
+      </c>
+      <c r="B10" s="16"/>
       <c r="D10" s="49" t="s">
-        <v>125</v>
-      </c>
-      <c r="E10" s="18"/>
+        <v>91</v>
+      </c>
+      <c r="E10" s="16"/>
       <c r="G10" s="49" t="s">
-        <v>132</v>
-      </c>
-      <c r="H10" s="18"/>
+        <v>100</v>
+      </c>
+      <c r="H10" s="16"/>
     </row>
     <row r="14" ht="21.75" customHeight="1">
-      <c r="A14" s="16" t="s">
-        <v>142</v>
-      </c>
-      <c r="B14" s="18"/>
-      <c r="D14" s="16" t="s">
-        <v>148</v>
-      </c>
-      <c r="E14" s="18"/>
-      <c r="G14" s="51" t="s">
-        <v>153</v>
-      </c>
-      <c r="H14" s="18"/>
+      <c r="A14" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="B14" s="16"/>
+      <c r="D14" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="E14" s="16"/>
+      <c r="G14" s="54" t="s">
+        <v>124</v>
+      </c>
+      <c r="H14" s="16"/>
     </row>
     <row r="15" ht="18.0" customHeight="1">
-      <c r="A15" s="24" t="s">
-        <v>161</v>
-      </c>
-      <c r="B15" s="18"/>
-      <c r="D15" s="24" t="s">
-        <v>168</v>
-      </c>
-      <c r="E15" s="18"/>
-      <c r="G15" s="53" t="s">
-        <v>173</v>
-      </c>
-      <c r="H15" s="18"/>
+      <c r="A15" s="20" t="s">
+        <v>133</v>
+      </c>
+      <c r="B15" s="16"/>
+      <c r="D15" s="20" t="s">
+        <v>139</v>
+      </c>
+      <c r="E15" s="16"/>
+      <c r="G15" s="55" t="s">
+        <v>150</v>
+      </c>
+      <c r="H15" s="16"/>
     </row>
     <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="B16" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="D16" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="E16" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="G16" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="H16" s="38" t="s">
-        <v>51</v>
+      <c r="A16" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="E16" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="G16" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="H16" s="30" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="17" ht="42.0" customHeight="1">
-      <c r="A17" s="45" t="s">
-        <v>188</v>
-      </c>
-      <c r="B17" s="44" t="s">
-        <v>190</v>
-      </c>
-      <c r="D17" s="45" t="s">
+      <c r="A17" s="37" t="s">
+        <v>172</v>
+      </c>
+      <c r="B17" s="36" t="s">
+        <v>175</v>
+      </c>
+      <c r="D17" s="37" t="s">
+        <v>177</v>
+      </c>
+      <c r="E17" s="56" t="s">
+        <v>183</v>
+      </c>
+      <c r="G17" s="35" t="s">
+        <v>189</v>
+      </c>
+      <c r="H17" s="56" t="s">
         <v>191</v>
       </c>
-      <c r="E17" s="56" t="s">
-        <v>193</v>
-      </c>
-      <c r="G17" s="42" t="s">
-        <v>196</v>
-      </c>
-      <c r="H17" s="56" t="s">
-        <v>198</v>
-      </c>
     </row>
     <row r="18" ht="15.0" customHeight="1">
-      <c r="A18" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="B18" s="46" t="s">
-        <v>90</v>
-      </c>
-      <c r="D18" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="E18" s="46" t="s">
-        <v>90</v>
-      </c>
-      <c r="G18" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="H18" s="46" t="s">
-        <v>90</v>
+      <c r="A18" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="B18" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="D18" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="E18" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="G18" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="H18" s="39" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="19" ht="27.75" customHeight="1">
-      <c r="A19" s="47" t="s">
-        <v>208</v>
-      </c>
-      <c r="B19" s="47" t="s">
-        <v>209</v>
-      </c>
-      <c r="D19" s="47" t="s">
-        <v>210</v>
-      </c>
-      <c r="E19" s="47" t="s">
-        <v>120</v>
-      </c>
-      <c r="G19" s="47" t="s">
-        <v>120</v>
-      </c>
-      <c r="H19" s="47" t="s">
-        <v>120</v>
+      <c r="A19" s="46" t="s">
+        <v>202</v>
+      </c>
+      <c r="B19" s="46" t="s">
+        <v>204</v>
+      </c>
+      <c r="D19" s="46" t="s">
+        <v>205</v>
+      </c>
+      <c r="E19" s="46" t="s">
+        <v>71</v>
+      </c>
+      <c r="G19" s="46" t="s">
+        <v>71</v>
+      </c>
+      <c r="H19" s="46" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="20" ht="18.0" customHeight="1">
       <c r="A20" s="49" t="s">
-        <v>211</v>
-      </c>
-      <c r="B20" s="18"/>
+        <v>213</v>
+      </c>
+      <c r="B20" s="16"/>
       <c r="D20" s="49" t="s">
-        <v>212</v>
-      </c>
-      <c r="E20" s="18"/>
-      <c r="G20" s="57" t="s">
-        <v>218</v>
-      </c>
-      <c r="H20" s="18"/>
+        <v>219</v>
+      </c>
+      <c r="E20" s="16"/>
+      <c r="G20" s="60" t="s">
+        <v>228</v>
+      </c>
+      <c r="H20" s="16"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
     <row r="23" ht="15.75" customHeight="1"/>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="51" t="s">
-        <v>220</v>
-      </c>
-      <c r="B24" s="18"/>
+      <c r="A24" s="54" t="s">
+        <v>240</v>
+      </c>
+      <c r="B24" s="16"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="53" t="s">
-        <v>227</v>
-      </c>
-      <c r="B25" s="18"/>
+      <c r="A25" s="55" t="s">
+        <v>247</v>
+      </c>
+      <c r="B25" s="16"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="B26" s="38" t="s">
-        <v>51</v>
+      <c r="A26" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B26" s="30" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="27" ht="44.25" customHeight="1">
-      <c r="A27" s="42" t="s">
-        <v>230</v>
+      <c r="A27" s="35" t="s">
+        <v>251</v>
       </c>
       <c r="B27" s="56" t="s">
-        <v>232</v>
+        <v>252</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="B28" s="46" t="s">
-        <v>90</v>
+      <c r="A28" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="B28" s="39" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="29" ht="27.75" customHeight="1">
-      <c r="A29" s="47" t="s">
-        <v>120</v>
-      </c>
-      <c r="B29" s="47" t="s">
-        <v>120</v>
+      <c r="A29" s="46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B29" s="46" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="57" t="s">
-        <v>234</v>
-      </c>
-      <c r="B30" s="18"/>
+      <c r="A30" s="60" t="s">
+        <v>254</v>
+      </c>
+      <c r="B30" s="16"/>
     </row>
     <row r="31" ht="15.75" customHeight="1"/>
     <row r="32" ht="15.75" customHeight="1"/>
@@ -6234,438 +6234,438 @@
   </cols>
   <sheetData>
     <row r="1" ht="27.75" customHeight="1">
-      <c r="A1" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="3"/>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="5"/>
     </row>
     <row r="2" ht="18.0" customHeight="1">
-      <c r="A2" s="11"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="3"/>
+      <c r="A2" s="10"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="5"/>
     </row>
     <row r="3">
-      <c r="B3" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>6</v>
+      <c r="B3" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="4" ht="24.0" customHeight="1">
-      <c r="A4" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" s="25" t="s">
-        <v>29</v>
-      </c>
-      <c r="C4" s="25" t="s">
-        <v>35</v>
-      </c>
-      <c r="D4" s="25" t="s">
-        <v>36</v>
-      </c>
-      <c r="E4" s="22" t="s">
-        <v>37</v>
+      <c r="A4" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="18" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="5" ht="21.75" customHeight="1">
-      <c r="A5" s="28" t="s">
-        <v>39</v>
-      </c>
-      <c r="B5" s="30" t="s">
-        <v>41</v>
-      </c>
-      <c r="C5" s="31" t="s">
-        <v>42</v>
-      </c>
-      <c r="D5" s="33" t="s">
-        <v>45</v>
-      </c>
-      <c r="E5" s="36" t="s">
+      <c r="A5" s="27" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" s="32" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5" s="34" t="s">
         <v>48</v>
       </c>
+      <c r="E5" s="38" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="6" ht="21.75" customHeight="1">
-      <c r="A6" s="40" t="s">
-        <v>52</v>
-      </c>
-      <c r="B6" s="41" t="s">
-        <v>54</v>
-      </c>
-      <c r="C6" s="31" t="s">
-        <v>57</v>
-      </c>
-      <c r="D6" s="33" t="s">
-        <v>58</v>
-      </c>
-      <c r="E6" s="43" t="s">
-        <v>59</v>
+      <c r="A6" s="42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B6" s="48" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" s="32" t="s">
+        <v>84</v>
+      </c>
+      <c r="D6" s="34" t="s">
+        <v>87</v>
+      </c>
+      <c r="E6" s="50" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="7" ht="21.75" customHeight="1">
-      <c r="A7" s="28" t="s">
-        <v>64</v>
-      </c>
-      <c r="B7" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="C7" s="31" t="s">
-        <v>66</v>
-      </c>
-      <c r="D7" s="33" t="s">
-        <v>69</v>
-      </c>
-      <c r="E7" s="36" t="s">
-        <v>71</v>
+      <c r="A7" s="27" t="s">
+        <v>93</v>
+      </c>
+      <c r="B7" s="31" t="s">
+        <v>94</v>
+      </c>
+      <c r="C7" s="32" t="s">
+        <v>96</v>
+      </c>
+      <c r="D7" s="34" t="s">
+        <v>97</v>
+      </c>
+      <c r="E7" s="38" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="8" ht="21.75" customHeight="1">
-      <c r="A8" s="40" t="s">
-        <v>74</v>
-      </c>
-      <c r="B8" s="41" t="s">
-        <v>41</v>
-      </c>
-      <c r="C8" s="31" t="s">
-        <v>78</v>
-      </c>
-      <c r="D8" s="33" t="s">
-        <v>81</v>
-      </c>
-      <c r="E8" s="43" t="s">
-        <v>82</v>
+      <c r="A8" s="42" t="s">
+        <v>101</v>
+      </c>
+      <c r="B8" s="48" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="32" t="s">
+        <v>102</v>
+      </c>
+      <c r="D8" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="E8" s="50" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="9" ht="21.75" customHeight="1">
-      <c r="A9" s="28" t="s">
-        <v>84</v>
-      </c>
-      <c r="B9" s="30" t="s">
-        <v>86</v>
-      </c>
-      <c r="C9" s="31" t="s">
-        <v>87</v>
-      </c>
-      <c r="D9" s="33" t="s">
-        <v>88</v>
-      </c>
-      <c r="E9" s="36" t="s">
-        <v>89</v>
+      <c r="A9" s="27" t="s">
+        <v>105</v>
+      </c>
+      <c r="B9" s="31" t="s">
+        <v>107</v>
+      </c>
+      <c r="C9" s="32" t="s">
+        <v>108</v>
+      </c>
+      <c r="D9" s="34" t="s">
+        <v>110</v>
+      </c>
+      <c r="E9" s="38" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="10" ht="21.75" customHeight="1">
-      <c r="A10" s="40" t="s">
-        <v>91</v>
-      </c>
-      <c r="B10" s="41" t="s">
-        <v>92</v>
-      </c>
-      <c r="C10" s="31" t="s">
-        <v>93</v>
-      </c>
-      <c r="D10" s="33" t="s">
-        <v>94</v>
-      </c>
-      <c r="E10" s="43" t="s">
-        <v>95</v>
+      <c r="A10" s="42" t="s">
+        <v>112</v>
+      </c>
+      <c r="B10" s="48" t="s">
+        <v>113</v>
+      </c>
+      <c r="C10" s="32" t="s">
+        <v>114</v>
+      </c>
+      <c r="D10" s="34" t="s">
+        <v>117</v>
+      </c>
+      <c r="E10" s="50" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="11" ht="21.75" customHeight="1">
-      <c r="A11" s="28" t="s">
-        <v>97</v>
-      </c>
-      <c r="B11" s="30" t="s">
-        <v>98</v>
-      </c>
-      <c r="C11" s="31" t="s">
-        <v>99</v>
-      </c>
-      <c r="D11" s="33" t="s">
-        <v>100</v>
-      </c>
-      <c r="E11" s="36" t="s">
+      <c r="A11" s="27" t="s">
+        <v>119</v>
+      </c>
+      <c r="B11" s="31" t="s">
+        <v>120</v>
+      </c>
+      <c r="C11" s="32" t="s">
+        <v>121</v>
+      </c>
+      <c r="D11" s="34" t="s">
+        <v>122</v>
+      </c>
+      <c r="E11" s="38" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="12" ht="21.75" customHeight="1">
+      <c r="A12" s="42" t="s">
+        <v>125</v>
+      </c>
+      <c r="B12" s="48" t="s">
+        <v>126</v>
+      </c>
+      <c r="C12" s="32" t="s">
+        <v>127</v>
+      </c>
+      <c r="D12" s="34" t="s">
+        <v>128</v>
+      </c>
+      <c r="E12" s="50" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="13" ht="21.75" customHeight="1">
+      <c r="A13" s="27" t="s">
+        <v>131</v>
+      </c>
+      <c r="B13" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="32" t="s">
+        <v>134</v>
+      </c>
+      <c r="D13" s="34" t="s">
+        <v>135</v>
+      </c>
+      <c r="E13" s="38" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="14" ht="21.75" customHeight="1">
+      <c r="A14" s="42" t="s">
+        <v>137</v>
+      </c>
+      <c r="B14" s="48" t="s">
+        <v>138</v>
+      </c>
+      <c r="C14" s="32" t="s">
+        <v>140</v>
+      </c>
+      <c r="D14" s="34" t="s">
+        <v>141</v>
+      </c>
+      <c r="E14" s="50" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="15" ht="21.75" customHeight="1">
+      <c r="A15" s="27" t="s">
+        <v>144</v>
+      </c>
+      <c r="B15" s="31" t="s">
+        <v>146</v>
+      </c>
+      <c r="C15" s="32" t="s">
+        <v>148</v>
+      </c>
+      <c r="D15" s="34" t="s">
+        <v>151</v>
+      </c>
+      <c r="E15" s="38" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="16" ht="21.75" customHeight="1">
+      <c r="A16" s="42" t="s">
+        <v>155</v>
+      </c>
+      <c r="B16" s="48" t="s">
+        <v>156</v>
+      </c>
+      <c r="C16" s="32" t="s">
+        <v>157</v>
+      </c>
+      <c r="D16" s="34" t="s">
+        <v>158</v>
+      </c>
+      <c r="E16" s="50" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="12" ht="21.75" customHeight="1">
-      <c r="A12" s="40" t="s">
-        <v>103</v>
-      </c>
-      <c r="B12" s="41" t="s">
-        <v>104</v>
-      </c>
-      <c r="C12" s="31" t="s">
-        <v>106</v>
-      </c>
-      <c r="D12" s="33" t="s">
-        <v>108</v>
-      </c>
-      <c r="E12" s="43" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="13" ht="21.75" customHeight="1">
-      <c r="A13" s="28" t="s">
-        <v>113</v>
-      </c>
-      <c r="B13" s="30" t="s">
-        <v>41</v>
-      </c>
-      <c r="C13" s="31" t="s">
-        <v>114</v>
-      </c>
-      <c r="D13" s="33" t="s">
-        <v>115</v>
-      </c>
-      <c r="E13" s="36" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="14" ht="21.75" customHeight="1">
-      <c r="A14" s="40" t="s">
-        <v>118</v>
-      </c>
-      <c r="B14" s="41" t="s">
-        <v>119</v>
-      </c>
-      <c r="C14" s="31" t="s">
-        <v>121</v>
-      </c>
-      <c r="D14" s="33" t="s">
-        <v>122</v>
-      </c>
-      <c r="E14" s="43" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="15" ht="21.75" customHeight="1">
-      <c r="A15" s="28" t="s">
-        <v>126</v>
-      </c>
-      <c r="B15" s="30" t="s">
-        <v>128</v>
-      </c>
-      <c r="C15" s="31" t="s">
-        <v>129</v>
-      </c>
-      <c r="D15" s="33" t="s">
+    <row r="17" ht="21.75" customHeight="1">
+      <c r="A17" s="27" t="s">
+        <v>162</v>
+      </c>
+      <c r="B17" s="31" t="s">
+        <v>164</v>
+      </c>
+      <c r="C17" s="32" t="s">
+        <v>166</v>
+      </c>
+      <c r="D17" s="34" t="s">
+        <v>168</v>
+      </c>
+      <c r="E17" s="38" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="18" ht="21.75" customHeight="1">
+      <c r="A18" s="42" t="s">
+        <v>171</v>
+      </c>
+      <c r="B18" s="48" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18" s="32" t="s">
+        <v>174</v>
+      </c>
+      <c r="D18" s="34" t="s">
+        <v>176</v>
+      </c>
+      <c r="E18" s="50" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="19" ht="21.75" customHeight="1">
+      <c r="A19" s="27" t="s">
         <v>130</v>
       </c>
-      <c r="E15" s="36" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="16" ht="21.75" customHeight="1">
-      <c r="A16" s="40" t="s">
-        <v>135</v>
-      </c>
-      <c r="B16" s="41" t="s">
-        <v>136</v>
-      </c>
-      <c r="C16" s="31" t="s">
-        <v>137</v>
-      </c>
-      <c r="D16" s="33" t="s">
-        <v>138</v>
-      </c>
-      <c r="E16" s="43" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="17" ht="21.75" customHeight="1">
-      <c r="A17" s="28" t="s">
-        <v>140</v>
-      </c>
-      <c r="B17" s="30" t="s">
-        <v>141</v>
-      </c>
-      <c r="C17" s="31" t="s">
-        <v>143</v>
-      </c>
-      <c r="D17" s="33" t="s">
-        <v>144</v>
-      </c>
-      <c r="E17" s="36" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="18" ht="21.75" customHeight="1">
-      <c r="A18" s="40" t="s">
-        <v>147</v>
-      </c>
-      <c r="B18" s="41" t="s">
-        <v>41</v>
-      </c>
-      <c r="C18" s="31" t="s">
-        <v>149</v>
-      </c>
-      <c r="D18" s="33" t="s">
-        <v>150</v>
-      </c>
-      <c r="E18" s="43" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="19" ht="21.75" customHeight="1">
-      <c r="A19" s="28" t="s">
-        <v>110</v>
-      </c>
-      <c r="B19" s="30" t="s">
-        <v>41</v>
-      </c>
-      <c r="C19" s="31" t="s">
-        <v>154</v>
-      </c>
-      <c r="D19" s="33" t="s">
-        <v>155</v>
-      </c>
-      <c r="E19" s="36" t="s">
-        <v>156</v>
+      <c r="B19" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" s="32" t="s">
+        <v>180</v>
+      </c>
+      <c r="D19" s="34" t="s">
+        <v>181</v>
+      </c>
+      <c r="E19" s="38" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="20" ht="21.75" customHeight="1">
-      <c r="A20" s="40" t="s">
-        <v>157</v>
-      </c>
-      <c r="B20" s="41" t="s">
-        <v>158</v>
-      </c>
-      <c r="C20" s="31" t="s">
-        <v>159</v>
-      </c>
-      <c r="D20" s="33" t="s">
-        <v>160</v>
-      </c>
-      <c r="E20" s="43" t="s">
-        <v>162</v>
+      <c r="A20" s="42" t="s">
+        <v>184</v>
+      </c>
+      <c r="B20" s="48" t="s">
+        <v>186</v>
+      </c>
+      <c r="C20" s="32" t="s">
+        <v>187</v>
+      </c>
+      <c r="D20" s="34" t="s">
+        <v>188</v>
+      </c>
+      <c r="E20" s="50" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="21" ht="21.75" customHeight="1">
-      <c r="A21" s="28" t="s">
-        <v>164</v>
-      </c>
-      <c r="B21" s="30" t="s">
-        <v>165</v>
-      </c>
-      <c r="C21" s="31" t="s">
-        <v>166</v>
-      </c>
-      <c r="D21" s="33" t="s">
-        <v>167</v>
-      </c>
-      <c r="E21" s="36" t="s">
-        <v>169</v>
+      <c r="A21" s="27" t="s">
+        <v>192</v>
+      </c>
+      <c r="B21" s="31" t="s">
+        <v>194</v>
+      </c>
+      <c r="C21" s="32" t="s">
+        <v>195</v>
+      </c>
+      <c r="D21" s="34" t="s">
+        <v>196</v>
+      </c>
+      <c r="E21" s="38" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="22" ht="21.75" customHeight="1">
-      <c r="A22" s="40" t="s">
-        <v>170</v>
-      </c>
-      <c r="B22" s="41" t="s">
-        <v>41</v>
-      </c>
-      <c r="C22" s="31" t="s">
-        <v>171</v>
-      </c>
-      <c r="D22" s="33" t="s">
-        <v>172</v>
-      </c>
-      <c r="E22" s="43" t="s">
-        <v>174</v>
+      <c r="A22" s="42" t="s">
+        <v>198</v>
+      </c>
+      <c r="B22" s="48" t="s">
+        <v>40</v>
+      </c>
+      <c r="C22" s="32" t="s">
+        <v>200</v>
+      </c>
+      <c r="D22" s="34" t="s">
+        <v>201</v>
+      </c>
+      <c r="E22" s="50" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="23" ht="21.75" customHeight="1">
-      <c r="A23" s="28" t="s">
-        <v>176</v>
-      </c>
-      <c r="B23" s="30" t="s">
-        <v>177</v>
-      </c>
-      <c r="C23" s="31" t="s">
-        <v>178</v>
-      </c>
-      <c r="D23" s="33" t="s">
-        <v>179</v>
-      </c>
-      <c r="E23" s="36" t="s">
-        <v>180</v>
+      <c r="A23" s="27" t="s">
+        <v>206</v>
+      </c>
+      <c r="B23" s="31" t="s">
+        <v>207</v>
+      </c>
+      <c r="C23" s="32" t="s">
+        <v>209</v>
+      </c>
+      <c r="D23" s="34" t="s">
+        <v>210</v>
+      </c>
+      <c r="E23" s="38" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="24" ht="21.75" customHeight="1">
-      <c r="A24" s="40" t="s">
-        <v>181</v>
-      </c>
-      <c r="B24" s="41" t="s">
-        <v>182</v>
-      </c>
-      <c r="C24" s="31" t="s">
-        <v>183</v>
-      </c>
-      <c r="D24" s="33" t="s">
-        <v>185</v>
-      </c>
-      <c r="E24" s="43" t="s">
-        <v>186</v>
+      <c r="A24" s="42" t="s">
+        <v>214</v>
+      </c>
+      <c r="B24" s="48" t="s">
+        <v>215</v>
+      </c>
+      <c r="C24" s="32" t="s">
+        <v>216</v>
+      </c>
+      <c r="D24" s="34" t="s">
+        <v>217</v>
+      </c>
+      <c r="E24" s="50" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="25" ht="21.75" customHeight="1">
-      <c r="A25" s="28" t="s">
-        <v>187</v>
-      </c>
-      <c r="B25" s="30" t="s">
-        <v>189</v>
-      </c>
-      <c r="C25" s="31" t="s">
-        <v>166</v>
-      </c>
-      <c r="D25" s="33" t="s">
-        <v>192</v>
-      </c>
-      <c r="E25" s="36" t="s">
-        <v>194</v>
+      <c r="A25" s="27" t="s">
+        <v>220</v>
+      </c>
+      <c r="B25" s="31" t="s">
+        <v>221</v>
+      </c>
+      <c r="C25" s="32" t="s">
+        <v>195</v>
+      </c>
+      <c r="D25" s="34" t="s">
+        <v>222</v>
+      </c>
+      <c r="E25" s="38" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="26" ht="21.75" customHeight="1">
-      <c r="A26" s="40" t="s">
-        <v>195</v>
-      </c>
-      <c r="B26" s="41" t="s">
-        <v>197</v>
-      </c>
-      <c r="C26" s="31" t="s">
-        <v>199</v>
-      </c>
-      <c r="D26" s="33" t="s">
-        <v>201</v>
-      </c>
-      <c r="E26" s="43" t="s">
-        <v>202</v>
+      <c r="A26" s="42" t="s">
+        <v>225</v>
+      </c>
+      <c r="B26" s="48" t="s">
+        <v>227</v>
+      </c>
+      <c r="C26" s="32" t="s">
+        <v>230</v>
+      </c>
+      <c r="D26" s="34" t="s">
+        <v>232</v>
+      </c>
+      <c r="E26" s="50" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="27" ht="21.75" customHeight="1">
-      <c r="A27" s="28" t="s">
-        <v>203</v>
-      </c>
-      <c r="B27" s="30" t="s">
-        <v>205</v>
-      </c>
-      <c r="C27" s="31" t="s">
-        <v>206</v>
-      </c>
-      <c r="D27" s="33" t="s">
-        <v>207</v>
-      </c>
-      <c r="E27" s="36" t="s">
-        <v>103</v>
+      <c r="A27" s="27" t="s">
+        <v>236</v>
+      </c>
+      <c r="B27" s="31" t="s">
+        <v>237</v>
+      </c>
+      <c r="C27" s="32" t="s">
+        <v>238</v>
+      </c>
+      <c r="D27" s="34" t="s">
+        <v>239</v>
+      </c>
+      <c r="E27" s="38" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1"/>

</xml_diff>